<commit_message>
IKD update: GaN CMOS 2026-02-23T23:36Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T230"/>
+  <dimension ref="A1:T234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17766,6 +17766,310 @@
       </c>
       <c r="T230" t="inlineStr"/>
     </row>
+    <row r="231">
+      <c r="A231" t="inlineStr"/>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Interleaved Resonant DC-DC with NPC Inverter and MSVPWM Control for Advanced EV Wireless Charging</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>K, Arulvendhan; P, Srinivasan</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr"/>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae4944</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae4944</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr"/>
+      <c r="O231" t="inlineStr"/>
+      <c r="P231" t="inlineStr"/>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>Interleaved Resonant DC-DC with NPC Inverter and MSVPWM Control for Advanced EV Wireless Charging</t>
+        </is>
+      </c>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="T231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr"/>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Interleaved Resonant DC-DC with NPC Inverter and MSVPWM Control for Advanced EV Wireless Charging</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>K, Arulvendhan; P, Srinivasan</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr"/>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae4944</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae4944</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr"/>
+      <c r="O232" t="inlineStr"/>
+      <c r="P232" t="inlineStr"/>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>Interleaved Resonant DC-DC with NPC Inverter and MSVPWM Control for Advanced EV Wireless Charging</t>
+        </is>
+      </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="T232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr"/>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Multi-channel TRNG based on Scalable Cascaded Full Feedback Ring Oscillator</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Association for Computing Machinery (ACM)</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>ACM Transactions on Design Automation of Electronic Systems</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Yao, Liang; Kang, Peiyang; Xu, Yaohua; Yang, Yun; Liang, Huaguo; Huang, Zhengfeng; Lu, Yingchun</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr"/>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>10.1145/3798101</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3798101</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr"/>
+      <c r="O233" t="inlineStr"/>
+      <c r="P233" t="inlineStr"/>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>Multi-channel TRNG based on Scalable Cascaded Full Feedback Ring Oscillator</t>
+        </is>
+      </c>
+      <c r="R233" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S233" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="T233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr"/>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Interleaved Resonant DC-DC with NPC Inverter and MSVPWM Control for Advanced EV Wireless Charging</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>K, Arulvendhan; P, Srinivasan</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr"/>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae4944</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae4944</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr"/>
+      <c r="O234" t="inlineStr"/>
+      <c r="P234" t="inlineStr"/>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>Interleaved Resonant DC-DC with NPC Inverter and MSVPWM Control for Advanced EV Wireless Charging</t>
+        </is>
+      </c>
+      <c r="R234" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-02-24T23:36Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T234"/>
+  <dimension ref="A1:T237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18070,6 +18070,226 @@
       </c>
       <c r="T234" t="inlineStr"/>
     </row>
+    <row r="235">
+      <c r="A235" t="inlineStr"/>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Advancing Nano sheet Transistor Modeling with Gradient based 
+Boosting Machines</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>mandrumaka, kiran; Gade, Francis Harish Reddy</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr"/>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8923546/v1</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8923546/v1</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N235" t="inlineStr"/>
+      <c r="O235" t="inlineStr"/>
+      <c r="P235" t="inlineStr"/>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>Advancing Nano sheet Transistor Modeling with Gradient based 
+Boosting Machines</t>
+        </is>
+      </c>
+      <c r="R235" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="T235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr"/>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Design and Implementation of an 8-Bit Logical Barrel Shifter Using Cadence Virtuoso and Xcelium in 45 nm CMOS Technology</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr"/>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Rajashekarappa, Abhay Surya</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr"/>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8930915/v1</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8930915/v1</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N236" t="inlineStr"/>
+      <c r="O236" t="inlineStr"/>
+      <c r="P236" t="inlineStr"/>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>Design and Implementation of an 8-Bit Logical Barrel Shifter Using Cadence Virtuoso and Xcelium in 45 nm CMOS Technology</t>
+        </is>
+      </c>
+      <c r="R236" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="T236" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr"/>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Advancing Nano sheet Transistor Modeling with Gradient based 
+Boosting Machines</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>mandrumaka, kiran; Gade, Francis Harish Reddy</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr"/>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8923546/v1</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8923546/v1</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr"/>
+      <c r="O237" t="inlineStr"/>
+      <c r="P237" t="inlineStr"/>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>Advancing Nano sheet Transistor Modeling with Gradient based 
+Boosting Machines</t>
+        </is>
+      </c>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S237" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="T237" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-02-25T23:31Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T237"/>
+  <dimension ref="A1:T245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18290,6 +18290,614 @@
       </c>
       <c r="T237" t="inlineStr"/>
     </row>
+    <row r="238">
+      <c r="A238" t="inlineStr"/>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>High-Speed Monolithic 3D Ternary CMOS Design with Junctionless FETs</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Ahn, Hyunho; Han, Jiwon; Kim, Sihyun; Kim, Janghyun; Kim, Sangwan</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr"/>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae4a45</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae4a45</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr"/>
+      <c r="O238" t="inlineStr"/>
+      <c r="P238" t="inlineStr"/>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>High-Speed Monolithic 3D Ternary CMOS Design with Junctionless FETs</t>
+        </is>
+      </c>
+      <c r="R238" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="T238" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr"/>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Lee, Kang Hee; Yang, Yeonsil; Heo, Junseok; Kim, Jang Hyun</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr"/>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr"/>
+      <c r="O239" t="inlineStr"/>
+      <c r="P239" t="inlineStr"/>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="T239" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr"/>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Lee, Kang Hee; Yang, Yeonsil; Heo, Junseok; Kim, Jang Hyun</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr"/>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr"/>
+      <c r="O240" t="inlineStr"/>
+      <c r="P240" t="inlineStr"/>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="T240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr"/>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Lee, Kang Hee; Yang, Yeonsil; Heo, Junseok; Kim, Jang Hyun</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr"/>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr"/>
+      <c r="O241" t="inlineStr"/>
+      <c r="P241" t="inlineStr"/>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R241" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="T241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr"/>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Lee, Kang Hee; Yang, Yeonsil; Heo, Junseok; Kim, Jang Hyun</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr"/>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr"/>
+      <c r="O242" t="inlineStr"/>
+      <c r="P242" t="inlineStr"/>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S242" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="T242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr"/>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Lee, Kang Hee; Yang, Yeonsil; Heo, Junseok; Kim, Jang Hyun</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr"/>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr"/>
+      <c r="O243" t="inlineStr"/>
+      <c r="P243" t="inlineStr"/>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S243" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="T243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr"/>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Lee, Kang Hee; Yang, Yeonsil; Heo, Junseok; Kim, Jang Hyun</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr"/>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr"/>
+      <c r="O244" t="inlineStr"/>
+      <c r="P244" t="inlineStr"/>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S244" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="T244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr"/>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Lee, Kang Hee; Yang, Yeonsil; Heo, Junseok; Kim, Jang Hyun</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr"/>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-41105-1</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr"/>
+      <c r="O245" t="inlineStr"/>
+      <c r="P245" t="inlineStr"/>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>Optimization of enhancement-mode MIS-GaN HEMT with dual channel for simple process using TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S245" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="T245" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-02-26T23:34Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T245"/>
+  <dimension ref="A1:T264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18898,6 +18898,1458 @@
       </c>
       <c r="T245" t="inlineStr"/>
     </row>
+    <row r="246">
+      <c r="A246" t="inlineStr"/>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr"/>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr"/>
+      <c r="O246" t="inlineStr"/>
+      <c r="P246" t="inlineStr"/>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R246" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S246" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr"/>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr"/>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N247" t="inlineStr"/>
+      <c r="O247" t="inlineStr"/>
+      <c r="P247" t="inlineStr"/>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R247" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S247" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr"/>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr"/>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr"/>
+      <c r="O248" t="inlineStr"/>
+      <c r="P248" t="inlineStr"/>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R248" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr"/>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Microcoating is a further improvement in the aesthetics of monolithic restorations (literature review)</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Media Sphere Publishing House</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Stomatology</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Losev, F.F.; Skugareva, D.K.; Dyakonenko, E.E.</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr"/>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>10.17116/stomat202610501180</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.17116/stomat202610501180</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N249" t="inlineStr"/>
+      <c r="O249" t="inlineStr"/>
+      <c r="P249" t="inlineStr"/>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>Microcoating is a further improvement in the aesthetics of monolithic restorations (literature review)</t>
+        </is>
+      </c>
+      <c r="R249" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S249" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr"/>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr"/>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr"/>
+      <c r="O250" t="inlineStr"/>
+      <c r="P250" t="inlineStr"/>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R250" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T250" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr"/>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr"/>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr"/>
+      <c r="O251" t="inlineStr"/>
+      <c r="P251" t="inlineStr"/>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T251" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr"/>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr"/>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr"/>
+      <c r="O252" t="inlineStr"/>
+      <c r="P252" t="inlineStr"/>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr"/>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr"/>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr"/>
+      <c r="O253" t="inlineStr"/>
+      <c r="P253" t="inlineStr"/>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr"/>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr"/>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr"/>
+      <c r="O254" t="inlineStr"/>
+      <c r="P254" t="inlineStr"/>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr"/>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr"/>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr"/>
+      <c r="O255" t="inlineStr"/>
+      <c r="P255" t="inlineStr"/>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R255" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T255" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr"/>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Characterization of Etching Damage Induced by O
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    /BCl
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    Atomic Layer Etching for Enhancement-Mode GaN-Based HEMTs</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Electron Devices</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Wang, Qiang; Li, Shengwen; Chen, Xueting; Li, Feiyang; Hou, Xuan</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr"/>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>10.1109/ted.2025.3648980</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ted.2025.3648980</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr"/>
+      <c r="O256" t="inlineStr"/>
+      <c r="P256" t="inlineStr"/>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>Characterization of Etching Damage Induced by O
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    /BCl
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    Atomic Layer Etching for Enhancement-Mode GaN-Based HEMTs</t>
+        </is>
+      </c>
+      <c r="R256" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr"/>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr"/>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr"/>
+      <c r="O257" t="inlineStr"/>
+      <c r="P257" t="inlineStr"/>
+      <c r="Q257" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R257" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr"/>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr"/>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr"/>
+      <c r="O258" t="inlineStr"/>
+      <c r="P258" t="inlineStr"/>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R258" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr"/>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr"/>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N259" t="inlineStr"/>
+      <c r="O259" t="inlineStr"/>
+      <c r="P259" t="inlineStr"/>
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R259" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S259" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr"/>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr"/>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N260" t="inlineStr"/>
+      <c r="O260" t="inlineStr"/>
+      <c r="P260" t="inlineStr"/>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R260" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S260" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr"/>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr"/>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N261" t="inlineStr"/>
+      <c r="O261" t="inlineStr"/>
+      <c r="P261" t="inlineStr"/>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R261" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S261" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr"/>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr"/>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N262" t="inlineStr"/>
+      <c r="O262" t="inlineStr"/>
+      <c r="P262" t="inlineStr"/>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R262" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S262" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr"/>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr"/>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N263" t="inlineStr"/>
+      <c r="O263" t="inlineStr"/>
+      <c r="P263" t="inlineStr"/>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S263" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr"/>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Zhang, Xinyao; Gong, Can; Mi, MinHan; Zhou, Yuwei; Meng, Ting; Liu, Tianhao; Hao, Yu; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr"/>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae4ab8</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N264" t="inlineStr"/>
+      <c r="O264" t="inlineStr"/>
+      <c r="P264" t="inlineStr"/>
+      <c r="Q264" t="inlineStr">
+        <is>
+          <t>Linearity enhancement of AlGaN/GaN/graded-Al 0.1-0.25 GaN: Si-doped/GaN double channel HEMT</t>
+        </is>
+      </c>
+      <c r="R264" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S264" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="T264" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-02-27T23:28Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T264"/>
+  <dimension ref="A1:T265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20350,6 +20350,82 @@
       </c>
       <c r="T264" t="inlineStr"/>
     </row>
+    <row r="265">
+      <c r="A265" t="inlineStr"/>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Electrical Properties and Performance Enhancement of AlGaN/GaN/Si HEMTs</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Mosbahi, Hana; Ali, Mohammed Khalil Mohammed; Gassoumi, Malek</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr"/>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>10.3390/mi17030297</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17030297</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N265" t="inlineStr"/>
+      <c r="O265" t="inlineStr"/>
+      <c r="P265" t="inlineStr"/>
+      <c r="Q265" t="inlineStr">
+        <is>
+          <t>Electrical Properties and Performance Enhancement of AlGaN/GaN/Si HEMTs</t>
+        </is>
+      </c>
+      <c r="R265" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S265" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="T265" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-02-28T23:26Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T265"/>
+  <dimension ref="A1:T270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20426,6 +20426,386 @@
       </c>
       <c r="T265" t="inlineStr"/>
     </row>
+    <row r="266">
+      <c r="A266" t="inlineStr"/>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>WHO Traditional Medicine Strategy 2025–2034: A Policy Analysis of Its People-Centered Framework</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Dutta, Abhijit</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr"/>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261426230</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261426230</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N266" t="inlineStr"/>
+      <c r="O266" t="inlineStr"/>
+      <c r="P266" t="inlineStr"/>
+      <c r="Q266" t="inlineStr">
+        <is>
+          <t>WHO Traditional Medicine Strategy 2025–2034: A Policy Analysis of Its People-Centered Framework</t>
+        </is>
+      </c>
+      <c r="R266" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S266" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="T266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr"/>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>WHO Traditional Medicine Strategy 2025–2034: A Policy Analysis of Its People-Centered Framework</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Dutta, Abhijit</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr"/>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261426230</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261426230</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N267" t="inlineStr"/>
+      <c r="O267" t="inlineStr"/>
+      <c r="P267" t="inlineStr"/>
+      <c r="Q267" t="inlineStr">
+        <is>
+          <t>WHO Traditional Medicine Strategy 2025–2034: A Policy Analysis of Its People-Centered Framework</t>
+        </is>
+      </c>
+      <c r="R267" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr"/>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Research on Temperature Monitoring and Control Technology for SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Dean &amp; Francis Press</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Science and Technology of Engineering, Chemistry and Environmental Protection</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Shen, Yichen</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr"/>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>10.61173/mj0y4f37</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.61173/mj0y4f37</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N268" t="inlineStr"/>
+      <c r="O268" t="inlineStr"/>
+      <c r="P268" t="inlineStr"/>
+      <c r="Q268" t="inlineStr">
+        <is>
+          <t>Research on Temperature Monitoring and Control Technology for SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="R268" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="T268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr"/>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Research on Temperature Monitoring and Control Technology for SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Dean &amp; Francis Press</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Science and Technology of Engineering, Chemistry and Environmental Protection</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Shen, Yichen</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr"/>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>10.61173/mj0y4f37</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.61173/mj0y4f37</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N269" t="inlineStr"/>
+      <c r="O269" t="inlineStr"/>
+      <c r="P269" t="inlineStr"/>
+      <c r="Q269" t="inlineStr">
+        <is>
+          <t>Research on Temperature Monitoring and Control Technology for SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="R269" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S269" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="T269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr"/>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Analysis of the Temperature-Dependent Mechanism of MIS-HEMT in Negative Bias Stress Under X-Ray Irradiation</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Electron Devices</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Lin, Cheng-Hsien; Yeh, Chien-Hung; Chen, Po-Hsun; Chang, Ting-Chang; Lee, Ya-Huan; Kuo, Ting-Tzu; Hsu, Jui-Tse; Lin, Jia-Hong; Chen, Yi-Huang; Tsai, Yu-Hsiang</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr"/>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>10.1109/ted.2025.3648979</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ted.2025.3648979</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N270" t="inlineStr"/>
+      <c r="O270" t="inlineStr"/>
+      <c r="P270" t="inlineStr"/>
+      <c r="Q270" t="inlineStr">
+        <is>
+          <t>Analysis of the Temperature-Dependent Mechanism of MIS-HEMT in Negative Bias Stress Under X-Ray Irradiation</t>
+        </is>
+      </c>
+      <c r="R270" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S270" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="T270" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-02T23:30Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T270"/>
+  <dimension ref="A1:T272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20806,6 +20806,158 @@
       </c>
       <c r="T270" t="inlineStr"/>
     </row>
+    <row r="271">
+      <c r="A271" t="inlineStr"/>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>First demonstration of 8-in. N-polar GaN HEMT wafer via wafer bonding and layer transfer</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>APL Materials</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Li, Chengguo; Shen, Andy</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr"/>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>10.1063/5.0297689</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0297689</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N271" t="inlineStr"/>
+      <c r="O271" t="inlineStr"/>
+      <c r="P271" t="inlineStr"/>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>First demonstration of 8-in. N-polar GaN HEMT wafer via wafer bonding and layer transfer</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="T271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr"/>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Investigation of Ti/Al/Ni/Au ohmic contacts for AlScN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Streicher, Isabel; Milazzo, Simone; Straňák, Patrik; Kirste, Lutz; Duarte, Teresa; Di Franco, Salvatore; Votadoro, Valerio; Leone, Stefano; Greco, Giuseppe; Roccaforte, Fabrizio</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr"/>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>10.1063/5.0314958</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0314958</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr"/>
+      <c r="O272" t="inlineStr"/>
+      <c r="P272" t="inlineStr"/>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>Investigation of Ti/Al/Ni/Au ohmic contacts for AlScN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R272" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="T272" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-03T23:31Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T272"/>
+  <dimension ref="A1:T273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20958,6 +20958,82 @@
       </c>
       <c r="T272" t="inlineStr"/>
     </row>
+    <row r="273">
+      <c r="A273" t="inlineStr"/>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>A Monolithic U-Shaped Rotor with Quasi-Zero Stiffness for Piezoelectric Ultrasonic Motors</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Symmetry</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Wu, Jintao; Li, Huafeng</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr"/>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>10.3390/sym18030436</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/sym18030436</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr"/>
+      <c r="O273" t="inlineStr"/>
+      <c r="P273" t="inlineStr"/>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>A Monolithic U-Shaped Rotor with Quasi-Zero Stiffness for Piezoelectric Ultrasonic Motors</t>
+        </is>
+      </c>
+      <c r="R273" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S273" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="T273" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-04T23:34Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T273"/>
+  <dimension ref="A1:T276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21034,6 +21034,234 @@
       </c>
       <c r="T273" t="inlineStr"/>
     </row>
+    <row r="274">
+      <c r="A274" t="inlineStr"/>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>A Monolithic Mechanosensitive 3D-printed Jaw with Piezoresistive Sensing for Grasp Force Estimation</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Mukherjee, Sourajit; Desarda, Kunal; Ambe, Yuichi; Takaki, Takeshi</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr"/>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae4cf6</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae4cf6</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N274" t="inlineStr"/>
+      <c r="O274" t="inlineStr"/>
+      <c r="P274" t="inlineStr"/>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>A Monolithic Mechanosensitive 3D-printed Jaw with Piezoresistive Sensing for Grasp Force Estimation</t>
+        </is>
+      </c>
+      <c r="R274" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr"/>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Data Augmentation via Auxiliary Classifier GAN for Enhanced Modeling of Gallium Nitride HEMT Devices</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Liu, Yifei; Qian, Yihan; Hu, Yefeng; Wu, Ye</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr"/>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15051067</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15051067</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr"/>
+      <c r="O275" t="inlineStr"/>
+      <c r="P275" t="inlineStr"/>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>Data Augmentation via Auxiliary Classifier GAN for Enhanced Modeling of Gallium Nitride HEMT Devices</t>
+        </is>
+      </c>
+      <c r="R275" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S275" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="T275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr"/>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Symbol detection in a MIMO wireless communication system using a FeFET-coupled CMOS ring oscillator array</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Neuromorphic Computing and Engineering</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Jadia, Harsh Kumar; Ghosh, Abhinaba; Ali, Md Hanif; Farid Uddin, Syed; N, Sathish; Mandal, Shirshendu; Raut, Nihal; Mulaosmanovic, Halid; Dünkel, Stefan; Beyer, Sven; Amonkar, Suraj; Ganguly, Udayan</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr"/>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>10.1088/2634-4386/ae4cc5</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2634-4386/ae4cc5</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N276" t="inlineStr"/>
+      <c r="O276" t="inlineStr"/>
+      <c r="P276" t="inlineStr"/>
+      <c r="Q276" t="inlineStr">
+        <is>
+          <t>Symbol detection in a MIMO wireless communication system using a FeFET-coupled CMOS ring oscillator array</t>
+        </is>
+      </c>
+      <c r="R276" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S276" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="T276" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-05T23:53Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T276"/>
+  <dimension ref="A1:T290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21262,6 +21262,1058 @@
       </c>
       <c r="T276" t="inlineStr"/>
     </row>
+    <row r="277">
+      <c r="A277" t="inlineStr"/>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Assessing Small-Signal System Strength Across Modes, Locations and Operating Conditions for Inverter Based Resource Connections</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr"/>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Hadjileonidas, Andreas; Zhu, Yue; Brahma, Debargha; Green, Timothy C.</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr"/>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>10.36227/techrxiv.177274582.25115226/v1</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.36227/techrxiv.177274582.25115226/v1</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N277" t="inlineStr"/>
+      <c r="O277" t="inlineStr"/>
+      <c r="P277" t="inlineStr"/>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>Assessing Small-Signal System Strength Across Modes, Locations and Operating Conditions for Inverter Based Resource Connections</t>
+        </is>
+      </c>
+      <c r="R277" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S277" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr"/>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>CMOS BEOL-compatible monolithic integration of high-temperature functional materials using on-chip microheaters</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>SPIE</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Integrated Optics: Devices, Materials, and Technologies XXX</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Xu, Zhiyun; Dao, Khoi; Chen, Rui; Hu, Juejun</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr"/>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>10.1117/12.3079909</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1117/12.3079909</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N278" t="inlineStr"/>
+      <c r="O278" t="inlineStr"/>
+      <c r="P278" t="inlineStr"/>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>CMOS BEOL-compatible monolithic integration of high-temperature functional materials using on-chip microheaters</t>
+        </is>
+      </c>
+      <c r="R278" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S278" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr"/>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>TCAD analysis on defect-induced degradation of electrical and retention characteristics in 3D DRAM</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Fatima, Bushra; Manhas, Sanjeev; Khan, Imtiyaz Ahmad; Raju, Harsh; Kumar, Arvind</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr"/>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae4dfb</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae4dfb</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N279" t="inlineStr"/>
+      <c r="O279" t="inlineStr"/>
+      <c r="P279" t="inlineStr"/>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>TCAD analysis on defect-induced degradation of electrical and retention characteristics in 3D DRAM</t>
+        </is>
+      </c>
+      <c r="R279" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S279" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr"/>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Adaptive Tuning Framework for MOSFET Gate Drive Parameters Based on PPO</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Wang, Yuhang; Zhu, Zhongbo; Bao, Qidong; Meng, Xiangyu; Sun, Xinglin</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr"/>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15051089</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15051089</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr"/>
+      <c r="O280" t="inlineStr"/>
+      <c r="P280" t="inlineStr"/>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>Adaptive Tuning Framework for MOSFET Gate Drive Parameters Based on PPO</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S280" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr"/>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Machine learning approach for non-destructive characterization of embedded nano-structure in Si MOSFET</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Lyu, Renxiang; Yamaguchi, Hyoto; KASAI, Seiya</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr"/>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae4dfc</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae4dfc</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr"/>
+      <c r="O281" t="inlineStr"/>
+      <c r="P281" t="inlineStr"/>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>Machine learning approach for non-destructive characterization of embedded nano-structure in Si MOSFET</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S281" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr"/>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Adaptive Tuning Framework for MOSFET Gate Drive Parameters Based on PPO</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Wang, Yuhang; Zhu, Zhongbo; Bao, Qidong; Meng, Xiangyu; Sun, Xinglin</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr"/>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15051089</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15051089</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr"/>
+      <c r="O282" t="inlineStr"/>
+      <c r="P282" t="inlineStr"/>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>Adaptive Tuning Framework for MOSFET Gate Drive Parameters Based on PPO</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S282" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr"/>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>TCAD analysis on defect-induced degradation of electrical and retention characteristics in 3D DRAM</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Fatima, Bushra; Manhas, Sanjeev; Khan, Imtiyaz Ahmad; Raju, Harsh; Kumar, Arvind</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr"/>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae4dfb</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae4dfb</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr"/>
+      <c r="O283" t="inlineStr"/>
+      <c r="P283" t="inlineStr"/>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>TCAD analysis on defect-induced degradation of electrical and retention characteristics in 3D DRAM</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S283" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr"/>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Adaptive Tuning Framework for MOSFET Gate Drive Parameters Based on PPO</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Wang, Yuhang; Zhu, Zhongbo; Bao, Qidong; Meng, Xiangyu; Sun, Xinglin</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr"/>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15051089</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15051089</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr"/>
+      <c r="O284" t="inlineStr"/>
+      <c r="P284" t="inlineStr"/>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>Adaptive Tuning Framework for MOSFET Gate Drive Parameters Based on PPO</t>
+        </is>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T284" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr"/>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Machine learning approach for non-destructive characterization of embedded nano-structure in Si MOSFET</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Lyu, Renxiang; Yamaguchi, Hyoto; KASAI, Seiya</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr"/>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae4dfc</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae4dfc</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr"/>
+      <c r="O285" t="inlineStr"/>
+      <c r="P285" t="inlineStr"/>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>Machine learning approach for non-destructive characterization of embedded nano-structure in Si MOSFET</t>
+        </is>
+      </c>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T285" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr"/>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Fabrication of a GaN-on-diamond HEMT device using 30-mm-square mosaic-diamond substrate</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Scripta Materialia</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Shirayanagi, Yusuke; Tomohisa, Shingo; Kasamura, Keiji; Toyoda, Hiroki; Matsumae, Takashi; Kurashima, Yuichi; Takagi, Hideki; Kubota, Akihisa; Takenaga, Takashi</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr"/>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>10.1016/j.scriptamat.2026.117260</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.scriptamat.2026.117260</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr"/>
+      <c r="O286" t="inlineStr"/>
+      <c r="P286" t="inlineStr"/>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>Fabrication of a GaN-on-diamond HEMT device using 30-mm-square mosaic-diamond substrate</t>
+        </is>
+      </c>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr"/>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>The Influence of Technological Parameters of Deposition of Dielectric Layers by the ICP CVD Method on Surface Leakage Currents in AlGaN/GaN HEMT</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Belarusian State University of Informatics and Radioelectronics</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Doklady BGUIR</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Demidovich, S.; Yunik, A.; Kovalchuk, N.; Solovjov, Ja.</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr"/>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>10.35596/1729-7648-2026-24-1-5-12</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35596/1729-7648-2026-24-1-5-12</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr"/>
+      <c r="O287" t="inlineStr"/>
+      <c r="P287" t="inlineStr"/>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>The Influence of Technological Parameters of Deposition of Dielectric Layers by the ICP CVD Method on Surface Leakage Currents in AlGaN/GaN HEMT</t>
+        </is>
+      </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T287" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr"/>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>TCAD analysis on defect-induced degradation of electrical and retention characteristics in 3D DRAM</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Fatima, Bushra; Manhas, Sanjeev; Khan, Imtiyaz Ahmad; Raju, Harsh; Kumar, Arvind</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr"/>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae4dfb</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae4dfb</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr"/>
+      <c r="O288" t="inlineStr"/>
+      <c r="P288" t="inlineStr"/>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>TCAD analysis on defect-induced degradation of electrical and retention characteristics in 3D DRAM</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr"/>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Assessing Small-Signal System Strength Across Modes, Locations and Operating Conditions for Inverter Based Resource Connections</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr"/>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Hadjileonidas, Andreas; Zhu, Yue; Brahma, Debargha; Green, Timothy C.</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr"/>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>10.36227/techrxiv.177274582.25115226/v1</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.36227/techrxiv.177274582.25115226/v1</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr"/>
+      <c r="O289" t="inlineStr"/>
+      <c r="P289" t="inlineStr"/>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>Assessing Small-Signal System Strength Across Modes, Locations and Operating Conditions for Inverter Based Resource Connections</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr"/>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Assessing Small-Signal System Strength Across Modes, Locations and Operating Conditions for Inverter Based Resource Connections</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr"/>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Hadjileonidas, Andreas; Zhu, Yue; Brahma, Debargha; Green, Timothy C.</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr"/>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>10.36227/techrxiv.177274582.25115226/v1</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.36227/techrxiv.177274582.25115226/v1</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr"/>
+      <c r="O290" t="inlineStr"/>
+      <c r="P290" t="inlineStr"/>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>Assessing Small-Signal System Strength Across Modes, Locations and Operating Conditions for Inverter Based Resource Connections</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S290" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="T290" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-06T23:31Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T290"/>
+  <dimension ref="A1:T291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22314,6 +22314,82 @@
       </c>
       <c r="T290" t="inlineStr"/>
     </row>
+    <row r="291">
+      <c r="A291" t="inlineStr"/>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Monolithic Hybrid Metalens Singlet for Broadband Aberration-Corrected LWIR Imaging</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>ACS Photonics</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Chen, Yan; Hou, Mingming; Li, Linhan; He, Yang; Liu, Sitan; Pu, Shiliang; Yi, Fei</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr"/>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>10.1021/acsphotonics.5c02539</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsphotonics.5c02539</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr"/>
+      <c r="O291" t="inlineStr"/>
+      <c r="P291" t="inlineStr"/>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>Monolithic Hybrid Metalens Singlet for Broadband Aberration-Corrected LWIR Imaging</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S291" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="T291" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-08T23:28Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T291"/>
+  <dimension ref="A1:T293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22390,6 +22390,158 @@
       </c>
       <c r="T291" t="inlineStr"/>
     </row>
+    <row r="292">
+      <c r="A292" t="inlineStr"/>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Junction temperature smooth control of SiC MOSFET by switch trajectory adjustment based on quasi-lossless snubber circuit</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Wu, Junke; Wu, Yuntao; Wei, Yunpeng; He, Siliang</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr"/>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107143</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107143</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr"/>
+      <c r="O292" t="inlineStr"/>
+      <c r="P292" t="inlineStr"/>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>Junction temperature smooth control of SiC MOSFET by switch trajectory adjustment based on quasi-lossless snubber circuit</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S292" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="T292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr"/>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Junction temperature smooth control of SiC MOSFET by switch trajectory adjustment based on quasi-lossless snubber circuit</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Wu, Junke; Wu, Yuntao; Wei, Yunpeng; He, Siliang</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr"/>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107143</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107143</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr"/>
+      <c r="O293" t="inlineStr"/>
+      <c r="P293" t="inlineStr"/>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>Junction temperature smooth control of SiC MOSFET by switch trajectory adjustment based on quasi-lossless snubber circuit</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S293" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="T293" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-09T23:31Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T293"/>
+  <dimension ref="A1:T298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22542,6 +22542,366 @@
       </c>
       <c r="T293" t="inlineStr"/>
     </row>
+    <row r="294">
+      <c r="A294" t="inlineStr"/>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr"/>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Wu, Di; Gan, ShengLong</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr"/>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr"/>
+      <c r="O294" t="inlineStr"/>
+      <c r="P294" t="inlineStr"/>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S294" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="T294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr"/>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr"/>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Wu, Di; Gan, ShengLong</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr"/>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr"/>
+      <c r="O295" t="inlineStr"/>
+      <c r="P295" t="inlineStr"/>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S295" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="T295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr"/>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr"/>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Wu, Di; Gan, ShengLong</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr"/>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr"/>
+      <c r="O296" t="inlineStr"/>
+      <c r="P296" t="inlineStr"/>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="R296" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S296" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr"/>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr"/>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Wu, Di; Gan, ShengLong</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr"/>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr"/>
+      <c r="O297" t="inlineStr"/>
+      <c r="P297" t="inlineStr"/>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="R297" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S297" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="T297" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr"/>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr"/>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Wu, Di; Gan, ShengLong</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr"/>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8528895/v1</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr"/>
+      <c r="O298" t="inlineStr"/>
+      <c r="P298" t="inlineStr"/>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>Few-shot Remote Sensing Scene Image Classification Method Based On Cross-Scale Efficient Hybrid Encoder</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S298" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="T298" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-10T23:32Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T298"/>
+  <dimension ref="A1:T299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22902,6 +22902,82 @@
       </c>
       <c r="T298" t="inlineStr"/>
     </row>
+    <row r="299">
+      <c r="A299" t="inlineStr"/>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Enhanced threshold voltage stability in GaN p-FETs via post-dielectric thermal anneal</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Li, Teng; Qi, Hengyuan; Yu, Jingjing; Duan, Jialin; Liu, Sihang; Wang, Maojun; Zhang, Meng; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr"/>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae4f1c</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae4f1c</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr"/>
+      <c r="O299" t="inlineStr"/>
+      <c r="P299" t="inlineStr"/>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>Enhanced threshold voltage stability in GaN p-FETs via post-dielectric thermal anneal</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="T299" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-11T23:30Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T299"/>
+  <dimension ref="A1:T310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22978,6 +22978,842 @@
       </c>
       <c r="T299" t="inlineStr"/>
     </row>
+    <row r="300">
+      <c r="A300" t="inlineStr"/>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Inverter topology with unipolar modulation of single-phase transformerless inverter topologies for grid-connected photovoltaic applications</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>GSC Online Press</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>World Journal of Advanced Engineering Technology and Sciences</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Alam, Md. Aftab</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr"/>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>10.30574/wjaets.2026.18.3.0143</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.30574/wjaets.2026.18.3.0143</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr"/>
+      <c r="O300" t="inlineStr"/>
+      <c r="P300" t="inlineStr"/>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>Inverter topology with unipolar modulation of single-phase transformerless inverter topologies for grid-connected photovoltaic applications</t>
+        </is>
+      </c>
+      <c r="R300" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S300" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr"/>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Inverter topology with unipolar modulation of single-phase transformerless inverter topologies for grid-connected photovoltaic applications</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>GSC Online Press</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>World Journal of Advanced Engineering Technology and Sciences</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Alam, Md. Aftab</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr"/>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>10.30574/wjaets.2026.18.3.0143</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.30574/wjaets.2026.18.3.0143</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N301" t="inlineStr"/>
+      <c r="O301" t="inlineStr"/>
+      <c r="P301" t="inlineStr"/>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>Inverter topology with unipolar modulation of single-phase transformerless inverter topologies for grid-connected photovoltaic applications</t>
+        </is>
+      </c>
+      <c r="R301" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S301" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr"/>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Threshold voltage and channel mobility in counter-doped SiC p-channel MOSFETs with nitrided gate oxides</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Ito, Ryoma; Inoue, Akira; Mikami, Kyota; Kaneko, Mitsuaki; KIMOTO, Tsunenobu</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr"/>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae500c</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae500c</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr"/>
+      <c r="O302" t="inlineStr"/>
+      <c r="P302" t="inlineStr"/>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>Threshold voltage and channel mobility in counter-doped SiC p-channel MOSFETs with nitrided gate oxides</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T302" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr"/>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>A 6–18 GHz High-Efficiency GaN Power Amplifier Using Transistor Stacking and Reactive Matching</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Wang, Cetian; Liao, Xuejie; Gong, Moquan; Xiao, Fei; Guan, He; Zhang, Fan; Zhou, Deyun</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr"/>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>10.3390/mi17030338</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17030338</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N303" t="inlineStr"/>
+      <c r="O303" t="inlineStr"/>
+      <c r="P303" t="inlineStr"/>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>A 6–18 GHz High-Efficiency GaN Power Amplifier Using Transistor Stacking and Reactive Matching</t>
+        </is>
+      </c>
+      <c r="R303" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S303" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr"/>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>A Scalable Asymmetric Triple-Metal Gate-All-Around Nanowire MOSFET Architecture with Hybrid SiGe/Ge/InGaAs Channel</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Ruchitha, V.; Kiran Kumar, E.; Balaji, B.; Cheerla, Sreevardhan; AGARWAL, VIPUL; Sreenivasa Rao, D.; Gowthami, Y; Singh, Lokendra; Jena, Biswajit</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr"/>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae5024</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae5024</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N304" t="inlineStr"/>
+      <c r="O304" t="inlineStr"/>
+      <c r="P304" t="inlineStr"/>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>A Scalable Asymmetric Triple-Metal Gate-All-Around Nanowire MOSFET Architecture with Hybrid SiGe/Ge/InGaAs Channel</t>
+        </is>
+      </c>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S304" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr"/>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>A Scalable Asymmetric Triple-Metal Gate-All-Around Nanowire MOSFET Architecture with Hybrid SiGe/Ge/InGaAs Channel</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Ruchitha, V.; Kiran Kumar, E.; Balaji, B.; Cheerla, Sreevardhan; AGARWAL, VIPUL; Sreenivasa Rao, D.; Gowthami, Y; Singh, Lokendra; Jena, Biswajit</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr"/>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae5024</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae5024</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr"/>
+      <c r="O305" t="inlineStr"/>
+      <c r="P305" t="inlineStr"/>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>A Scalable Asymmetric Triple-Metal Gate-All-Around Nanowire MOSFET Architecture with Hybrid SiGe/Ge/InGaAs Channel</t>
+        </is>
+      </c>
+      <c r="R305" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S305" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr"/>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Inverter topology with unipolar modulation of single-phase transformerless inverter topologies for grid-connected photovoltaic applications</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>GSC Online Press</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>World Journal of Advanced Engineering Technology and Sciences</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Alam, Md. Aftab</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr"/>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>10.30574/wjaets.2026.18.3.0143</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.30574/wjaets.2026.18.3.0143</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N306" t="inlineStr"/>
+      <c r="O306" t="inlineStr"/>
+      <c r="P306" t="inlineStr"/>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>Inverter topology with unipolar modulation of single-phase transformerless inverter topologies for grid-connected photovoltaic applications</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S306" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr"/>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Implementation of hybrid random number generator on FPGA: Combining lorenz chaotic system with carry chain based ring oscillator</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Analog Integrated Circuits and Signal Processing</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Fan, Baoshuo; Zeng, Xiangye; Wang, Jingyi; Luo, Mingming; Li, Xiaoyu; Liu, Jianfei; Lu, Jia; Ma, Jie</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr"/>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>10.1007/s10470-026-02572-8</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10470-026-02572-8</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr"/>
+      <c r="O307" t="inlineStr"/>
+      <c r="P307" t="inlineStr"/>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>Implementation of hybrid random number generator on FPGA: Combining lorenz chaotic system with carry chain based ring oscillator</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S307" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr"/>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Inverter topology with unipolar modulation of single-phase transformerless inverter topologies for grid-connected photovoltaic applications</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>GSC Online Press</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>World Journal of Advanced Engineering Technology and Sciences</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Alam, Md. Aftab</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr"/>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>10.30574/wjaets.2026.18.3.0143</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.30574/wjaets.2026.18.3.0143</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr"/>
+      <c r="O308" t="inlineStr"/>
+      <c r="P308" t="inlineStr"/>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>Inverter topology with unipolar modulation of single-phase transformerless inverter topologies for grid-connected photovoltaic applications</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S308" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr"/>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>A 6–18 GHz High-Efficiency GaN Power Amplifier Using Transistor Stacking and Reactive Matching</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Wang, Cetian; Liao, Xuejie; Gong, Moquan; Xiao, Fei; Guan, He; Zhang, Fan; Zhou, Deyun</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr"/>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>10.3390/mi17030338</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17030338</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr"/>
+      <c r="O309" t="inlineStr"/>
+      <c r="P309" t="inlineStr"/>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>A 6–18 GHz High-Efficiency GaN Power Amplifier Using Transistor Stacking and Reactive Matching</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S309" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr"/>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Threshold voltage and channel mobility in counter-doped SiC p-channel MOSFETs with nitrided gate oxides</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Ito, Ryoma; Inoue, Akira; Mikami, Kyota; Kaneko, Mitsuaki; KIMOTO, Tsunenobu</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr"/>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae500c</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae500c</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr"/>
+      <c r="O310" t="inlineStr"/>
+      <c r="P310" t="inlineStr"/>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>Threshold voltage and channel mobility in counter-doped SiC p-channel MOSFETs with nitrided gate oxides</t>
+        </is>
+      </c>
+      <c r="R310" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S310" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="T310" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-12T23:31Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T310"/>
+  <dimension ref="A1:T311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23814,6 +23814,82 @@
       </c>
       <c r="T310" t="inlineStr"/>
     </row>
+    <row r="311">
+      <c r="A311" t="inlineStr"/>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Atomic Layer Deposition in Transistors and Monolithic 3D Integration</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Advanced Functional Materials</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Liu, Yue; Zou, Taoyu; Xu, Cheng‐Yan; Zhen, Liang; Li, Yang; Noh, Yong‐Young</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr"/>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>10.1002/adfm.74729</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/adfm.74729</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N311" t="inlineStr"/>
+      <c r="O311" t="inlineStr"/>
+      <c r="P311" t="inlineStr"/>
+      <c r="Q311" t="inlineStr">
+        <is>
+          <t>Atomic Layer Deposition in Transistors and Monolithic 3D Integration</t>
+        </is>
+      </c>
+      <c r="R311" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S311" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="T311" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-13T23:33Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T311"/>
+  <dimension ref="A1:T320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23890,6 +23890,678 @@
       </c>
       <c r="T311" t="inlineStr"/>
     </row>
+    <row r="312">
+      <c r="A312" t="inlineStr"/>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>A Wide-Voltage-Range Input High-Power-Density Three-Phase Grid-Frequency Isolated Inverter</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr"/>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Tang, Yong; Tang, Huiying; Wang, Bo</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr"/>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8947226/v1</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8947226/v1</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N312" t="inlineStr"/>
+      <c r="O312" t="inlineStr"/>
+      <c r="P312" t="inlineStr"/>
+      <c r="Q312" t="inlineStr">
+        <is>
+          <t>A Wide-Voltage-Range Input High-Power-Density Three-Phase Grid-Frequency Isolated Inverter</t>
+        </is>
+      </c>
+      <c r="R312" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S312" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="T312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr"/>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>A Wide-Voltage-Range Input High-Power-Density Three-Phase Grid-Frequency Isolated Inverter</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr"/>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Tang, Yong; Tang, Huiying; Wang, Bo</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr"/>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8947226/v1</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8947226/v1</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N313" t="inlineStr"/>
+      <c r="O313" t="inlineStr"/>
+      <c r="P313" t="inlineStr"/>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>A Wide-Voltage-Range Input High-Power-Density Three-Phase Grid-Frequency Isolated Inverter</t>
+        </is>
+      </c>
+      <c r="R313" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S313" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="T313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr"/>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Machine learning-driven optimization of monolithic gold plasmonic sensors: Achieving ultrahigh sensitivity with interpretable linear models</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Public Library of Science (PLoS)</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>PLOS One</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Akter, Sonia; Abdullah, Hasan</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr"/>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>10.1371/journal.pone.0343113</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1371/journal.pone.0343113</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N314" t="inlineStr"/>
+      <c r="O314" t="inlineStr"/>
+      <c r="P314" t="inlineStr"/>
+      <c r="Q314" t="inlineStr">
+        <is>
+          <t>Machine learning-driven optimization of monolithic gold plasmonic sensors: Achieving ultrahigh sensitivity with interpretable linear models</t>
+        </is>
+      </c>
+      <c r="R314" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S314" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="T314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr"/>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Single-Event Burnout Mitigation in Silicon VDMOS Power Devices: An Electro-Thermal TCAD Study</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Rodrigo, Eusebio; Rebollo, José; Jordà, Xavier; Camps, José; Latorre, Llorenç; Vellvehi, Miquel</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr"/>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15061201</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15061201</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N315" t="inlineStr"/>
+      <c r="O315" t="inlineStr"/>
+      <c r="P315" t="inlineStr"/>
+      <c r="Q315" t="inlineStr">
+        <is>
+          <t>Single-Event Burnout Mitigation in Silicon VDMOS Power Devices: An Electro-Thermal TCAD Study</t>
+        </is>
+      </c>
+      <c r="R315" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S315" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="T315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr"/>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Single-Event Burnout Mitigation in Silicon VDMOS Power Devices: An Electro-Thermal TCAD Study</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Rodrigo, Eusebio; Rebollo, José; Jordà, Xavier; Camps, José; Latorre, Llorenç; Vellvehi, Miquel</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr"/>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15061201</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15061201</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N316" t="inlineStr"/>
+      <c r="O316" t="inlineStr"/>
+      <c r="P316" t="inlineStr"/>
+      <c r="Q316" t="inlineStr">
+        <is>
+          <t>Single-Event Burnout Mitigation in Silicon VDMOS Power Devices: An Electro-Thermal TCAD Study</t>
+        </is>
+      </c>
+      <c r="R316" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S316" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="T316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr"/>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Single-Event Burnout Mitigation in Silicon VDMOS Power Devices: An Electro-Thermal TCAD Study</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Rodrigo, Eusebio; Rebollo, José; Jordà, Xavier; Camps, José; Latorre, Llorenç; Vellvehi, Miquel</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr"/>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15061201</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15061201</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N317" t="inlineStr"/>
+      <c r="O317" t="inlineStr"/>
+      <c r="P317" t="inlineStr"/>
+      <c r="Q317" t="inlineStr">
+        <is>
+          <t>Single-Event Burnout Mitigation in Silicon VDMOS Power Devices: An Electro-Thermal TCAD Study</t>
+        </is>
+      </c>
+      <c r="R317" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S317" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="T317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr"/>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>A Wide-Voltage-Range Input High-Power-Density Three-Phase Grid-Frequency Isolated Inverter</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr"/>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Tang, Yong; Tang, Huiying; Wang, Bo</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr"/>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8947226/v1</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8947226/v1</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N318" t="inlineStr"/>
+      <c r="O318" t="inlineStr"/>
+      <c r="P318" t="inlineStr"/>
+      <c r="Q318" t="inlineStr">
+        <is>
+          <t>A Wide-Voltage-Range Input High-Power-Density Three-Phase Grid-Frequency Isolated Inverter</t>
+        </is>
+      </c>
+      <c r="R318" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S318" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="T318" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr"/>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>A Wide-Voltage-Range Input High-Power-Density Three-Phase Grid-Frequency Isolated Inverter</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr"/>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Tang, Yong; Tang, Huiying; Wang, Bo</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr"/>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8947226/v1</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8947226/v1</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N319" t="inlineStr"/>
+      <c r="O319" t="inlineStr"/>
+      <c r="P319" t="inlineStr"/>
+      <c r="Q319" t="inlineStr">
+        <is>
+          <t>A Wide-Voltage-Range Input High-Power-Density Three-Phase Grid-Frequency Isolated Inverter</t>
+        </is>
+      </c>
+      <c r="R319" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S319" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="T319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr"/>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Dual‐Gate Ambipolar MoTe
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    Transistor Enabled Reconfigurable Logic and Memory for Next‐Generation Computing</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Advanced Functional Materials</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Lu, Haoyue; Wang, Yan; Sun, Hao; Liu, Jing</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr"/>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>10.1002/adfm.202525471</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/adfm.202525471</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N320" t="inlineStr"/>
+      <c r="O320" t="inlineStr"/>
+      <c r="P320" t="inlineStr"/>
+      <c r="Q320" t="inlineStr">
+        <is>
+          <t>Dual‐Gate Ambipolar MoTe
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    Transistor Enabled Reconfigurable Logic and Memory for Next‐Generation Computing</t>
+        </is>
+      </c>
+      <c r="R320" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S320" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="T320" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-14T23:31Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T320"/>
+  <dimension ref="A1:T326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24562,6 +24562,454 @@
       </c>
       <c r="T320" t="inlineStr"/>
     </row>
+    <row r="321">
+      <c r="A321" t="inlineStr"/>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>PSD based Multi-Layer Protection for Inverter Interfaced Microgrids</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Roy, Subhamita; Debnath, Anushka; Debnath, Sudipta</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr"/>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae51e9</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae51e9</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N321" t="inlineStr"/>
+      <c r="O321" t="inlineStr"/>
+      <c r="P321" t="inlineStr"/>
+      <c r="Q321" t="inlineStr">
+        <is>
+          <t>PSD based Multi-Layer Protection for Inverter Interfaced Microgrids</t>
+        </is>
+      </c>
+      <c r="R321" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S321" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="T321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr"/>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Beyond Good Practices: Designing Scientific Software for Contribution and Reuse</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Copernicus GmbH</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr"/>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Hutton, Eric; Tucker, Gregory; Piper, Mark; Gan, Tian</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr"/>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>10.5194/egusphere-egu26-16877</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5194/egusphere-egu26-16877</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N322" t="inlineStr"/>
+      <c r="O322" t="inlineStr"/>
+      <c r="P322" t="inlineStr"/>
+      <c r="Q322" t="inlineStr">
+        <is>
+          <t>Beyond Good Practices: Designing Scientific Software for Contribution and Reuse</t>
+        </is>
+      </c>
+      <c r="R322" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S322" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="T322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr"/>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>PSD based Multi-Layer Protection for Inverter Interfaced Microgrids</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Roy, Subhamita; Debnath, Anushka; Debnath, Sudipta</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr"/>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae51e9</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae51e9</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N323" t="inlineStr"/>
+      <c r="O323" t="inlineStr"/>
+      <c r="P323" t="inlineStr"/>
+      <c r="Q323" t="inlineStr">
+        <is>
+          <t>PSD based Multi-Layer Protection for Inverter Interfaced Microgrids</t>
+        </is>
+      </c>
+      <c r="R323" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S323" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="T323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr"/>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>PSD based Multi-Layer Protection for Inverter Interfaced Microgrids</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Roy, Subhamita; Debnath, Anushka; Debnath, Sudipta</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr"/>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae51e9</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae51e9</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N324" t="inlineStr"/>
+      <c r="O324" t="inlineStr"/>
+      <c r="P324" t="inlineStr"/>
+      <c r="Q324" t="inlineStr">
+        <is>
+          <t>PSD based Multi-Layer Protection for Inverter Interfaced Microgrids</t>
+        </is>
+      </c>
+      <c r="R324" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S324" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="T324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr"/>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Ultrathin GaOx Tunneling Contact for 2D Transition-metal Dichalcogenides Transistor</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>International Journal of Extreme Manufacturing</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Li, Yun; Yun, Tinghe; Fang, Wuqing; Cui, Nan; Wei, Bohan; Mu, Haoran; Du, Luojun; Zhang, Song; Zhang, Guangyu; Lin, Shenghuang</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr"/>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>10.1088/2631-7990/ae51d2</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-7990/ae51d2</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N325" t="inlineStr"/>
+      <c r="O325" t="inlineStr"/>
+      <c r="P325" t="inlineStr"/>
+      <c r="Q325" t="inlineStr">
+        <is>
+          <t>Ultrathin GaOx Tunneling Contact for 2D Transition-metal Dichalcogenides Transistor</t>
+        </is>
+      </c>
+      <c r="R325" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S325" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="T325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr"/>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Seasonal and diel variations of electrical resistivity in a beech tree stem using time-lapse electrical resistivity imaging</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Copernicus GmbH</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr"/>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Watlet, Arnaud; Gourdol, Laurent; Schymanski, Stanislaus; Hissler, Christophe; Costantini, Andrea; Tailliez, Cyrille; Iffly, Jean-François; Keim, Richard</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr"/>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>10.5194/egusphere-egu26-20808</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5194/egusphere-egu26-20808</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N326" t="inlineStr"/>
+      <c r="O326" t="inlineStr"/>
+      <c r="P326" t="inlineStr"/>
+      <c r="Q326" t="inlineStr">
+        <is>
+          <t>Seasonal and diel variations of electrical resistivity in a beech tree stem using time-lapse electrical resistivity imaging</t>
+        </is>
+      </c>
+      <c r="R326" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S326" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="T326" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-15T23:33Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T326"/>
+  <dimension ref="A1:T327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25010,6 +25010,82 @@
       </c>
       <c r="T326" t="inlineStr"/>
     </row>
+    <row r="327">
+      <c r="A327" t="inlineStr"/>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Optimized Asymmetric Multilevel Inverter with Smart Control for Efficient Renewable Grid Systems</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Asian Research Association</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>International Research Journal of Multidisciplinary Technovation</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>C, Dinakaran; T, Padmavathi</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr"/>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>10.54392/irjmt2627</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54392/irjmt2627</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N327" t="inlineStr"/>
+      <c r="O327" t="inlineStr"/>
+      <c r="P327" t="inlineStr"/>
+      <c r="Q327" t="inlineStr">
+        <is>
+          <t>Optimized Asymmetric Multilevel Inverter with Smart Control for Efficient Renewable Grid Systems</t>
+        </is>
+      </c>
+      <c r="R327" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S327" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="T327" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-16T23:35Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T327"/>
+  <dimension ref="A1:T333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25086,6 +25086,448 @@
       </c>
       <c r="T327" t="inlineStr"/>
     </row>
+    <row r="328">
+      <c r="A328" t="inlineStr"/>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Hybrid Energy Source Fed Hystersis Current Control Algorithm for Cascaded Multi Level Inverter</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr"/>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Jayaprakasam, Vinothini; Ravindran, Ramkumar; S, Ravi</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr"/>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8861291/v1</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8861291/v1</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N328" t="inlineStr"/>
+      <c r="O328" t="inlineStr"/>
+      <c r="P328" t="inlineStr"/>
+      <c r="Q328" t="inlineStr">
+        <is>
+          <t>Hybrid Energy Source Fed Hystersis Current Control Algorithm for Cascaded Multi Level Inverter</t>
+        </is>
+      </c>
+      <c r="R328" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S328" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="T328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr"/>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Hybrid Energy Source Fed Hystersis Current Control Algorithm for Cascaded Multi Level Inverter</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr"/>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Jayaprakasam, Vinothini; Ravindran, Ramkumar; S, Ravi</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr"/>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8861291/v1</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8861291/v1</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N329" t="inlineStr"/>
+      <c r="O329" t="inlineStr"/>
+      <c r="P329" t="inlineStr"/>
+      <c r="Q329" t="inlineStr">
+        <is>
+          <t>Hybrid Energy Source Fed Hystersis Current Control Algorithm for Cascaded Multi Level Inverter</t>
+        </is>
+      </c>
+      <c r="R329" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S329" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="T329" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr"/>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>SiC hybrid channel MOSFET with low ON-resistance and low OFF-state oxide field</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Journal of Power Electronics</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>He, Yawei; Sang, Ling; He, Feng; Niu, Xiping; Li, Xinyu; Dong, Shaohua; Hao, Xiamin; Li, Zheyang; Jin, Rui</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr"/>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>10.1007/s43236-025-01247-3</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s43236-025-01247-3</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N330" t="inlineStr"/>
+      <c r="O330" t="inlineStr"/>
+      <c r="P330" t="inlineStr"/>
+      <c r="Q330" t="inlineStr">
+        <is>
+          <t>SiC hybrid channel MOSFET with low ON-resistance and low OFF-state oxide field</t>
+        </is>
+      </c>
+      <c r="R330" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S330" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="T330" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr"/>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>&lt;i&gt;In situ&lt;/i&gt;
+                    XRD study of strain evolution in AlGaN/GaN HEMT at high temperatures up to 1000 °C</t>
+        </is>
+      </c>
+      <c r="C331" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Li, Botong; Duersch, Bobby G.; Ellis, Hunter; Rahaman, Imteaz; Belanger, Aidan; Aksamija, Zlatan; Van Devener, Brian Roy; Anderson, Kathy; Fu, Kai</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr"/>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>10.1063/5.0316124</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0316124</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N331" t="inlineStr"/>
+      <c r="O331" t="inlineStr"/>
+      <c r="P331" t="inlineStr"/>
+      <c r="Q331" t="inlineStr">
+        <is>
+          <t>&lt;i&gt;In situ&lt;/i&gt;
+                    XRD study of strain evolution in AlGaN/GaN HEMT at high temperatures up to 1000 °C</t>
+        </is>
+      </c>
+      <c r="R331" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S331" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="T331" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr"/>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Hybrid Energy Source Fed Hystersis Current Control Algorithm for Cascaded Multi Level Inverter</t>
+        </is>
+      </c>
+      <c r="C332" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr"/>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Jayaprakasam, Vinothini; Ravindran, Ramkumar; S, Ravi</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr"/>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8861291/v1</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8861291/v1</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N332" t="inlineStr"/>
+      <c r="O332" t="inlineStr"/>
+      <c r="P332" t="inlineStr"/>
+      <c r="Q332" t="inlineStr">
+        <is>
+          <t>Hybrid Energy Source Fed Hystersis Current Control Algorithm for Cascaded Multi Level Inverter</t>
+        </is>
+      </c>
+      <c r="R332" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S332" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="T332" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr"/>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Hybrid Energy Source Fed Hystersis Current Control Algorithm for Cascaded Multi Level Inverter</t>
+        </is>
+      </c>
+      <c r="C333" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr"/>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Jayaprakasam, Vinothini; Ravindran, Ramkumar; S, Ravi</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr"/>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-8861291/v1</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-8861291/v1</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N333" t="inlineStr"/>
+      <c r="O333" t="inlineStr"/>
+      <c r="P333" t="inlineStr"/>
+      <c r="Q333" t="inlineStr">
+        <is>
+          <t>Hybrid Energy Source Fed Hystersis Current Control Algorithm for Cascaded Multi Level Inverter</t>
+        </is>
+      </c>
+      <c r="R333" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S333" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="T333" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-17T23:36Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T333"/>
+  <dimension ref="A1:T342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25528,6 +25528,678 @@
       </c>
       <c r="T333" t="inlineStr"/>
     </row>
+    <row r="334">
+      <c r="A334" t="inlineStr"/>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>The Privacy Risks of PV Inverter Telemetry: A Systematic Analysis of Leakage Vectors in Modern DER Ecosystems</t>
+        </is>
+      </c>
+      <c r="C334" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr"/>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Salas, V.</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr"/>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>10.20944/preprints202603.1181.v1</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20944/preprints202603.1181.v1</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N334" t="inlineStr"/>
+      <c r="O334" t="inlineStr"/>
+      <c r="P334" t="inlineStr"/>
+      <c r="Q334" t="inlineStr">
+        <is>
+          <t>The Privacy Risks of PV Inverter Telemetry: A Systematic Analysis of Leakage Vectors in Modern DER Ecosystems</t>
+        </is>
+      </c>
+      <c r="R334" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S334" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="T334" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr"/>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Metal Packaging: From Monolithic Containers to Hybrid Architectures</t>
+        </is>
+      </c>
+      <c r="C335" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Pagnotta, Leonardo</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr"/>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>10.3390/ma19061177</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma19061177</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N335" t="inlineStr"/>
+      <c r="O335" t="inlineStr"/>
+      <c r="P335" t="inlineStr"/>
+      <c r="Q335" t="inlineStr">
+        <is>
+          <t>Metal Packaging: From Monolithic Containers to Hybrid Architectures</t>
+        </is>
+      </c>
+      <c r="R335" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S335" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="T335" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr"/>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Electrothermal catalysis: paradigm shift from monolithic Joule heating to interparticle electrical promotion</t>
+        </is>
+      </c>
+      <c r="C336" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Oxford University Press (OUP)</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>National Science Review</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Mei, Xueyi; Zhang, Yexin; Zhang, Zhaoliang; Zhang, Jian</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr"/>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>10.1093/nsr/nwag167</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1093/nsr/nwag167</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N336" t="inlineStr"/>
+      <c r="O336" t="inlineStr"/>
+      <c r="P336" t="inlineStr"/>
+      <c r="Q336" t="inlineStr">
+        <is>
+          <t>Electrothermal catalysis: paradigm shift from monolithic Joule heating to interparticle electrical promotion</t>
+        </is>
+      </c>
+      <c r="R336" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S336" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="T336" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr"/>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Gate health state assessment of SiC MOSFET based on clustering algorithm and 2D-cloud modeling</t>
+        </is>
+      </c>
+      <c r="C337" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Circuit World</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Tang, Chenhao; Sun, Pengju; Wu, Junke; He, Chun</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr"/>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>10.1108/cw-01-2026-0003</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/cw-01-2026-0003</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N337" t="inlineStr"/>
+      <c r="O337" t="inlineStr"/>
+      <c r="P337" t="inlineStr"/>
+      <c r="Q337" t="inlineStr">
+        <is>
+          <t>Gate health state assessment of SiC MOSFET based on clustering algorithm and 2D-cloud modeling</t>
+        </is>
+      </c>
+      <c r="R337" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S337" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="T337" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr"/>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Impact of Low-Frequency RF Injection on Leakage Behavior in Nanoscale NMOS Devices</t>
+        </is>
+      </c>
+      <c r="C338" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Abedi, Mohammad; Abedi, Zahra; Zarkesh-Ha, Payman; Hemmady, Sameer; Schamiloglu, Edl</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr"/>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15061244</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15061244</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N338" t="inlineStr"/>
+      <c r="O338" t="inlineStr"/>
+      <c r="P338" t="inlineStr"/>
+      <c r="Q338" t="inlineStr">
+        <is>
+          <t>Impact of Low-Frequency RF Injection on Leakage Behavior in Nanoscale NMOS Devices</t>
+        </is>
+      </c>
+      <c r="R338" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S338" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="T338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr"/>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Gate health state assessment of SiC MOSFET based on clustering algorithm and 2D-cloud modeling</t>
+        </is>
+      </c>
+      <c r="C339" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Circuit World</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Tang, Chenhao; Sun, Pengju; Wu, Junke; He, Chun</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr"/>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>10.1108/cw-01-2026-0003</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/cw-01-2026-0003</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N339" t="inlineStr"/>
+      <c r="O339" t="inlineStr"/>
+      <c r="P339" t="inlineStr"/>
+      <c r="Q339" t="inlineStr">
+        <is>
+          <t>Gate health state assessment of SiC MOSFET based on clustering algorithm and 2D-cloud modeling</t>
+        </is>
+      </c>
+      <c r="R339" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S339" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="T339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr"/>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Gate health state assessment of SiC MOSFET based on clustering algorithm and 2D-cloud modeling</t>
+        </is>
+      </c>
+      <c r="C340" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Circuit World</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Tang, Chenhao; Sun, Pengju; Wu, Junke; He, Chun</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr"/>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>10.1108/cw-01-2026-0003</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/cw-01-2026-0003</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N340" t="inlineStr"/>
+      <c r="O340" t="inlineStr"/>
+      <c r="P340" t="inlineStr"/>
+      <c r="Q340" t="inlineStr">
+        <is>
+          <t>Gate health state assessment of SiC MOSFET based on clustering algorithm and 2D-cloud modeling</t>
+        </is>
+      </c>
+      <c r="R340" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S340" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="T340" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr"/>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>The Privacy Risks of PV Inverter Telemetry: A Systematic Analysis of Leakage Vectors in Modern DER Ecosystems</t>
+        </is>
+      </c>
+      <c r="C341" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr"/>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Salas, V.</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr"/>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>10.20944/preprints202603.1181.v1</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20944/preprints202603.1181.v1</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K341" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N341" t="inlineStr"/>
+      <c r="O341" t="inlineStr"/>
+      <c r="P341" t="inlineStr"/>
+      <c r="Q341" t="inlineStr">
+        <is>
+          <t>The Privacy Risks of PV Inverter Telemetry: A Systematic Analysis of Leakage Vectors in Modern DER Ecosystems</t>
+        </is>
+      </c>
+      <c r="R341" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S341" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="T341" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr"/>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>The Privacy Risks of PV Inverter Telemetry: A Systematic Analysis of Leakage Vectors in Modern DER Ecosystems</t>
+        </is>
+      </c>
+      <c r="C342" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr"/>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Salas, V.</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr"/>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>10.20944/preprints202603.1181.v1</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20944/preprints202603.1181.v1</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N342" t="inlineStr"/>
+      <c r="O342" t="inlineStr"/>
+      <c r="P342" t="inlineStr"/>
+      <c r="Q342" t="inlineStr">
+        <is>
+          <t>The Privacy Risks of PV Inverter Telemetry: A Systematic Analysis of Leakage Vectors in Modern DER Ecosystems</t>
+        </is>
+      </c>
+      <c r="R342" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S342" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="T342" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-19T23:33Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T342"/>
+  <dimension ref="A1:T351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26200,6 +26200,694 @@
       </c>
       <c r="T342" t="inlineStr"/>
     </row>
+    <row r="343">
+      <c r="A343" t="inlineStr"/>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="C343" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Chen, Hong-You; Lee, Hsin-Ying; Lee, Hao; Wu, Yuh-Renn; Lee, Ching-Ting</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr"/>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K343" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N343" t="inlineStr"/>
+      <c r="O343" t="inlineStr"/>
+      <c r="P343" t="inlineStr"/>
+      <c r="Q343" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="R343" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S343" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="T343" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr"/>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="C344" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Chen, Hong-You; Lee, Hsin-Ying; Lee, Hao; Wu, Yuh-Renn; Lee, Ching-Ting</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr"/>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K344" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N344" t="inlineStr"/>
+      <c r="O344" t="inlineStr"/>
+      <c r="P344" t="inlineStr"/>
+      <c r="Q344" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="R344" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S344" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="T344" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr"/>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>TCAD-Machine Learning Enabled TID Compact Model Development for Commercial SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="C345" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Association for Computing Machinery (ACM)</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>ACM Transactions on Design Automation of Electronic Systems</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Gao, Xujiao; Ray, Jaideep; Rummel, Brian; Glaser, Caleb; Rhoades, Elaine; Young, Joshua; Musson, Larry; Buchheit, Thomas</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr"/>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>10.1145/3766551</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3766551</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K345" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N345" t="inlineStr"/>
+      <c r="O345" t="inlineStr"/>
+      <c r="P345" t="inlineStr"/>
+      <c r="Q345" t="inlineStr">
+        <is>
+          <t>TCAD-Machine Learning Enabled TID Compact Model Development for Commercial SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="R345" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S345" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="T345" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr"/>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>TCAD-Machine Learning Enabled TID Compact Model Development for Commercial SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="C346" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Association for Computing Machinery (ACM)</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>ACM Transactions on Design Automation of Electronic Systems</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Gao, Xujiao; Ray, Jaideep; Rummel, Brian; Glaser, Caleb; Rhoades, Elaine; Young, Joshua; Musson, Larry; Buchheit, Thomas</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr"/>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>10.1145/3766551</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3766551</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K346" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N346" t="inlineStr"/>
+      <c r="O346" t="inlineStr"/>
+      <c r="P346" t="inlineStr"/>
+      <c r="Q346" t="inlineStr">
+        <is>
+          <t>TCAD-Machine Learning Enabled TID Compact Model Development for Commercial SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="R346" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S346" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="T346" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr"/>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Self-delamination based double-sided MOSFET fabrication on single crystalline ultrathin silicon</t>
+        </is>
+      </c>
+      <c r="C347" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>International Journal of Extreme Manufacturing</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Lee, Sangyeop; Kim, Seungbeom; Kim, Junhyung; Son, ChangHee; Kim, Seok</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr"/>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>10.1088/2631-7990/ae542f</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-7990/ae542f</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K347" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N347" t="inlineStr"/>
+      <c r="O347" t="inlineStr"/>
+      <c r="P347" t="inlineStr"/>
+      <c r="Q347" t="inlineStr">
+        <is>
+          <t>Self-delamination based double-sided MOSFET fabrication on single crystalline ultrathin silicon</t>
+        </is>
+      </c>
+      <c r="R347" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S347" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="T347" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr"/>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="C348" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Chen, Hong-You; Lee, Hsin-Ying; Lee, Hao; Wu, Yuh-Renn; Lee, Ching-Ting</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr"/>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K348" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N348" t="inlineStr"/>
+      <c r="O348" t="inlineStr"/>
+      <c r="P348" t="inlineStr"/>
+      <c r="Q348" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="R348" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S348" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="T348" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr"/>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="C349" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Chen, Hong-You; Lee, Hsin-Ying; Lee, Hao; Wu, Yuh-Renn; Lee, Ching-Ting</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr"/>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K349" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N349" t="inlineStr"/>
+      <c r="O349" t="inlineStr"/>
+      <c r="P349" t="inlineStr"/>
+      <c r="Q349" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="R349" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S349" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="T349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr"/>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Design a dopingless optimized core shell GAA nanotube TFET with INGAAS source and ZrO
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    gate dielectric based on hybrid optimization for leakage current reduction</t>
+        </is>
+      </c>
+      <c r="C350" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Kumar, Pankaj; Raman, Ashish</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr"/>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae5425</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae5425</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K350" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N350" t="inlineStr"/>
+      <c r="O350" t="inlineStr"/>
+      <c r="P350" t="inlineStr"/>
+      <c r="Q350" t="inlineStr">
+        <is>
+          <t>Design a dopingless optimized core shell GAA nanotube TFET with INGAAS source and ZrO
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    gate dielectric based on hybrid optimization for leakage current reduction</t>
+        </is>
+      </c>
+      <c r="R350" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S350" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="T350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr"/>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="C351" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Chen, Hong-You; Lee, Hsin-Ying; Lee, Hao; Wu, Yuh-Renn; Lee, Ching-Ting</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr"/>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma19061209</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N351" t="inlineStr"/>
+      <c r="O351" t="inlineStr"/>
+      <c r="P351" t="inlineStr"/>
+      <c r="Q351" t="inlineStr">
+        <is>
+          <t>Source Field Plate Incorporated Monolithic Inverters Composed of GaN-Based CMOS-HEMTs with Double-2DEG Channels and Fin-Gated Multiple Nanochannels</t>
+        </is>
+      </c>
+      <c r="R351" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S351" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="T351" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-20T23:33Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T351"/>
+  <dimension ref="A1:T352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26888,6 +26888,82 @@
       </c>
       <c r="T351" t="inlineStr"/>
     </row>
+    <row r="352">
+      <c r="A352" t="inlineStr"/>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>The utility of transplanted CMOs: do China’s collective copyright management organizations deliver market benefits?</t>
+        </is>
+      </c>
+      <c r="C352" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Oxford University Press (OUP)</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Journal of Intellectual Property Law &amp;amp; Practice</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Liu, Jie</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr"/>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>10.1093/jiplp/jpag013</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1093/jiplp/jpag013</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N352" t="inlineStr"/>
+      <c r="O352" t="inlineStr"/>
+      <c r="P352" t="inlineStr"/>
+      <c r="Q352" t="inlineStr">
+        <is>
+          <t>The utility of transplanted CMOs: do China’s collective copyright management organizations deliver market benefits?</t>
+        </is>
+      </c>
+      <c r="R352" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S352" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="T352" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-23T23:36Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T352"/>
+  <dimension ref="A1:T354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26964,6 +26964,158 @@
       </c>
       <c r="T352" t="inlineStr"/>
     </row>
+    <row r="353">
+      <c r="A353" t="inlineStr"/>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Impact of Polarization Charges on Threshold Voltage and Band Offset in AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="C353" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Suemitsu, Tetsuya; Imabayashi, Hiroki; Shiojima, Kenji</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr"/>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.202501001</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.202501001</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N353" t="inlineStr"/>
+      <c r="O353" t="inlineStr"/>
+      <c r="P353" t="inlineStr"/>
+      <c r="Q353" t="inlineStr">
+        <is>
+          <t>Impact of Polarization Charges on Threshold Voltage and Band Offset in AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="R353" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S353" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="T353" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr"/>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Impact of Polarization Charges on Threshold Voltage and Band Offset in AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="C354" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Suemitsu, Tetsuya; Imabayashi, Hiroki; Shiojima, Kenji</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr"/>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.202501001</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.202501001</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N354" t="inlineStr"/>
+      <c r="O354" t="inlineStr"/>
+      <c r="P354" t="inlineStr"/>
+      <c r="Q354" t="inlineStr">
+        <is>
+          <t>Impact of Polarization Charges on Threshold Voltage and Band Offset in AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="R354" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S354" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="T354" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-24T23:36Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T354"/>
+  <dimension ref="A1:T361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27116,6 +27116,538 @@
       </c>
       <c r="T354" t="inlineStr"/>
     </row>
+    <row r="355">
+      <c r="A355" t="inlineStr"/>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Phase Locked Loop Based Soft Switching Implementation of Class D Series Resonant Inverter</t>
+        </is>
+      </c>
+      <c r="C355" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Bitlis Eren Universitesi Fen Bilimleri Dergisi</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Bitlis Eren Üniversitesi Fen Bilimleri Dergisi</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Eker, Kadir; Öncü, Selim</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr"/>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>10.17798/bitlisfen.1806088</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.17798/bitlisfen.1806088</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N355" t="inlineStr"/>
+      <c r="O355" t="inlineStr"/>
+      <c r="P355" t="inlineStr"/>
+      <c r="Q355" t="inlineStr">
+        <is>
+          <t>Phase Locked Loop Based Soft Switching Implementation of Class D Series Resonant Inverter</t>
+        </is>
+      </c>
+      <c r="R355" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S355" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="T355" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr"/>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>A Monolithic CMOS-MEMS SoC with 1.8 mm/s and 2 mK Resolution for Flow and Temperature Sensing via a Microcantilever Array</t>
+        </is>
+      </c>
+      <c r="C356" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Microsystems &amp;amp; Nanoengineering</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Wang, Feiyun; Ouyang, Xuan; Hong, Linze; Song, Xiangyu; Xu, Wei</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr"/>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>10.1038/s41378-026-01220-5</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41378-026-01220-5</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K356" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M356" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N356" t="inlineStr"/>
+      <c r="O356" t="inlineStr"/>
+      <c r="P356" t="inlineStr"/>
+      <c r="Q356" t="inlineStr">
+        <is>
+          <t>A Monolithic CMOS-MEMS SoC with 1.8 mm/s and 2 mK Resolution for Flow and Temperature Sensing via a Microcantilever Array</t>
+        </is>
+      </c>
+      <c r="R356" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S356" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="T356" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr"/>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>A Driver Source Based on 120‐GHz GaN Monolithic Integrated Frequency Multiplier</t>
+        </is>
+      </c>
+      <c r="C357" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>International Journal of Circuit Theory and Applications</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Li, Yuhang; Shi, Jun; Zheng, Xiaomeng; Meng, Jin; Zhang, Dehai</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr"/>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>10.1002/cta.70414</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/cta.70414</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K357" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N357" t="inlineStr"/>
+      <c r="O357" t="inlineStr"/>
+      <c r="P357" t="inlineStr"/>
+      <c r="Q357" t="inlineStr">
+        <is>
+          <t>A Driver Source Based on 120‐GHz GaN Monolithic Integrated Frequency Multiplier</t>
+        </is>
+      </c>
+      <c r="R357" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S357" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="T357" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr"/>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Phase Locked Loop Based Soft Switching Implementation of Class D Series Resonant Inverter</t>
+        </is>
+      </c>
+      <c r="C358" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Bitlis Eren Universitesi Fen Bilimleri Dergisi</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Bitlis Eren Üniversitesi Fen Bilimleri Dergisi</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Eker, Kadir; Öncü, Selim</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr"/>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>10.17798/bitlisfen.1806088</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.17798/bitlisfen.1806088</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N358" t="inlineStr"/>
+      <c r="O358" t="inlineStr"/>
+      <c r="P358" t="inlineStr"/>
+      <c r="Q358" t="inlineStr">
+        <is>
+          <t>Phase Locked Loop Based Soft Switching Implementation of Class D Series Resonant Inverter</t>
+        </is>
+      </c>
+      <c r="R358" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S358" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="T358" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr"/>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>A Driver Source Based on 120‐GHz GaN Monolithic Integrated Frequency Multiplier</t>
+        </is>
+      </c>
+      <c r="C359" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>International Journal of Circuit Theory and Applications</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Li, Yuhang; Shi, Jun; Zheng, Xiaomeng; Meng, Jin; Zhang, Dehai</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr"/>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>10.1002/cta.70414</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/cta.70414</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N359" t="inlineStr"/>
+      <c r="O359" t="inlineStr"/>
+      <c r="P359" t="inlineStr"/>
+      <c r="Q359" t="inlineStr">
+        <is>
+          <t>A Driver Source Based on 120‐GHz GaN Monolithic Integrated Frequency Multiplier</t>
+        </is>
+      </c>
+      <c r="R359" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S359" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="T359" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr"/>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Towards a low resistance ohmic contact to p-type Mg doped multilayer hBN</t>
+        </is>
+      </c>
+      <c r="C360" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>2D Materials</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Marye, Shambel Abate; Kumar, Ravi Ranjan; Tumilty, Niall</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr"/>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>10.1088/2053-1583/ae55b4</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2053-1583/ae55b4</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N360" t="inlineStr"/>
+      <c r="O360" t="inlineStr"/>
+      <c r="P360" t="inlineStr"/>
+      <c r="Q360" t="inlineStr">
+        <is>
+          <t>Towards a low resistance ohmic contact to p-type Mg doped multilayer hBN</t>
+        </is>
+      </c>
+      <c r="R360" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S360" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="T360" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr"/>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Towards a low resistance ohmic contact to p-type Mg doped multilayer hBN</t>
+        </is>
+      </c>
+      <c r="C361" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>2D Materials</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Marye, Shambel Abate; Kumar, Ravi Ranjan; Tumilty, Niall</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr"/>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>10.1088/2053-1583/ae55b4</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2053-1583/ae55b4</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N361" t="inlineStr"/>
+      <c r="O361" t="inlineStr"/>
+      <c r="P361" t="inlineStr"/>
+      <c r="Q361" t="inlineStr">
+        <is>
+          <t>Towards a low resistance ohmic contact to p-type Mg doped multilayer hBN</t>
+        </is>
+      </c>
+      <c r="R361" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S361" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="T361" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-25T23:39Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T361"/>
+  <dimension ref="A1:T366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27648,6 +27648,382 @@
       </c>
       <c r="T361" t="inlineStr"/>
     </row>
+    <row r="362">
+      <c r="A362" t="inlineStr"/>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>2.9-kV Enhancement-Mode GaN Monolithic Bidirectional Switch Based on Gate Post-Annealing-Free Oxygen Plasma Treatment</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Qu, Zifeng; Li, Ang; Xu, Yunsong; Zhang, Xiaodong; Yu, Guohao; Long, Chao; Liu, Wen; Wen, Huiqing</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr"/>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3661591</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3661591</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N362" t="inlineStr"/>
+      <c r="O362" t="inlineStr"/>
+      <c r="P362" t="inlineStr"/>
+      <c r="Q362" t="inlineStr">
+        <is>
+          <t>2.9-kV Enhancement-Mode GaN Monolithic Bidirectional Switch Based on Gate Post-Annealing-Free Oxygen Plasma Treatment</t>
+        </is>
+      </c>
+      <c r="R362" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S362" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="T362" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr"/>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Beyond Remediation: An Irreversibility Threshold for Preventive AI Governance</t>
+        </is>
+      </c>
+      <c r="C363" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Center for Open Science</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr"/>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Duseja, Sushil</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr"/>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>10.31235/osf.io/g3rnj_v1</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.31235/osf.io/g3rnj_v1</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K363" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N363" t="inlineStr"/>
+      <c r="O363" t="inlineStr"/>
+      <c r="P363" t="inlineStr"/>
+      <c r="Q363" t="inlineStr">
+        <is>
+          <t>Beyond Remediation: An Irreversibility Threshold for Preventive AI Governance</t>
+        </is>
+      </c>
+      <c r="R363" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S363" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="T363" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr"/>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>2.9-kV Enhancement-Mode GaN Monolithic Bidirectional Switch Based on Gate Post-Annealing-Free Oxygen Plasma Treatment</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Qu, Zifeng; Li, Ang; Xu, Yunsong; Zhang, Xiaodong; Yu, Guohao; Long, Chao; Liu, Wen; Wen, Huiqing</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr"/>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3661591</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3661591</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N364" t="inlineStr"/>
+      <c r="O364" t="inlineStr"/>
+      <c r="P364" t="inlineStr"/>
+      <c r="Q364" t="inlineStr">
+        <is>
+          <t>2.9-kV Enhancement-Mode GaN Monolithic Bidirectional Switch Based on Gate Post-Annealing-Free Oxygen Plasma Treatment</t>
+        </is>
+      </c>
+      <c r="R364" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S364" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="T364" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr"/>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>A Dual-Mode Memristor-Based Oscillator for Energy-Efficient Biomedical Wireless Systems</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Barraj, Imen; Masmoudi, Mohamed</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr"/>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>10.3390/mi17040393</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17040393</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K365" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N365" t="inlineStr"/>
+      <c r="O365" t="inlineStr"/>
+      <c r="P365" t="inlineStr"/>
+      <c r="Q365" t="inlineStr">
+        <is>
+          <t>A Dual-Mode Memristor-Based Oscillator for Energy-Efficient Biomedical Wireless Systems</t>
+        </is>
+      </c>
+      <c r="R365" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S365" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="T365" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr"/>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>2.9-kV Enhancement-Mode GaN Monolithic Bidirectional Switch Based on Gate Post-Annealing-Free Oxygen Plasma Treatment</t>
+        </is>
+      </c>
+      <c r="C366" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Qu, Zifeng; Li, Ang; Xu, Yunsong; Zhang, Xiaodong; Yu, Guohao; Long, Chao; Liu, Wen; Wen, Huiqing</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr"/>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3661591</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3661591</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K366" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N366" t="inlineStr"/>
+      <c r="O366" t="inlineStr"/>
+      <c r="P366" t="inlineStr"/>
+      <c r="Q366" t="inlineStr">
+        <is>
+          <t>2.9-kV Enhancement-Mode GaN Monolithic Bidirectional Switch Based on Gate Post-Annealing-Free Oxygen Plasma Treatment</t>
+        </is>
+      </c>
+      <c r="R366" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S366" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="T366" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-26T23:36Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T366"/>
+  <dimension ref="A1:T368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28024,6 +28024,158 @@
       </c>
       <c r="T366" t="inlineStr"/>
     </row>
+    <row r="367">
+      <c r="A367" t="inlineStr"/>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Comparative Analysis of Sliding-Mode Control Techniques in Five-Level Active Neutral Point Clamped Flying Capacitor Inverter</t>
+        </is>
+      </c>
+      <c r="C367" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Fesli, Ugur</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr"/>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15071383</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15071383</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K367" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N367" t="inlineStr"/>
+      <c r="O367" t="inlineStr"/>
+      <c r="P367" t="inlineStr"/>
+      <c r="Q367" t="inlineStr">
+        <is>
+          <t>Comparative Analysis of Sliding-Mode Control Techniques in Five-Level Active Neutral Point Clamped Flying Capacitor Inverter</t>
+        </is>
+      </c>
+      <c r="R367" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S367" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="T367" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr"/>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Comparative Analysis of Sliding-Mode Control Techniques in Five-Level Active Neutral Point Clamped Flying Capacitor Inverter</t>
+        </is>
+      </c>
+      <c r="C368" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Fesli, Ugur</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr"/>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15071383</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15071383</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K368" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M368" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N368" t="inlineStr"/>
+      <c r="O368" t="inlineStr"/>
+      <c r="P368" t="inlineStr"/>
+      <c r="Q368" t="inlineStr">
+        <is>
+          <t>Comparative Analysis of Sliding-Mode Control Techniques in Five-Level Active Neutral Point Clamped Flying Capacitor Inverter</t>
+        </is>
+      </c>
+      <c r="R368" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S368" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="T368" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-27T23:37Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T368"/>
+  <dimension ref="A1:T371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28176,6 +28176,234 @@
       </c>
       <c r="T368" t="inlineStr"/>
     </row>
+    <row r="369">
+      <c r="A369" t="inlineStr"/>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Design and Comparative Analysis of Hybrid DG‐MOSFET with Conventional CMOS Using Visual TCAD</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Micro and Nano Semiconductor Devices for Digital, Analog and Sensor Design</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Kushagra; Tripathi, Suman Lata; Raj, Balwinder</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr"/>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>10.1002/9781394307340.ch3</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/9781394307340.ch3</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K369" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N369" t="inlineStr"/>
+      <c r="O369" t="inlineStr"/>
+      <c r="P369" t="inlineStr"/>
+      <c r="Q369" t="inlineStr">
+        <is>
+          <t>Design and Comparative Analysis of Hybrid DG‐MOSFET with Conventional CMOS Using Visual TCAD</t>
+        </is>
+      </c>
+      <c r="R369" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S369" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="T369" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr"/>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Design and Comparative Analysis of Hybrid DG‐MOSFET with Conventional CMOS Using Visual TCAD</t>
+        </is>
+      </c>
+      <c r="C370" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Micro and Nano Semiconductor Devices for Digital, Analog and Sensor Design</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Kushagra; Tripathi, Suman Lata; Raj, Balwinder</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr"/>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>10.1002/9781394307340.ch3</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/9781394307340.ch3</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K370" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N370" t="inlineStr"/>
+      <c r="O370" t="inlineStr"/>
+      <c r="P370" t="inlineStr"/>
+      <c r="Q370" t="inlineStr">
+        <is>
+          <t>Design and Comparative Analysis of Hybrid DG‐MOSFET with Conventional CMOS Using Visual TCAD</t>
+        </is>
+      </c>
+      <c r="R370" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S370" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="T370" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr"/>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Design and Comparative Analysis of Hybrid DG‐MOSFET with Conventional CMOS Using Visual TCAD</t>
+        </is>
+      </c>
+      <c r="C371" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Micro and Nano Semiconductor Devices for Digital, Analog and Sensor Design</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Kushagra; Tripathi, Suman Lata; Raj, Balwinder</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr"/>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>10.1002/9781394307340.ch3</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/9781394307340.ch3</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N371" t="inlineStr"/>
+      <c r="O371" t="inlineStr"/>
+      <c r="P371" t="inlineStr"/>
+      <c r="Q371" t="inlineStr">
+        <is>
+          <t>Design and Comparative Analysis of Hybrid DG‐MOSFET with Conventional CMOS Using Visual TCAD</t>
+        </is>
+      </c>
+      <c r="R371" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S371" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="T371" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-28T23:35Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T371"/>
+  <dimension ref="A1:T380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28404,6 +28404,738 @@
       </c>
       <c r="T371" t="inlineStr"/>
     </row>
+    <row r="372">
+      <c r="A372" t="inlineStr"/>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>High‐Density and Scalable Graphene Hall Sensor Arrays Through Monolithic CMOS Integration</t>
+        </is>
+      </c>
+      <c r="C372" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Advanced Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Iyer, Vasant; Shah, Nishal; Johnson, A. T. Charlie; Issadore, David A.; Aflatouni, Firooz</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr"/>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>10.1002/aelm.202500776</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/aelm.202500776</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K372" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N372" t="inlineStr"/>
+      <c r="O372" t="inlineStr"/>
+      <c r="P372" t="inlineStr"/>
+      <c r="Q372" t="inlineStr">
+        <is>
+          <t>High‐Density and Scalable Graphene Hall Sensor Arrays Through Monolithic CMOS Integration</t>
+        </is>
+      </c>
+      <c r="R372" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S372" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="T372" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr"/>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="C373" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Ge, Mei; Zhang, Wenqian; Lu, Meijing; Gao, Yingyuan; Li, Yi; Yu, Chenhui; Chen, Dunjun</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr"/>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N373" t="inlineStr"/>
+      <c r="O373" t="inlineStr"/>
+      <c r="P373" t="inlineStr"/>
+      <c r="Q373" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="R373" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S373" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="T373" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr"/>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="C374" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Ge, Mei; Zhang, Wenqian; Lu, Meijing; Gao, Yingyuan; Li, Yi; Yu, Chenhui; Chen, Dunjun</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr"/>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N374" t="inlineStr"/>
+      <c r="O374" t="inlineStr"/>
+      <c r="P374" t="inlineStr"/>
+      <c r="Q374" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="R374" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S374" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="T374" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr"/>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="C375" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Ge, Mei; Zhang, Wenqian; Lu, Meijing; Gao, Yingyuan; Li, Yi; Yu, Chenhui; Chen, Dunjun</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr"/>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N375" t="inlineStr"/>
+      <c r="O375" t="inlineStr"/>
+      <c r="P375" t="inlineStr"/>
+      <c r="Q375" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="R375" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S375" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="T375" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr"/>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Ge, Mei; Zhang, Wenqian; Lu, Meijing; Gao, Yingyuan; Li, Yi; Yu, Chenhui; Chen, Dunjun</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr"/>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N376" t="inlineStr"/>
+      <c r="O376" t="inlineStr"/>
+      <c r="P376" t="inlineStr"/>
+      <c r="Q376" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="R376" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S376" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="T376" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr"/>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Heteroepitaxial β‐Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    Trench‐Gate MOSFET on 4H‐SiC: Trap, Thermal, and Breakdown Optimization</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Alam, Md Zafar; Khan, Imran Ahmed; Amin, Syed Intekhab; Anam, Aadil</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr"/>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.202500848</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.202500848</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N377" t="inlineStr"/>
+      <c r="O377" t="inlineStr"/>
+      <c r="P377" t="inlineStr"/>
+      <c r="Q377" t="inlineStr">
+        <is>
+          <t>Heteroepitaxial β‐Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    Trench‐Gate MOSFET on 4H‐SiC: Trap, Thermal, and Breakdown Optimization</t>
+        </is>
+      </c>
+      <c r="R377" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S377" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="T377" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr"/>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Transformer Less Grid Feeding Current Source Inverter for Solar Photovoltaic System</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>International Journal for Research in Applied Science and Engineering Technology (IJRASET)</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>International Journal for Research in Applied Science and Engineering Technology</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Venkatesh, Boini</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr"/>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>10.22214/ijraset.2026.78730</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22214/ijraset.2026.78730</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N378" t="inlineStr"/>
+      <c r="O378" t="inlineStr"/>
+      <c r="P378" t="inlineStr"/>
+      <c r="Q378" t="inlineStr">
+        <is>
+          <t>Transformer Less Grid Feeding Current Source Inverter for Solar Photovoltaic System</t>
+        </is>
+      </c>
+      <c r="R378" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S378" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="T378" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr"/>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Three-Transistor Antifuse OTP Memory: Design, Simulation and Behavioral Verification</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Lattice Science Publication (LSP)</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Indian Journal of VLSI Design</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Thakur, Jyoti; Soni, Prof. Bhavesh</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr"/>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>10.54105/ijvlsid.b1235.06010326</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54105/ijvlsid.b1235.06010326</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N379" t="inlineStr"/>
+      <c r="O379" t="inlineStr"/>
+      <c r="P379" t="inlineStr"/>
+      <c r="Q379" t="inlineStr">
+        <is>
+          <t>Three-Transistor Antifuse OTP Memory: Design, Simulation and Behavioral Verification</t>
+        </is>
+      </c>
+      <c r="R379" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S379" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="T379" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr"/>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Ge, Mei; Zhang, Wenqian; Lu, Meijing; Gao, Yingyuan; Li, Yi; Yu, Chenhui; Chen, Dunjun</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr"/>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae585d</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N380" t="inlineStr"/>
+      <c r="O380" t="inlineStr"/>
+      <c r="P380" t="inlineStr"/>
+      <c r="Q380" t="inlineStr">
+        <is>
+          <t>An enhancement-mode GaN based p-channel heterostructure field effect transistor with Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    /AlGaN hybrid barrier layer</t>
+        </is>
+      </c>
+      <c r="R380" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S380" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="T380" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-29T23:37Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T380"/>
+  <dimension ref="A1:T381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29136,6 +29136,82 @@
       </c>
       <c r="T380" t="inlineStr"/>
     </row>
+    <row r="381">
+      <c r="A381" t="inlineStr"/>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Beyond Large Language Models: How Small, Specialized Agents are Replacing Monolithic Systems</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Edtech Publishers (OPC) Private Limited</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>International Journal of Science, Strategic Management and Technology</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Nandi, Pritha; Manna, Subhajit</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr"/>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>10.55041/ijsmt.v2i3.380</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.55041/ijsmt.v2i3.380</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N381" t="inlineStr"/>
+      <c r="O381" t="inlineStr"/>
+      <c r="P381" t="inlineStr"/>
+      <c r="Q381" t="inlineStr">
+        <is>
+          <t>Beyond Large Language Models: How Small, Specialized Agents are Replacing Monolithic Systems</t>
+        </is>
+      </c>
+      <c r="R381" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S381" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="T381" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-30T23:39Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T381"/>
+  <dimension ref="A1:T386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29212,6 +29212,386 @@
       </c>
       <c r="T381" t="inlineStr"/>
     </row>
+    <row r="382">
+      <c r="A382" t="inlineStr"/>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Compact Monolithic Star Tracker System</t>
+        </is>
+      </c>
+      <c r="C382" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Optics</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Zuber, Kamil; Wright, Duncan; Choi, Jebum; Sytsma, Joni; Hall, Colin</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr"/>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>10.3390/opt7020025</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/opt7020025</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N382" t="inlineStr"/>
+      <c r="O382" t="inlineStr"/>
+      <c r="P382" t="inlineStr"/>
+      <c r="Q382" t="inlineStr">
+        <is>
+          <t>Compact Monolithic Star Tracker System</t>
+        </is>
+      </c>
+      <c r="R382" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S382" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="T382" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr"/>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Cryogenic Temperature Electrical Characterization of Enhancement-Mode Thin Barrier AlGaN/GaN HEMT With Hybrid Ferroelectric Charge Trap Gate-Stack</t>
+        </is>
+      </c>
+      <c r="C383" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Electron Devices</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Rai, Rahul; Nguyen, Khanh Quoc; Ho, Viet Quoc; Tran, Hung Duy; Mazhari, Baquer; Chang, Edward Yi</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr"/>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>10.1109/ted.2026.3663344</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ted.2026.3663344</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N383" t="inlineStr"/>
+      <c r="O383" t="inlineStr"/>
+      <c r="P383" t="inlineStr"/>
+      <c r="Q383" t="inlineStr">
+        <is>
+          <t>Cryogenic Temperature Electrical Characterization of Enhancement-Mode Thin Barrier AlGaN/GaN HEMT With Hybrid Ferroelectric Charge Trap Gate-Stack</t>
+        </is>
+      </c>
+      <c r="R383" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S383" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="T383" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr"/>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Electro-Thermal Reliability Analysis and Performance Evaluation of a 1.2-kV Cascode GaN HEMT for High-Power-Density Applications</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Nanotechnology</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Chong, Chen; Liu, Hongxia; Wang, Shulong; Chen, Shupeng</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr"/>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6528/ae5880</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6528/ae5880</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N384" t="inlineStr"/>
+      <c r="O384" t="inlineStr"/>
+      <c r="P384" t="inlineStr"/>
+      <c r="Q384" t="inlineStr">
+        <is>
+          <t>Electro-Thermal Reliability Analysis and Performance Evaluation of a 1.2-kV Cascode GaN HEMT for High-Power-Density Applications</t>
+        </is>
+      </c>
+      <c r="R384" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S384" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="T384" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr"/>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Cryogenic Temperature Electrical Characterization of Enhancement-Mode Thin Barrier AlGaN/GaN HEMT With Hybrid Ferroelectric Charge Trap Gate-Stack</t>
+        </is>
+      </c>
+      <c r="C385" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Electron Devices</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Rai, Rahul; Nguyen, Khanh Quoc; Ho, Viet Quoc; Tran, Hung Duy; Mazhari, Baquer; Chang, Edward Yi</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr"/>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>10.1109/ted.2026.3663344</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ted.2026.3663344</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N385" t="inlineStr"/>
+      <c r="O385" t="inlineStr"/>
+      <c r="P385" t="inlineStr"/>
+      <c r="Q385" t="inlineStr">
+        <is>
+          <t>Cryogenic Temperature Electrical Characterization of Enhancement-Mode Thin Barrier AlGaN/GaN HEMT With Hybrid Ferroelectric Charge Trap Gate-Stack</t>
+        </is>
+      </c>
+      <c r="R385" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S385" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="T385" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr"/>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Gate Oxide Degradation and Interface-Trap Mechanisms in Planar SiC MOSFETs Under Dynamic Gate Stress</t>
+        </is>
+      </c>
+      <c r="C386" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Electron Devices</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Cao, Jiaying; Tang, Jiuyang; Kong, Liudan; Duan, Yuhan; Chang, Yifei; Zhang, Qingchun Jon; Liu, Pan</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr"/>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>10.1109/ted.2026.3665857</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ted.2026.3665857</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N386" t="inlineStr"/>
+      <c r="O386" t="inlineStr"/>
+      <c r="P386" t="inlineStr"/>
+      <c r="Q386" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Gate Oxide Degradation and Interface-Trap Mechanisms in Planar SiC MOSFETs Under Dynamic Gate Stress</t>
+        </is>
+      </c>
+      <c r="R386" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S386" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="T386" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-03-31T23:38Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T386"/>
+  <dimension ref="A1:T395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29592,6 +29592,690 @@
       </c>
       <c r="T386" t="inlineStr"/>
     </row>
+    <row r="387">
+      <c r="A387" t="inlineStr"/>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Monolithic excitable photonic neuron</t>
+        </is>
+      </c>
+      <c r="C387" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Optics Express</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Liston, Odhran; Sheehan, Robert N.; Peters, Frank H.; Kelleher, Bryan</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr"/>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>10.1364/oe.590413</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/oe.590413</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N387" t="inlineStr"/>
+      <c r="O387" t="inlineStr"/>
+      <c r="P387" t="inlineStr"/>
+      <c r="Q387" t="inlineStr">
+        <is>
+          <t>Monolithic excitable photonic neuron</t>
+        </is>
+      </c>
+      <c r="R387" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S387" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="T387" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr"/>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Si Power and SiC MOSFET, IGBT, and HEMT GaN at Cryogenic Temperature for Superconducting Propulsion System</t>
+        </is>
+      </c>
+      <c r="C388" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Applied Superconductivity</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Laïb, Yanis; Berger, Kévin; Raël, Stéphane; Lévêque, Jean</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr"/>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>10.1109/tasc.2026.3674548</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tasc.2026.3674548</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N388" t="inlineStr"/>
+      <c r="O388" t="inlineStr"/>
+      <c r="P388" t="inlineStr"/>
+      <c r="Q388" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Si Power and SiC MOSFET, IGBT, and HEMT GaN at Cryogenic Temperature for Superconducting Propulsion System</t>
+        </is>
+      </c>
+      <c r="R388" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S388" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="T388" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr"/>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Si Power and SiC MOSFET, IGBT, and HEMT GaN at Cryogenic Temperature for Superconducting Propulsion System</t>
+        </is>
+      </c>
+      <c r="C389" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Applied Superconductivity</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Laïb, Yanis; Berger, Kévin; Raël, Stéphane; Lévêque, Jean</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr"/>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>10.1109/tasc.2026.3674548</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tasc.2026.3674548</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N389" t="inlineStr"/>
+      <c r="O389" t="inlineStr"/>
+      <c r="P389" t="inlineStr"/>
+      <c r="Q389" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Si Power and SiC MOSFET, IGBT, and HEMT GaN at Cryogenic Temperature for Superconducting Propulsion System</t>
+        </is>
+      </c>
+      <c r="R389" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S389" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="T389" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr"/>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Si Power and SiC MOSFET, IGBT, and HEMT GaN at Cryogenic Temperature for Superconducting Propulsion System</t>
+        </is>
+      </c>
+      <c r="C390" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Applied Superconductivity</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Laïb, Yanis; Berger, Kévin; Raël, Stéphane; Lévêque, Jean</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr"/>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>10.1109/tasc.2026.3674548</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tasc.2026.3674548</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N390" t="inlineStr"/>
+      <c r="O390" t="inlineStr"/>
+      <c r="P390" t="inlineStr"/>
+      <c r="Q390" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Si Power and SiC MOSFET, IGBT, and HEMT GaN at Cryogenic Temperature for Superconducting Propulsion System</t>
+        </is>
+      </c>
+      <c r="R390" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S390" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="T390" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr"/>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Design of GaN HEMT Buck Converter for BCM Operation</t>
+        </is>
+      </c>
+      <c r="C391" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Hsieh, Yueh-Tsung; Chen, Chun-Hao; Chen, Tsung-Lin; Chieng, Wei-Hua; Chang, Edward-Yi</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr"/>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>10.3390/en19071700</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19071700</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N391" t="inlineStr"/>
+      <c r="O391" t="inlineStr"/>
+      <c r="P391" t="inlineStr"/>
+      <c r="Q391" t="inlineStr">
+        <is>
+          <t>Design of GaN HEMT Buck Converter for BCM Operation</t>
+        </is>
+      </c>
+      <c r="R391" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S391" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="T391" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr"/>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Si Power and SiC MOSFET, IGBT, and HEMT GaN at Cryogenic Temperature for Superconducting Propulsion System</t>
+        </is>
+      </c>
+      <c r="C392" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Applied Superconductivity</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Laïb, Yanis; Berger, Kévin; Raël, Stéphane; Lévêque, Jean</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr"/>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>10.1109/tasc.2026.3674548</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tasc.2026.3674548</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N392" t="inlineStr"/>
+      <c r="O392" t="inlineStr"/>
+      <c r="P392" t="inlineStr"/>
+      <c r="Q392" t="inlineStr">
+        <is>
+          <t>Performance Evaluation of Si Power and SiC MOSFET, IGBT, and HEMT GaN at Cryogenic Temperature for Superconducting Propulsion System</t>
+        </is>
+      </c>
+      <c r="R392" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S392" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="T392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr"/>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>ANPC-5L Inverter Floating Capacitor Pre-Charge Solution Design</t>
+        </is>
+      </c>
+      <c r="C393" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Darcy &amp; Roy Press Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Academic Journal of Science and Technology</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Yuan, Haohui; He, Qiwei; Wang, Yu</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr"/>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>10.54097/ywe9we28</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54097/ywe9we28</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N393" t="inlineStr"/>
+      <c r="O393" t="inlineStr"/>
+      <c r="P393" t="inlineStr"/>
+      <c r="Q393" t="inlineStr">
+        <is>
+          <t>ANPC-5L Inverter Floating Capacitor Pre-Charge Solution Design</t>
+        </is>
+      </c>
+      <c r="R393" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S393" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="T393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr"/>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Research Progress on CMOS Leakage Current Optimization and Low-Power Design</t>
+        </is>
+      </c>
+      <c r="C394" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Darcy &amp; Roy Press Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Academic Journal of Science and Technology</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Sun, Yujian</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr"/>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>10.54097/6hfpvg60</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54097/6hfpvg60</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N394" t="inlineStr"/>
+      <c r="O394" t="inlineStr"/>
+      <c r="P394" t="inlineStr"/>
+      <c r="Q394" t="inlineStr">
+        <is>
+          <t>Research Progress on CMOS Leakage Current Optimization and Low-Power Design</t>
+        </is>
+      </c>
+      <c r="R394" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S394" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="T394" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr"/>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Analysis and Optimization of Optical Logic Gate Technology</t>
+        </is>
+      </c>
+      <c r="C395" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Darcy &amp; Roy Press Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Academic Journal of Science and Technology</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Han, Wenhua</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr"/>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>10.54097/75tcm209</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54097/75tcm209</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N395" t="inlineStr"/>
+      <c r="O395" t="inlineStr"/>
+      <c r="P395" t="inlineStr"/>
+      <c r="Q395" t="inlineStr">
+        <is>
+          <t>Analysis and Optimization of Optical Logic Gate Technology</t>
+        </is>
+      </c>
+      <c r="R395" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S395" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="T395" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-01T23:39Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T395"/>
+  <dimension ref="A1:T396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30276,6 +30276,82 @@
       </c>
       <c r="T395" t="inlineStr"/>
     </row>
+    <row r="396">
+      <c r="A396" t="inlineStr"/>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Comparative Analysis of Heat Dissipation Distribution in Double‐Sided Cooling Si‐IGBT and SiC‐MOSFET Power Semiconductor Modules</t>
+        </is>
+      </c>
+      <c r="C396" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Electrical Engineering in Japan</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Yasui, Kan; Morikawa, Takahiro; Kushima, Takayuki; Funaki, Tsuyoshi</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr"/>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>10.1002/eej.70027</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/eej.70027</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N396" t="inlineStr"/>
+      <c r="O396" t="inlineStr"/>
+      <c r="P396" t="inlineStr"/>
+      <c r="Q396" t="inlineStr">
+        <is>
+          <t>Comparative Analysis of Heat Dissipation Distribution in Double‐Sided Cooling Si‐IGBT and SiC‐MOSFET Power Semiconductor Modules</t>
+        </is>
+      </c>
+      <c r="R396" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S396" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="T396" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-02T23:39Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T396"/>
+  <dimension ref="A1:T397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30352,6 +30352,78 @@
       </c>
       <c r="T396" t="inlineStr"/>
     </row>
+    <row r="397">
+      <c r="A397" t="inlineStr"/>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Emergence of a complex logic gate from the integration of slippage-induced frameshift mechanisms</t>
+        </is>
+      </c>
+      <c r="C397" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>openRxiv</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr"/>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Bhatti, Rushik; Saikrishnan, Kayarat</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr"/>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>10.64898/2026.04.01.715767</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.04.01.715767</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N397" t="inlineStr"/>
+      <c r="O397" t="inlineStr"/>
+      <c r="P397" t="inlineStr"/>
+      <c r="Q397" t="inlineStr">
+        <is>
+          <t>Emergence of a complex logic gate from the integration of slippage-induced frameshift mechanisms</t>
+        </is>
+      </c>
+      <c r="R397" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S397" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="T397" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-03T23:38Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T397"/>
+  <dimension ref="A1:T404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30424,6 +30424,538 @@
       </c>
       <c r="T397" t="inlineStr"/>
     </row>
+    <row r="398">
+      <c r="A398" t="inlineStr"/>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>TNFRSF17 as a complementary biomarker to PD-L1 for predicting the response to immunotherapy in urothelial bladder cancer</t>
+        </is>
+      </c>
+      <c r="C398" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Public Library of Science (PLoS)</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>PLOS One</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Chen, Jiawen; Li, Bingsheng; Gan, Yu; Li, Pan</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr"/>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>10.1371/journal.pone.0346131</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1371/journal.pone.0346131</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N398" t="inlineStr"/>
+      <c r="O398" t="inlineStr"/>
+      <c r="P398" t="inlineStr"/>
+      <c r="Q398" t="inlineStr">
+        <is>
+          <t>TNFRSF17 as a complementary biomarker to PD-L1 for predicting the response to immunotherapy in urothelial bladder cancer</t>
+        </is>
+      </c>
+      <c r="R398" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S398" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="T398" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr"/>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Monolithic integration of VCSELs with graphene/PEDOT:PSS photodetectors for compact optoelectronics</t>
+        </is>
+      </c>
+      <c r="C399" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Optics Express</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Mei, Yu; Xing, Yanhui; Cui, Ning; Zhang, Feng; Fu, Lishan; Guan, Baolu</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr"/>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>10.1364/oe.586609</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/oe.586609</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N399" t="inlineStr"/>
+      <c r="O399" t="inlineStr"/>
+      <c r="P399" t="inlineStr"/>
+      <c r="Q399" t="inlineStr">
+        <is>
+          <t>Monolithic integration of VCSELs with graphene/PEDOT:PSS photodetectors for compact optoelectronics</t>
+        </is>
+      </c>
+      <c r="R399" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S399" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="T399" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr"/>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>TNFRSF17 as a complementary biomarker to PD-L1 for predicting the response to immunotherapy in urothelial bladder cancer</t>
+        </is>
+      </c>
+      <c r="C400" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Public Library of Science (PLoS)</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>PLOS One</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Chen, Jiawen; Li, Bingsheng; Gan, Yu; Li, Pan</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr"/>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>10.1371/journal.pone.0346131</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1371/journal.pone.0346131</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N400" t="inlineStr"/>
+      <c r="O400" t="inlineStr"/>
+      <c r="P400" t="inlineStr"/>
+      <c r="Q400" t="inlineStr">
+        <is>
+          <t>TNFRSF17 as a complementary biomarker to PD-L1 for predicting the response to immunotherapy in urothelial bladder cancer</t>
+        </is>
+      </c>
+      <c r="R400" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S400" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="T400" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr"/>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Implementation Of Low Power and High Speed Dadda Multiplier Using XOR-XNOR Cell Based Hybrid Logic Full Adder Using Power Gating NMOS</t>
+        </is>
+      </c>
+      <c r="C401" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Edtech Publishers (OPC) Private Limited</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>INTERNATIONAL JOURNAL OF SCIENTIFIC RESEARCH IN ENGINEERING AND MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Raju, A. David; Surekha, Ms. M.; Swetha, K.; Sudheer, M.; Kumar, K. Manoj; Bhavana, M.</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr"/>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>10.55041/ijsrem58982</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.55041/ijsrem58982</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N401" t="inlineStr"/>
+      <c r="O401" t="inlineStr"/>
+      <c r="P401" t="inlineStr"/>
+      <c r="Q401" t="inlineStr">
+        <is>
+          <t>Implementation Of Low Power and High Speed Dadda Multiplier Using XOR-XNOR Cell Based Hybrid Logic Full Adder Using Power Gating NMOS</t>
+        </is>
+      </c>
+      <c r="R401" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S401" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="T401" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr"/>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>A novel 1200V SiC trench MOSFET based on superjunction and shielded gate technologies for reduced power loss</t>
+        </is>
+      </c>
+      <c r="C402" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Zhang, Xin; Cui, Pengfei; Liu, Qirui; Hu, Canbo; Wang, Dejun</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr"/>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae5aca</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae5aca</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N402" t="inlineStr"/>
+      <c r="O402" t="inlineStr"/>
+      <c r="P402" t="inlineStr"/>
+      <c r="Q402" t="inlineStr">
+        <is>
+          <t>A novel 1200V SiC trench MOSFET based on superjunction and shielded gate technologies for reduced power loss</t>
+        </is>
+      </c>
+      <c r="R402" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S402" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="T402" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr"/>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>A novel 1200V SiC trench MOSFET based on superjunction and shielded gate technologies for reduced power loss</t>
+        </is>
+      </c>
+      <c r="C403" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Zhang, Xin; Cui, Pengfei; Liu, Qirui; Hu, Canbo; Wang, Dejun</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr"/>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae5aca</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae5aca</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N403" t="inlineStr"/>
+      <c r="O403" t="inlineStr"/>
+      <c r="P403" t="inlineStr"/>
+      <c r="Q403" t="inlineStr">
+        <is>
+          <t>A novel 1200V SiC trench MOSFET based on superjunction and shielded gate technologies for reduced power loss</t>
+        </is>
+      </c>
+      <c r="R403" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S403" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="T403" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr"/>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Effects of electron irradiation and thermal cycling on electrical properties of GaN HEMT</t>
+        </is>
+      </c>
+      <c r="C404" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Soldering &amp;amp; Surface Mount Technology</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Han, Dan; Chen, Xiao; Shen, Zicai; Chen, Rui; Cao, Rongxing; Liu, Yang; Liu, Hanxun; Xue, Yuxiong</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr"/>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>10.1108/ssmt-11-2025-0063</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/ssmt-11-2025-0063</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N404" t="inlineStr"/>
+      <c r="O404" t="inlineStr"/>
+      <c r="P404" t="inlineStr"/>
+      <c r="Q404" t="inlineStr">
+        <is>
+          <t>Effects of electron irradiation and thermal cycling on electrical properties of GaN HEMT</t>
+        </is>
+      </c>
+      <c r="R404" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S404" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="T404" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-05T23:38Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T404"/>
+  <dimension ref="A1:T405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30956,6 +30956,82 @@
       </c>
       <c r="T404" t="inlineStr"/>
     </row>
+    <row r="405">
+      <c r="A405" t="inlineStr"/>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>A hybrid NCA-CNN deep learning approach for high-accuracy parametric fault diagnosis in MOSFET-C analog circuits</t>
+        </is>
+      </c>
+      <c r="C405" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>AEU - International Journal of Electronics and Communications</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Erkal, Keziban; Turhal, Umit Cigdem; Onal, Yasemin; Yesil, Abdullah</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr"/>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>10.1016/j.aeue.2026.156306</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.aeue.2026.156306</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N405" t="inlineStr"/>
+      <c r="O405" t="inlineStr"/>
+      <c r="P405" t="inlineStr"/>
+      <c r="Q405" t="inlineStr">
+        <is>
+          <t>A hybrid NCA-CNN deep learning approach for high-accuracy parametric fault diagnosis in MOSFET-C analog circuits</t>
+        </is>
+      </c>
+      <c r="R405" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S405" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="T405" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-06T23:39Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T405"/>
+  <dimension ref="A1:T406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31032,6 +31032,82 @@
       </c>
       <c r="T405" t="inlineStr"/>
     </row>
+    <row r="406">
+      <c r="A406" t="inlineStr"/>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Characterization of the H2M monolithic CMOS sensor</t>
+        </is>
+      </c>
+      <c r="C406" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Nuclear Instruments and Methods in Physics Research Section A: Accelerators, Spectrometers, Detectors and Associated Equipment</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Ballabriga, Rafael; Buschmann, Eric; Campbell, Michael; Mohr, Raimon Casanova; Dannheim, Dominik; Dilg, Jona; Dorda, Ana; Feyens, Ono; King, Finn; Gadow, Philipp; Gregor, Ingrid-Maria; Hansen, Karsten</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr"/>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>10.1016/j.nima.2026.171353</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.nima.2026.171353</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N406" t="inlineStr"/>
+      <c r="O406" t="inlineStr"/>
+      <c r="P406" t="inlineStr"/>
+      <c r="Q406" t="inlineStr">
+        <is>
+          <t>Characterization of the H2M monolithic CMOS sensor</t>
+        </is>
+      </c>
+      <c r="R406" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S406" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="T406" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-08T23:41Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T406"/>
+  <dimension ref="A1:T412"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31108,6 +31108,462 @@
       </c>
       <c r="T406" t="inlineStr"/>
     </row>
+    <row r="407">
+      <c r="A407" t="inlineStr"/>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>All-GaN monolithic integration of 2T1C pixel circuits with μLEDs</t>
+        </is>
+      </c>
+      <c r="C407" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Optics Letters</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Gao, Yipin; Liu, Chao</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr"/>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>10.1364/ol.593095</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/ol.593095</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N407" t="inlineStr"/>
+      <c r="O407" t="inlineStr"/>
+      <c r="P407" t="inlineStr"/>
+      <c r="Q407" t="inlineStr">
+        <is>
+          <t>All-GaN monolithic integration of 2T1C pixel circuits with μLEDs</t>
+        </is>
+      </c>
+      <c r="R407" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S407" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="T407" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr"/>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>TCAD and experimental study of geometric components in charge pumping current for accurate characterization of interface trap density in SiC pMOSFETs</t>
+        </is>
+      </c>
+      <c r="C408" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Shimura, Kazuma; Okamoto, Dai; Taguchi, Yuta; Kimata, Kenta; SOMETANI, Mitsuru; Hirai, Hirohisa; Okamoto, Mitsuo; HATAKEYAMA, Tetsuo</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr"/>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae5c0c</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae5c0c</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N408" t="inlineStr"/>
+      <c r="O408" t="inlineStr"/>
+      <c r="P408" t="inlineStr"/>
+      <c r="Q408" t="inlineStr">
+        <is>
+          <t>TCAD and experimental study of geometric components in charge pumping current for accurate characterization of interface trap density in SiC pMOSFETs</t>
+        </is>
+      </c>
+      <c r="R408" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S408" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="T408" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr"/>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>TCAD and experimental study of geometric components in charge pumping current for accurate characterization of interface trap density in SiC pMOSFETs</t>
+        </is>
+      </c>
+      <c r="C409" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Shimura, Kazuma; Okamoto, Dai; Taguchi, Yuta; Kimata, Kenta; SOMETANI, Mitsuru; Hirai, Hirohisa; Okamoto, Mitsuo; HATAKEYAMA, Tetsuo</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr"/>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae5c0c</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae5c0c</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N409" t="inlineStr"/>
+      <c r="O409" t="inlineStr"/>
+      <c r="P409" t="inlineStr"/>
+      <c r="Q409" t="inlineStr">
+        <is>
+          <t>TCAD and experimental study of geometric components in charge pumping current for accurate characterization of interface trap density in SiC pMOSFETs</t>
+        </is>
+      </c>
+      <c r="R409" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S409" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="T409" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr"/>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>TCAD and experimental study of geometric components in charge pumping current for accurate characterization of interface trap density in SiC pMOSFETs</t>
+        </is>
+      </c>
+      <c r="C410" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Shimura, Kazuma; Okamoto, Dai; Taguchi, Yuta; Kimata, Kenta; SOMETANI, Mitsuru; Hirai, Hirohisa; Okamoto, Mitsuo; HATAKEYAMA, Tetsuo</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr"/>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae5c0c</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae5c0c</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N410" t="inlineStr"/>
+      <c r="O410" t="inlineStr"/>
+      <c r="P410" t="inlineStr"/>
+      <c r="Q410" t="inlineStr">
+        <is>
+          <t>TCAD and experimental study of geometric components in charge pumping current for accurate characterization of interface trap density in SiC pMOSFETs</t>
+        </is>
+      </c>
+      <c r="R410" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S410" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="T410" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr"/>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>AI-Assisted Low Power Optimization in CMOS VLSI Circuits Using Machine Learning Technique</t>
+        </is>
+      </c>
+      <c r="C411" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Naksh Solutions</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>International Journal of Advanced Research in Science Communication and Technology</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Dr Malijeddi Murali, Dr A Rajesh, Mr. R. Narender; Mr. P. Kiran Kumar</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr"/>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>10.48175/ijarsct-32714</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48175/ijarsct-32714</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N411" t="inlineStr"/>
+      <c r="O411" t="inlineStr"/>
+      <c r="P411" t="inlineStr"/>
+      <c r="Q411" t="inlineStr">
+        <is>
+          <t>AI-Assisted Low Power Optimization in CMOS VLSI Circuits Using Machine Learning Technique</t>
+        </is>
+      </c>
+      <c r="R411" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S411" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="T411" t="inlineStr"/>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr"/>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>All-GaN monolithic integration of 2T1C pixel circuits with μLEDs</t>
+        </is>
+      </c>
+      <c r="C412" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Optics Letters</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Gao, Yipin; Liu, Chao</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr"/>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>10.1364/ol.593095</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/ol.593095</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N412" t="inlineStr"/>
+      <c r="O412" t="inlineStr"/>
+      <c r="P412" t="inlineStr"/>
+      <c r="Q412" t="inlineStr">
+        <is>
+          <t>All-GaN monolithic integration of 2T1C pixel circuits with μLEDs</t>
+        </is>
+      </c>
+      <c r="R412" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S412" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="T412" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-10T23:39Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T412"/>
+  <dimension ref="A1:T421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31564,6 +31564,682 @@
       </c>
       <c r="T412" t="inlineStr"/>
     </row>
+    <row r="413">
+      <c r="A413" t="inlineStr"/>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Differential Protection Based on Virtual Short-Circuit Current Considering Both Grid-Forming Inverter and Grid-Following Inverter for New Energy Bases</t>
+        </is>
+      </c>
+      <c r="C413" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Su, Zehua; Chen, Qian; Wang, Sijin; Qin, Zhehan; Gao, Jingyu</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr"/>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>10.3390/en19081853</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19081853</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N413" t="inlineStr"/>
+      <c r="O413" t="inlineStr"/>
+      <c r="P413" t="inlineStr"/>
+      <c r="Q413" t="inlineStr">
+        <is>
+          <t>Differential Protection Based on Virtual Short-Circuit Current Considering Both Grid-Forming Inverter and Grid-Following Inverter for New Energy Bases</t>
+        </is>
+      </c>
+      <c r="R413" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S413" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="T413" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr"/>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Differential Protection Based on Virtual Short-Circuit Current Considering Both Grid-Forming Inverter and Grid-Following Inverter for New Energy Bases</t>
+        </is>
+      </c>
+      <c r="C414" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Su, Zehua; Chen, Qian; Wang, Sijin; Qin, Zhehan; Gao, Jingyu</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr"/>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>10.3390/en19081853</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19081853</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N414" t="inlineStr"/>
+      <c r="O414" t="inlineStr"/>
+      <c r="P414" t="inlineStr"/>
+      <c r="Q414" t="inlineStr">
+        <is>
+          <t>Differential Protection Based on Virtual Short-Circuit Current Considering Both Grid-Forming Inverter and Grid-Following Inverter for New Energy Bases</t>
+        </is>
+      </c>
+      <c r="R414" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S414" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="T414" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr"/>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Realizing High-Q Quasi-BIC Through Monolithic Dimer Metasurface in SOI Platform</t>
+        </is>
+      </c>
+      <c r="C415" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr"/>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Bin Shams, Abdullah; Aitchison, J. Stewart; Sharar, Shadman Shahriar</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr"/>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>10.1364/opticaopen.31967694</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/opticaopen.31967694</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N415" t="inlineStr"/>
+      <c r="O415" t="inlineStr"/>
+      <c r="P415" t="inlineStr"/>
+      <c r="Q415" t="inlineStr">
+        <is>
+          <t>Realizing High-Q Quasi-BIC Through Monolithic Dimer Metasurface in SOI Platform</t>
+        </is>
+      </c>
+      <c r="R415" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S415" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="T415" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr"/>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Realizing High-Q Quasi-BIC Through Monolithic Dimer Metasurface in SOI Platform</t>
+        </is>
+      </c>
+      <c r="C416" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr"/>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Bin Shams, Abdullah; Aitchison, J. Stewart; Sharar, Shadman Shahriar</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr"/>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>10.1364/opticaopen.31967694.v1</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/opticaopen.31967694.v1</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N416" t="inlineStr"/>
+      <c r="O416" t="inlineStr"/>
+      <c r="P416" t="inlineStr"/>
+      <c r="Q416" t="inlineStr">
+        <is>
+          <t>Realizing High-Q Quasi-BIC Through Monolithic Dimer Metasurface in SOI Platform</t>
+        </is>
+      </c>
+      <c r="R416" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S416" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="T416" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr"/>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Monolithic integration for self-contained skin electronics</t>
+        </is>
+      </c>
+      <c r="C417" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>International Journal of Extreme Manufacturing</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Kim, Daegun; Lee, Giwon; Park, Sungjun</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr"/>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>10.1088/2631-7990/ae5d9e</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-7990/ae5d9e</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N417" t="inlineStr"/>
+      <c r="O417" t="inlineStr"/>
+      <c r="P417" t="inlineStr"/>
+      <c r="Q417" t="inlineStr">
+        <is>
+          <t>Monolithic integration for self-contained skin electronics</t>
+        </is>
+      </c>
+      <c r="R417" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S417" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="T417" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr"/>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Counting, Likert scaling or entropy? Measuring channel diversity of omni-channel marketing</t>
+        </is>
+      </c>
+      <c r="C418" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Industrial Management &amp;amp; Data Systems</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Li, Sihan; Zhuang, Guijun</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr"/>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>10.1108/imds-02-2025-0213</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/imds-02-2025-0213</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N418" t="inlineStr"/>
+      <c r="O418" t="inlineStr"/>
+      <c r="P418" t="inlineStr"/>
+      <c r="Q418" t="inlineStr">
+        <is>
+          <t>Counting, Likert scaling or entropy? Measuring channel diversity of omni-channel marketing</t>
+        </is>
+      </c>
+      <c r="R418" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S418" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="T418" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr"/>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Counting, Likert scaling or entropy? Measuring channel diversity of omni-channel marketing</t>
+        </is>
+      </c>
+      <c r="C419" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Industrial Management &amp;amp; Data Systems</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Li, Sihan; Zhuang, Guijun</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr"/>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>10.1108/imds-02-2025-0213</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/imds-02-2025-0213</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K419" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N419" t="inlineStr"/>
+      <c r="O419" t="inlineStr"/>
+      <c r="P419" t="inlineStr"/>
+      <c r="Q419" t="inlineStr">
+        <is>
+          <t>Counting, Likert scaling or entropy? Measuring channel diversity of omni-channel marketing</t>
+        </is>
+      </c>
+      <c r="R419" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S419" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="T419" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr"/>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Differential Protection Based on Virtual Short-Circuit Current Considering Both Grid-Forming Inverter and Grid-Following Inverter for New Energy Bases</t>
+        </is>
+      </c>
+      <c r="C420" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Su, Zehua; Chen, Qian; Wang, Sijin; Qin, Zhehan; Gao, Jingyu</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr"/>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>10.3390/en19081853</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19081853</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K420" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N420" t="inlineStr"/>
+      <c r="O420" t="inlineStr"/>
+      <c r="P420" t="inlineStr"/>
+      <c r="Q420" t="inlineStr">
+        <is>
+          <t>Differential Protection Based on Virtual Short-Circuit Current Considering Both Grid-Forming Inverter and Grid-Following Inverter for New Energy Bases</t>
+        </is>
+      </c>
+      <c r="R420" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S420" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="T420" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr"/>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Differential Protection Based on Virtual Short-Circuit Current Considering Both Grid-Forming Inverter and Grid-Following Inverter for New Energy Bases</t>
+        </is>
+      </c>
+      <c r="C421" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Su, Zehua; Chen, Qian; Wang, Sijin; Qin, Zhehan; Gao, Jingyu</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr"/>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>10.3390/en19081853</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19081853</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K421" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N421" t="inlineStr"/>
+      <c r="O421" t="inlineStr"/>
+      <c r="P421" t="inlineStr"/>
+      <c r="Q421" t="inlineStr">
+        <is>
+          <t>Differential Protection Based on Virtual Short-Circuit Current Considering Both Grid-Forming Inverter and Grid-Following Inverter for New Energy Bases</t>
+        </is>
+      </c>
+      <c r="R421" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S421" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="T421" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-13T23:48Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T421"/>
+  <dimension ref="A1:T429"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32240,6 +32240,602 @@
       </c>
       <c r="T421" t="inlineStr"/>
     </row>
+    <row r="422">
+      <c r="A422" t="inlineStr"/>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>The Monolithic Topology of Quasi-BIC Resonances in Dimer Metasurface</t>
+        </is>
+      </c>
+      <c r="C422" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr"/>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Bin Shams, Abdullah; Aitchison, J. Stewart</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr"/>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>10.1364/opticaopen.31974969.v1</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/opticaopen.31974969.v1</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N422" t="inlineStr"/>
+      <c r="O422" t="inlineStr"/>
+      <c r="P422" t="inlineStr"/>
+      <c r="Q422" t="inlineStr">
+        <is>
+          <t>The Monolithic Topology of Quasi-BIC Resonances in Dimer Metasurface</t>
+        </is>
+      </c>
+      <c r="R422" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S422" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="T422" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr"/>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>The Monolithic Topology of Quasi-BIC Resonances in Dimer Metasurface</t>
+        </is>
+      </c>
+      <c r="C423" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr"/>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Bin Shams, Abdullah; Aitchison, J. Stewart</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr"/>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>10.1364/opticaopen.31974969</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/opticaopen.31974969</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N423" t="inlineStr"/>
+      <c r="O423" t="inlineStr"/>
+      <c r="P423" t="inlineStr"/>
+      <c r="Q423" t="inlineStr">
+        <is>
+          <t>The Monolithic Topology of Quasi-BIC Resonances in Dimer Metasurface</t>
+        </is>
+      </c>
+      <c r="R423" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S423" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="T423" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr"/>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Electromagnetically Induced Transparency on All-Dielectric Monolithic Dimer Metasurface in SOI Platform</t>
+        </is>
+      </c>
+      <c r="C424" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr"/>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Bin Shams, Abdullah; Aitchison, J. Stewart; Sharar, Shadman Shahriar</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr"/>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>10.1364/opticaopen.31975218.v1</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/opticaopen.31975218.v1</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N424" t="inlineStr"/>
+      <c r="O424" t="inlineStr"/>
+      <c r="P424" t="inlineStr"/>
+      <c r="Q424" t="inlineStr">
+        <is>
+          <t>Electromagnetically Induced Transparency on All-Dielectric Monolithic Dimer Metasurface in SOI Platform</t>
+        </is>
+      </c>
+      <c r="R424" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S424" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="T424" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr"/>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Electromagnetically Induced Transparency on All-Dielectric Monolithic Dimer Metasurface in SOI Platform</t>
+        </is>
+      </c>
+      <c r="C425" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr"/>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Bin Shams, Abdullah; Aitchison, J. Stewart; Sharar, Shadman Shahriar</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr"/>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>10.1364/opticaopen.31975218</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/opticaopen.31975218</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N425" t="inlineStr"/>
+      <c r="O425" t="inlineStr"/>
+      <c r="P425" t="inlineStr"/>
+      <c r="Q425" t="inlineStr">
+        <is>
+          <t>Electromagnetically Induced Transparency on All-Dielectric Monolithic Dimer Metasurface in SOI Platform</t>
+        </is>
+      </c>
+      <c r="R425" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S425" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="T425" t="inlineStr"/>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr"/>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Negative capacitance double-gate junctionless MOS transistor for biosensing applications</t>
+        </is>
+      </c>
+      <c r="C426" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Kumar, Amit; Chaturvedi, Saurabh; Kumar, Satyendra</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr"/>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae5ed4</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae5ed4</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N426" t="inlineStr"/>
+      <c r="O426" t="inlineStr"/>
+      <c r="P426" t="inlineStr"/>
+      <c r="Q426" t="inlineStr">
+        <is>
+          <t>Negative capacitance double-gate junctionless MOS transistor for biosensing applications</t>
+        </is>
+      </c>
+      <c r="R426" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S426" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="T426" t="inlineStr"/>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr"/>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>DESIGN AND IMPLEMENTATION OF SOFT- SWITCHING DC DC CONVERTER USING SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="C427" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Edtech Publishers (OPC) Private Limited</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>International Scientific Journal of Engineering and Management</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>P, Siddhi</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr"/>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>10.55041/isjem06339</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.55041/isjem06339</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N427" t="inlineStr"/>
+      <c r="O427" t="inlineStr"/>
+      <c r="P427" t="inlineStr"/>
+      <c r="Q427" t="inlineStr">
+        <is>
+          <t>DESIGN AND IMPLEMENTATION OF SOFT- SWITCHING DC DC CONVERTER USING SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="R427" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S427" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="T427" t="inlineStr"/>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr"/>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>DESIGN AND IMPLEMENTATION OF SOFT- SWITCHING DC DC CONVERTER USING SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="C428" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Edtech Publishers (OPC) Private Limited</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>International Scientific Journal of Engineering and Management</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>P, Siddhi</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr"/>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>10.55041/isjem06339</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.55041/isjem06339</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N428" t="inlineStr"/>
+      <c r="O428" t="inlineStr"/>
+      <c r="P428" t="inlineStr"/>
+      <c r="Q428" t="inlineStr">
+        <is>
+          <t>DESIGN AND IMPLEMENTATION OF SOFT- SWITCHING DC DC CONVERTER USING SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="R428" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S428" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="T428" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr"/>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>SiO
+                    &lt;sub&gt;x&lt;/sub&gt;
+                    ‐Based Probabilistic Bits Enabling Invertible Logic Gate for Cryptographic Applications</t>
+        </is>
+      </c>
+      <c r="C429" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Advanced Intelligent Systems</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Kim, Jihyun; Choi, Hyeonsik; Woo, Jiyong</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr"/>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>10.1002/aisy.70365</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/aisy.70365</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N429" t="inlineStr"/>
+      <c r="O429" t="inlineStr"/>
+      <c r="P429" t="inlineStr"/>
+      <c r="Q429" t="inlineStr">
+        <is>
+          <t>SiO
+                    &lt;sub&gt;x&lt;/sub&gt;
+                    ‐Based Probabilistic Bits Enabling Invertible Logic Gate for Cryptographic Applications</t>
+        </is>
+      </c>
+      <c r="R429" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S429" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="T429" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-14T23:46Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T429"/>
+  <dimension ref="A1:T433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32836,6 +32836,310 @@
       </c>
       <c r="T429" t="inlineStr"/>
     </row>
+    <row r="430">
+      <c r="A430" t="inlineStr"/>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Three New Philosophical Categories for Holistically Assessing Complementary Medicine, Derived from the History and Theory of Medicine</t>
+        </is>
+      </c>
+      <c r="C430" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>S. Karger AG</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Complementary Medicine Research</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Schmidt, Josef M.</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr"/>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>10.1159/000551108</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1159/000551108</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N430" t="inlineStr"/>
+      <c r="O430" t="inlineStr"/>
+      <c r="P430" t="inlineStr"/>
+      <c r="Q430" t="inlineStr">
+        <is>
+          <t>Three New Philosophical Categories for Holistically Assessing Complementary Medicine, Derived from the History and Theory of Medicine</t>
+        </is>
+      </c>
+      <c r="R430" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S430" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="T430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr"/>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Monolithic Potentiometric Cell Using Fused Filament Fabrication</t>
+        </is>
+      </c>
+      <c r="C431" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Analytical Chemistry</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Torricelli, Dario; Rojas, Daniel; Crespo, Gastón; Cuartero, María</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr"/>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>10.1021/acs.analchem.6c00156</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acs.analchem.6c00156</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N431" t="inlineStr"/>
+      <c r="O431" t="inlineStr"/>
+      <c r="P431" t="inlineStr"/>
+      <c r="Q431" t="inlineStr">
+        <is>
+          <t>Monolithic Potentiometric Cell Using Fused Filament Fabrication</t>
+        </is>
+      </c>
+      <c r="R431" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S431" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="T431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr"/>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>From Monolithic Models to Cognitive Hives: A Framework for Multimodal Reasoning Systems</t>
+        </is>
+      </c>
+      <c r="C432" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Al-Kindi Center for Research and Development</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Journal of Computer Science and Technology Studies</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Inesh Hettiarachchi</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr"/>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>10.32996/jcsts.2026.8.5.14</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.32996/jcsts.2026.8.5.14</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N432" t="inlineStr"/>
+      <c r="O432" t="inlineStr"/>
+      <c r="P432" t="inlineStr"/>
+      <c r="Q432" t="inlineStr">
+        <is>
+          <t>From Monolithic Models to Cognitive Hives: A Framework for Multimodal Reasoning Systems</t>
+        </is>
+      </c>
+      <c r="R432" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S432" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="T432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr"/>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Three New Philosophical Categories for Holistically Assessing Complementary Medicine, Derived from the History and Theory of Medicine</t>
+        </is>
+      </c>
+      <c r="C433" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>S. Karger AG</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Complementary Medicine Research</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Schmidt, Josef M.</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr"/>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>10.1159/000551108</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1159/000551108</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N433" t="inlineStr"/>
+      <c r="O433" t="inlineStr"/>
+      <c r="P433" t="inlineStr"/>
+      <c r="Q433" t="inlineStr">
+        <is>
+          <t>Three New Philosophical Categories for Holistically Assessing Complementary Medicine, Derived from the History and Theory of Medicine</t>
+        </is>
+      </c>
+      <c r="R433" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S433" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="T433" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-16T23:44Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T433"/>
+  <dimension ref="A1:T436"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33140,6 +33140,234 @@
       </c>
       <c r="T433" t="inlineStr"/>
     </row>
+    <row r="434">
+      <c r="A434" t="inlineStr"/>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Mg Doping Gradient Engineering by MOCVD for Threshold Voltage Enhancement in Si-Based p-GaN E-Mode HEMTs</t>
+        </is>
+      </c>
+      <c r="C434" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Coatings</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Chen, Changyao; Zhang, Shuhan; Fan, Qian; Ni, Xianfeng; Gu, Xing</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr"/>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>10.3390/coatings16040476</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/coatings16040476</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K434" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N434" t="inlineStr"/>
+      <c r="O434" t="inlineStr"/>
+      <c r="P434" t="inlineStr"/>
+      <c r="Q434" t="inlineStr">
+        <is>
+          <t>Mg Doping Gradient Engineering by MOCVD for Threshold Voltage Enhancement in Si-Based p-GaN E-Mode HEMTs</t>
+        </is>
+      </c>
+      <c r="R434" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S434" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="T434" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr"/>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Mg Doping Gradient Engineering by MOCVD for Threshold Voltage Enhancement in Si-Based p-GaN E-Mode HEMTs</t>
+        </is>
+      </c>
+      <c r="C435" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Coatings</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Chen, Changyao; Zhang, Shuhan; Fan, Qian; Ni, Xianfeng; Gu, Xing</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr"/>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>10.3390/coatings16040476</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/coatings16040476</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K435" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N435" t="inlineStr"/>
+      <c r="O435" t="inlineStr"/>
+      <c r="P435" t="inlineStr"/>
+      <c r="Q435" t="inlineStr">
+        <is>
+          <t>Mg Doping Gradient Engineering by MOCVD for Threshold Voltage Enhancement in Si-Based p-GaN E-Mode HEMTs</t>
+        </is>
+      </c>
+      <c r="R435" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S435" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="T435" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr"/>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Total ionizing dose and single-event transient effects in 22nm-FDSOI technology by TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C436" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Huang, Kai; Bi, Jinshun; Aierken, Abuduwayiti; Liu, Xuefei; Liu, Mingqiang; Gao, Changsong; Wang, Gang; Wang, Degui; Xuan, Yundong</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr"/>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae6097</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae6097</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K436" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N436" t="inlineStr"/>
+      <c r="O436" t="inlineStr"/>
+      <c r="P436" t="inlineStr"/>
+      <c r="Q436" t="inlineStr">
+        <is>
+          <t>Total ionizing dose and single-event transient effects in 22nm-FDSOI technology by TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R436" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S436" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="T436" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-17T23:42Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T436"/>
+  <dimension ref="A1:T439"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33368,6 +33368,242 @@
       </c>
       <c r="T436" t="inlineStr"/>
     </row>
+    <row r="437">
+      <c r="A437" t="inlineStr"/>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Published Databases Resources for Traditional, Complementary, and Integrative Medicine: Update of a Systematic Review</t>
+        </is>
+      </c>
+      <c r="C437" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Raak, Christa K.; Martin, David D.; Boehm, Katja; Hacke, Daniela; Unger, Sebastian; Ostermann, Thomas</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr"/>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261441386</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261441386</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N437" t="inlineStr"/>
+      <c r="O437" t="inlineStr"/>
+      <c r="P437" t="inlineStr"/>
+      <c r="Q437" t="inlineStr">
+        <is>
+          <t>Published Databases Resources for Traditional, Complementary, and Integrative Medicine: Update of a Systematic Review</t>
+        </is>
+      </c>
+      <c r="R437" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S437" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="T437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr"/>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Published Databases Resources for Traditional, Complementary, and Integrative Medicine: Update of a Systematic Review</t>
+        </is>
+      </c>
+      <c r="C438" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Raak, Christa K.; Martin, David D.; Boehm, Katja; Hacke, Daniela; Unger, Sebastian; Ostermann, Thomas</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr"/>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261441386</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261441386</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N438" t="inlineStr"/>
+      <c r="O438" t="inlineStr"/>
+      <c r="P438" t="inlineStr"/>
+      <c r="Q438" t="inlineStr">
+        <is>
+          <t>Published Databases Resources for Traditional, Complementary, and Integrative Medicine: Update of a Systematic Review</t>
+        </is>
+      </c>
+      <c r="R438" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S438" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="T438" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr"/>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Enhanced Dopant Activation and Reduced Specific Contact Resistivity in Ti/n
+                    &lt;sup&gt;+&lt;/sup&gt;
+                    -Si Contacts by O
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    Ambient Spike Annealing</t>
+        </is>
+      </c>
+      <c r="C439" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>liu, jianhong; Xu, Jing; ji, xiaoxue; Liu, Jinbiao; Xu, Binbin; Liu, Chang; Gao, Haisu; Guo, Yanxiang; Han, Yaxuan; Liu, Xiangsheng; Luo, Jun</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr"/>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae613e</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae613e</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N439" t="inlineStr"/>
+      <c r="O439" t="inlineStr"/>
+      <c r="P439" t="inlineStr"/>
+      <c r="Q439" t="inlineStr">
+        <is>
+          <t>Enhanced Dopant Activation and Reduced Specific Contact Resistivity in Ti/n
+                    &lt;sup&gt;+&lt;/sup&gt;
+                    -Si Contacts by O
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    Ambient Spike Annealing</t>
+        </is>
+      </c>
+      <c r="R439" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S439" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="T439" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-19T23:41Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T439"/>
+  <dimension ref="A1:T440"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33604,6 +33604,78 @@
       </c>
       <c r="T439" t="inlineStr"/>
     </row>
+    <row r="440">
+      <c r="A440" t="inlineStr"/>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Monolithic solution and null-space condensation of internal variables in finite viscoelasticity</t>
+        </is>
+      </c>
+      <c r="C440" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr"/>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Sethuraman, A. K.K.; Hesch, C.</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr"/>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9245077/v1</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9245077/v1</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N440" t="inlineStr"/>
+      <c r="O440" t="inlineStr"/>
+      <c r="P440" t="inlineStr"/>
+      <c r="Q440" t="inlineStr">
+        <is>
+          <t>Monolithic solution and null-space condensation of internal variables in finite viscoelasticity</t>
+        </is>
+      </c>
+      <c r="R440" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S440" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="T440" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-20T23:46Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T440"/>
+  <dimension ref="A1:T451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33676,6 +33676,842 @@
       </c>
       <c r="T440" t="inlineStr"/>
     </row>
+    <row r="441">
+      <c r="A441" t="inlineStr"/>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Emerging multilevel inverter architectures for high-performance photovoltaic systems: a review</t>
+        </is>
+      </c>
+      <c r="C441" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Interactions</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Kamalaselvan, A.; Murugesan, Muthukumar; Sitharaj, Ajithkumar; Rajiv, S.; Kalaivanan, K.</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr"/>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>10.1007/s10751-026-02509-7</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10751-026-02509-7</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N441" t="inlineStr"/>
+      <c r="O441" t="inlineStr"/>
+      <c r="P441" t="inlineStr"/>
+      <c r="Q441" t="inlineStr">
+        <is>
+          <t>Emerging multilevel inverter architectures for high-performance photovoltaic systems: a review</t>
+        </is>
+      </c>
+      <c r="R441" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S441" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T441" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr"/>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>THE ROLE OF ACUPUNCTURE IN OVERCOMING COMPLAINTS OF CARPAL TUNNEL SYNDROME</t>
+        </is>
+      </c>
+      <c r="C442" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>International Islamic Medical Forum</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>International Journal of Islamic and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Ramona, Dela; Septadina, Indri Seta</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr"/>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>10.55116/ijicm.v7i1.112</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.55116/ijicm.v7i1.112</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N442" t="inlineStr"/>
+      <c r="O442" t="inlineStr"/>
+      <c r="P442" t="inlineStr"/>
+      <c r="Q442" t="inlineStr">
+        <is>
+          <t>THE ROLE OF ACUPUNCTURE IN OVERCOMING COMPLAINTS OF CARPAL TUNNEL SYNDROME</t>
+        </is>
+      </c>
+      <c r="R442" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S442" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T442" t="inlineStr"/>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr"/>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Düşük Gerilim Düşük Güçlü MOSFET Tasarım Yöntemlerinin İncelenmesi</t>
+        </is>
+      </c>
+      <c r="C443" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Politeknik Dergisi</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Journal of Polytechnic</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Doğan Sekreter, Pelin; Uygur, Atilla; Alçı, Mustafa</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr"/>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>10.2339/politeknik.1338855</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2339/politeknik.1338855</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N443" t="inlineStr"/>
+      <c r="O443" t="inlineStr"/>
+      <c r="P443" t="inlineStr"/>
+      <c r="Q443" t="inlineStr">
+        <is>
+          <t>Düşük Gerilim Düşük Güçlü MOSFET Tasarım Yöntemlerinin İncelenmesi</t>
+        </is>
+      </c>
+      <c r="R443" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S443" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T443" t="inlineStr"/>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr"/>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Influence of p-GaN body contact on output characteristics of vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="C444" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Kusunoki, Nami; Ichikawa, Yuki; Oka, Tohru; Tanaka, Nariaki; Hasegawa, Kazuya; Izumi, Takatomi; Niwa, Takaki; Suda, Jun</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr"/>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae620d</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae620d</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N444" t="inlineStr"/>
+      <c r="O444" t="inlineStr"/>
+      <c r="P444" t="inlineStr"/>
+      <c r="Q444" t="inlineStr">
+        <is>
+          <t>Influence of p-GaN body contact on output characteristics of vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="R444" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S444" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T444" t="inlineStr"/>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr"/>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>A compact antenna aperture tuner with high voltage enhancement-mode p-GaN HEMT switch</t>
+        </is>
+      </c>
+      <c r="C445" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Cambridge University Press (CUP)</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>International Journal of Microwave and Wireless Technologies</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Yu, Chia Hao; Chiu, Hsien-Chin; Lin, Chia-Han; Huang, Chong-Rong; Kao, Hsuan-Ling; Lin, Shinn-Yn; Lin, Chia-Fu</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr"/>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>10.1017/s1759078726103134</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1017/s1759078726103134</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N445" t="inlineStr"/>
+      <c r="O445" t="inlineStr"/>
+      <c r="P445" t="inlineStr"/>
+      <c r="Q445" t="inlineStr">
+        <is>
+          <t>A compact antenna aperture tuner with high voltage enhancement-mode p-GaN HEMT switch</t>
+        </is>
+      </c>
+      <c r="R445" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S445" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T445" t="inlineStr"/>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr"/>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Düşük Gerilim Düşük Güçlü MOSFET Tasarım Yöntemlerinin İncelenmesi</t>
+        </is>
+      </c>
+      <c r="C446" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Politeknik Dergisi</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>Journal of Polytechnic</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Doğan Sekreter, Pelin; Uygur, Atilla; Alçı, Mustafa</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr"/>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>10.2339/politeknik.1338855</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2339/politeknik.1338855</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K446" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N446" t="inlineStr"/>
+      <c r="O446" t="inlineStr"/>
+      <c r="P446" t="inlineStr"/>
+      <c r="Q446" t="inlineStr">
+        <is>
+          <t>Düşük Gerilim Düşük Güçlü MOSFET Tasarım Yöntemlerinin İncelenmesi</t>
+        </is>
+      </c>
+      <c r="R446" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S446" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T446" t="inlineStr"/>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr"/>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>A compact antenna aperture tuner with high voltage enhancement-mode p-GaN HEMT switch</t>
+        </is>
+      </c>
+      <c r="C447" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Cambridge University Press (CUP)</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>International Journal of Microwave and Wireless Technologies</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Yu, Chia Hao; Chiu, Hsien-Chin; Lin, Chia-Han; Huang, Chong-Rong; Kao, Hsuan-Ling; Lin, Shinn-Yn; Lin, Chia-Fu</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr"/>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>10.1017/s1759078726103134</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1017/s1759078726103134</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K447" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N447" t="inlineStr"/>
+      <c r="O447" t="inlineStr"/>
+      <c r="P447" t="inlineStr"/>
+      <c r="Q447" t="inlineStr">
+        <is>
+          <t>A compact antenna aperture tuner with high voltage enhancement-mode p-GaN HEMT switch</t>
+        </is>
+      </c>
+      <c r="R447" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S447" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T447" t="inlineStr"/>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr"/>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Emerging multilevel inverter architectures for high-performance photovoltaic systems: a review</t>
+        </is>
+      </c>
+      <c r="C448" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Interactions</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Kamalaselvan, A.; Murugesan, Muthukumar; Sitharaj, Ajithkumar; Rajiv, S.; Kalaivanan, K.</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr"/>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>10.1007/s10751-026-02509-7</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10751-026-02509-7</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K448" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N448" t="inlineStr"/>
+      <c r="O448" t="inlineStr"/>
+      <c r="P448" t="inlineStr"/>
+      <c r="Q448" t="inlineStr">
+        <is>
+          <t>Emerging multilevel inverter architectures for high-performance photovoltaic systems: a review</t>
+        </is>
+      </c>
+      <c r="R448" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S448" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T448" t="inlineStr"/>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr"/>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Influence of p-GaN body contact on output characteristics of vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="C449" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Kusunoki, Nami; Ichikawa, Yuki; Oka, Tohru; Tanaka, Nariaki; Hasegawa, Kazuya; Izumi, Takatomi; Niwa, Takaki; Suda, Jun</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr"/>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae620d</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae620d</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K449" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N449" t="inlineStr"/>
+      <c r="O449" t="inlineStr"/>
+      <c r="P449" t="inlineStr"/>
+      <c r="Q449" t="inlineStr">
+        <is>
+          <t>Influence of p-GaN body contact on output characteristics of vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="R449" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S449" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T449" t="inlineStr"/>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr"/>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Influence of p-GaN body contact on output characteristics of vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="C450" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Kusunoki, Nami; Ichikawa, Yuki; Oka, Tohru; Tanaka, Nariaki; Hasegawa, Kazuya; Izumi, Takatomi; Niwa, Takaki; Suda, Jun</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr"/>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae620d</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae620d</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N450" t="inlineStr"/>
+      <c r="O450" t="inlineStr"/>
+      <c r="P450" t="inlineStr"/>
+      <c r="Q450" t="inlineStr">
+        <is>
+          <t>Influence of p-GaN body contact on output characteristics of vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="R450" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S450" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T450" t="inlineStr"/>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr"/>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Influence of p-GaN body contact on output characteristics of vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="C451" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Kusunoki, Nami; Ichikawa, Yuki; Oka, Tohru; Tanaka, Nariaki; Hasegawa, Kazuya; Izumi, Takatomi; Niwa, Takaki; Suda, Jun</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr"/>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae620d</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae620d</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K451" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N451" t="inlineStr"/>
+      <c r="O451" t="inlineStr"/>
+      <c r="P451" t="inlineStr"/>
+      <c r="Q451" t="inlineStr">
+        <is>
+          <t>Influence of p-GaN body contact on output characteristics of vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="R451" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S451" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="T451" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-21T23:38Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T451"/>
+  <dimension ref="A1:T452"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34512,6 +34512,82 @@
       </c>
       <c r="T451" t="inlineStr"/>
     </row>
+    <row r="452">
+      <c r="A452" t="inlineStr"/>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Cost-effective single-source 25-level inverter achieving twelvefold voltage gain with redundant switching and hybrid modulation</t>
+        </is>
+      </c>
+      <c r="C452" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Hosseinpour, Majid; Mansourizadeh, Hossein; Seifi, Ali</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr"/>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-49547-3</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-49547-3</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N452" t="inlineStr"/>
+      <c r="O452" t="inlineStr"/>
+      <c r="P452" t="inlineStr"/>
+      <c r="Q452" t="inlineStr">
+        <is>
+          <t>Cost-effective single-source 25-level inverter achieving twelvefold voltage gain with redundant switching and hybrid modulation</t>
+        </is>
+      </c>
+      <c r="R452" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S452" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="T452" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-22T23:50Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T452"/>
+  <dimension ref="A1:T458"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34588,6 +34588,462 @@
       </c>
       <c r="T452" t="inlineStr"/>
     </row>
+    <row r="453">
+      <c r="A453" t="inlineStr"/>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Associations Between Social and Religious Characteristics and the Use of Religion-Based and Complementary Healing Practices Among Muslim Women in Chicago: A Cross-Sectional Community Survey</t>
+        </is>
+      </c>
+      <c r="C453" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Abdulbaseer, Ummesalmah; Yunus, Raudah M.; Padela, Aasim I.</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr"/>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261445326</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261445326</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K453" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N453" t="inlineStr"/>
+      <c r="O453" t="inlineStr"/>
+      <c r="P453" t="inlineStr"/>
+      <c r="Q453" t="inlineStr">
+        <is>
+          <t>Associations Between Social and Religious Characteristics and the Use of Religion-Based and Complementary Healing Practices Among Muslim Women in Chicago: A Cross-Sectional Community Survey</t>
+        </is>
+      </c>
+      <c r="R453" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S453" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="T453" t="inlineStr"/>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr"/>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Associations Between Social and Religious Characteristics and the Use of Religion-Based and Complementary Healing Practices Among Muslim Women in Chicago: A Cross-Sectional Community Survey</t>
+        </is>
+      </c>
+      <c r="C454" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Abdulbaseer, Ummesalmah; Yunus, Raudah M.; Padela, Aasim I.</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr"/>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261445326</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261445326</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K454" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N454" t="inlineStr"/>
+      <c r="O454" t="inlineStr"/>
+      <c r="P454" t="inlineStr"/>
+      <c r="Q454" t="inlineStr">
+        <is>
+          <t>Associations Between Social and Religious Characteristics and the Use of Religion-Based and Complementary Healing Practices Among Muslim Women in Chicago: A Cross-Sectional Community Survey</t>
+        </is>
+      </c>
+      <c r="R454" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S454" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="T454" t="inlineStr"/>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr"/>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Review on ultrathin-barrier AlGaN(&amp;lt;6 nm)/GaN enhancement-mode technology: concept, device fabrication, and integration prospects</t>
+        </is>
+      </c>
+      <c r="C455" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Huang, Sen; Zheng, Yang; Zhang, Kaiwei; Zhang, Yang; Tan, Huan; Li, Dong; Zhao, Zichen; Lai, Senfa; He, Yaoyao; Gao, Xinguo; Wang, Xinhua; Wei, Ke</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr"/>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae634c</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae634c</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K455" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N455" t="inlineStr"/>
+      <c r="O455" t="inlineStr"/>
+      <c r="P455" t="inlineStr"/>
+      <c r="Q455" t="inlineStr">
+        <is>
+          <t>Review on ultrathin-barrier AlGaN(&amp;lt;6 nm)/GaN enhancement-mode technology: concept, device fabrication, and integration prospects</t>
+        </is>
+      </c>
+      <c r="R455" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S455" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="T455" t="inlineStr"/>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr"/>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Suppression of Interface Traps and Improved Breakdown in Recessed-Gate AlGaN/GaN MISHEMTs Using Low-Temperature Nitrogen Passivation</t>
+        </is>
+      </c>
+      <c r="C456" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>ACS Omega</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Chen, Hsin-Chu; Liu, An-Chen; Lin, Cheng-Hsien; Chou, Sheng-Yao; Chang, Ting-Chang; Kao, Tsung-Sheng; Kuo, Hao-Chung</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr"/>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>10.1021/acsomega.5c10644</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsomega.5c10644</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K456" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N456" t="inlineStr"/>
+      <c r="O456" t="inlineStr"/>
+      <c r="P456" t="inlineStr"/>
+      <c r="Q456" t="inlineStr">
+        <is>
+          <t>Suppression of Interface Traps and Improved Breakdown in Recessed-Gate AlGaN/GaN MISHEMTs Using Low-Temperature Nitrogen Passivation</t>
+        </is>
+      </c>
+      <c r="R456" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S456" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="T456" t="inlineStr"/>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr"/>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Suppression of Interface Traps and Improved Breakdown in Recessed-Gate AlGaN/GaN MISHEMTs Using Low-Temperature Nitrogen Passivation</t>
+        </is>
+      </c>
+      <c r="C457" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>ACS Omega</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Chen, Hsin-Chu; Liu, An-Chen; Lin, Cheng-Hsien; Chou, Sheng-Yao; Chang, Ting-Chang; Kao, Tsung-Sheng; Kuo, Hao-Chung</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr"/>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>10.1021/acsomega.5c10644</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsomega.5c10644</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K457" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N457" t="inlineStr"/>
+      <c r="O457" t="inlineStr"/>
+      <c r="P457" t="inlineStr"/>
+      <c r="Q457" t="inlineStr">
+        <is>
+          <t>Suppression of Interface Traps and Improved Breakdown in Recessed-Gate AlGaN/GaN MISHEMTs Using Low-Temperature Nitrogen Passivation</t>
+        </is>
+      </c>
+      <c r="R457" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S457" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="T457" t="inlineStr"/>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr"/>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Ohmic Contact Engineering in Strained Si/SiGe Heterostructures for Cryo‐Electronics Operating at 1.5 K</t>
+        </is>
+      </c>
+      <c r="C458" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Fidorra, Fabian; Mistroni, Alberto; Hnida-Gut, Katarzyna E.; Reichmann, Felix; Adnadane, Meriem; Wen, Wei-Chen; Yamamoto, Yuji; Bärwolf, Florian; Schubert, Markus Andreas; Lisker, Marco</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr"/>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.202501036</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.202501036</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K458" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N458" t="inlineStr"/>
+      <c r="O458" t="inlineStr"/>
+      <c r="P458" t="inlineStr"/>
+      <c r="Q458" t="inlineStr">
+        <is>
+          <t>Ohmic Contact Engineering in Strained Si/SiGe Heterostructures for Cryo‐Electronics Operating at 1.5 K</t>
+        </is>
+      </c>
+      <c r="R458" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S458" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="T458" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-23T23:51Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T458"/>
+  <dimension ref="A1:T461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35044,6 +35044,254 @@
       </c>
       <c r="T458" t="inlineStr"/>
     </row>
+    <row r="459">
+      <c r="A459" t="inlineStr"/>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Tailoring the Sensitivity-Range Tradeoff in Monolithic InGaN/GaN Temperature Sensing Devices via Indium Content Engineering</t>
+        </is>
+      </c>
+      <c r="C459" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Electron Devices</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Yang, Hongying; An, Xiaoshuai; Li, Kwai Hei</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr"/>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>10.1109/ted.2026.3679655</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ted.2026.3679655</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K459" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N459" t="inlineStr"/>
+      <c r="O459" t="inlineStr"/>
+      <c r="P459" t="inlineStr"/>
+      <c r="Q459" t="inlineStr">
+        <is>
+          <t>Tailoring the Sensitivity-Range Tradeoff in Monolithic InGaN/GaN Temperature Sensing Devices via Indium Content Engineering</t>
+        </is>
+      </c>
+      <c r="R459" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S459" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="T459" t="inlineStr"/>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr"/>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>First-Principles Study of N
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    or H
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    /N
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    Plasma Pretreatment: Effects on the Interface Properties in Si
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    N
+                    &lt;sub&gt;4&lt;/sub&gt;
+                    /AlN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="C460" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Electron Devices</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Yang, Jiaofen; Tao, Ming; Xiao, Jing; Tang, Kai; Chen, Yilan; Zhang, Wenjing; Zhang, Bin; Huang, Bowen; Liu, Jie; Wang, Hongyue; Wang, Jinyan; Wang, Maojun</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr"/>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>10.1109/ted.2026.3678928</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ted.2026.3678928</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K460" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N460" t="inlineStr"/>
+      <c r="O460" t="inlineStr"/>
+      <c r="P460" t="inlineStr"/>
+      <c r="Q460" t="inlineStr">
+        <is>
+          <t>First-Principles Study of N
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    or H
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    /N
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    Plasma Pretreatment: Effects on the Interface Properties in Si
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    N
+                    &lt;sub&gt;4&lt;/sub&gt;
+                    /AlN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="R460" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S460" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="T460" t="inlineStr"/>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr"/>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Tailoring the Sensitivity-Range Tradeoff in Monolithic InGaN/GaN Temperature Sensing Devices via Indium Content Engineering</t>
+        </is>
+      </c>
+      <c r="C461" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Electron Devices</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Yang, Hongying; An, Xiaoshuai; Li, Kwai Hei</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr"/>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>10.1109/ted.2026.3679655</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ted.2026.3679655</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K461" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N461" t="inlineStr"/>
+      <c r="O461" t="inlineStr"/>
+      <c r="P461" t="inlineStr"/>
+      <c r="Q461" t="inlineStr">
+        <is>
+          <t>Tailoring the Sensitivity-Range Tradeoff in Monolithic InGaN/GaN Temperature Sensing Devices via Indium Content Engineering</t>
+        </is>
+      </c>
+      <c r="R461" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S461" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="T461" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-24T23:42Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T461"/>
+  <dimension ref="A1:T466"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35292,6 +35292,386 @@
       </c>
       <c r="T461" t="inlineStr"/>
     </row>
+    <row r="462">
+      <c r="A462" t="inlineStr"/>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>High-performance power electronic management systems using MOSFET technology for electric vehicle energy storage</t>
+        </is>
+      </c>
+      <c r="C462" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Inderscience Publishers</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>International Journal of Power Electronics</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Basri, Omar Kanaan Al; Nnori, Fayrooz Kanaan</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr"/>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>10.1504/ijpelec.2027.10077958</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1504/ijpelec.2027.10077958</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K462" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N462" t="inlineStr"/>
+      <c r="O462" t="inlineStr"/>
+      <c r="P462" t="inlineStr"/>
+      <c r="Q462" t="inlineStr">
+        <is>
+          <t>High-performance power electronic management systems using MOSFET technology for electric vehicle energy storage</t>
+        </is>
+      </c>
+      <c r="R462" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S462" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="T462" t="inlineStr"/>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr"/>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Design of a High-Speed, Low-Power Dadda Multiplier Based on XOR–XNOR Hybrid Full Adder and NMOS Power Gating</t>
+        </is>
+      </c>
+      <c r="C463" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Edtech Publishers (OPC) Private Limited</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>INTERNATIONAL JOURNAL OF SCIENTIFIC RESEARCH IN ENGINEERING AND MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>KUMAR, DR. N. SATHEESH; NANDINI, KAKUMANI RAJA</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr"/>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>10.55041/ijsrem60775</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.55041/ijsrem60775</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K463" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N463" t="inlineStr"/>
+      <c r="O463" t="inlineStr"/>
+      <c r="P463" t="inlineStr"/>
+      <c r="Q463" t="inlineStr">
+        <is>
+          <t>Design of a High-Speed, Low-Power Dadda Multiplier Based on XOR–XNOR Hybrid Full Adder and NMOS Power Gating</t>
+        </is>
+      </c>
+      <c r="R463" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S463" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="T463" t="inlineStr"/>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr"/>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Study of Ferroelectric Stack Thickness and Annealing Sequence Effects on GaN HEMTs with Hybrid Ferroelectric Stacks Gate</t>
+        </is>
+      </c>
+      <c r="C464" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>ACS Applied Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Liao, Po-Chuan; Chang, Hao-Wei; Rana, Siddharth; Hsiao, Chien-Nan; Seong, Tae-Yeon; Wuu, Dong-Sing; Kašalynas, Irmantas; Horng, Ray-Hua</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr"/>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>10.1021/acsaelm.6c00387</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsaelm.6c00387</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N464" t="inlineStr"/>
+      <c r="O464" t="inlineStr"/>
+      <c r="P464" t="inlineStr"/>
+      <c r="Q464" t="inlineStr">
+        <is>
+          <t>Study of Ferroelectric Stack Thickness and Annealing Sequence Effects on GaN HEMTs with Hybrid Ferroelectric Stacks Gate</t>
+        </is>
+      </c>
+      <c r="R464" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S464" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="T464" t="inlineStr"/>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr"/>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>High-performance power electronic management systems using MOSFET technology for electric vehicle energy storage</t>
+        </is>
+      </c>
+      <c r="C465" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Inderscience Publishers</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>International Journal of Power Electronics</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Basri, Omar Kanaan Al; Nnori, Fayrooz Kanaan</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr"/>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>10.1504/ijpelec.2027.10077958</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1504/ijpelec.2027.10077958</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K465" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N465" t="inlineStr"/>
+      <c r="O465" t="inlineStr"/>
+      <c r="P465" t="inlineStr"/>
+      <c r="Q465" t="inlineStr">
+        <is>
+          <t>High-performance power electronic management systems using MOSFET technology for electric vehicle energy storage</t>
+        </is>
+      </c>
+      <c r="R465" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S465" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="T465" t="inlineStr"/>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr"/>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Distance Protection for Power Grids with Inverter-Based Resources: Challenges, Probable Solutions and Future Research Opportunities</t>
+        </is>
+      </c>
+      <c r="C466" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Sarode, Gajanan; Bhatkar, Mangalkumar; Paladhi, Subhadeep</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr"/>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>10.3390/electricity7020037</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electricity7020037</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N466" t="inlineStr"/>
+      <c r="O466" t="inlineStr"/>
+      <c r="P466" t="inlineStr"/>
+      <c r="Q466" t="inlineStr">
+        <is>
+          <t>Distance Protection for Power Grids with Inverter-Based Resources: Challenges, Probable Solutions and Future Research Opportunities</t>
+        </is>
+      </c>
+      <c r="R466" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S466" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="T466" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-25T23:41Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T466"/>
+  <dimension ref="A1:T467"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35672,6 +35672,82 @@
       </c>
       <c r="T466" t="inlineStr"/>
     </row>
+    <row r="467">
+      <c r="A467" t="inlineStr"/>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Theoretical Foundations of Integrating Microservices Architecture into Monolithic Enterprise Systems</t>
+        </is>
+      </c>
+      <c r="C467" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>International Journal of Science and Research</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>International Journal of Science and Research (IJSR)</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Nadeem Mohammed, Abdul</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr"/>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>10.21275/sr26421181425</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21275/sr26421181425</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K467" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N467" t="inlineStr"/>
+      <c r="O467" t="inlineStr"/>
+      <c r="P467" t="inlineStr"/>
+      <c r="Q467" t="inlineStr">
+        <is>
+          <t>Theoretical Foundations of Integrating Microservices Architecture into Monolithic Enterprise Systems</t>
+        </is>
+      </c>
+      <c r="R467" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S467" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="T467" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-27T23:57Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T467"/>
+  <dimension ref="A1:T471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35748,6 +35748,310 @@
       </c>
       <c r="T467" t="inlineStr"/>
     </row>
+    <row r="468">
+      <c r="A468" t="inlineStr"/>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>AI ENHANCED INTELLIGENT INVERTER CONTROL USING GRNN FOR RESILIENT AC/DC HYBRID MICROGRID</t>
+        </is>
+      </c>
+      <c r="C468" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Thamilmaran, A; Shanmugam, Prabhakar Karthikeyan</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr"/>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae6553</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae6553</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N468" t="inlineStr"/>
+      <c r="O468" t="inlineStr"/>
+      <c r="P468" t="inlineStr"/>
+      <c r="Q468" t="inlineStr">
+        <is>
+          <t>AI ENHANCED INTELLIGENT INVERTER CONTROL USING GRNN FOR RESILIENT AC/DC HYBRID MICROGRID</t>
+        </is>
+      </c>
+      <c r="R468" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S468" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="T468" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr"/>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Optical gradient and translucency behavior of three multilayer monolithic zirconia systems: a spectrophotometric study</t>
+        </is>
+      </c>
+      <c r="C469" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Özişçi, Özlem</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr"/>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-50564-5</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-50564-5</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N469" t="inlineStr"/>
+      <c r="O469" t="inlineStr"/>
+      <c r="P469" t="inlineStr"/>
+      <c r="Q469" t="inlineStr">
+        <is>
+          <t>Optical gradient and translucency behavior of three multilayer monolithic zirconia systems: a spectrophotometric study</t>
+        </is>
+      </c>
+      <c r="R469" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S469" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="T469" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr"/>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>AI ENHANCED INTELLIGENT INVERTER CONTROL USING GRNN FOR RESILIENT AC/DC HYBRID MICROGRID</t>
+        </is>
+      </c>
+      <c r="C470" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Thamilmaran, A; Shanmugam, Prabhakar Karthikeyan</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr"/>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae6553</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae6553</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N470" t="inlineStr"/>
+      <c r="O470" t="inlineStr"/>
+      <c r="P470" t="inlineStr"/>
+      <c r="Q470" t="inlineStr">
+        <is>
+          <t>AI ENHANCED INTELLIGENT INVERTER CONTROL USING GRNN FOR RESILIENT AC/DC HYBRID MICROGRID</t>
+        </is>
+      </c>
+      <c r="R470" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S470" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="T470" t="inlineStr"/>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr"/>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Gate-length scaling of AlGaN/GaN HEMTs for cryogenic low-noise operation</t>
+        </is>
+      </c>
+      <c r="C471" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Mebarki, Mohamed Aniss; Ragnar, Ferrand Drake Del Castillo; Joint, François; Meledin, Denis; Sundin, Erik; Thorsell, Mattias; Rorsman, Niklas; Belitsky, Victor; Desmaris, Vincent</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr"/>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325467</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325467</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K471" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N471" t="inlineStr"/>
+      <c r="O471" t="inlineStr"/>
+      <c r="P471" t="inlineStr"/>
+      <c r="Q471" t="inlineStr">
+        <is>
+          <t>Gate-length scaling of AlGaN/GaN HEMTs for cryogenic low-noise operation</t>
+        </is>
+      </c>
+      <c r="R471" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S471" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="T471" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-28T23:57Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T471"/>
+  <dimension ref="A1:T477"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36052,6 +36052,462 @@
       </c>
       <c r="T471" t="inlineStr"/>
     </row>
+    <row r="472">
+      <c r="A472" t="inlineStr"/>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Construction Management Template on Erecting Walls from Monolithic Expanded Polystyrene Concrete</t>
+        </is>
+      </c>
+      <c r="C472" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Buildings</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Čolak, Ivo; Meneylyuk, Oleksandr; Kos, Zeljko; Nikiforov, Oleksii</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr"/>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>10.3390/buildings16091727</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/buildings16091727</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N472" t="inlineStr"/>
+      <c r="O472" t="inlineStr"/>
+      <c r="P472" t="inlineStr"/>
+      <c r="Q472" t="inlineStr">
+        <is>
+          <t>Construction Management Template on Erecting Walls from Monolithic Expanded Polystyrene Concrete</t>
+        </is>
+      </c>
+      <c r="R472" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S472" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="T472" t="inlineStr"/>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr"/>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Terahertz Antenna-Coupled Wire-Channel Field-Effect Transistors Based on AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="C473" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Moscotin, Maxim; Jorudas, Justinas; Prystawko, Pawel; Saniuk, Miroslav; Kovalevskij, Vitalij; Kašalynas, Irmantas</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr"/>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>10.3390/s26092701</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/s26092701</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K473" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N473" t="inlineStr"/>
+      <c r="O473" t="inlineStr"/>
+      <c r="P473" t="inlineStr"/>
+      <c r="Q473" t="inlineStr">
+        <is>
+          <t>Terahertz Antenna-Coupled Wire-Channel Field-Effect Transistors Based on AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="R473" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S473" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="T473" t="inlineStr"/>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr"/>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Terahertz Antenna-Coupled Wire-Channel Field-Effect Transistors Based on AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="C474" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Moscotin, Maxim; Jorudas, Justinas; Prystawko, Pawel; Saniuk, Miroslav; Kovalevskij, Vitalij; Kašalynas, Irmantas</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr"/>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>10.3390/s26092701</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/s26092701</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K474" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N474" t="inlineStr"/>
+      <c r="O474" t="inlineStr"/>
+      <c r="P474" t="inlineStr"/>
+      <c r="Q474" t="inlineStr">
+        <is>
+          <t>Terahertz Antenna-Coupled Wire-Channel Field-Effect Transistors Based on AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="R474" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S474" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="T474" t="inlineStr"/>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr"/>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Solid-state exciplex emission and logic gate behavior in modified o-carboranes</t>
+        </is>
+      </c>
+      <c r="C475" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Academia.edu Journals</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Academia Nano: Science, Materials, Technology</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Nishiyama, Shunsuke; Yanagihara, Takumi; Tanaka, Kazuo</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr"/>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>10.20935/acadnano8280</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20935/acadnano8280</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N475" t="inlineStr"/>
+      <c r="O475" t="inlineStr"/>
+      <c r="P475" t="inlineStr"/>
+      <c r="Q475" t="inlineStr">
+        <is>
+          <t>Solid-state exciplex emission and logic gate behavior in modified o-carboranes</t>
+        </is>
+      </c>
+      <c r="R475" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S475" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="T475" t="inlineStr"/>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr"/>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>pH-Dependent Luminescence of Flufenamic Acid Utilizing Molecular Logic Gate Operations</t>
+        </is>
+      </c>
+      <c r="C476" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Applied Spectroscopy</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Prachalith, N.C.; Vibha, K.; Suresh Kumar, H.M.; Thipperudrappa, J.; Khadke, Udaykumar V.</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr"/>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>10.1177/00037028261438136</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/00037028261438136</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N476" t="inlineStr"/>
+      <c r="O476" t="inlineStr"/>
+      <c r="P476" t="inlineStr"/>
+      <c r="Q476" t="inlineStr">
+        <is>
+          <t>pH-Dependent Luminescence of Flufenamic Acid Utilizing Molecular Logic Gate Operations</t>
+        </is>
+      </c>
+      <c r="R476" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S476" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="T476" t="inlineStr"/>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr"/>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Terahertz Antenna-Coupled Wire-Channel Field-Effect Transistors Based on AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="C477" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Moscotin, Maxim; Jorudas, Justinas; Prystawko, Pawel; Saniuk, Miroslav; Kovalevskij, Vitalij; Kašalynas, Irmantas</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr"/>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>10.3390/s26092701</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/s26092701</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N477" t="inlineStr"/>
+      <c r="O477" t="inlineStr"/>
+      <c r="P477" t="inlineStr"/>
+      <c r="Q477" t="inlineStr">
+        <is>
+          <t>Terahertz Antenna-Coupled Wire-Channel Field-Effect Transistors Based on AlGaN/GaN Heterostructures</t>
+        </is>
+      </c>
+      <c r="R477" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S477" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="T477" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-04-29T23:57Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T477"/>
+  <dimension ref="A1:T479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36508,6 +36508,154 @@
       </c>
       <c r="T477" t="inlineStr"/>
     </row>
+    <row r="478">
+      <c r="A478" t="inlineStr"/>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Device Optimization of Non-Ideal Ion-Sensitive Back Barrier β-(AlGa)2O3/Ga2O3 HEMT for pH Sensor application </t>
+        </is>
+      </c>
+      <c r="C478" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr"/>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Ranjan, Ravi; Kashyap, Nitesh; Raman, Ashish; Kumar, Naveen; Kumar, Prateek; Singh, Sarabdeep</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr"/>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9396349/v1</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9396349/v1</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N478" t="inlineStr"/>
+      <c r="O478" t="inlineStr"/>
+      <c r="P478" t="inlineStr"/>
+      <c r="Q478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Device Optimization of Non-Ideal Ion-Sensitive Back Barrier β-(AlGa)2O3/Ga2O3 HEMT for pH Sensor application </t>
+        </is>
+      </c>
+      <c r="R478" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S478" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="T478" t="inlineStr"/>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr"/>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Growth, electron transport, and transistors of N-polar distributed polarization-doped AlGaN channel on single-crystal AlN substrates</t>
+        </is>
+      </c>
+      <c r="C479" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Kim, Eungkyun; Yu, Changkai; Singhal, Jashan; Zhang, Zexuan; Jena, Debdeep; Xing, Huili Grace</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr"/>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>10.1063/5.0307703</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0307703</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K479" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N479" t="inlineStr"/>
+      <c r="O479" t="inlineStr"/>
+      <c r="P479" t="inlineStr"/>
+      <c r="Q479" t="inlineStr">
+        <is>
+          <t>Growth, electron transport, and transistors of N-polar distributed polarization-doped AlGaN channel on single-crystal AlN substrates</t>
+        </is>
+      </c>
+      <c r="R479" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S479" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="T479" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-05T23:51Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T479"/>
+  <dimension ref="A1:T483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36656,6 +36656,310 @@
       </c>
       <c r="T479" t="inlineStr"/>
     </row>
+    <row r="480">
+      <c r="A480" t="inlineStr"/>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Adaptation of Distributed Microservice System Patterns for In-Process Interaction in Monolithic Applications</t>
+        </is>
+      </c>
+      <c r="C480" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Universal Library Open Access Publications LLC</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>Universal Library of Multidisciplinary</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Butorin, I. D.</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr"/>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>10.70315/uloap.ulmdi.2026.0301009</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.70315/uloap.ulmdi.2026.0301009</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N480" t="inlineStr"/>
+      <c r="O480" t="inlineStr"/>
+      <c r="P480" t="inlineStr"/>
+      <c r="Q480" t="inlineStr">
+        <is>
+          <t>Adaptation of Distributed Microservice System Patterns for In-Process Interaction in Monolithic Applications</t>
+        </is>
+      </c>
+      <c r="R480" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S480" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="T480" t="inlineStr"/>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr"/>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Tool design simulation and experimental validation of a monolithic hard-shell rooftop</t>
+        </is>
+      </c>
+      <c r="C481" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Discover Vehicles</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Chirinda, Gibson P.; Matope, Stephen; Sterzing, Andreas; Nagel, Matthias</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr"/>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>10.1007/s44465-026-00016-1</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s44465-026-00016-1</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N481" t="inlineStr"/>
+      <c r="O481" t="inlineStr"/>
+      <c r="P481" t="inlineStr"/>
+      <c r="Q481" t="inlineStr">
+        <is>
+          <t>Tool design simulation and experimental validation of a monolithic hard-shell rooftop</t>
+        </is>
+      </c>
+      <c r="R481" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S481" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="T481" t="inlineStr"/>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr"/>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Sensitivity Prediction in Triple-Material Dielectric-Stack Gate-All-Around (TM-DS-GAA) MOSFET Biosensors Using Random Forest Machine Learning</t>
+        </is>
+      </c>
+      <c r="C482" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Gupta, Rashmi; Gupta, Neeraj; Kumar, Prashant</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr"/>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae68be</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae68be</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N482" t="inlineStr"/>
+      <c r="O482" t="inlineStr"/>
+      <c r="P482" t="inlineStr"/>
+      <c r="Q482" t="inlineStr">
+        <is>
+          <t>Sensitivity Prediction in Triple-Material Dielectric-Stack Gate-All-Around (TM-DS-GAA) MOSFET Biosensors Using Random Forest Machine Learning</t>
+        </is>
+      </c>
+      <c r="R482" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S482" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="T482" t="inlineStr"/>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr"/>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Sensitivity Prediction in Triple-Material Dielectric-Stack Gate-All-Around (TM-DS-GAA) MOSFET Biosensors Using Random Forest Machine Learning</t>
+        </is>
+      </c>
+      <c r="C483" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Gupta, Rashmi; Gupta, Neeraj; Kumar, Prashant</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr"/>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae68be</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae68be</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N483" t="inlineStr"/>
+      <c r="O483" t="inlineStr"/>
+      <c r="P483" t="inlineStr"/>
+      <c r="Q483" t="inlineStr">
+        <is>
+          <t>Sensitivity Prediction in Triple-Material Dielectric-Stack Gate-All-Around (TM-DS-GAA) MOSFET Biosensors Using Random Forest Machine Learning</t>
+        </is>
+      </c>
+      <c r="R483" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S483" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="T483" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-06T23:54Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T483"/>
+  <dimension ref="A1:T501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36960,6 +36960,1374 @@
       </c>
       <c r="T483" t="inlineStr"/>
     </row>
+    <row r="484">
+      <c r="A484" t="inlineStr"/>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Monolithically Integrated GaN Hysteresis Comparator Based on Complementary Logic</t>
+        </is>
+      </c>
+      <c r="C484" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Ma, Shaoyan; Jiang, Qimeng; Huang, Sen; Yang, Yang; Zhang, Xuanming; Liu, Jianfei; Liu, Wen; Wang, Xinhua; Wei, Ke; Gao, Xinguo; Cen, Lizhao; Liu, Xinyu</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr"/>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae693f</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae693f</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N484" t="inlineStr"/>
+      <c r="O484" t="inlineStr"/>
+      <c r="P484" t="inlineStr"/>
+      <c r="Q484" t="inlineStr">
+        <is>
+          <t>Monolithically Integrated GaN Hysteresis Comparator Based on Complementary Logic</t>
+        </is>
+      </c>
+      <c r="R484" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S484" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T484" t="inlineStr"/>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr"/>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Monolithically Integrated GaN Hysteresis Comparator Based on Complementary Logic</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Ma, Shaoyan; Jiang, Qimeng; Huang, Sen; Yang, Yang; Zhang, Xuanming; Liu, Jianfei; Liu, Wen; Wang, Xinhua; Wei, Ke; Gao, Xinguo; Cen, Lizhao; Liu, Xinyu</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr"/>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae693f</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae693f</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K485" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M485" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N485" t="inlineStr"/>
+      <c r="O485" t="inlineStr"/>
+      <c r="P485" t="inlineStr"/>
+      <c r="Q485" t="inlineStr">
+        <is>
+          <t>Monolithically Integrated GaN Hysteresis Comparator Based on Complementary Logic</t>
+        </is>
+      </c>
+      <c r="R485" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S485" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T485" t="inlineStr"/>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr"/>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Liao, Tsung-I; Kuo, Chun-Chih; Chang, Sheng-Po; Chen, Jone F.; Chang, Shoou-Jinn</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr"/>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N486" t="inlineStr"/>
+      <c r="O486" t="inlineStr"/>
+      <c r="P486" t="inlineStr"/>
+      <c r="Q486" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R486" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S486" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T486" t="inlineStr"/>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr"/>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>High-Responsivity 3.2 THz Detector Design and TCAD Modeling in 28 nm CMOS Technology</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Li, Wenlong; Zhang, Xin; Wang, Yongqiang; Yan, Ningning; Hou, Yuefeng; Ma, Kaixue</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr"/>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15091958</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15091958</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K487" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M487" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N487" t="inlineStr"/>
+      <c r="O487" t="inlineStr"/>
+      <c r="P487" t="inlineStr"/>
+      <c r="Q487" t="inlineStr">
+        <is>
+          <t>High-Responsivity 3.2 THz Detector Design and TCAD Modeling in 28 nm CMOS Technology</t>
+        </is>
+      </c>
+      <c r="R487" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S487" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T487" t="inlineStr"/>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr"/>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>A Novel 1.2kV GaN Trench MOSFET with Reduced Saturation Current</t>
+        </is>
+      </c>
+      <c r="C488" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Jamal, Rashid; Gupta, Parthasarathi; Rahman, Hafizur</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr"/>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae6940</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae6940</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K488" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M488" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N488" t="inlineStr"/>
+      <c r="O488" t="inlineStr"/>
+      <c r="P488" t="inlineStr"/>
+      <c r="Q488" t="inlineStr">
+        <is>
+          <t>A Novel 1.2kV GaN Trench MOSFET with Reduced Saturation Current</t>
+        </is>
+      </c>
+      <c r="R488" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S488" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T488" t="inlineStr"/>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr"/>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C489" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Liao, Tsung-I; Kuo, Chun-Chih; Chang, Sheng-Po; Chen, Jone F.; Chang, Shoou-Jinn</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr"/>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K489" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M489" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N489" t="inlineStr"/>
+      <c r="O489" t="inlineStr"/>
+      <c r="P489" t="inlineStr"/>
+      <c r="Q489" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R489" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S489" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T489" t="inlineStr"/>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr"/>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>A Novel 1.2kV GaN Trench MOSFET with Reduced Saturation Current</t>
+        </is>
+      </c>
+      <c r="C490" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Jamal, Rashid; Gupta, Parthasarathi; Rahman, Hafizur</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr"/>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae6940</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae6940</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M490" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N490" t="inlineStr"/>
+      <c r="O490" t="inlineStr"/>
+      <c r="P490" t="inlineStr"/>
+      <c r="Q490" t="inlineStr">
+        <is>
+          <t>A Novel 1.2kV GaN Trench MOSFET with Reduced Saturation Current</t>
+        </is>
+      </c>
+      <c r="R490" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S490" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T490" t="inlineStr"/>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr"/>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C491" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Liao, Tsung-I; Kuo, Chun-Chih; Chang, Sheng-Po; Chen, Jone F.; Chang, Shoou-Jinn</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr"/>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K491" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M491" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N491" t="inlineStr"/>
+      <c r="O491" t="inlineStr"/>
+      <c r="P491" t="inlineStr"/>
+      <c r="Q491" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R491" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S491" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T491" t="inlineStr"/>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr"/>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C492" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Liao, Tsung-I; Kuo, Chun-Chih; Chang, Sheng-Po; Chen, Jone F.; Chang, Shoou-Jinn</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr"/>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K492" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M492" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N492" t="inlineStr"/>
+      <c r="O492" t="inlineStr"/>
+      <c r="P492" t="inlineStr"/>
+      <c r="Q492" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R492" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S492" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T492" t="inlineStr"/>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr"/>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>A Novel 1.2kV GaN Trench MOSFET with Reduced Saturation Current</t>
+        </is>
+      </c>
+      <c r="C493" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Jamal, Rashid; Gupta, Parthasarathi; Rahman, Hafizur</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr"/>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae6940</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae6940</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M493" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N493" t="inlineStr"/>
+      <c r="O493" t="inlineStr"/>
+      <c r="P493" t="inlineStr"/>
+      <c r="Q493" t="inlineStr">
+        <is>
+          <t>A Novel 1.2kV GaN Trench MOSFET with Reduced Saturation Current</t>
+        </is>
+      </c>
+      <c r="R493" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S493" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T493" t="inlineStr"/>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr"/>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>High-Responsivity 3.2 THz Detector Design and TCAD Modeling in 28 nm CMOS Technology</t>
+        </is>
+      </c>
+      <c r="C494" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Li, Wenlong; Zhang, Xin; Wang, Yongqiang; Yan, Ningning; Hou, Yuefeng; Ma, Kaixue</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr"/>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15091958</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15091958</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M494" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N494" t="inlineStr"/>
+      <c r="O494" t="inlineStr"/>
+      <c r="P494" t="inlineStr"/>
+      <c r="Q494" t="inlineStr">
+        <is>
+          <t>High-Responsivity 3.2 THz Detector Design and TCAD Modeling in 28 nm CMOS Technology</t>
+        </is>
+      </c>
+      <c r="R494" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S494" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T494" t="inlineStr"/>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr"/>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C495" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Liao, Tsung-I; Kuo, Chun-Chih; Chang, Sheng-Po; Chen, Jone F.; Chang, Shoou-Jinn</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr"/>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K495" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M495" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N495" t="inlineStr"/>
+      <c r="O495" t="inlineStr"/>
+      <c r="P495" t="inlineStr"/>
+      <c r="Q495" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R495" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S495" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T495" t="inlineStr"/>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr"/>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>High-Responsivity 3.2 THz Detector Design and TCAD Modeling in 28 nm CMOS Technology</t>
+        </is>
+      </c>
+      <c r="C496" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Li, Wenlong; Zhang, Xin; Wang, Yongqiang; Yan, Ningning; Hou, Yuefeng; Ma, Kaixue</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr"/>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15091958</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15091958</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M496" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N496" t="inlineStr"/>
+      <c r="O496" t="inlineStr"/>
+      <c r="P496" t="inlineStr"/>
+      <c r="Q496" t="inlineStr">
+        <is>
+          <t>High-Responsivity 3.2 THz Detector Design and TCAD Modeling in 28 nm CMOS Technology</t>
+        </is>
+      </c>
+      <c r="R496" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S496" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T496" t="inlineStr"/>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr"/>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Polynomial Computation Using Multiplexer-Based Stochastic Logic in VLSI</t>
+        </is>
+      </c>
+      <c r="C497" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>International Journal for Multidisciplinary Research (IJFMR)</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>International Journal For Multidisciplinary Research</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>kumar, konda; Rajeev, Garikapati; Reddy, Kapuluru; Valarmathi, M</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr"/>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>10.36948/ijfmr.2026.v08i03.75123</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.36948/ijfmr.2026.v08i03.75123</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K497" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M497" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N497" t="inlineStr"/>
+      <c r="O497" t="inlineStr"/>
+      <c r="P497" t="inlineStr"/>
+      <c r="Q497" t="inlineStr">
+        <is>
+          <t>Polynomial Computation Using Multiplexer-Based Stochastic Logic in VLSI</t>
+        </is>
+      </c>
+      <c r="R497" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S497" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T497" t="inlineStr"/>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr"/>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C498" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Liao, Tsung-I; Kuo, Chun-Chih; Chang, Sheng-Po; Chen, Jone F.; Chang, Shoou-Jinn</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr"/>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M498" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N498" t="inlineStr"/>
+      <c r="O498" t="inlineStr"/>
+      <c r="P498" t="inlineStr"/>
+      <c r="Q498" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R498" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S498" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T498" t="inlineStr"/>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr"/>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>A high-performance quasi-solid-state supercapacitor diode for flexible logic gate</t>
+        </is>
+      </c>
+      <c r="C499" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>OAE Publishing Inc.</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Energy Materials</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Zhai, Dongmei; Yan, Zefeng; Dong, Keyi; Tang, Weiyang; Sun, Quanhu; Li, Xiao; Yang, Jiaxin; Lv, Tian; Chen, Tao</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr"/>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>10.20517/energymater.2026.11</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20517/energymater.2026.11</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K499" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M499" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N499" t="inlineStr"/>
+      <c r="O499" t="inlineStr"/>
+      <c r="P499" t="inlineStr"/>
+      <c r="Q499" t="inlineStr">
+        <is>
+          <t>A high-performance quasi-solid-state supercapacitor diode for flexible logic gate</t>
+        </is>
+      </c>
+      <c r="R499" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S499" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T499" t="inlineStr"/>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr"/>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Monolithically Integrated GaN Hysteresis Comparator Based on Complementary Logic</t>
+        </is>
+      </c>
+      <c r="C500" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Ma, Shaoyan; Jiang, Qimeng; Huang, Sen; Yang, Yang; Zhang, Xuanming; Liu, Jianfei; Liu, Wen; Wang, Xinhua; Wei, Ke; Gao, Xinguo; Cen, Lizhao; Liu, Xinyu</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr"/>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae693f</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae693f</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M500" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N500" t="inlineStr"/>
+      <c r="O500" t="inlineStr"/>
+      <c r="P500" t="inlineStr"/>
+      <c r="Q500" t="inlineStr">
+        <is>
+          <t>Monolithically Integrated GaN Hysteresis Comparator Based on Complementary Logic</t>
+        </is>
+      </c>
+      <c r="R500" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S500" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T500" t="inlineStr"/>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr"/>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C501" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Liao, Tsung-I; Kuo, Chun-Chih; Chang, Sheng-Po; Chen, Jone F.; Chang, Shoou-Jinn</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr"/>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae6948</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M501" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N501" t="inlineStr"/>
+      <c r="O501" t="inlineStr"/>
+      <c r="P501" t="inlineStr"/>
+      <c r="Q501" t="inlineStr">
+        <is>
+          <t>TCAD Analysis of Etching-Depth-Dependent Electrical Behavior in p-GaN Gate AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R501" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S501" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="T501" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-07T23:56Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T501"/>
+  <dimension ref="A1:T508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38328,6 +38328,538 @@
       </c>
       <c r="T501" t="inlineStr"/>
     </row>
+    <row r="502">
+      <c r="A502" t="inlineStr"/>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>CMOS inverter on flexible plastic substrate using junctionless double-gate polycrystalline Ge thin-film transistors fabricated via Cu-based metal-induced crystallization</t>
+        </is>
+      </c>
+      <c r="C502" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Kurihara, Akito; Okuyama, Tetsuo; Tsuchiya, Toshiyuki; Hara, Akito</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr"/>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae6a56</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae6a56</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M502" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N502" t="inlineStr"/>
+      <c r="O502" t="inlineStr"/>
+      <c r="P502" t="inlineStr"/>
+      <c r="Q502" t="inlineStr">
+        <is>
+          <t>CMOS inverter on flexible plastic substrate using junctionless double-gate polycrystalline Ge thin-film transistors fabricated via Cu-based metal-induced crystallization</t>
+        </is>
+      </c>
+      <c r="R502" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S502" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="T502" t="inlineStr"/>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr"/>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Strategies for Migrating Monolithic Enterprise Applications to Modular Microservices Architecture</t>
+        </is>
+      </c>
+      <c r="C503" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>European International Journal of Multidisciplinary Research and Management Studies</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>International Journal of Computer Science &amp;amp; Information System</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Abduaziz, Abdukhalimov</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr"/>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>10.55640/ijcsis/volume11issue05-02</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.55640/ijcsis/volume11issue05-02</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M503" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N503" t="inlineStr"/>
+      <c r="O503" t="inlineStr"/>
+      <c r="P503" t="inlineStr"/>
+      <c r="Q503" t="inlineStr">
+        <is>
+          <t>Strategies for Migrating Monolithic Enterprise Applications to Modular Microservices Architecture</t>
+        </is>
+      </c>
+      <c r="R503" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S503" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="T503" t="inlineStr"/>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr"/>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Enhancement-mode AlN/GaN/AlN HEMTs</t>
+        </is>
+      </c>
+      <c r="C504" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>Applied Physics Express</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Chen, Yu-Hsin; Nomoto, Kazuki; Chaudhuri, Reet; Encomendero, Jimy; Agrawal, Shivali; Kim, Eungkyun; Kim, Jeongwoo; Ma, Siyuan; Xing, Huili G.; Jena, Debdeep</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr"/>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>10.35848/1882-0786/ae6a5b</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1882-0786/ae6a5b</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K504" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M504" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N504" t="inlineStr"/>
+      <c r="O504" t="inlineStr"/>
+      <c r="P504" t="inlineStr"/>
+      <c r="Q504" t="inlineStr">
+        <is>
+          <t>Enhancement-mode AlN/GaN/AlN HEMTs</t>
+        </is>
+      </c>
+      <c r="R504" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S504" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="T504" t="inlineStr"/>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr"/>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>HPM-Induced Damage Mechanisms and Protection Strategies for AlGaN/GaN HEMTs with Graded Al Barriers and Gate-Misaligned Designs</t>
+        </is>
+      </c>
+      <c r="C505" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>Gao, Sheng; Yuan, Jiancheng; Jing, Liang; Wang, Manjing; Wang, Qi</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr"/>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae6a16</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae6a16</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K505" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M505" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N505" t="inlineStr"/>
+      <c r="O505" t="inlineStr"/>
+      <c r="P505" t="inlineStr"/>
+      <c r="Q505" t="inlineStr">
+        <is>
+          <t>HPM-Induced Damage Mechanisms and Protection Strategies for AlGaN/GaN HEMTs with Graded Al Barriers and Gate-Misaligned Designs</t>
+        </is>
+      </c>
+      <c r="R505" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S505" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="T505" t="inlineStr"/>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr"/>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>HPM-Induced Damage Mechanisms and Protection Strategies for AlGaN/GaN HEMTs with Graded Al Barriers and Gate-Misaligned Designs</t>
+        </is>
+      </c>
+      <c r="C506" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Gao, Sheng; Yuan, Jiancheng; Jing, Liang; Wang, Manjing; Wang, Qi</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr"/>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae6a16</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae6a16</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K506" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M506" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N506" t="inlineStr"/>
+      <c r="O506" t="inlineStr"/>
+      <c r="P506" t="inlineStr"/>
+      <c r="Q506" t="inlineStr">
+        <is>
+          <t>HPM-Induced Damage Mechanisms and Protection Strategies for AlGaN/GaN HEMTs with Graded Al Barriers and Gate-Misaligned Designs</t>
+        </is>
+      </c>
+      <c r="R506" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S506" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="T506" t="inlineStr"/>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr"/>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Strategies for Migrating Monolithic Enterprise Applications to Modular Microservices Architecture</t>
+        </is>
+      </c>
+      <c r="C507" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>European International Journal of Multidisciplinary Research and Management Studies</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>International Journal of Computer Science &amp;amp; Information System</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Abduaziz, Abdukhalimov</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr"/>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>10.55640/ijcsis/volume11issue05-02</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.55640/ijcsis/volume11issue05-02</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K507" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M507" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N507" t="inlineStr"/>
+      <c r="O507" t="inlineStr"/>
+      <c r="P507" t="inlineStr"/>
+      <c r="Q507" t="inlineStr">
+        <is>
+          <t>Strategies for Migrating Monolithic Enterprise Applications to Modular Microservices Architecture</t>
+        </is>
+      </c>
+      <c r="R507" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S507" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="T507" t="inlineStr"/>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr"/>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>HPM-Induced Damage Mechanisms and Protection Strategies for AlGaN/GaN HEMTs with Graded Al Barriers and Gate-Misaligned Designs</t>
+        </is>
+      </c>
+      <c r="C508" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Gao, Sheng; Yuan, Jiancheng; Jing, Liang; Wang, Manjing; Wang, Qi</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr"/>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae6a16</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae6a16</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K508" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M508" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N508" t="inlineStr"/>
+      <c r="O508" t="inlineStr"/>
+      <c r="P508" t="inlineStr"/>
+      <c r="Q508" t="inlineStr">
+        <is>
+          <t>HPM-Induced Damage Mechanisms and Protection Strategies for AlGaN/GaN HEMTs with Graded Al Barriers and Gate-Misaligned Designs</t>
+        </is>
+      </c>
+      <c r="R508" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S508" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="T508" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-08T23:59Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T508"/>
+  <dimension ref="A1:T510"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38860,6 +38860,158 @@
       </c>
       <c r="T508" t="inlineStr"/>
     </row>
+    <row r="509">
+      <c r="A509" t="inlineStr"/>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Monolithically integrated GaN MicroLED and microfluidic channel probe for simultaneous optogenetic stimulation and drug delivery</t>
+        </is>
+      </c>
+      <c r="C509" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>Oya, Kakeru; Kai, Nobuyuki; Shinohara, Gota; Ishikawa, Mikiko; Nishikawa, Atsushi; Loesing, Alexander; Ohkawa, Noriaki; SEKIGUCHI, Hiroto</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr"/>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae6ae8</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae6ae8</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K509" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M509" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N509" t="inlineStr"/>
+      <c r="O509" t="inlineStr"/>
+      <c r="P509" t="inlineStr"/>
+      <c r="Q509" t="inlineStr">
+        <is>
+          <t>Monolithically integrated GaN MicroLED and microfluidic channel probe for simultaneous optogenetic stimulation and drug delivery</t>
+        </is>
+      </c>
+      <c r="R509" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S509" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="T509" t="inlineStr"/>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr"/>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Monolithically integrated GaN MicroLED and microfluidic channel probe for simultaneous optogenetic stimulation and drug delivery</t>
+        </is>
+      </c>
+      <c r="C510" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>Oya, Kakeru; Kai, Nobuyuki; Shinohara, Gota; Ishikawa, Mikiko; Nishikawa, Atsushi; Loesing, Alexander; Ohkawa, Noriaki; SEKIGUCHI, Hiroto</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr"/>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae6ae8</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae6ae8</t>
+        </is>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K510" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M510" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N510" t="inlineStr"/>
+      <c r="O510" t="inlineStr"/>
+      <c r="P510" t="inlineStr"/>
+      <c r="Q510" t="inlineStr">
+        <is>
+          <t>Monolithically integrated GaN MicroLED and microfluidic channel probe for simultaneous optogenetic stimulation and drug delivery</t>
+        </is>
+      </c>
+      <c r="R510" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S510" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="T510" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-09T23:53Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T510"/>
+  <dimension ref="A1:T513"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39012,6 +39012,222 @@
       </c>
       <c r="T510" t="inlineStr"/>
     </row>
+    <row r="511">
+      <c r="A511" t="inlineStr"/>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Correction to “Large‐Scale Fabrication of Meta‐Axicon With Circular Polarization on CMOS Platform”</t>
+        </is>
+      </c>
+      <c r="C511" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Nanophotonics</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr"/>
+      <c r="G511" t="inlineStr"/>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>10.1002/nap2.70127</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/nap2.70127</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K511" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M511" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N511" t="inlineStr"/>
+      <c r="O511" t="inlineStr"/>
+      <c r="P511" t="inlineStr"/>
+      <c r="Q511" t="inlineStr">
+        <is>
+          <t>Correction to “Large‐Scale Fabrication of Meta‐Axicon With Circular Polarization on CMOS Platform”</t>
+        </is>
+      </c>
+      <c r="R511" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S511" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="T511" t="inlineStr"/>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr"/>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Correction to “Large‐Scale Fabrication of Meta‐Axicon With Circular Polarization on CMOS Platform”</t>
+        </is>
+      </c>
+      <c r="C512" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Nanophotonics</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr"/>
+      <c r="G512" t="inlineStr"/>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>10.1002/nap2.70127</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/nap2.70127</t>
+        </is>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K512" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M512" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N512" t="inlineStr"/>
+      <c r="O512" t="inlineStr"/>
+      <c r="P512" t="inlineStr"/>
+      <c r="Q512" t="inlineStr">
+        <is>
+          <t>Correction to “Large‐Scale Fabrication of Meta‐Axicon With Circular Polarization on CMOS Platform”</t>
+        </is>
+      </c>
+      <c r="R512" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S512" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="T512" t="inlineStr"/>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr"/>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Correction to “Large‐Scale Fabrication of Meta‐Axicon With Circular Polarization on CMOS Platform”</t>
+        </is>
+      </c>
+      <c r="C513" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Nanophotonics</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr"/>
+      <c r="G513" t="inlineStr"/>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>10.1002/nap2.70127</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/nap2.70127</t>
+        </is>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K513" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M513" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N513" t="inlineStr"/>
+      <c r="O513" t="inlineStr"/>
+      <c r="P513" t="inlineStr"/>
+      <c r="Q513" t="inlineStr">
+        <is>
+          <t>Correction to “Large‐Scale Fabrication of Meta‐Axicon With Circular Polarization on CMOS Platform”</t>
+        </is>
+      </c>
+      <c r="R513" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S513" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="T513" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-13T00:03Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T513"/>
+  <dimension ref="A1:T524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39228,6 +39228,818 @@
       </c>
       <c r="T513" t="inlineStr"/>
     </row>
+    <row r="514">
+      <c r="A514" t="inlineStr"/>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Ballistic Transport in n-type MoTe2 Junctionless Gate-All-Around Nanowire FETs: Temperature-Dependent Performance, CMOS Complementarity, and Benchmarking</t>
+        </is>
+      </c>
+      <c r="C514" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr"/>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>Majumdar, SANDIP</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr"/>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>10.22541/authorea.15003102/v1</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22541/authorea.15003102/v1</t>
+        </is>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K514" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M514" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N514" t="inlineStr"/>
+      <c r="O514" t="inlineStr"/>
+      <c r="P514" t="inlineStr"/>
+      <c r="Q514" t="inlineStr">
+        <is>
+          <t>Ballistic Transport in n-type MoTe2 Junctionless Gate-All-Around Nanowire FETs: Temperature-Dependent Performance, CMOS Complementarity, and Benchmarking</t>
+        </is>
+      </c>
+      <c r="R514" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S514" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T514" t="inlineStr"/>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr"/>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>A Compendium of Reporting Guidelines for Traditional, Complementary, and Integrative Medicine from the Enhancing the QUAlity and Transparency Of health Research (EQUATOR) Network</t>
+        </is>
+      </c>
+      <c r="C515" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Walter de Gruyter GmbH</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Journal of Complementary and Integrative Medicine</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>Ng, Jeremy Y.; Syed, Niveen; Moher, David</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr"/>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>10.1515/jcim-2026-0073</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1515/jcim-2026-0073</t>
+        </is>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K515" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M515" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N515" t="inlineStr"/>
+      <c r="O515" t="inlineStr"/>
+      <c r="P515" t="inlineStr"/>
+      <c r="Q515" t="inlineStr">
+        <is>
+          <t>A Compendium of Reporting Guidelines for Traditional, Complementary, and Integrative Medicine from the Enhancing the QUAlity and Transparency Of health Research (EQUATOR) Network</t>
+        </is>
+      </c>
+      <c r="R515" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S515" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T515" t="inlineStr"/>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr"/>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Ballistic Transport in n-type MoTe2 Junctionless Gate-All-Around Nanowire FETs: Temperature-Dependent Performance, CMOS Complementarity, and Benchmarking</t>
+        </is>
+      </c>
+      <c r="C516" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr"/>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>Majumdar, SANDIP</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr"/>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>10.22541/authorea.15003102/v1</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22541/authorea.15003102/v1</t>
+        </is>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K516" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M516" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N516" t="inlineStr"/>
+      <c r="O516" t="inlineStr"/>
+      <c r="P516" t="inlineStr"/>
+      <c r="Q516" t="inlineStr">
+        <is>
+          <t>Ballistic Transport in n-type MoTe2 Junctionless Gate-All-Around Nanowire FETs: Temperature-Dependent Performance, CMOS Complementarity, and Benchmarking</t>
+        </is>
+      </c>
+      <c r="R516" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S516" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T516" t="inlineStr"/>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr"/>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Cross-Platform Experimental Validation of Multi-Stage Adaptive Gate Driving for MOSFET Switching Loss Reduction in Transformer Boost Circuits</t>
+        </is>
+      </c>
+      <c r="C517" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr"/>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>CHENG, Jiale; WANG, Yabin; WANG, Zhongyu; SUN, Hao; ZHANG, Haibo; GUO, Fang</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr"/>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9439736/v1</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9439736/v1</t>
+        </is>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K517" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M517" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N517" t="inlineStr"/>
+      <c r="O517" t="inlineStr"/>
+      <c r="P517" t="inlineStr"/>
+      <c r="Q517" t="inlineStr">
+        <is>
+          <t>Cross-Platform Experimental Validation of Multi-Stage Adaptive Gate Driving for MOSFET Switching Loss Reduction in Transformer Boost Circuits</t>
+        </is>
+      </c>
+      <c r="R517" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S517" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T517" t="inlineStr"/>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr"/>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Cross-Platform Experimental Validation of Multi-Stage Adaptive Gate Driving for MOSFET Switching Loss Reduction in Transformer Boost Circuits</t>
+        </is>
+      </c>
+      <c r="C518" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr"/>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>CHENG, Jiale; WANG, Yabin; WANG, Zhongyu; SUN, Hao; ZHANG, Haibo; GUO, Fang</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr"/>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9439736/v1</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9439736/v1</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K518" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M518" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N518" t="inlineStr"/>
+      <c r="O518" t="inlineStr"/>
+      <c r="P518" t="inlineStr"/>
+      <c r="Q518" t="inlineStr">
+        <is>
+          <t>Cross-Platform Experimental Validation of Multi-Stage Adaptive Gate Driving for MOSFET Switching Loss Reduction in Transformer Boost Circuits</t>
+        </is>
+      </c>
+      <c r="R518" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S518" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T518" t="inlineStr"/>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr"/>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Cross-Platform Experimental Validation of Multi-Stage Adaptive Gate Driving for MOSFET Switching Loss Reduction in Transformer Boost Circuits</t>
+        </is>
+      </c>
+      <c r="C519" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr"/>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>CHENG, Jiale; WANG, Yabin; WANG, Zhongyu; SUN, Hao; ZHANG, Haibo; GUO, Fang</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr"/>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9439736/v1</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9439736/v1</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K519" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L519" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M519" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N519" t="inlineStr"/>
+      <c r="O519" t="inlineStr"/>
+      <c r="P519" t="inlineStr"/>
+      <c r="Q519" t="inlineStr">
+        <is>
+          <t>Cross-Platform Experimental Validation of Multi-Stage Adaptive Gate Driving for MOSFET Switching Loss Reduction in Transformer Boost Circuits</t>
+        </is>
+      </c>
+      <c r="R519" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S519" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T519" t="inlineStr"/>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr"/>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Dynamic characteristic of 1200V p-GaN HEMT with ±20V gate operating range on the Si Substrates</t>
+        </is>
+      </c>
+      <c r="C520" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>Zhao, Yaopeng; Hao, Jiamao; Shi, Jiahao; Luo, Pan; Li, Ang; Luo, Jingtao; Wang, Chong; Wang, Jianyuan; Liu, Kai; Yang, Lei; Wen, Haibing; Tan, Cher Ming</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr"/>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae67bb</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae67bb</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K520" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L520" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M520" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N520" t="inlineStr"/>
+      <c r="O520" t="inlineStr"/>
+      <c r="P520" t="inlineStr"/>
+      <c r="Q520" t="inlineStr">
+        <is>
+          <t>Dynamic characteristic of 1200V p-GaN HEMT with ±20V gate operating range on the Si Substrates</t>
+        </is>
+      </c>
+      <c r="R520" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S520" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T520" t="inlineStr"/>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr"/>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Ballistic Transport in n-type MoTe2 Junctionless Gate-All-Around Nanowire FETs: Temperature-Dependent Performance, CMOS Complementarity, and Benchmarking</t>
+        </is>
+      </c>
+      <c r="C521" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr"/>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>Majumdar, SANDIP</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr"/>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>10.22541/authorea.15003102/v1</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22541/authorea.15003102/v1</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K521" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M521" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N521" t="inlineStr"/>
+      <c r="O521" t="inlineStr"/>
+      <c r="P521" t="inlineStr"/>
+      <c r="Q521" t="inlineStr">
+        <is>
+          <t>Ballistic Transport in n-type MoTe2 Junctionless Gate-All-Around Nanowire FETs: Temperature-Dependent Performance, CMOS Complementarity, and Benchmarking</t>
+        </is>
+      </c>
+      <c r="R521" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S521" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T521" t="inlineStr"/>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr"/>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Dynamic characteristic of 1200V p-GaN HEMT with ±20V gate operating range on the Si Substrates</t>
+        </is>
+      </c>
+      <c r="C522" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>Zhao, Yaopeng; Hao, Jiamao; Shi, Jiahao; Luo, Pan; Li, Ang; Luo, Jingtao; Wang, Chong; Wang, Jianyuan; Liu, Kai; Yang, Lei; Wen, Haibing; Tan, Cher Ming</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr"/>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae67bb</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae67bb</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K522" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L522" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M522" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N522" t="inlineStr"/>
+      <c r="O522" t="inlineStr"/>
+      <c r="P522" t="inlineStr"/>
+      <c r="Q522" t="inlineStr">
+        <is>
+          <t>Dynamic characteristic of 1200V p-GaN HEMT with ±20V gate operating range on the Si Substrates</t>
+        </is>
+      </c>
+      <c r="R522" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S522" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T522" t="inlineStr"/>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr"/>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Diffusion of contact metals in GaN/AlGaN stacks</t>
+        </is>
+      </c>
+      <c r="C523" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>Bilke, Marie-Louise; Siegrist, Theo; Gärtner, Jan; Szabo, Nadine; Großer, Andreas; Mikolajick, Thomas; Schmult, Stefan</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr"/>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>10.1063/5.0316421</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0316421</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K523" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L523" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M523" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N523" t="inlineStr"/>
+      <c r="O523" t="inlineStr"/>
+      <c r="P523" t="inlineStr"/>
+      <c r="Q523" t="inlineStr">
+        <is>
+          <t>Diffusion of contact metals in GaN/AlGaN stacks</t>
+        </is>
+      </c>
+      <c r="R523" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S523" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T523" t="inlineStr"/>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr"/>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Diffusion of contact metals in GaN/AlGaN stacks</t>
+        </is>
+      </c>
+      <c r="C524" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>Bilke, Marie-Louise; Siegrist, Theo; Gärtner, Jan; Szabo, Nadine; Großer, Andreas; Mikolajick, Thomas; Schmult, Stefan</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr"/>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>10.1063/5.0316421</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0316421</t>
+        </is>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K524" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L524" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M524" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N524" t="inlineStr"/>
+      <c r="O524" t="inlineStr"/>
+      <c r="P524" t="inlineStr"/>
+      <c r="Q524" t="inlineStr">
+        <is>
+          <t>Diffusion of contact metals in GaN/AlGaN stacks</t>
+        </is>
+      </c>
+      <c r="R524" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S524" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="T524" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-14T00:03Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T524"/>
+  <dimension ref="A1:T529"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40040,6 +40040,386 @@
       </c>
       <c r="T524" t="inlineStr"/>
     </row>
+    <row r="525">
+      <c r="A525" t="inlineStr"/>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Validated Instruments for Measuring Health Literacy Among Traditional, Complementary, and Integrative Medicine Users: A Critical, Systematic Review</t>
+        </is>
+      </c>
+      <c r="C525" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>Carter, Tristan; Foley, Hope; Adams, Jon; Graham, Kim; Steel, Amie</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr"/>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261445329</t>
+        </is>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261445329</t>
+        </is>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K525" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L525" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M525" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N525" t="inlineStr"/>
+      <c r="O525" t="inlineStr"/>
+      <c r="P525" t="inlineStr"/>
+      <c r="Q525" t="inlineStr">
+        <is>
+          <t>Validated Instruments for Measuring Health Literacy Among Traditional, Complementary, and Integrative Medicine Users: A Critical, Systematic Review</t>
+        </is>
+      </c>
+      <c r="R525" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S525" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="T525" t="inlineStr"/>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr"/>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Validated Instruments for Measuring Health Literacy Among Traditional, Complementary, and Integrative Medicine Users: A Critical, Systematic Review</t>
+        </is>
+      </c>
+      <c r="C526" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>Carter, Tristan; Foley, Hope; Adams, Jon; Graham, Kim; Steel, Amie</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr"/>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261445329</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261445329</t>
+        </is>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K526" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L526" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M526" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N526" t="inlineStr"/>
+      <c r="O526" t="inlineStr"/>
+      <c r="P526" t="inlineStr"/>
+      <c r="Q526" t="inlineStr">
+        <is>
+          <t>Validated Instruments for Measuring Health Literacy Among Traditional, Complementary, and Integrative Medicine Users: A Critical, Systematic Review</t>
+        </is>
+      </c>
+      <c r="R526" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S526" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="T526" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr"/>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Reconfigurable logic MOSFET based on bidirectional single-transistor latch operation</t>
+        </is>
+      </c>
+      <c r="C527" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>Lim, Doohyeok</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr"/>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae6d45</t>
+        </is>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae6d45</t>
+        </is>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K527" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L527" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M527" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N527" t="inlineStr"/>
+      <c r="O527" t="inlineStr"/>
+      <c r="P527" t="inlineStr"/>
+      <c r="Q527" t="inlineStr">
+        <is>
+          <t>Reconfigurable logic MOSFET based on bidirectional single-transistor latch operation</t>
+        </is>
+      </c>
+      <c r="R527" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S527" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="T527" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr"/>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Reconfigurable logic MOSFET based on bidirectional single-transistor latch operation</t>
+        </is>
+      </c>
+      <c r="C528" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>Lim, Doohyeok</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr"/>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae6d45</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae6d45</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K528" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L528" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M528" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N528" t="inlineStr"/>
+      <c r="O528" t="inlineStr"/>
+      <c r="P528" t="inlineStr"/>
+      <c r="Q528" t="inlineStr">
+        <is>
+          <t>Reconfigurable logic MOSFET based on bidirectional single-transistor latch operation</t>
+        </is>
+      </c>
+      <c r="R528" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S528" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="T528" t="inlineStr"/>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr"/>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Reconfigurable logic MOSFET based on bidirectional single-transistor latch operation</t>
+        </is>
+      </c>
+      <c r="C529" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>Lim, Doohyeok</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr"/>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae6d45</t>
+        </is>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae6d45</t>
+        </is>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K529" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L529" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M529" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N529" t="inlineStr"/>
+      <c r="O529" t="inlineStr"/>
+      <c r="P529" t="inlineStr"/>
+      <c r="Q529" t="inlineStr">
+        <is>
+          <t>Reconfigurable logic MOSFET based on bidirectional single-transistor latch operation</t>
+        </is>
+      </c>
+      <c r="R529" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S529" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="T529" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-15T00:00Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T529"/>
+  <dimension ref="A1:T530"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40420,6 +40420,82 @@
       </c>
       <c r="T529" t="inlineStr"/>
     </row>
+    <row r="530">
+      <c r="A530" t="inlineStr"/>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Mechanically Driven, Self‐Powered Hydrogel Iontronics for Visualized Tactile Logic Gate Circuit</t>
+        </is>
+      </c>
+      <c r="C530" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>Ouyang, Yaowen; Xiang, Xing; Zhang, Yuyang; Li, Xiang; Zhou, Yanguang; Wang, Zhong Lin; Wei, Di</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr"/>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>10.1002/smll.73728</t>
+        </is>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/smll.73728</t>
+        </is>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K530" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L530" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M530" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N530" t="inlineStr"/>
+      <c r="O530" t="inlineStr"/>
+      <c r="P530" t="inlineStr"/>
+      <c r="Q530" t="inlineStr">
+        <is>
+          <t>Mechanically Driven, Self‐Powered Hydrogel Iontronics for Visualized Tactile Logic Gate Circuit</t>
+        </is>
+      </c>
+      <c r="R530" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S530" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="T530" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-15T23:56Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T530"/>
+  <dimension ref="A1:T540"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40496,6 +40496,754 @@
       </c>
       <c r="T530" t="inlineStr"/>
     </row>
+    <row r="531">
+      <c r="A531" t="inlineStr"/>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Technical, Regulatory, and Market Challenges of 100% Inverter-Based Grids: A Review</t>
+        </is>
+      </c>
+      <c r="C531" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>Mostova, Viktoriya; Vaccaro, Alfredo</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr"/>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>10.3390/en19102375</t>
+        </is>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19102375</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K531" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L531" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M531" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N531" t="inlineStr"/>
+      <c r="O531" t="inlineStr"/>
+      <c r="P531" t="inlineStr"/>
+      <c r="Q531" t="inlineStr">
+        <is>
+          <t>Technical, Regulatory, and Market Challenges of 100% Inverter-Based Grids: A Review</t>
+        </is>
+      </c>
+      <c r="R531" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S531" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T531" t="inlineStr"/>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr"/>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Sensorless Control of Compressor Motor Considering Inverter Nonlinearities and Parameter Estimation</t>
+        </is>
+      </c>
+      <c r="C532" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>Sapmaz, Tunahan; Bakan, Ahmet Faruk</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr"/>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>10.3390/en19102374</t>
+        </is>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19102374</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K532" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L532" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M532" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N532" t="inlineStr"/>
+      <c r="O532" t="inlineStr"/>
+      <c r="P532" t="inlineStr"/>
+      <c r="Q532" t="inlineStr">
+        <is>
+          <t>Sensorless Control of Compressor Motor Considering Inverter Nonlinearities and Parameter Estimation</t>
+        </is>
+      </c>
+      <c r="R532" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S532" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T532" t="inlineStr"/>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr"/>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Cell-scale autonomous CMOS motes for intracellular bioelectronics</t>
+        </is>
+      </c>
+      <c r="C533" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>openRxiv</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr"/>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>Ramakrishnan, Girish; Cardoso, Filipe Arroyo; Stoy, William; Andino-Pavlovsky, Vicky; Goes, Joaquim; Shepard, Kenneth</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr"/>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>10.64898/2026.05.12.724193</t>
+        </is>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.05.12.724193</t>
+        </is>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K533" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L533" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M533" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N533" t="inlineStr"/>
+      <c r="O533" t="inlineStr"/>
+      <c r="P533" t="inlineStr"/>
+      <c r="Q533" t="inlineStr">
+        <is>
+          <t>Cell-scale autonomous CMOS motes for intracellular bioelectronics</t>
+        </is>
+      </c>
+      <c r="R533" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S533" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T533" t="inlineStr"/>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr"/>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Cell-scale autonomous CMOS motes for intracellular bioelectronics</t>
+        </is>
+      </c>
+      <c r="C534" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>openRxiv</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr"/>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>Ramakrishnan, Girish; Cardoso, Filipe Arroyo; Stoy, William; Andino-Pavlovsky, Vicky; Goes, Joaquim; Shepard, Kenneth</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr"/>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>10.64898/2026.05.12.724193</t>
+        </is>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.05.12.724193</t>
+        </is>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K534" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L534" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M534" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N534" t="inlineStr"/>
+      <c r="O534" t="inlineStr"/>
+      <c r="P534" t="inlineStr"/>
+      <c r="Q534" t="inlineStr">
+        <is>
+          <t>Cell-scale autonomous CMOS motes for intracellular bioelectronics</t>
+        </is>
+      </c>
+      <c r="R534" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S534" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T534" t="inlineStr"/>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr"/>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Technical, Regulatory, and Market Challenges of 100% Inverter-Based Grids: A Review</t>
+        </is>
+      </c>
+      <c r="C535" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>Mostova, Viktoriya; Vaccaro, Alfredo</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr"/>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>10.3390/en19102375</t>
+        </is>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19102375</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K535" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L535" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M535" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N535" t="inlineStr"/>
+      <c r="O535" t="inlineStr"/>
+      <c r="P535" t="inlineStr"/>
+      <c r="Q535" t="inlineStr">
+        <is>
+          <t>Technical, Regulatory, and Market Challenges of 100% Inverter-Based Grids: A Review</t>
+        </is>
+      </c>
+      <c r="R535" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S535" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T535" t="inlineStr"/>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr"/>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Sensorless Control of Compressor Motor Considering Inverter Nonlinearities and Parameter Estimation</t>
+        </is>
+      </c>
+      <c r="C536" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>Sapmaz, Tunahan; Bakan, Ahmet Faruk</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr"/>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>10.3390/en19102374</t>
+        </is>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19102374</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K536" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L536" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M536" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N536" t="inlineStr"/>
+      <c r="O536" t="inlineStr"/>
+      <c r="P536" t="inlineStr"/>
+      <c r="Q536" t="inlineStr">
+        <is>
+          <t>Sensorless Control of Compressor Motor Considering Inverter Nonlinearities and Parameter Estimation</t>
+        </is>
+      </c>
+      <c r="R536" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S536" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T536" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr"/>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Cell-scale autonomous CMOS motes for intracellular bioelectronics</t>
+        </is>
+      </c>
+      <c r="C537" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>openRxiv</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr"/>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>Ramakrishnan, Girish; Cardoso, Filipe Arroyo; Stoy, William; Andino-Pavlovsky, Vicky; Goes, Joaquim; Shepard, Kenneth</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr"/>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>10.64898/2026.05.12.724193</t>
+        </is>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.05.12.724193</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K537" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L537" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M537" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N537" t="inlineStr"/>
+      <c r="O537" t="inlineStr"/>
+      <c r="P537" t="inlineStr"/>
+      <c r="Q537" t="inlineStr">
+        <is>
+          <t>Cell-scale autonomous CMOS motes for intracellular bioelectronics</t>
+        </is>
+      </c>
+      <c r="R537" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S537" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T537" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr"/>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Technical, Regulatory, and Market Challenges of 100% Inverter-Based Grids: A Review</t>
+        </is>
+      </c>
+      <c r="C538" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>Mostova, Viktoriya; Vaccaro, Alfredo</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr"/>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>10.3390/en19102375</t>
+        </is>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19102375</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K538" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L538" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M538" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N538" t="inlineStr"/>
+      <c r="O538" t="inlineStr"/>
+      <c r="P538" t="inlineStr"/>
+      <c r="Q538" t="inlineStr">
+        <is>
+          <t>Technical, Regulatory, and Market Challenges of 100% Inverter-Based Grids: A Review</t>
+        </is>
+      </c>
+      <c r="R538" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S538" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T538" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr"/>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Sensorless Control of Compressor Motor Considering Inverter Nonlinearities and Parameter Estimation</t>
+        </is>
+      </c>
+      <c r="C539" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>Sapmaz, Tunahan; Bakan, Ahmet Faruk</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr"/>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>10.3390/en19102374</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19102374</t>
+        </is>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K539" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L539" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M539" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N539" t="inlineStr"/>
+      <c r="O539" t="inlineStr"/>
+      <c r="P539" t="inlineStr"/>
+      <c r="Q539" t="inlineStr">
+        <is>
+          <t>Sensorless Control of Compressor Motor Considering Inverter Nonlinearities and Parameter Estimation</t>
+        </is>
+      </c>
+      <c r="R539" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S539" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T539" t="inlineStr"/>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr"/>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Effects of 673K Temperature Anneal on a 4H-SiC CMOS NOT Logic Gate</t>
+        </is>
+      </c>
+      <c r="C540" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Materials Science Forum</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>Rinaldi, Nicola; di Benedetto, Luigi; Rommel, Mathias; May, Alexander; Baier, Leander; Liguori, Rosalba; Rubino, Alfredo; Licciardo, Gian Domenico</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr"/>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>10.4028/p-4zjeap</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-4zjeap</t>
+        </is>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K540" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L540" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M540" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N540" t="inlineStr"/>
+      <c r="O540" t="inlineStr"/>
+      <c r="P540" t="inlineStr"/>
+      <c r="Q540" t="inlineStr">
+        <is>
+          <t>Effects of 673K Temperature Anneal on a 4H-SiC CMOS NOT Logic Gate</t>
+        </is>
+      </c>
+      <c r="R540" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S540" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="T540" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-17T23:59Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T540"/>
+  <dimension ref="A1:T542"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41244,6 +41244,158 @@
       </c>
       <c r="T540" t="inlineStr"/>
     </row>
+    <row r="541">
+      <c r="A541" t="inlineStr"/>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Numerical simulation and modeling of HgCdTe and MoS₂ heterostructure MOSFET using polynomial fitting extrapolation technique</t>
+        </is>
+      </c>
+      <c r="C541" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Micro and Nanostructures</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>Malu, U.; Pravin, J. Charles; Babu, A. Ramesh</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr"/>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>10.1016/j.micrna.2026.208737</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.micrna.2026.208737</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K541" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L541" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M541" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N541" t="inlineStr"/>
+      <c r="O541" t="inlineStr"/>
+      <c r="P541" t="inlineStr"/>
+      <c r="Q541" t="inlineStr">
+        <is>
+          <t>Numerical simulation and modeling of HgCdTe and MoS₂ heterostructure MOSFET using polynomial fitting extrapolation technique</t>
+        </is>
+      </c>
+      <c r="R541" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S541" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="T541" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr"/>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Numerical simulation and modeling of HgCdTe and MoS₂ heterostructure MOSFET using polynomial fitting extrapolation technique</t>
+        </is>
+      </c>
+      <c r="C542" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Micro and Nanostructures</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>Malu, U.; Pravin, J. Charles; Babu, A. Ramesh</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr"/>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>10.1016/j.micrna.2026.208737</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.micrna.2026.208737</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K542" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L542" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M542" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N542" t="inlineStr"/>
+      <c r="O542" t="inlineStr"/>
+      <c r="P542" t="inlineStr"/>
+      <c r="Q542" t="inlineStr">
+        <is>
+          <t>Numerical simulation and modeling of HgCdTe and MoS₂ heterostructure MOSFET using polynomial fitting extrapolation technique</t>
+        </is>
+      </c>
+      <c r="R542" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S542" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="T542" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-19T00:11Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T542"/>
+  <dimension ref="A1:T562"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41396,6 +41396,1526 @@
       </c>
       <c r="T542" t="inlineStr"/>
     </row>
+    <row r="543">
+      <c r="A543" t="inlineStr"/>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="C543" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>Chang, Cheng; Lin, Chenyang; Luo, Shisong; Chen, Huayi; Qiu, Chufan; Lau, Lucas; Zhang, Zonghao; Li, Tao; Emon, Md Jahidul Hoq; Rahad, Rummanur; Lou, Jun; Zhao, Yuji</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr"/>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K543" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L543" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M543" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N543" t="inlineStr"/>
+      <c r="O543" t="inlineStr"/>
+      <c r="P543" t="inlineStr"/>
+      <c r="Q543" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="R543" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S543" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T543" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr"/>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Design Optimization of 600V 4H-SiC Lateral Bi-Directional MOSFET (L-BiD-MOSFET) with 3D TCAD Simulation</t>
+        </is>
+      </c>
+      <c r="C544" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>Jang, Seung Yup; deBoer, Skylar; Sung, Woongje</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr"/>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>10.4028/p-t04lti</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-t04lti</t>
+        </is>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K544" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L544" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M544" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N544" t="inlineStr"/>
+      <c r="O544" t="inlineStr"/>
+      <c r="P544" t="inlineStr"/>
+      <c r="Q544" t="inlineStr">
+        <is>
+          <t>Design Optimization of 600V 4H-SiC Lateral Bi-Directional MOSFET (L-BiD-MOSFET) with 3D TCAD Simulation</t>
+        </is>
+      </c>
+      <c r="R544" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S544" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T544" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr"/>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="C545" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>Chang, Cheng; Lin, Chenyang; Luo, Shisong; Chen, Huayi; Qiu, Chufan; Lau, Lucas; Zhang, Zonghao; Li, Tao; Emon, Md Jahidul Hoq; Rahad, Rummanur; Lou, Jun; Zhao, Yuji</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr"/>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K545" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L545" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M545" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N545" t="inlineStr"/>
+      <c r="O545" t="inlineStr"/>
+      <c r="P545" t="inlineStr"/>
+      <c r="Q545" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="R545" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S545" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T545" t="inlineStr"/>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr"/>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Design Optimization of 600V 4H-SiC Lateral Bi-Directional MOSFET (L-BiD-MOSFET) with 3D TCAD Simulation</t>
+        </is>
+      </c>
+      <c r="C546" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>Jang, Seung Yup; deBoer, Skylar; Sung, Woongje</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr"/>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>10.4028/p-t04lti</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-t04lti</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K546" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L546" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M546" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N546" t="inlineStr"/>
+      <c r="O546" t="inlineStr"/>
+      <c r="P546" t="inlineStr"/>
+      <c r="Q546" t="inlineStr">
+        <is>
+          <t>Design Optimization of 600V 4H-SiC Lateral Bi-Directional MOSFET (L-BiD-MOSFET) with 3D TCAD Simulation</t>
+        </is>
+      </c>
+      <c r="R546" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S546" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T546" t="inlineStr"/>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr"/>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Dynamic HV-H³TRB Test on 3.3 kV SiC MOSFET Modules</t>
+        </is>
+      </c>
+      <c r="C547" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>Peters, Jan Hendrik; Hanf, Michael; Clausner, Sven; Kaminski, Nando</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr"/>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>10.4028/p-tv6uj9</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-tv6uj9</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K547" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L547" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M547" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N547" t="inlineStr"/>
+      <c r="O547" t="inlineStr"/>
+      <c r="P547" t="inlineStr"/>
+      <c r="Q547" t="inlineStr">
+        <is>
+          <t>Dynamic HV-H³TRB Test on 3.3 kV SiC MOSFET Modules</t>
+        </is>
+      </c>
+      <c r="R547" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S547" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T547" t="inlineStr"/>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr"/>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Low-Inductance Packaging Design for SiC Power MOSFET Modules</t>
+        </is>
+      </c>
+      <c r="C548" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>Zhang, Zhao Bo; Yu, Renze; Jahdi, Saeed; Alatise, Olayiwola; Iannuzzo, Francesco; Stark, Bernard</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr"/>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>10.4028/p-kuni9m</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-kuni9m</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K548" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L548" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M548" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N548" t="inlineStr"/>
+      <c r="O548" t="inlineStr"/>
+      <c r="P548" t="inlineStr"/>
+      <c r="Q548" t="inlineStr">
+        <is>
+          <t>Low-Inductance Packaging Design for SiC Power MOSFET Modules</t>
+        </is>
+      </c>
+      <c r="R548" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S548" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T548" t="inlineStr"/>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr"/>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Peak Voltage and Switching Slope Dependency of Gate Switching Instability in SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="C549" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>Schnitzler, Ruben; Fink, Tobias; Halmer, David; Koch, Dominik; Kallfass, Ingmar</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr"/>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>10.4028/p-kxtj4u</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-kxtj4u</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K549" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L549" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M549" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N549" t="inlineStr"/>
+      <c r="O549" t="inlineStr"/>
+      <c r="P549" t="inlineStr"/>
+      <c r="Q549" t="inlineStr">
+        <is>
+          <t>Peak Voltage and Switching Slope Dependency of Gate Switching Instability in SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="R549" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S549" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T549" t="inlineStr"/>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr"/>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Peak Voltage and Switching Slope Dependency of Gate Switching Instability in SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="C550" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>Schnitzler, Ruben; Fink, Tobias; Halmer, David; Koch, Dominik; Kallfass, Ingmar</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr"/>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>10.4028/p-kxtj4u</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-kxtj4u</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K550" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L550" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M550" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N550" t="inlineStr"/>
+      <c r="O550" t="inlineStr"/>
+      <c r="P550" t="inlineStr"/>
+      <c r="Q550" t="inlineStr">
+        <is>
+          <t>Peak Voltage and Switching Slope Dependency of Gate Switching Instability in SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="R550" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S550" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T550" t="inlineStr"/>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr"/>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Normally-off GaN HEMT Device Technology and Performance Enhancement Methods</t>
+        </is>
+      </c>
+      <c r="C551" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>EWA Publishing</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Theoretical and Natural Science</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>Wang, Haotian</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr"/>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>10.54254/2753-8818/2026.33563</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54254/2753-8818/2026.33563</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K551" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L551" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M551" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N551" t="inlineStr"/>
+      <c r="O551" t="inlineStr"/>
+      <c r="P551" t="inlineStr"/>
+      <c r="Q551" t="inlineStr">
+        <is>
+          <t>Normally-off GaN HEMT Device Technology and Performance Enhancement Methods</t>
+        </is>
+      </c>
+      <c r="R551" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S551" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T551" t="inlineStr"/>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr"/>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="C552" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>Chang, Cheng; Lin, Chenyang; Luo, Shisong; Chen, Huayi; Qiu, Chufan; Lau, Lucas; Zhang, Zonghao; Li, Tao; Emon, Md Jahidul Hoq; Rahad, Rummanur; Lou, Jun; Zhao, Yuji</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr"/>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K552" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L552" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M552" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N552" t="inlineStr"/>
+      <c r="O552" t="inlineStr"/>
+      <c r="P552" t="inlineStr"/>
+      <c r="Q552" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="R552" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S552" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T552" t="inlineStr"/>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr"/>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Design Optimization of 600V 4H-SiC Lateral Bi-Directional MOSFET (L-BiD-MOSFET) with 3D TCAD Simulation</t>
+        </is>
+      </c>
+      <c r="C553" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>Jang, Seung Yup; deBoer, Skylar; Sung, Woongje</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr"/>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>10.4028/p-t04lti</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-t04lti</t>
+        </is>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K553" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L553" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M553" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N553" t="inlineStr"/>
+      <c r="O553" t="inlineStr"/>
+      <c r="P553" t="inlineStr"/>
+      <c r="Q553" t="inlineStr">
+        <is>
+          <t>Design Optimization of 600V 4H-SiC Lateral Bi-Directional MOSFET (L-BiD-MOSFET) with 3D TCAD Simulation</t>
+        </is>
+      </c>
+      <c r="R553" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S553" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T553" t="inlineStr"/>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr"/>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Dynamic HV-H³TRB Test on 3.3 kV SiC MOSFET Modules</t>
+        </is>
+      </c>
+      <c r="C554" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>Peters, Jan Hendrik; Hanf, Michael; Clausner, Sven; Kaminski, Nando</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr"/>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>10.4028/p-tv6uj9</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-tv6uj9</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K554" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L554" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M554" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N554" t="inlineStr"/>
+      <c r="O554" t="inlineStr"/>
+      <c r="P554" t="inlineStr"/>
+      <c r="Q554" t="inlineStr">
+        <is>
+          <t>Dynamic HV-H³TRB Test on 3.3 kV SiC MOSFET Modules</t>
+        </is>
+      </c>
+      <c r="R554" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S554" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T554" t="inlineStr"/>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr"/>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Low-Inductance Packaging Design for SiC Power MOSFET Modules</t>
+        </is>
+      </c>
+      <c r="C555" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>Zhang, Zhao Bo; Yu, Renze; Jahdi, Saeed; Alatise, Olayiwola; Iannuzzo, Francesco; Stark, Bernard</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr"/>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>10.4028/p-kuni9m</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-kuni9m</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K555" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L555" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M555" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N555" t="inlineStr"/>
+      <c r="O555" t="inlineStr"/>
+      <c r="P555" t="inlineStr"/>
+      <c r="Q555" t="inlineStr">
+        <is>
+          <t>Low-Inductance Packaging Design for SiC Power MOSFET Modules</t>
+        </is>
+      </c>
+      <c r="R555" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S555" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T555" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr"/>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Peak Voltage and Switching Slope Dependency of Gate Switching Instability in SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="C556" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>Schnitzler, Ruben; Fink, Tobias; Halmer, David; Koch, Dominik; Kallfass, Ingmar</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr"/>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>10.4028/p-kxtj4u</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-kxtj4u</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K556" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L556" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M556" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N556" t="inlineStr"/>
+      <c r="O556" t="inlineStr"/>
+      <c r="P556" t="inlineStr"/>
+      <c r="Q556" t="inlineStr">
+        <is>
+          <t>Peak Voltage and Switching Slope Dependency of Gate Switching Instability in SiC MOSFET</t>
+        </is>
+      </c>
+      <c r="R556" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S556" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T556" t="inlineStr"/>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr"/>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Normally-off GaN HEMT Device Technology and Performance Enhancement Methods</t>
+        </is>
+      </c>
+      <c r="C557" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>EWA Publishing</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Theoretical and Natural Science</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>Wang, Haotian</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr"/>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>10.54254/2753-8818/2026.33563</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54254/2753-8818/2026.33563</t>
+        </is>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K557" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L557" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M557" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N557" t="inlineStr"/>
+      <c r="O557" t="inlineStr"/>
+      <c r="P557" t="inlineStr"/>
+      <c r="Q557" t="inlineStr">
+        <is>
+          <t>Normally-off GaN HEMT Device Technology and Performance Enhancement Methods</t>
+        </is>
+      </c>
+      <c r="R557" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S557" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T557" t="inlineStr"/>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr"/>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Coherently grown AlN/GaN HEMT heterostructures on AlN buffer on SiC substrate—Impact of coherent growth on electrical and thermal characteristics</t>
+        </is>
+      </c>
+      <c r="C558" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>Lingaparthi, Ravikiran; Jiang, Yi; Seah, Tian Long Alex; Khanum, Rizwana; Dharmarasu, Nethaji; Koh, Yee Kan; Radhakrishnan, K.; Ng, Geok Ing</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr"/>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>10.1063/5.0318670</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0318670</t>
+        </is>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K558" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L558" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M558" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N558" t="inlineStr"/>
+      <c r="O558" t="inlineStr"/>
+      <c r="P558" t="inlineStr"/>
+      <c r="Q558" t="inlineStr">
+        <is>
+          <t>Coherently grown AlN/GaN HEMT heterostructures on AlN buffer on SiC substrate—Impact of coherent growth on electrical and thermal characteristics</t>
+        </is>
+      </c>
+      <c r="R558" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S558" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T558" t="inlineStr"/>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr"/>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Design Optimization of 600V 4H-SiC Lateral Bi-Directional MOSFET (L-BiD-MOSFET) with 3D TCAD Simulation</t>
+        </is>
+      </c>
+      <c r="C559" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>Jang, Seung Yup; deBoer, Skylar; Sung, Woongje</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr"/>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>10.4028/p-t04lti</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-t04lti</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K559" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L559" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M559" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N559" t="inlineStr"/>
+      <c r="O559" t="inlineStr"/>
+      <c r="P559" t="inlineStr"/>
+      <c r="Q559" t="inlineStr">
+        <is>
+          <t>Design Optimization of 600V 4H-SiC Lateral Bi-Directional MOSFET (L-BiD-MOSFET) with 3D TCAD Simulation</t>
+        </is>
+      </c>
+      <c r="R559" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S559" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T559" t="inlineStr"/>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr"/>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="C560" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>Chang, Cheng; Lin, Chenyang; Luo, Shisong; Chen, Huayi; Qiu, Chufan; Lau, Lucas; Zhang, Zonghao; Li, Tao; Emon, Md Jahidul Hoq; Rahad, Rummanur; Lou, Jun; Zhao, Yuji</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr"/>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K560" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L560" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M560" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N560" t="inlineStr"/>
+      <c r="O560" t="inlineStr"/>
+      <c r="P560" t="inlineStr"/>
+      <c r="Q560" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="R560" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S560" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T560" t="inlineStr"/>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr"/>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>A new dual-functional sensing system for glucose detection and logic gate construction based on PNIPAM-GOD/Co-MoS2 binary architecture intelligent films</t>
+        </is>
+      </c>
+      <c r="C561" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Bioelectrochemistry</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>Chen, Wen; Yang, Changyi; Li, Jiawei; Shi, Keren; Bai, Ruyu; Zhou, Yongzhong; Meng, Lingchen; Yao, Huiqin</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr"/>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>10.1016/j.bioelechem.2026.109331</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.bioelechem.2026.109331</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K561" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L561" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M561" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N561" t="inlineStr"/>
+      <c r="O561" t="inlineStr"/>
+      <c r="P561" t="inlineStr"/>
+      <c r="Q561" t="inlineStr">
+        <is>
+          <t>A new dual-functional sensing system for glucose detection and logic gate construction based on PNIPAM-GOD/Co-MoS2 binary architecture intelligent films</t>
+        </is>
+      </c>
+      <c r="R561" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S561" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T561" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr"/>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="C562" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>Chang, Cheng; Lin, Chenyang; Luo, Shisong; Chen, Huayi; Qiu, Chufan; Lau, Lucas; Zhang, Zonghao; Li, Tao; Emon, Md Jahidul Hoq; Rahad, Rummanur; Lou, Jun; Zhao, Yuji</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr"/>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325223</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K562" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L562" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M562" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N562" t="inlineStr"/>
+      <c r="O562" t="inlineStr"/>
+      <c r="P562" t="inlineStr"/>
+      <c r="Q562" t="inlineStr">
+        <is>
+          <t>Gate leakage suppression in p-GaN/AlGaN p-channel transistors via transferred BN gate dielectric for high-temperature operation</t>
+        </is>
+      </c>
+      <c r="R562" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S562" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="T562" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-20T00:10Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T562"/>
+  <dimension ref="A1:T569"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42916,6 +42916,538 @@
       </c>
       <c r="T562" t="inlineStr"/>
     </row>
+    <row r="563">
+      <c r="A563" t="inlineStr"/>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Analysis of current-voltage characteristics of npn structures for the estimation of acceptor concentration of a buried p-type layer in vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="C563" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>Oka, Tohru; Suda, Jun</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr"/>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae6fff</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae6fff</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K563" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L563" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M563" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N563" t="inlineStr"/>
+      <c r="O563" t="inlineStr"/>
+      <c r="P563" t="inlineStr"/>
+      <c r="Q563" t="inlineStr">
+        <is>
+          <t>Analysis of current-voltage characteristics of npn structures for the estimation of acceptor concentration of a buried p-type layer in vertical GaN trench metal-oxide-semiconductor field effect transistors</t>
+        </is>
+      </c>
+      <c r="R563" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S563" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="T563" t="inlineStr"/>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr"/>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>1.2 kV SiC MOSFET with Reduced Dynamic Losses Enabled by SiN Gate Dielectric</t>
+        </is>
+      </c>
+      <c r="C564" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>Stecconi, Tommaso; Stark, Roger; Reigosa, Paula; Schneider, Nick; Li, Coris; Liang, Leon; Knoll, Lars</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr"/>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>10.4028/p-6bms4c</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-6bms4c</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K564" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L564" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M564" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N564" t="inlineStr"/>
+      <c r="O564" t="inlineStr"/>
+      <c r="P564" t="inlineStr"/>
+      <c r="Q564" t="inlineStr">
+        <is>
+          <t>1.2 kV SiC MOSFET with Reduced Dynamic Losses Enabled by SiN Gate Dielectric</t>
+        </is>
+      </c>
+      <c r="R564" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S564" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="T564" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr"/>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Body Diode Reliability and Reverse Recovery Characteristics of Short Tapered SJ-MOSFET Fabricated by MeV Al Ion Implantation</t>
+        </is>
+      </c>
+      <c r="C565" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>Tawara, Takeshi; Takenaka, Kensuke; Narita, Syunki; Harada, Shinsuke</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr"/>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>10.4028/p-q9p090</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-q9p090</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K565" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L565" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M565" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N565" t="inlineStr"/>
+      <c r="O565" t="inlineStr"/>
+      <c r="P565" t="inlineStr"/>
+      <c r="Q565" t="inlineStr">
+        <is>
+          <t>Body Diode Reliability and Reverse Recovery Characteristics of Short Tapered SJ-MOSFET Fabricated by MeV Al Ion Implantation</t>
+        </is>
+      </c>
+      <c r="R565" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S565" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="T565" t="inlineStr"/>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr"/>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>1.2 kV SiC MOSFET with Reduced Dynamic Losses Enabled by SiN Gate Dielectric</t>
+        </is>
+      </c>
+      <c r="C566" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>Stecconi, Tommaso; Stark, Roger; Reigosa, Paula; Schneider, Nick; Li, Coris; Liang, Leon; Knoll, Lars</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr"/>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>10.4028/p-6bms4c</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-6bms4c</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K566" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L566" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M566" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N566" t="inlineStr"/>
+      <c r="O566" t="inlineStr"/>
+      <c r="P566" t="inlineStr"/>
+      <c r="Q566" t="inlineStr">
+        <is>
+          <t>1.2 kV SiC MOSFET with Reduced Dynamic Losses Enabled by SiN Gate Dielectric</t>
+        </is>
+      </c>
+      <c r="R566" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S566" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="T566" t="inlineStr"/>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr"/>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Experimental Analysis of 4H-SiC CMOS NOT Logic Gate Down to 100K</t>
+        </is>
+      </c>
+      <c r="C567" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>di Benedetto, Luigi; Rinaldi, Nicola; Rommel, Mathias; May, Alexander; Baier, Leander; Liguori, Rosalba; Rubino, Alfredo; Licciardo, Gian Domenico</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr"/>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>10.4028/p-3xeutp</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-3xeutp</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L567" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M567" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N567" t="inlineStr"/>
+      <c r="O567" t="inlineStr"/>
+      <c r="P567" t="inlineStr"/>
+      <c r="Q567" t="inlineStr">
+        <is>
+          <t>Experimental Analysis of 4H-SiC CMOS NOT Logic Gate Down to 100K</t>
+        </is>
+      </c>
+      <c r="R567" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S567" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="T567" t="inlineStr"/>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr"/>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Hybrid quantum encryption with an ultrafast rGO/Ni all-optical logic gate</t>
+        </is>
+      </c>
+      <c r="C568" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>Optical Materials Express</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>Hernández-Acosta, Marco Antonio; Córdova-Morales, Pablo; Torres-Torres, Carlos; Martinez-Rivas, Adrian; Valdez-Pérez, Donato; Rangel-Rojo, Raúl</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr"/>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>10.1364/ome.585024</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/ome.585024</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L568" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M568" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N568" t="inlineStr"/>
+      <c r="O568" t="inlineStr"/>
+      <c r="P568" t="inlineStr"/>
+      <c r="Q568" t="inlineStr">
+        <is>
+          <t>Hybrid quantum encryption with an ultrafast rGO/Ni all-optical logic gate</t>
+        </is>
+      </c>
+      <c r="R568" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S568" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="T568" t="inlineStr"/>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr"/>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>1.2 kV SiC MOSFET with Reduced Dynamic Losses Enabled by SiN Gate Dielectric</t>
+        </is>
+      </c>
+      <c r="C569" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>Stecconi, Tommaso; Stark, Roger; Reigosa, Paula; Schneider, Nick; Li, Coris; Liang, Leon; Knoll, Lars</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr"/>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>10.4028/p-6bms4c</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-6bms4c</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L569" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M569" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N569" t="inlineStr"/>
+      <c r="O569" t="inlineStr"/>
+      <c r="P569" t="inlineStr"/>
+      <c r="Q569" t="inlineStr">
+        <is>
+          <t>1.2 kV SiC MOSFET with Reduced Dynamic Losses Enabled by SiN Gate Dielectric</t>
+        </is>
+      </c>
+      <c r="R569" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S569" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="T569" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-21T00:10Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T569"/>
+  <dimension ref="A1:T570"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43448,6 +43448,78 @@
       </c>
       <c r="T569" t="inlineStr"/>
     </row>
+    <row r="570">
+      <c r="A570" t="inlineStr"/>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Simulation Study of Short Channel Effects in New Hemispherical Gate-All-Around (HGAA)  MOS Devices</t>
+        </is>
+      </c>
+      <c r="C570" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr"/>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>Balestra, Francis; Ghibaudo, Gerard</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr"/>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>10.20944/preprints202605.1292.v1</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20944/preprints202605.1292.v1</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K570" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L570" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M570" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N570" t="inlineStr"/>
+      <c r="O570" t="inlineStr"/>
+      <c r="P570" t="inlineStr"/>
+      <c r="Q570" t="inlineStr">
+        <is>
+          <t>Simulation Study of Short Channel Effects in New Hemispherical Gate-All-Around (HGAA)  MOS Devices</t>
+        </is>
+      </c>
+      <c r="R570" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S570" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="T570" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-23T00:10Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T570"/>
+  <dimension ref="A1:T574"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43520,6 +43520,310 @@
       </c>
       <c r="T570" t="inlineStr"/>
     </row>
+    <row r="571">
+      <c r="A571" t="inlineStr"/>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Semiconducting p-GaN gate HEMT with avalanche-like non-destructive breakdown capability</t>
+        </is>
+      </c>
+      <c r="C571" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>Yu, Jingjing; Yang, Junjie; Zheng, Qian; Liu, Sihang; Wang, Maojun; Yang, Xuelin; Shen, Bo; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr"/>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>10.1063/5.0319233</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0319233</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K571" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L571" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M571" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N571" t="inlineStr"/>
+      <c r="O571" t="inlineStr"/>
+      <c r="P571" t="inlineStr"/>
+      <c r="Q571" t="inlineStr">
+        <is>
+          <t>Semiconducting p-GaN gate HEMT with avalanche-like non-destructive breakdown capability</t>
+        </is>
+      </c>
+      <c r="R571" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S571" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="T571" t="inlineStr"/>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr"/>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Semiconducting p-GaN gate HEMT with avalanche-like non-destructive breakdown capability</t>
+        </is>
+      </c>
+      <c r="C572" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>Yu, Jingjing; Yang, Junjie; Zheng, Qian; Liu, Sihang; Wang, Maojun; Yang, Xuelin; Shen, Bo; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr"/>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>10.1063/5.0319233</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0319233</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K572" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L572" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M572" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N572" t="inlineStr"/>
+      <c r="O572" t="inlineStr"/>
+      <c r="P572" t="inlineStr"/>
+      <c r="Q572" t="inlineStr">
+        <is>
+          <t>Semiconducting p-GaN gate HEMT with avalanche-like non-destructive breakdown capability</t>
+        </is>
+      </c>
+      <c r="R572" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S572" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="T572" t="inlineStr"/>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr"/>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Semiconducting p-GaN gate HEMT with avalanche-like non-destructive breakdown capability</t>
+        </is>
+      </c>
+      <c r="C573" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>Yu, Jingjing; Yang, Junjie; Zheng, Qian; Liu, Sihang; Wang, Maojun; Yang, Xuelin; Shen, Bo; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr"/>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>10.1063/5.0319233</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0319233</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K573" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L573" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M573" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N573" t="inlineStr"/>
+      <c r="O573" t="inlineStr"/>
+      <c r="P573" t="inlineStr"/>
+      <c r="Q573" t="inlineStr">
+        <is>
+          <t>Semiconducting p-GaN gate HEMT with avalanche-like non-destructive breakdown capability</t>
+        </is>
+      </c>
+      <c r="R573" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S573" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="T573" t="inlineStr"/>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr"/>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Semiconducting p-GaN gate HEMT with avalanche-like non-destructive breakdown capability</t>
+        </is>
+      </c>
+      <c r="C574" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>Yu, Jingjing; Yang, Junjie; Zheng, Qian; Liu, Sihang; Wang, Maojun; Yang, Xuelin; Shen, Bo; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr"/>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>10.1063/5.0319233</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0319233</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K574" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L574" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M574" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N574" t="inlineStr"/>
+      <c r="O574" t="inlineStr"/>
+      <c r="P574" t="inlineStr"/>
+      <c r="Q574" t="inlineStr">
+        <is>
+          <t>Semiconducting p-GaN gate HEMT with avalanche-like non-destructive breakdown capability</t>
+        </is>
+      </c>
+      <c r="R574" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S574" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="T574" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-26T00:09Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T574"/>
+  <dimension ref="A1:T580"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43824,6 +43824,462 @@
       </c>
       <c r="T574" t="inlineStr"/>
     </row>
+    <row r="575">
+      <c r="A575" t="inlineStr"/>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>A Systematic Review and Benchmarking of Subthreshold / Weak-Inversion CMOS Inverter-Based Ultra-Low-Power Amplifiers: Performance Trade-Offs and Design Guidelines</t>
+        </is>
+      </c>
+      <c r="C575" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>EWA Publishing</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Applied and Computational Engineering</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>Li, Yitong</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr"/>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>10.54254/2755-2721/2026.bj33823</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54254/2755-2721/2026.bj33823</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K575" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L575" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M575" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N575" t="inlineStr"/>
+      <c r="O575" t="inlineStr"/>
+      <c r="P575" t="inlineStr"/>
+      <c r="Q575" t="inlineStr">
+        <is>
+          <t>A Systematic Review and Benchmarking of Subthreshold / Weak-Inversion CMOS Inverter-Based Ultra-Low-Power Amplifiers: Performance Trade-Offs and Design Guidelines</t>
+        </is>
+      </c>
+      <c r="R575" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S575" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="T575" t="inlineStr"/>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr"/>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Continuous-Time Transient Stability Assessment of Inverter-Dominated Microgrids viaPhysics-Informed Neural ODEs</t>
+        </is>
+      </c>
+      <c r="C576" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Fakultas Teknik, Universitas Negeri Makassar</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Journal of Electrical Engineering and Informatics</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>Andi Nur Faisal</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr"/>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>10.59562/jeeni.v3i2.12701</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.59562/jeeni.v3i2.12701</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K576" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L576" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M576" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N576" t="inlineStr"/>
+      <c r="O576" t="inlineStr"/>
+      <c r="P576" t="inlineStr"/>
+      <c r="Q576" t="inlineStr">
+        <is>
+          <t>Continuous-Time Transient Stability Assessment of Inverter-Dominated Microgrids viaPhysics-Informed Neural ODEs</t>
+        </is>
+      </c>
+      <c r="R576" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S576" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="T576" t="inlineStr"/>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr"/>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Epitaxial growth and characterization of AlGaN/GaN HEMT structures on 4 inch directly bonded GaN/SiC substrates</t>
+        </is>
+      </c>
+      <c r="C577" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>Nonaka, Kentaro; Kishimoto, Ryozo; Isoda, Yoshinori; Kobayashi, Hiroki; Kuraoka, Yoshitaka; Sato, Kei; Yoshino, Takashi</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr"/>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae6c7c</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae6c7c</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K577" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L577" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M577" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N577" t="inlineStr"/>
+      <c r="O577" t="inlineStr"/>
+      <c r="P577" t="inlineStr"/>
+      <c r="Q577" t="inlineStr">
+        <is>
+          <t>Epitaxial growth and characterization of AlGaN/GaN HEMT structures on 4 inch directly bonded GaN/SiC substrates</t>
+        </is>
+      </c>
+      <c r="R577" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S577" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="T577" t="inlineStr"/>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr"/>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Epitaxial growth and characterization of AlGaN/GaN HEMT structures on 4 inch directly bonded GaN/SiC substrates</t>
+        </is>
+      </c>
+      <c r="C578" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>Nonaka, Kentaro; Kishimoto, Ryozo; Isoda, Yoshinori; Kobayashi, Hiroki; Kuraoka, Yoshitaka; Sato, Kei; Yoshino, Takashi</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr"/>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae6c7c</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae6c7c</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K578" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L578" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M578" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N578" t="inlineStr"/>
+      <c r="O578" t="inlineStr"/>
+      <c r="P578" t="inlineStr"/>
+      <c r="Q578" t="inlineStr">
+        <is>
+          <t>Epitaxial growth and characterization of AlGaN/GaN HEMT structures on 4 inch directly bonded GaN/SiC substrates</t>
+        </is>
+      </c>
+      <c r="R578" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S578" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="T578" t="inlineStr"/>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr"/>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Continuous-Time Transient Stability Assessment of Inverter-Dominated Microgrids viaPhysics-Informed Neural ODEs</t>
+        </is>
+      </c>
+      <c r="C579" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Fakultas Teknik, Universitas Negeri Makassar</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Journal of Electrical Engineering and Informatics</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>Andi Nur Faisal</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr"/>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>10.59562/jeeni.v3i2.12701</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.59562/jeeni.v3i2.12701</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K579" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L579" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M579" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N579" t="inlineStr"/>
+      <c r="O579" t="inlineStr"/>
+      <c r="P579" t="inlineStr"/>
+      <c r="Q579" t="inlineStr">
+        <is>
+          <t>Continuous-Time Transient Stability Assessment of Inverter-Dominated Microgrids viaPhysics-Informed Neural ODEs</t>
+        </is>
+      </c>
+      <c r="R579" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S579" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="T579" t="inlineStr"/>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr"/>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>The Grid-Forming Operation of a Modified Delta-Connected Cascaded H-Bridge Multilevel Inverter with PV Integration</t>
+        </is>
+      </c>
+      <c r="C580" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Machines</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>Noman, Abdullah M.</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr"/>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>10.3390/machines14060581</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/machines14060581</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K580" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L580" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M580" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N580" t="inlineStr"/>
+      <c r="O580" t="inlineStr"/>
+      <c r="P580" t="inlineStr"/>
+      <c r="Q580" t="inlineStr">
+        <is>
+          <t>The Grid-Forming Operation of a Modified Delta-Connected Cascaded H-Bridge Multilevel Inverter with PV Integration</t>
+        </is>
+      </c>
+      <c r="R580" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S580" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="T580" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-27T00:10Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T580"/>
+  <dimension ref="A1:T594"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44280,6 +44280,1070 @@
       </c>
       <c r="T580" t="inlineStr"/>
     </row>
+    <row r="581">
+      <c r="A581" t="inlineStr"/>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Adaptive Control Strategy for a Single-Inverter Dual-PMSM System Under Load Disturbance</t>
+        </is>
+      </c>
+      <c r="C581" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>Wang, Siling; Li, Dongsheng</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr"/>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15112302</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15112302</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K581" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L581" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M581" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N581" t="inlineStr"/>
+      <c r="O581" t="inlineStr"/>
+      <c r="P581" t="inlineStr"/>
+      <c r="Q581" t="inlineStr">
+        <is>
+          <t>Adaptive Control Strategy for a Single-Inverter Dual-PMSM System Under Load Disturbance</t>
+        </is>
+      </c>
+      <c r="R581" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S581" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T581" t="inlineStr"/>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr"/>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>A Rapid-prototyping CMOS-RRAM Integration Strategy</t>
+        </is>
+      </c>
+      <c r="C582" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Microsystems &amp;amp; Nanoengineering</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>Tsiamis, Andreas; Stathopoulos, Spyros; Prodromakis, Themis</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr"/>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>10.1038/s41378-026-01335-9</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41378-026-01335-9</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K582" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L582" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M582" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N582" t="inlineStr"/>
+      <c r="O582" t="inlineStr"/>
+      <c r="P582" t="inlineStr"/>
+      <c r="Q582" t="inlineStr">
+        <is>
+          <t>A Rapid-prototyping CMOS-RRAM Integration Strategy</t>
+        </is>
+      </c>
+      <c r="R582" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S582" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T582" t="inlineStr"/>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr"/>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Exploring Oncology Referral Practices for Complementary and Alternative Medicine: A Scoping Review</t>
+        </is>
+      </c>
+      <c r="C583" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>Malur Rangaiah, Usha Rani; Ghoshal, Arunangshu; Sowjanya, Dumbala; Subramani, Vinod Kumar; Dhyani, Vijay Shree; Karmbadka, Ashwini; Maharana, Satyapriya; Salins, Naveen</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr"/>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261451651</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261451651</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K583" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L583" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M583" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N583" t="inlineStr"/>
+      <c r="O583" t="inlineStr"/>
+      <c r="P583" t="inlineStr"/>
+      <c r="Q583" t="inlineStr">
+        <is>
+          <t>Exploring Oncology Referral Practices for Complementary and Alternative Medicine: A Scoping Review</t>
+        </is>
+      </c>
+      <c r="R583" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S583" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T583" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr"/>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Foundations of Modular AI—Shifting from Monolithic Systems</t>
+        </is>
+      </c>
+      <c r="C584" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>CRC Press</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Agentic Intelligence</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>Hutson, James</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr"/>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>10.1201/9781003688013-2</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1201/9781003688013-2</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K584" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L584" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M584" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N584" t="inlineStr"/>
+      <c r="O584" t="inlineStr"/>
+      <c r="P584" t="inlineStr"/>
+      <c r="Q584" t="inlineStr">
+        <is>
+          <t>Foundations of Modular AI—Shifting from Monolithic Systems</t>
+        </is>
+      </c>
+      <c r="R584" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S584" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T584" t="inlineStr"/>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr"/>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>A Rapid-prototyping CMOS-RRAM Integration Strategy</t>
+        </is>
+      </c>
+      <c r="C585" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Microsystems &amp;amp; Nanoengineering</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>Tsiamis, Andreas; Stathopoulos, Spyros; Prodromakis, Themis</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr"/>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>10.1038/s41378-026-01335-9</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41378-026-01335-9</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K585" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L585" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M585" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N585" t="inlineStr"/>
+      <c r="O585" t="inlineStr"/>
+      <c r="P585" t="inlineStr"/>
+      <c r="Q585" t="inlineStr">
+        <is>
+          <t>A Rapid-prototyping CMOS-RRAM Integration Strategy</t>
+        </is>
+      </c>
+      <c r="R585" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S585" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T585" t="inlineStr"/>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr"/>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Exploring Oncology Referral Practices for Complementary and Alternative Medicine: A Scoping Review</t>
+        </is>
+      </c>
+      <c r="C586" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>Malur Rangaiah, Usha Rani; Ghoshal, Arunangshu; Sowjanya, Dumbala; Subramani, Vinod Kumar; Dhyani, Vijay Shree; Karmbadka, Ashwini; Maharana, Satyapriya; Salins, Naveen</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr"/>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261451651</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261451651</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K586" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L586" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M586" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N586" t="inlineStr"/>
+      <c r="O586" t="inlineStr"/>
+      <c r="P586" t="inlineStr"/>
+      <c r="Q586" t="inlineStr">
+        <is>
+          <t>Exploring Oncology Referral Practices for Complementary and Alternative Medicine: A Scoping Review</t>
+        </is>
+      </c>
+      <c r="R586" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S586" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T586" t="inlineStr"/>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr"/>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Enhancement-mode tri-gate GaN MIS-HEMTs with PEALD-AlN/HfO2 dual-gate dielectric</t>
+        </is>
+      </c>
+      <c r="C587" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>Rai, Rahul; Ho, Viet Quoc; Nguyen, Khanh Quoc; Kuo, Hao Chung; Chang, Edward Yi</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr"/>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>10.1063/5.0320099</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0320099</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K587" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L587" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M587" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N587" t="inlineStr"/>
+      <c r="O587" t="inlineStr"/>
+      <c r="P587" t="inlineStr"/>
+      <c r="Q587" t="inlineStr">
+        <is>
+          <t>Enhancement-mode tri-gate GaN MIS-HEMTs with PEALD-AlN/HfO2 dual-gate dielectric</t>
+        </is>
+      </c>
+      <c r="R587" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S587" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T587" t="inlineStr"/>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr"/>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Enhancement-mode tri-gate GaN MIS-HEMTs with PEALD-AlN/HfO2 dual-gate dielectric</t>
+        </is>
+      </c>
+      <c r="C588" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>Rai, Rahul; Ho, Viet Quoc; Nguyen, Khanh Quoc; Kuo, Hao Chung; Chang, Edward Yi</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr"/>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>10.1063/5.0320099</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0320099</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K588" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L588" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M588" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N588" t="inlineStr"/>
+      <c r="O588" t="inlineStr"/>
+      <c r="P588" t="inlineStr"/>
+      <c r="Q588" t="inlineStr">
+        <is>
+          <t>Enhancement-mode tri-gate GaN MIS-HEMTs with PEALD-AlN/HfO2 dual-gate dielectric</t>
+        </is>
+      </c>
+      <c r="R588" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S588" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T588" t="inlineStr"/>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr"/>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Adaptive Control Strategy for a Single-Inverter Dual-PMSM System Under Load Disturbance</t>
+        </is>
+      </c>
+      <c r="C589" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>Wang, Siling; Li, Dongsheng</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr"/>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15112302</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15112302</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K589" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L589" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M589" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N589" t="inlineStr"/>
+      <c r="O589" t="inlineStr"/>
+      <c r="P589" t="inlineStr"/>
+      <c r="Q589" t="inlineStr">
+        <is>
+          <t>Adaptive Control Strategy for a Single-Inverter Dual-PMSM System Under Load Disturbance</t>
+        </is>
+      </c>
+      <c r="R589" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S589" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T589" t="inlineStr"/>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr"/>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>A Rapid-prototyping CMOS-RRAM Integration Strategy</t>
+        </is>
+      </c>
+      <c r="C590" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>Microsystems &amp;amp; Nanoengineering</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>Tsiamis, Andreas; Stathopoulos, Spyros; Prodromakis, Themis</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr"/>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>10.1038/s41378-026-01335-9</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41378-026-01335-9</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K590" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L590" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M590" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N590" t="inlineStr"/>
+      <c r="O590" t="inlineStr"/>
+      <c r="P590" t="inlineStr"/>
+      <c r="Q590" t="inlineStr">
+        <is>
+          <t>A Rapid-prototyping CMOS-RRAM Integration Strategy</t>
+        </is>
+      </c>
+      <c r="R590" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S590" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T590" t="inlineStr"/>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr"/>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Noise Optimization of VCO-ADCs Based on Ring Oscillators with Cascoded Inverter Delay Cells</t>
+        </is>
+      </c>
+      <c r="C591" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>Granizo, Javier; Garvi, Ruben; Fernandez, Javier; de la Torre, Jorge; Hernandez, Luis</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr"/>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15112299</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15112299</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K591" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L591" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M591" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N591" t="inlineStr"/>
+      <c r="O591" t="inlineStr"/>
+      <c r="P591" t="inlineStr"/>
+      <c r="Q591" t="inlineStr">
+        <is>
+          <t>Noise Optimization of VCO-ADCs Based on Ring Oscillators with Cascoded Inverter Delay Cells</t>
+        </is>
+      </c>
+      <c r="R591" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S591" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T591" t="inlineStr"/>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr"/>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Adaptive Control Strategy for a Single-Inverter Dual-PMSM System Under Load Disturbance</t>
+        </is>
+      </c>
+      <c r="C592" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>Wang, Siling; Li, Dongsheng</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr"/>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15112302</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15112302</t>
+        </is>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K592" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L592" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M592" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N592" t="inlineStr"/>
+      <c r="O592" t="inlineStr"/>
+      <c r="P592" t="inlineStr"/>
+      <c r="Q592" t="inlineStr">
+        <is>
+          <t>Adaptive Control Strategy for a Single-Inverter Dual-PMSM System Under Load Disturbance</t>
+        </is>
+      </c>
+      <c r="R592" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S592" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T592" t="inlineStr"/>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr"/>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Enhancement-mode tri-gate GaN MIS-HEMTs with PEALD-AlN/HfO2 dual-gate dielectric</t>
+        </is>
+      </c>
+      <c r="C593" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>Rai, Rahul; Ho, Viet Quoc; Nguyen, Khanh Quoc; Kuo, Hao Chung; Chang, Edward Yi</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr"/>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>10.1063/5.0320099</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0320099</t>
+        </is>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K593" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L593" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M593" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N593" t="inlineStr"/>
+      <c r="O593" t="inlineStr"/>
+      <c r="P593" t="inlineStr"/>
+      <c r="Q593" t="inlineStr">
+        <is>
+          <t>Enhancement-mode tri-gate GaN MIS-HEMTs with PEALD-AlN/HfO2 dual-gate dielectric</t>
+        </is>
+      </c>
+      <c r="R593" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S593" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T593" t="inlineStr"/>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr"/>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Enhancement-mode tri-gate GaN MIS-HEMTs with PEALD-AlN/HfO2 dual-gate dielectric</t>
+        </is>
+      </c>
+      <c r="C594" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>Rai, Rahul; Ho, Viet Quoc; Nguyen, Khanh Quoc; Kuo, Hao Chung; Chang, Edward Yi</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr"/>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>10.1063/5.0320099</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0320099</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K594" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L594" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M594" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N594" t="inlineStr"/>
+      <c r="O594" t="inlineStr"/>
+      <c r="P594" t="inlineStr"/>
+      <c r="Q594" t="inlineStr">
+        <is>
+          <t>Enhancement-mode tri-gate GaN MIS-HEMTs with PEALD-AlN/HfO2 dual-gate dielectric</t>
+        </is>
+      </c>
+      <c r="R594" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S594" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="T594" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-29T00:14Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T594"/>
+  <dimension ref="A1:T596"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45344,6 +45344,150 @@
       </c>
       <c r="T594" t="inlineStr"/>
     </row>
+    <row r="595">
+      <c r="A595" t="inlineStr"/>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Development of a Scalable Modular Monolithic Academic Management System for Educational Institutions</t>
+        </is>
+      </c>
+      <c r="C595" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>International Research Journal of Modernization in Engineering Technology and Science</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>International Research Journal of Modernization in Engineering Technology &amp;amp; Science</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr"/>
+      <c r="G595" t="inlineStr"/>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>10.56726/irjmets98983</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.56726/irjmets98983</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K595" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L595" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M595" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N595" t="inlineStr"/>
+      <c r="O595" t="inlineStr"/>
+      <c r="P595" t="inlineStr"/>
+      <c r="Q595" t="inlineStr">
+        <is>
+          <t>Development of a Scalable Modular Monolithic Academic Management System for Educational Institutions</t>
+        </is>
+      </c>
+      <c r="R595" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S595" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="T595" t="inlineStr"/>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr"/>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Numerical Validation of a MOSFET-Based Control Circuit for High-Power Intelligent Reflecting Surfaces for Wireless Power Transfer Applications</t>
+        </is>
+      </c>
+      <c r="C596" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr"/>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>Ichikawa, Gakuto; Omori, Eisuke; Nagata, Atsuko; Kumashiro, Akise; Kizaki, Kazuhiro; Saruwatari, Shunsuke; Wakatsuchi, Hiroki</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr"/>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9596944/v1</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9596944/v1</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K596" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L596" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M596" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N596" t="inlineStr"/>
+      <c r="O596" t="inlineStr"/>
+      <c r="P596" t="inlineStr"/>
+      <c r="Q596" t="inlineStr">
+        <is>
+          <t>Numerical Validation of a MOSFET-Based Control Circuit for High-Power Intelligent Reflecting Surfaces for Wireless Power Transfer Applications</t>
+        </is>
+      </c>
+      <c r="R596" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S596" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="T596" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-05-30T00:11Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T596"/>
+  <dimension ref="A1:T602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45488,6 +45488,462 @@
       </c>
       <c r="T596" t="inlineStr"/>
     </row>
+    <row r="597">
+      <c r="A597" t="inlineStr"/>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Evaluation of lateral soil pressure for monolithic column foundation of industrial buildings</t>
+        </is>
+      </c>
+      <c r="C597" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Ukrainian State University of Science and Technologies</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>Bridges and tunnels: theory, research, practice</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>Bakan, I. M.</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr"/>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>10.15802/bttrp2026-29-02</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.15802/bttrp2026-29-02</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K597" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L597" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M597" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N597" t="inlineStr"/>
+      <c r="O597" t="inlineStr"/>
+      <c r="P597" t="inlineStr"/>
+      <c r="Q597" t="inlineStr">
+        <is>
+          <t>Evaluation of lateral soil pressure for monolithic column foundation of industrial buildings</t>
+        </is>
+      </c>
+      <c r="R597" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S597" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="T597" t="inlineStr"/>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr"/>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Recent progress on GaN-on-GaN technology for RF applications</t>
+        </is>
+      </c>
+      <c r="C598" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>Chen, Hongda; Wu, Mei; Li, Shiming; Sun, Haolun; Xiang, Yuanmeng; Dong, Zishuo; Yang, Ling; Zhang, Meng; Lu, Hao; Hou, Bin; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr"/>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae74df</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae74df</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K598" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L598" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M598" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N598" t="inlineStr"/>
+      <c r="O598" t="inlineStr"/>
+      <c r="P598" t="inlineStr"/>
+      <c r="Q598" t="inlineStr">
+        <is>
+          <t>Recent progress on GaN-on-GaN technology for RF applications</t>
+        </is>
+      </c>
+      <c r="R598" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S598" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="T598" t="inlineStr"/>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr"/>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Dynamic On-resistance Degradation Mechanism of 1200 V Enhancement-mode GaN Schottky-Gate HEMT Devices on the Si Substrates</t>
+        </is>
+      </c>
+      <c r="C599" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>Zhao, Yaopeng; Shi, Jiahao; Li, Ang; Luo, Pan; Peng, Shutao; Luo, Jingtao; Yang, Lei; Wen, Hai-Bing; Liu, Kai; Wang, Chong; Wang, Jianyuan; Tan, Cher M</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr"/>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae753c</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae753c</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K599" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L599" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M599" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N599" t="inlineStr"/>
+      <c r="O599" t="inlineStr"/>
+      <c r="P599" t="inlineStr"/>
+      <c r="Q599" t="inlineStr">
+        <is>
+          <t>Dynamic On-resistance Degradation Mechanism of 1200 V Enhancement-mode GaN Schottky-Gate HEMT Devices on the Si Substrates</t>
+        </is>
+      </c>
+      <c r="R599" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S599" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="T599" t="inlineStr"/>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr"/>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Dynamic On-resistance Degradation Mechanism of 1200 V Enhancement-mode GaN Schottky-Gate HEMT Devices on the Si Substrates</t>
+        </is>
+      </c>
+      <c r="C600" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>Zhao, Yaopeng; Shi, Jiahao; Li, Ang; Luo, Pan; Peng, Shutao; Luo, Jingtao; Yang, Lei; Wen, Hai-Bing; Liu, Kai; Wang, Chong; Wang, Jianyuan; Tan, Cher M</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr"/>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae753c</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae753c</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K600" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L600" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M600" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N600" t="inlineStr"/>
+      <c r="O600" t="inlineStr"/>
+      <c r="P600" t="inlineStr"/>
+      <c r="Q600" t="inlineStr">
+        <is>
+          <t>Dynamic On-resistance Degradation Mechanism of 1200 V Enhancement-mode GaN Schottky-Gate HEMT Devices on the Si Substrates</t>
+        </is>
+      </c>
+      <c r="R600" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S600" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="T600" t="inlineStr"/>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr"/>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Diagnostic model of the CMOS integrated circuit output translator</t>
+        </is>
+      </c>
+      <c r="C601" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Metascience</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>Communication informatization and cybersecurity systems and technologies</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>Kuzavkov, V.; Fatty, A.</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr"/>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>10.58254/viti.9.2026.22.275</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.58254/viti.9.2026.22.275</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K601" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L601" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M601" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N601" t="inlineStr"/>
+      <c r="O601" t="inlineStr"/>
+      <c r="P601" t="inlineStr"/>
+      <c r="Q601" t="inlineStr">
+        <is>
+          <t>Diagnostic model of the CMOS integrated circuit output translator</t>
+        </is>
+      </c>
+      <c r="R601" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S601" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="T601" t="inlineStr"/>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr"/>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Theoretical study of a topological layered metastructure integrating NOR logic gate and multiphysical sensing functions</t>
+        </is>
+      </c>
+      <c r="C602" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Optics Express</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Du, Rui; Sui, Jun-Yang; Yao, Ting-Shuo; Zhang, Hai-Feng</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr"/>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>10.1364/oe.592675</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/oe.592675</t>
+        </is>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K602" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L602" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M602" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N602" t="inlineStr"/>
+      <c r="O602" t="inlineStr"/>
+      <c r="P602" t="inlineStr"/>
+      <c r="Q602" t="inlineStr">
+        <is>
+          <t>Theoretical study of a topological layered metastructure integrating NOR logic gate and multiphysical sensing functions</t>
+        </is>
+      </c>
+      <c r="R602" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S602" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="T602" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-01T00:10Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T602"/>
+  <dimension ref="A1:T603"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45944,6 +45944,82 @@
       </c>
       <c r="T602" t="inlineStr"/>
     </row>
+    <row r="603">
+      <c r="A603" t="inlineStr"/>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Low Insertion‐Loss High Power X‐Band SPDT Transmit/Receive Switches in 250 nm GaN HEMT</t>
+        </is>
+      </c>
+      <c r="C603" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Microwave and Optical Technology Letters</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>Kim, Tae‐Hoon; Lee, Mun‐Kyo; Hong, Soonyoung; Park, Jung‐Dong</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr"/>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>10.1002/mop.70649</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/mop.70649</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K603" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L603" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M603" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N603" t="inlineStr"/>
+      <c r="O603" t="inlineStr"/>
+      <c r="P603" t="inlineStr"/>
+      <c r="Q603" t="inlineStr">
+        <is>
+          <t>Low Insertion‐Loss High Power X‐Band SPDT Transmit/Receive Switches in 250 nm GaN HEMT</t>
+        </is>
+      </c>
+      <c r="R603" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S603" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="T603" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-02T00:17Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T603"/>
+  <dimension ref="A1:T604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46020,6 +46020,82 @@
       </c>
       <c r="T603" t="inlineStr"/>
     </row>
+    <row r="604">
+      <c r="A604" t="inlineStr"/>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Negative-bias temperature instability in AlSiO/p-type GaN metal-oxide-semiconductor field-effect transistors with ultrathin AlN interfacial layer</t>
+        </is>
+      </c>
+      <c r="C604" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>Iguchi, Hiroko; Narita, Tetsuo; Ito, Kenji; Iwasaki, Shiro; Kano, Emi; Ikarashi, Nobuyuki; Tomita, Kazuyoshi; Kikuta, Daigo</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr"/>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325347</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325347</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K604" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L604" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M604" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N604" t="inlineStr"/>
+      <c r="O604" t="inlineStr"/>
+      <c r="P604" t="inlineStr"/>
+      <c r="Q604" t="inlineStr">
+        <is>
+          <t>Negative-bias temperature instability in AlSiO/p-type GaN metal-oxide-semiconductor field-effect transistors with ultrathin AlN interfacial layer</t>
+        </is>
+      </c>
+      <c r="R604" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S604" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="T604" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-03T01:42Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T604"/>
+  <dimension ref="A1:T614"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46096,6 +46096,750 @@
       </c>
       <c r="T604" t="inlineStr"/>
     </row>
+    <row r="605">
+      <c r="A605" t="inlineStr"/>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Stator Resistance Compensation for PI-Based Field-Oriented Control of SPMSM Drives Using a Multilevel Inverter</t>
+        </is>
+      </c>
+      <c r="C605" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr"/>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>Quan, Nguyen Vinh; Son, Nguyen Ngoc</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr"/>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9591331/v1</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9591331/v1</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K605" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L605" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M605" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N605" t="inlineStr"/>
+      <c r="O605" t="inlineStr"/>
+      <c r="P605" t="inlineStr"/>
+      <c r="Q605" t="inlineStr">
+        <is>
+          <t>Stator Resistance Compensation for PI-Based Field-Oriented Control of SPMSM Drives Using a Multilevel Inverter</t>
+        </is>
+      </c>
+      <c r="R605" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S605" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T605" t="inlineStr"/>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr"/>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>A robust and energy-efficient CNTFET ternary SRAM cell utilizing a controllable inverter-based access mechanism</t>
+        </is>
+      </c>
+      <c r="C606" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Mousavi, Rasool; Ebrahimi, Behzad; Eslami, Mahdi</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr"/>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae7655</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae7655</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K606" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L606" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M606" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N606" t="inlineStr"/>
+      <c r="O606" t="inlineStr"/>
+      <c r="P606" t="inlineStr"/>
+      <c r="Q606" t="inlineStr">
+        <is>
+          <t>A robust and energy-efficient CNTFET ternary SRAM cell utilizing a controllable inverter-based access mechanism</t>
+        </is>
+      </c>
+      <c r="R606" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S606" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T606" t="inlineStr"/>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr"/>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Stator Resistance Compensation for PI-Based Field-Oriented Control of SPMSM Drives Using a Multilevel Inverter</t>
+        </is>
+      </c>
+      <c r="C607" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr"/>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>Quan, Nguyen Vinh; Son, Nguyen Ngoc</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr"/>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9591331/v1</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9591331/v1</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K607" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L607" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M607" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N607" t="inlineStr"/>
+      <c r="O607" t="inlineStr"/>
+      <c r="P607" t="inlineStr"/>
+      <c r="Q607" t="inlineStr">
+        <is>
+          <t>Stator Resistance Compensation for PI-Based Field-Oriented Control of SPMSM Drives Using a Multilevel Inverter</t>
+        </is>
+      </c>
+      <c r="R607" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S607" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T607" t="inlineStr"/>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr"/>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Urea-mediated interstitial N-doped α-MnO2/Al2O3 monolithic catalyst for enhanced room-temperature formaldehyde oxidation</t>
+        </is>
+      </c>
+      <c r="C608" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>Applied Surface Science</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>Song, Shi-Jia; Liu, Yang; Zhou, Hao; Yi, Xianliang</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr"/>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>10.1016/j.apsusc.2026.167163</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.apsusc.2026.167163</t>
+        </is>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K608" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L608" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M608" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N608" t="inlineStr"/>
+      <c r="O608" t="inlineStr"/>
+      <c r="P608" t="inlineStr"/>
+      <c r="Q608" t="inlineStr">
+        <is>
+          <t>Urea-mediated interstitial N-doped α-MnO2/Al2O3 monolithic catalyst for enhanced room-temperature formaldehyde oxidation</t>
+        </is>
+      </c>
+      <c r="R608" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S608" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T608" t="inlineStr"/>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr"/>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Decoupling and Optimization of Intrinsic Vertical Breakdown in 8-Inch GaN-on-Si HEMT Buffer</t>
+        </is>
+      </c>
+      <c r="C609" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>Dong, Wei; Zhang, Shuhan; Fan, Qian; Ni, Xianfeng; Gu, Xing</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr"/>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15112423</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15112423</t>
+        </is>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K609" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L609" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M609" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N609" t="inlineStr"/>
+      <c r="O609" t="inlineStr"/>
+      <c r="P609" t="inlineStr"/>
+      <c r="Q609" t="inlineStr">
+        <is>
+          <t>Decoupling and Optimization of Intrinsic Vertical Breakdown in 8-Inch GaN-on-Si HEMT Buffer</t>
+        </is>
+      </c>
+      <c r="R609" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S609" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T609" t="inlineStr"/>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr"/>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Small-signal model of RF InAlGaN/GaN HEMT and on-chip calibration structures</t>
+        </is>
+      </c>
+      <c r="C610" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Polish Academy of Sciences Chancellery</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>International Journal of Electronics and Telecommunications</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Florovič, Martin; Dzuriš, Michal; Krchnák, Jakub; Chvála, Aleš; Kováč, jr., Jaroslav; Kováčová, Soňa; Kováč, Jaroslav; Harťanský, René; Stuchlíková, Ľubica; Matuš, Matej</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr"/>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>10.24425/ijet.2026.157914</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.24425/ijet.2026.157914</t>
+        </is>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K610" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L610" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M610" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N610" t="inlineStr"/>
+      <c r="O610" t="inlineStr"/>
+      <c r="P610" t="inlineStr"/>
+      <c r="Q610" t="inlineStr">
+        <is>
+          <t>Small-signal model of RF InAlGaN/GaN HEMT and on-chip calibration structures</t>
+        </is>
+      </c>
+      <c r="R610" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S610" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T610" t="inlineStr"/>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr"/>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Stator Resistance Compensation for PI-Based Field-Oriented Control of SPMSM Drives Using a Multilevel Inverter</t>
+        </is>
+      </c>
+      <c r="C611" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr"/>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>Quan, Nguyen Vinh; Son, Nguyen Ngoc</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr"/>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9591331/v1</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9591331/v1</t>
+        </is>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K611" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L611" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M611" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N611" t="inlineStr"/>
+      <c r="O611" t="inlineStr"/>
+      <c r="P611" t="inlineStr"/>
+      <c r="Q611" t="inlineStr">
+        <is>
+          <t>Stator Resistance Compensation for PI-Based Field-Oriented Control of SPMSM Drives Using a Multilevel Inverter</t>
+        </is>
+      </c>
+      <c r="R611" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S611" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T611" t="inlineStr"/>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr"/>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>A robust and energy-efficient CNTFET ternary SRAM cell utilizing a controllable inverter-based access mechanism</t>
+        </is>
+      </c>
+      <c r="C612" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>Mousavi, Rasool; Ebrahimi, Behzad; Eslami, Mahdi</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr"/>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae7655</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae7655</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K612" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L612" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M612" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N612" t="inlineStr"/>
+      <c r="O612" t="inlineStr"/>
+      <c r="P612" t="inlineStr"/>
+      <c r="Q612" t="inlineStr">
+        <is>
+          <t>A robust and energy-efficient CNTFET ternary SRAM cell utilizing a controllable inverter-based access mechanism</t>
+        </is>
+      </c>
+      <c r="R612" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S612" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T612" t="inlineStr"/>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr"/>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Accurate closed-form delay formulas for interconnected CMOS gates based on first-order thresholded hybrid systems</t>
+        </is>
+      </c>
+      <c r="C613" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Ferdowsi, Arman; Függer, Matthias; Salzmann, Josef; Schmid, Ulrich</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr"/>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>10.1016/j.vlsi.2026.102701</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.vlsi.2026.102701</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K613" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L613" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M613" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N613" t="inlineStr"/>
+      <c r="O613" t="inlineStr"/>
+      <c r="P613" t="inlineStr"/>
+      <c r="Q613" t="inlineStr">
+        <is>
+          <t>Accurate closed-form delay formulas for interconnected CMOS gates based on first-order thresholded hybrid systems</t>
+        </is>
+      </c>
+      <c r="R613" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S613" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T613" t="inlineStr"/>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr"/>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Stator Resistance Compensation for PI-Based Field-Oriented Control of SPMSM Drives Using a Multilevel Inverter</t>
+        </is>
+      </c>
+      <c r="C614" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr"/>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>Quan, Nguyen Vinh; Son, Nguyen Ngoc</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr"/>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9591331/v1</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9591331/v1</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K614" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L614" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M614" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N614" t="inlineStr"/>
+      <c r="O614" t="inlineStr"/>
+      <c r="P614" t="inlineStr"/>
+      <c r="Q614" t="inlineStr">
+        <is>
+          <t>Stator Resistance Compensation for PI-Based Field-Oriented Control of SPMSM Drives Using a Multilevel Inverter</t>
+        </is>
+      </c>
+      <c r="R614" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S614" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="T614" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-04T01:44Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T614"/>
+  <dimension ref="A1:T618"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46840,6 +46840,302 @@
       </c>
       <c r="T614" t="inlineStr"/>
     </row>
+    <row r="615">
+      <c r="A615" t="inlineStr"/>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Traditional, complementary and alternative medicine: anaesthestic implications</t>
+        </is>
+      </c>
+      <c r="C615" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>World Federation of Societies of Anaesthesiologists</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr"/>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>Makanisi, Hylda; Hadebe, Simphiwe</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr"/>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>10.28923/atotw.576</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.28923/atotw.576</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K615" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L615" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M615" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N615" t="inlineStr"/>
+      <c r="O615" t="inlineStr"/>
+      <c r="P615" t="inlineStr"/>
+      <c r="Q615" t="inlineStr">
+        <is>
+          <t>Traditional, complementary and alternative medicine: anaesthestic implications</t>
+        </is>
+      </c>
+      <c r="R615" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S615" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="T615" t="inlineStr"/>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr"/>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Traditional, complementary and alternative medicine: anaesthestic implications</t>
+        </is>
+      </c>
+      <c r="C616" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>World Federation of Societies of Anaesthesiologists</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr"/>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Makanisi, Hylda; Hadebe, Simphiwe</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr"/>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>10.28923/atotw.576</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.28923/atotw.576</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K616" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L616" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M616" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N616" t="inlineStr"/>
+      <c r="O616" t="inlineStr"/>
+      <c r="P616" t="inlineStr"/>
+      <c r="Q616" t="inlineStr">
+        <is>
+          <t>Traditional, complementary and alternative medicine: anaesthestic implications</t>
+        </is>
+      </c>
+      <c r="R616" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S616" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="T616" t="inlineStr"/>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr"/>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Cylindrical FE–FE–DE heterostructure – assisted MOSFET for improved ON/OFF ratio and subthreshold swing</t>
+        </is>
+      </c>
+      <c r="C617" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Journal of Physics Communications</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>S, Pratheeksha; Nanjappa, Yashwanth; Mishra, Vikash; Awadhiya, Bhaskar</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr"/>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>10.1088/2399-6528/ae779d</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2399-6528/ae779d</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K617" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L617" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M617" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N617" t="inlineStr"/>
+      <c r="O617" t="inlineStr"/>
+      <c r="P617" t="inlineStr"/>
+      <c r="Q617" t="inlineStr">
+        <is>
+          <t>Cylindrical FE–FE–DE heterostructure – assisted MOSFET for improved ON/OFF ratio and subthreshold swing</t>
+        </is>
+      </c>
+      <c r="R617" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S617" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="T617" t="inlineStr"/>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr"/>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Cylindrical FE–FE–DE heterostructure – assisted MOSFET for improved ON/OFF ratio and subthreshold swing</t>
+        </is>
+      </c>
+      <c r="C618" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Journal of Physics Communications</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>S, Pratheeksha; Nanjappa, Yashwanth; Mishra, Vikash; Awadhiya, Bhaskar</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr"/>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>10.1088/2399-6528/ae779d</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2399-6528/ae779d</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K618" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L618" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M618" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N618" t="inlineStr"/>
+      <c r="O618" t="inlineStr"/>
+      <c r="P618" t="inlineStr"/>
+      <c r="Q618" t="inlineStr">
+        <is>
+          <t>Cylindrical FE–FE–DE heterostructure – assisted MOSFET for improved ON/OFF ratio and subthreshold swing</t>
+        </is>
+      </c>
+      <c r="R618" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S618" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="T618" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-05T00:13Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T618"/>
+  <dimension ref="A1:T631"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47136,6 +47136,994 @@
       </c>
       <c r="T618" t="inlineStr"/>
     </row>
+    <row r="619">
+      <c r="A619" t="inlineStr"/>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C619" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr"/>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K619" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L619" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M619" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N619" t="inlineStr"/>
+      <c r="O619" t="inlineStr"/>
+      <c r="P619" t="inlineStr"/>
+      <c r="Q619" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R619" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S619" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T619" t="inlineStr"/>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr"/>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C620" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr"/>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K620" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L620" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M620" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N620" t="inlineStr"/>
+      <c r="O620" t="inlineStr"/>
+      <c r="P620" t="inlineStr"/>
+      <c r="Q620" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R620" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S620" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T620" t="inlineStr"/>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr"/>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C621" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr"/>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K621" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L621" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M621" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N621" t="inlineStr"/>
+      <c r="O621" t="inlineStr"/>
+      <c r="P621" t="inlineStr"/>
+      <c r="Q621" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R621" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S621" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T621" t="inlineStr"/>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr"/>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Nested Monolithic Supercapacitor Patch Simultaneously Achieving High Stretchability, Stability, and Facile Integration for Flexible Electronics</t>
+        </is>
+      </c>
+      <c r="C622" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Advanced Functional Materials</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>Ye, Pengyuan; Mu, Chuanling; Fu, Lu; Zhang, Xiaojiang; Zuo, Wenjie; Li, Wen</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr"/>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>10.1002/adfm.76318</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/adfm.76318</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K622" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L622" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M622" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N622" t="inlineStr"/>
+      <c r="O622" t="inlineStr"/>
+      <c r="P622" t="inlineStr"/>
+      <c r="Q622" t="inlineStr">
+        <is>
+          <t>Nested Monolithic Supercapacitor Patch Simultaneously Achieving High Stretchability, Stability, and Facile Integration for Flexible Electronics</t>
+        </is>
+      </c>
+      <c r="R622" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S622" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T622" t="inlineStr"/>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr"/>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C623" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr"/>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K623" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L623" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M623" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N623" t="inlineStr"/>
+      <c r="O623" t="inlineStr"/>
+      <c r="P623" t="inlineStr"/>
+      <c r="Q623" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R623" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S623" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T623" t="inlineStr"/>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr"/>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C624" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr"/>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K624" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L624" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M624" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N624" t="inlineStr"/>
+      <c r="O624" t="inlineStr"/>
+      <c r="P624" t="inlineStr"/>
+      <c r="Q624" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R624" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S624" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T624" t="inlineStr"/>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr"/>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C625" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr"/>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K625" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L625" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M625" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N625" t="inlineStr"/>
+      <c r="O625" t="inlineStr"/>
+      <c r="P625" t="inlineStr"/>
+      <c r="Q625" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R625" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S625" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T625" t="inlineStr"/>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr"/>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C626" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr"/>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K626" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L626" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M626" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N626" t="inlineStr"/>
+      <c r="O626" t="inlineStr"/>
+      <c r="P626" t="inlineStr"/>
+      <c r="Q626" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R626" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S626" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T626" t="inlineStr"/>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr"/>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C627" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr"/>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K627" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L627" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M627" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N627" t="inlineStr"/>
+      <c r="O627" t="inlineStr"/>
+      <c r="P627" t="inlineStr"/>
+      <c r="Q627" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R627" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S627" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T627" t="inlineStr"/>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr"/>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C628" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr"/>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K628" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L628" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M628" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N628" t="inlineStr"/>
+      <c r="O628" t="inlineStr"/>
+      <c r="P628" t="inlineStr"/>
+      <c r="Q628" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R628" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S628" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T628" t="inlineStr"/>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr"/>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C629" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr"/>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K629" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L629" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M629" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N629" t="inlineStr"/>
+      <c r="O629" t="inlineStr"/>
+      <c r="P629" t="inlineStr"/>
+      <c r="Q629" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R629" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S629" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T629" t="inlineStr"/>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr"/>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C630" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr"/>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K630" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L630" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M630" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N630" t="inlineStr"/>
+      <c r="O630" t="inlineStr"/>
+      <c r="P630" t="inlineStr"/>
+      <c r="Q630" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R630" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S630" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T630" t="inlineStr"/>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr"/>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="C631" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Chinese Physics B</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>Xu, Shihao; Yang, Cui; Mao, Wei; Liu, Zhihong; Duan, Yu; He, Zhengda; Tang, Bowen; Zhang, Jincheng; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr"/>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1674-1056/ae77d1</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K631" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L631" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M631" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N631" t="inlineStr"/>
+      <c r="O631" t="inlineStr"/>
+      <c r="P631" t="inlineStr"/>
+      <c r="Q631" t="inlineStr">
+        <is>
+          <t>1980 V Vertical GaN-on-GaN Trench MOSFET with Step-Etched Implanted Guard Ring</t>
+        </is>
+      </c>
+      <c r="R631" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S631" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="T631" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-06T00:10Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T631"/>
+  <dimension ref="A1:T633"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48124,6 +48124,158 @@
       </c>
       <c r="T631" t="inlineStr"/>
     </row>
+    <row r="632">
+      <c r="A632" t="inlineStr"/>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Highly Reliable Common-Ground Single-Phase PV Grid-Connected Inverter</t>
+        </is>
+      </c>
+      <c r="C632" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>Do, Duc-Tuan; Nguyen Le, Huy-Bang; Tran, Viet-Hong; Tran, Anh-Tuan; Dinh, Van-Nghiep</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr"/>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15112493</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15112493</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K632" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L632" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M632" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N632" t="inlineStr"/>
+      <c r="O632" t="inlineStr"/>
+      <c r="P632" t="inlineStr"/>
+      <c r="Q632" t="inlineStr">
+        <is>
+          <t>Highly Reliable Common-Ground Single-Phase PV Grid-Connected Inverter</t>
+        </is>
+      </c>
+      <c r="R632" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S632" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="T632" t="inlineStr"/>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr"/>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Pendulum-actuated fiber-optic polarization-based torsion sensor for high-precision open-channel flow velocity measurement: Demonstration and modelling</t>
+        </is>
+      </c>
+      <c r="C633" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Measurement Science and Technology</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>MONDAL, SAIKAT; Roy Chaudhuri, Abhimanyu; Hanmaiahgari, Prashanth Reddy; ROY CHAUDHURI, PARTHA</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr"/>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6501/ae78f1</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6501/ae78f1</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K633" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L633" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M633" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N633" t="inlineStr"/>
+      <c r="O633" t="inlineStr"/>
+      <c r="P633" t="inlineStr"/>
+      <c r="Q633" t="inlineStr">
+        <is>
+          <t>Pendulum-actuated fiber-optic polarization-based torsion sensor for high-precision open-channel flow velocity measurement: Demonstration and modelling</t>
+        </is>
+      </c>
+      <c r="R633" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S633" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="T633" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-07T00:07Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T633"/>
+  <dimension ref="A1:T634"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48276,6 +48276,82 @@
       </c>
       <c r="T633" t="inlineStr"/>
     </row>
+    <row r="634">
+      <c r="A634" t="inlineStr"/>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Sustainable materials engineering of plasmonic Al–ZnO nanostructures for CMOS-compatible and reliable deep-UV photodetection</t>
+        </is>
+      </c>
+      <c r="C634" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Discover Materials</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>Qassim, Rami A.; Al Mashhadany, Yousif; Arsad, Norhana</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr"/>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>10.1007/s43939-026-00750-z</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s43939-026-00750-z</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K634" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L634" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M634" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N634" t="inlineStr"/>
+      <c r="O634" t="inlineStr"/>
+      <c r="P634" t="inlineStr"/>
+      <c r="Q634" t="inlineStr">
+        <is>
+          <t>Sustainable materials engineering of plasmonic Al–ZnO nanostructures for CMOS-compatible and reliable deep-UV photodetection</t>
+        </is>
+      </c>
+      <c r="R634" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S634" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="T634" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-08T00:12Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T634"/>
+  <dimension ref="A1:T635"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48352,6 +48352,82 @@
       </c>
       <c r="T634" t="inlineStr"/>
     </row>
+    <row r="635">
+      <c r="A635" t="inlineStr"/>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>PINN-Based Design of Cold Bent Monolithic Glass</t>
+        </is>
+      </c>
+      <c r="C635" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Stichting OpenAccess Foundation</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Challenging Glass Conference Proceedings</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>Laurs, Maximilian; Feldmann, Markus; Kraus, Michael</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr"/>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>10.47982/cgc.10.714</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.47982/cgc.10.714</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K635" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L635" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M635" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N635" t="inlineStr"/>
+      <c r="O635" t="inlineStr"/>
+      <c r="P635" t="inlineStr"/>
+      <c r="Q635" t="inlineStr">
+        <is>
+          <t>PINN-Based Design of Cold Bent Monolithic Glass</t>
+        </is>
+      </c>
+      <c r="R635" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S635" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="T635" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-09T00:09Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T635"/>
+  <dimension ref="A1:T638"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48428,6 +48428,234 @@
       </c>
       <c r="T635" t="inlineStr"/>
     </row>
+    <row r="636">
+      <c r="A636" t="inlineStr"/>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Clinically Significant Omega-3 Health Benefits From Stearidonic Acid and Buglossoides Oil: Plant-Based, Fish-Free Omega-3 that Converts Effectively to Eicosapentaenoic Acid/Docosahexaenoic Acid</t>
+        </is>
+      </c>
+      <c r="C636" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Integrative and Complementary Therapies</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>Hanaway, Patrick</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr"/>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>10.1177/27683192261456168</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683192261456168</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K636" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L636" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M636" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N636" t="inlineStr"/>
+      <c r="O636" t="inlineStr"/>
+      <c r="P636" t="inlineStr"/>
+      <c r="Q636" t="inlineStr">
+        <is>
+          <t>Clinically Significant Omega-3 Health Benefits From Stearidonic Acid and Buglossoides Oil: Plant-Based, Fish-Free Omega-3 that Converts Effectively to Eicosapentaenoic Acid/Docosahexaenoic Acid</t>
+        </is>
+      </c>
+      <c r="R636" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S636" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="T636" t="inlineStr"/>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr"/>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Precast-monolithic beam reinforced concrete floors with aerated concrete blocks</t>
+        </is>
+      </c>
+      <c r="C637" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>JVE International Ltd.</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Vibroengineering Procedia</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>Abdullayev, Ibrohim; Yunusaliev, Elmurod; Alakhanov, Zokir; Mukhammadyoqubov, Xusanboy</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr"/>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>10.21595/vp.2025.25505</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21595/vp.2025.25505</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K637" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L637" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M637" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N637" t="inlineStr"/>
+      <c r="O637" t="inlineStr"/>
+      <c r="P637" t="inlineStr"/>
+      <c r="Q637" t="inlineStr">
+        <is>
+          <t>Precast-monolithic beam reinforced concrete floors with aerated concrete blocks</t>
+        </is>
+      </c>
+      <c r="R637" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S637" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="T637" t="inlineStr"/>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr"/>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Impact of Channel Width on Electrical Characteristics for Inversion Mode N-channel TFT on Polycrystalline Ge by Solid Phase Crystallization</t>
+        </is>
+      </c>
+      <c r="C638" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>HUANG, LINYU; Igura, Kota; Wang, Dong; Toko, Kaoru; Yamamoto, Keisuke</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr"/>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae79a7</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae79a7</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K638" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L638" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M638" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N638" t="inlineStr"/>
+      <c r="O638" t="inlineStr"/>
+      <c r="P638" t="inlineStr"/>
+      <c r="Q638" t="inlineStr">
+        <is>
+          <t>Impact of Channel Width on Electrical Characteristics for Inversion Mode N-channel TFT on Polycrystalline Ge by Solid Phase Crystallization</t>
+        </is>
+      </c>
+      <c r="R638" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S638" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="T638" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-10T00:19Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T638"/>
+  <dimension ref="A1:T650"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48656,6 +48656,958 @@
       </c>
       <c r="T638" t="inlineStr"/>
     </row>
+    <row r="639">
+      <c r="A639" t="inlineStr"/>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Grid-Forming Inverter Control for Renewable-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="C639" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Eduschool Academic Research and Publishers</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>International Journal of Technical Research Studies (IJTRS)</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>A H, Deepesh</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr"/>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>10.63090/ijtrs/3139.1788.0014</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.63090/ijtrs/3139.1788.0014</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K639" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L639" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M639" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N639" t="inlineStr"/>
+      <c r="O639" t="inlineStr"/>
+      <c r="P639" t="inlineStr"/>
+      <c r="Q639" t="inlineStr">
+        <is>
+          <t>Grid-Forming Inverter Control for Renewable-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="R639" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S639" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T639" t="inlineStr"/>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr"/>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Correction: Ahmadimonfared, Z.; Eichner, S. Stability Assessment of Fully Inverter-Based Power Systems Using Grid-Forming Controls. Electronics 2025, 14, 4202</t>
+        </is>
+      </c>
+      <c r="C640" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>Ahmadimonfared, Zahra; Eichner, Stefan</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr"/>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122540</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122540</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K640" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L640" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M640" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N640" t="inlineStr"/>
+      <c r="O640" t="inlineStr"/>
+      <c r="P640" t="inlineStr"/>
+      <c r="Q640" t="inlineStr">
+        <is>
+          <t>Correction: Ahmadimonfared, Z.; Eichner, S. Stability Assessment of Fully Inverter-Based Power Systems Using Grid-Forming Controls. Electronics 2025, 14, 4202</t>
+        </is>
+      </c>
+      <c r="R640" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S640" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T640" t="inlineStr"/>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr"/>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Grid-Forming Inverter Control for Renewable-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="C641" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Eduschool Academic Research and Publishers</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>International Journal of Technical Research Studies (IJTRS)</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>A H, Deepesh</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr"/>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>10.63090/ijtrs/3139.1788.0014</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.63090/ijtrs/3139.1788.0014</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K641" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L641" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M641" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N641" t="inlineStr"/>
+      <c r="O641" t="inlineStr"/>
+      <c r="P641" t="inlineStr"/>
+      <c r="Q641" t="inlineStr">
+        <is>
+          <t>Grid-Forming Inverter Control for Renewable-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="R641" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S641" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T641" t="inlineStr"/>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr"/>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Design of monolithic piezoelectric bimorph mirrors made from lithium niobate</t>
+        </is>
+      </c>
+      <c r="C642" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Optics Express</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>Marzari, Francesco; Cutler, Grant; Goldberg, Kenneth A.</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr"/>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>10.1364/oe.596443</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/oe.596443</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K642" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L642" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M642" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N642" t="inlineStr"/>
+      <c r="O642" t="inlineStr"/>
+      <c r="P642" t="inlineStr"/>
+      <c r="Q642" t="inlineStr">
+        <is>
+          <t>Design of monolithic piezoelectric bimorph mirrors made from lithium niobate</t>
+        </is>
+      </c>
+      <c r="R642" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S642" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T642" t="inlineStr"/>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr"/>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="C643" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>Narita, Tetsuo; Ito, Kenji; Iguchi, Hiroko; Tomita, Kazuyoshi; Horita, Masahiro; Iwasaki, Shiro; Kikuta, Daigo</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr"/>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K643" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L643" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M643" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N643" t="inlineStr"/>
+      <c r="O643" t="inlineStr"/>
+      <c r="P643" t="inlineStr"/>
+      <c r="Q643" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="R643" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S643" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T643" t="inlineStr"/>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr"/>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="C644" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>Narita, Tetsuo; Ito, Kenji; Iguchi, Hiroko; Tomita, Kazuyoshi; Horita, Masahiro; Iwasaki, Shiro; Kikuta, Daigo</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr"/>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K644" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L644" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M644" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N644" t="inlineStr"/>
+      <c r="O644" t="inlineStr"/>
+      <c r="P644" t="inlineStr"/>
+      <c r="Q644" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="R644" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S644" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T644" t="inlineStr"/>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr"/>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="C645" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>Narita, Tetsuo; Ito, Kenji; Iguchi, Hiroko; Tomita, Kazuyoshi; Horita, Masahiro; Iwasaki, Shiro; Kikuta, Daigo</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr"/>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K645" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L645" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M645" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N645" t="inlineStr"/>
+      <c r="O645" t="inlineStr"/>
+      <c r="P645" t="inlineStr"/>
+      <c r="Q645" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="R645" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S645" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T645" t="inlineStr"/>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr"/>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Grid-Forming Inverter Control for Renewable-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="C646" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Eduschool Academic Research and Publishers</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>International Journal of Technical Research Studies (IJTRS)</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>A H, Deepesh</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr"/>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>10.63090/ijtrs/3139.1788.0014</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.63090/ijtrs/3139.1788.0014</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K646" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L646" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M646" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N646" t="inlineStr"/>
+      <c r="O646" t="inlineStr"/>
+      <c r="P646" t="inlineStr"/>
+      <c r="Q646" t="inlineStr">
+        <is>
+          <t>Grid-Forming Inverter Control for Renewable-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="R646" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S646" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T646" t="inlineStr"/>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr"/>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Correction: Ahmadimonfared, Z.; Eichner, S. Stability Assessment of Fully Inverter-Based Power Systems Using Grid-Forming Controls. Electronics 2025, 14, 4202</t>
+        </is>
+      </c>
+      <c r="C647" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Ahmadimonfared, Zahra; Eichner, Stefan</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr"/>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122540</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122540</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K647" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L647" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M647" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N647" t="inlineStr"/>
+      <c r="O647" t="inlineStr"/>
+      <c r="P647" t="inlineStr"/>
+      <c r="Q647" t="inlineStr">
+        <is>
+          <t>Correction: Ahmadimonfared, Z.; Eichner, S. Stability Assessment of Fully Inverter-Based Power Systems Using Grid-Forming Controls. Electronics 2025, 14, 4202</t>
+        </is>
+      </c>
+      <c r="R647" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S647" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T647" t="inlineStr"/>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr"/>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Grid-Forming Inverter Control for Renewable-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="C648" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Eduschool Academic Research and Publishers</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>International Journal of Technical Research Studies (IJTRS)</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>A H, Deepesh</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr"/>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>10.63090/ijtrs/3139.1788.0014</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.63090/ijtrs/3139.1788.0014</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K648" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L648" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M648" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N648" t="inlineStr"/>
+      <c r="O648" t="inlineStr"/>
+      <c r="P648" t="inlineStr"/>
+      <c r="Q648" t="inlineStr">
+        <is>
+          <t>Grid-Forming Inverter Control for Renewable-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="R648" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S648" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T648" t="inlineStr"/>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr"/>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="C649" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Narita, Tetsuo; Ito, Kenji; Iguchi, Hiroko; Tomita, Kazuyoshi; Horita, Masahiro; Iwasaki, Shiro; Kikuta, Daigo</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr"/>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K649" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L649" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M649" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N649" t="inlineStr"/>
+      <c r="O649" t="inlineStr"/>
+      <c r="P649" t="inlineStr"/>
+      <c r="Q649" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="R649" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S649" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T649" t="inlineStr"/>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr"/>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="C650" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>Narita, Tetsuo; Ito, Kenji; Iguchi, Hiroko; Tomita, Kazuyoshi; Horita, Masahiro; Iwasaki, Shiro; Kikuta, Daigo</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr"/>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0324229</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K650" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L650" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M650" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N650" t="inlineStr"/>
+      <c r="O650" t="inlineStr"/>
+      <c r="P650" t="inlineStr"/>
+      <c r="Q650" t="inlineStr">
+        <is>
+          <t>Investigation of Coulomb scattering centers using a substrate bias effect in
+                    &lt;i&gt;n&lt;/i&gt;
+                    -channel metal–oxide–semiconductor field-effect transistors with AlSiO/AlN/
+                    &lt;i&gt;p&lt;/i&gt;
+                    -type GaN gate structures</t>
+        </is>
+      </c>
+      <c r="R650" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S650" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="T650" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-11T00:19Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T650"/>
+  <dimension ref="A1:T653"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49608,6 +49608,234 @@
       </c>
       <c r="T650" t="inlineStr"/>
     </row>
+    <row r="651">
+      <c r="A651" t="inlineStr"/>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Retail channel, direct channel, or dual channels: which works better for manufacturers' trade-ins?</t>
+        </is>
+      </c>
+      <c r="C651" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Asia Pacific Journal of Marketing and Logistics</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>Tang, Fei; Dai, Ying; Ma, Zujun</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr"/>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>10.1108/apjml-10-2025-2270</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/apjml-10-2025-2270</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K651" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L651" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M651" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N651" t="inlineStr"/>
+      <c r="O651" t="inlineStr"/>
+      <c r="P651" t="inlineStr"/>
+      <c r="Q651" t="inlineStr">
+        <is>
+          <t>Retail channel, direct channel, or dual channels: which works better for manufacturers' trade-ins?</t>
+        </is>
+      </c>
+      <c r="R651" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S651" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="T651" t="inlineStr"/>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr"/>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Electro-Thermal Characteristics of E-Mode GaN HEMTs with Ohmic and Schottky Gates</t>
+        </is>
+      </c>
+      <c r="C652" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>Kim, Minji; Oh, Jiun; Han, Younghun; Song, June-O; Kwak, Joon Seop</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr"/>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122560</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122560</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K652" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L652" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M652" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N652" t="inlineStr"/>
+      <c r="O652" t="inlineStr"/>
+      <c r="P652" t="inlineStr"/>
+      <c r="Q652" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Electro-Thermal Characteristics of E-Mode GaN HEMTs with Ohmic and Schottky Gates</t>
+        </is>
+      </c>
+      <c r="R652" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S652" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="T652" t="inlineStr"/>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr"/>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Electro-Thermal Characteristics of E-Mode GaN HEMTs with Ohmic and Schottky Gates</t>
+        </is>
+      </c>
+      <c r="C653" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Kim, Minji; Oh, Jiun; Han, Younghun; Song, June-O; Kwak, Joon Seop</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr"/>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122560</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122560</t>
+        </is>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K653" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L653" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M653" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N653" t="inlineStr"/>
+      <c r="O653" t="inlineStr"/>
+      <c r="P653" t="inlineStr"/>
+      <c r="Q653" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Electro-Thermal Characteristics of E-Mode GaN HEMTs with Ohmic and Schottky Gates</t>
+        </is>
+      </c>
+      <c r="R653" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S653" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="T653" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-12T00:20Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T653"/>
+  <dimension ref="A1:T660"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49836,6 +49836,530 @@
       </c>
       <c r="T653" t="inlineStr"/>
     </row>
+    <row r="654">
+      <c r="A654" t="inlineStr"/>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Integrated Satellite Avionics with High Reliability and Low Cost Based on a Monolithic System-on-Programmable-Chip</t>
+        </is>
+      </c>
+      <c r="C654" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Fang, Sichao; Dai, Lu; Zou, Jiwei; Wang, Junbo; Chen, Tao</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr"/>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122574</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122574</t>
+        </is>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K654" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L654" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M654" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N654" t="inlineStr"/>
+      <c r="O654" t="inlineStr"/>
+      <c r="P654" t="inlineStr"/>
+      <c r="Q654" t="inlineStr">
+        <is>
+          <t>Integrated Satellite Avionics with High Reliability and Low Cost Based on a Monolithic System-on-Programmable-Chip</t>
+        </is>
+      </c>
+      <c r="R654" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S654" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="T654" t="inlineStr"/>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr"/>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Monolithic and hybrid integrated on chip optical filters for compact multi- and hyperspectral imaging payloads</t>
+        </is>
+      </c>
+      <c r="C655" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>SPIE</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Sensors and Systems for Space Applications XIX</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Delauré, B.; Berteloot, B.; Tack, K.</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr"/>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>10.1117/12.3094858</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1117/12.3094858</t>
+        </is>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K655" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L655" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M655" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N655" t="inlineStr"/>
+      <c r="O655" t="inlineStr"/>
+      <c r="P655" t="inlineStr"/>
+      <c r="Q655" t="inlineStr">
+        <is>
+          <t>Monolithic and hybrid integrated on chip optical filters for compact multi- and hyperspectral imaging payloads</t>
+        </is>
+      </c>
+      <c r="R655" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S655" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="T655" t="inlineStr"/>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr"/>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>DESIGN AND OPTIMIZATION OF A 7.7 GHZ RF POWER AMPLIFIER USING GAN HEMT TRANSISTOR ON ROGERS 5880LZ SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="C656" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City University of Industry and Trade</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Tạp chí Khoa học Đại học Công Thương</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Hoai Nam Tran; Manh Dan Do; Xuan Quynh Le; Van Tu Dinh</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr"/>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>10.62985/j.huit_ojs.vol26.no2e.384</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.62985/j.huit_ojs.vol26.no2e.384</t>
+        </is>
+      </c>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K656" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L656" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M656" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N656" t="inlineStr"/>
+      <c r="O656" t="inlineStr"/>
+      <c r="P656" t="inlineStr"/>
+      <c r="Q656" t="inlineStr">
+        <is>
+          <t>DESIGN AND OPTIMIZATION OF A 7.7 GHZ RF POWER AMPLIFIER USING GAN HEMT TRANSISTOR ON ROGERS 5880LZ SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="R656" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S656" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="T656" t="inlineStr"/>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr"/>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Lightweight Hybrid Additively Manufactured Liquid Cooler for 10 kV SiC MOSFET Power Module</t>
+        </is>
+      </c>
+      <c r="C657" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Open Engineering Inc</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr"/>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Pierson, Stephen; Wu, Qiang; Li, Xiaoling; Pandey, Hari; Weems, Ethan; Mantooth, H. Alan; Hu, Han</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr"/>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>10.31224/7304</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.31224/7304</t>
+        </is>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K657" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L657" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M657" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N657" t="inlineStr"/>
+      <c r="O657" t="inlineStr"/>
+      <c r="P657" t="inlineStr"/>
+      <c r="Q657" t="inlineStr">
+        <is>
+          <t>Lightweight Hybrid Additively Manufactured Liquid Cooler for 10 kV SiC MOSFET Power Module</t>
+        </is>
+      </c>
+      <c r="R657" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S657" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="T657" t="inlineStr"/>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr"/>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Lightweight Hybrid Additively Manufactured Liquid Cooler for 10 kV SiC MOSFET Power Module</t>
+        </is>
+      </c>
+      <c r="C658" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Open Engineering Inc</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr"/>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Pierson, Stephen; Wu, Qiang; Li, Xiaoling; Pandey, Hari; Weems, Ethan; Mantooth, H. Alan; Hu, Han</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr"/>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>10.31224/7304</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.31224/7304</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K658" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L658" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M658" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N658" t="inlineStr"/>
+      <c r="O658" t="inlineStr"/>
+      <c r="P658" t="inlineStr"/>
+      <c r="Q658" t="inlineStr">
+        <is>
+          <t>Lightweight Hybrid Additively Manufactured Liquid Cooler for 10 kV SiC MOSFET Power Module</t>
+        </is>
+      </c>
+      <c r="R658" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S658" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="T658" t="inlineStr"/>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr"/>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>DESIGN AND OPTIMIZATION OF A 7.7 GHZ RF POWER AMPLIFIER USING GAN HEMT TRANSISTOR ON ROGERS 5880LZ SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="C659" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City University of Industry and Trade</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Tạp chí Khoa học Đại học Công Thương</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Hoai Nam Tran; Manh Dan Do; Xuan Quynh Le; Van Tu Dinh</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr"/>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>10.62985/j.huit_ojs.vol26.no2e.384</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.62985/j.huit_ojs.vol26.no2e.384</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K659" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L659" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M659" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N659" t="inlineStr"/>
+      <c r="O659" t="inlineStr"/>
+      <c r="P659" t="inlineStr"/>
+      <c r="Q659" t="inlineStr">
+        <is>
+          <t>DESIGN AND OPTIMIZATION OF A 7.7 GHZ RF POWER AMPLIFIER USING GAN HEMT TRANSISTOR ON ROGERS 5880LZ SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="R659" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S659" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="T659" t="inlineStr"/>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr"/>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>DESIGN AND OPTIMIZATION OF A 7.7 GHZ RF POWER AMPLIFIER USING GAN HEMT TRANSISTOR ON ROGERS 5880LZ SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="C660" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City University of Industry and Trade</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Tạp chí Khoa học Đại học Công Thương</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>Hoai Nam Tran; Manh Dan Do; Xuan Quynh Le; Van Tu Dinh</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr"/>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>10.62985/j.huit_ojs.vol26.no2e.384</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.62985/j.huit_ojs.vol26.no2e.384</t>
+        </is>
+      </c>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K660" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L660" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M660" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N660" t="inlineStr"/>
+      <c r="O660" t="inlineStr"/>
+      <c r="P660" t="inlineStr"/>
+      <c r="Q660" t="inlineStr">
+        <is>
+          <t>DESIGN AND OPTIMIZATION OF A 7.7 GHZ RF POWER AMPLIFIER USING GAN HEMT TRANSISTOR ON ROGERS 5880LZ SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="R660" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S660" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="T660" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-13T00:22Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T660"/>
+  <dimension ref="A1:T662"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50360,6 +50360,158 @@
       </c>
       <c r="T660" t="inlineStr"/>
     </row>
+    <row r="661">
+      <c r="A661" t="inlineStr"/>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Stable low-resistance ohmic contact on GaN via an oxynitride interlayer over 20–200 °C: Mechanisms and performance</t>
+        </is>
+      </c>
+      <c r="C661" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>Xie, Shujie; Xu, Hengyu; Wan, Caiping; Hu, Zongyang; Cheng, Zhe; Wu, Xuankun; Mi, Chanxin; Yi, Boyang; Lian, Mengxiao; He, Yingrui; Zhang, Yun</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr"/>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>10.1063/5.0324776</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0324776</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K661" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L661" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M661" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N661" t="inlineStr"/>
+      <c r="O661" t="inlineStr"/>
+      <c r="P661" t="inlineStr"/>
+      <c r="Q661" t="inlineStr">
+        <is>
+          <t>Stable low-resistance ohmic contact on GaN via an oxynitride interlayer over 20–200 °C: Mechanisms and performance</t>
+        </is>
+      </c>
+      <c r="R661" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S661" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="T661" t="inlineStr"/>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr"/>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Stable low-resistance ohmic contact on GaN via an oxynitride interlayer over 20–200 °C: Mechanisms and performance</t>
+        </is>
+      </c>
+      <c r="C662" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Xie, Shujie; Xu, Hengyu; Wan, Caiping; Hu, Zongyang; Cheng, Zhe; Wu, Xuankun; Mi, Chanxin; Yi, Boyang; Lian, Mengxiao; He, Yingrui; Zhang, Yun</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr"/>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>10.1063/5.0324776</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0324776</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L662" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M662" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N662" t="inlineStr"/>
+      <c r="O662" t="inlineStr"/>
+      <c r="P662" t="inlineStr"/>
+      <c r="Q662" t="inlineStr">
+        <is>
+          <t>Stable low-resistance ohmic contact on GaN via an oxynitride interlayer over 20–200 °C: Mechanisms and performance</t>
+        </is>
+      </c>
+      <c r="R662" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S662" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="T662" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-16T01:42Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T662"/>
+  <dimension ref="A1:T666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50512,6 +50512,306 @@
       </c>
       <c r="T662" t="inlineStr"/>
     </row>
+    <row r="663">
+      <c r="A663" t="inlineStr"/>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Simulation Research on PID Control of Single-Phase Full-Bridge Inverter Based on MATLAB/Simulink</t>
+        </is>
+      </c>
+      <c r="C663" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>EWA Publishing</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Applied and Computational Engineering</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Su, Zerui</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr"/>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>10.54254/2755-2721/2026.34397</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54254/2755-2721/2026.34397</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K663" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L663" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M663" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N663" t="inlineStr"/>
+      <c r="O663" t="inlineStr"/>
+      <c r="P663" t="inlineStr"/>
+      <c r="Q663" t="inlineStr">
+        <is>
+          <t>Simulation Research on PID Control of Single-Phase Full-Bridge Inverter Based on MATLAB/Simulink</t>
+        </is>
+      </c>
+      <c r="R663" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S663" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="T663" t="inlineStr"/>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr"/>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>A monolithic component mode synthesis two-way fluid-structure interaction approach for hydrodynamic lubricated journal and slider plain bearings</t>
+        </is>
+      </c>
+      <c r="C664" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr"/>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Resch, Reinhard</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr"/>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-9671897/v1</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-9671897/v1</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K664" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L664" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M664" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N664" t="inlineStr"/>
+      <c r="O664" t="inlineStr"/>
+      <c r="P664" t="inlineStr"/>
+      <c r="Q664" t="inlineStr">
+        <is>
+          <t>A monolithic component mode synthesis two-way fluid-structure interaction approach for hydrodynamic lubricated journal and slider plain bearings</t>
+        </is>
+      </c>
+      <c r="R664" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S664" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="T664" t="inlineStr"/>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr"/>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Origin of threshold voltage instability in vertical GaN trench MOSFETs characterized by charge pumping</t>
+        </is>
+      </c>
+      <c r="C665" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>Luo, Haowen; Zhu, Renqiang; Fan, Xuancong; Yang, Wen; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr"/>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>10.1063/5.0331928</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0331928</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K665" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L665" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M665" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N665" t="inlineStr"/>
+      <c r="O665" t="inlineStr"/>
+      <c r="P665" t="inlineStr"/>
+      <c r="Q665" t="inlineStr">
+        <is>
+          <t>Origin of threshold voltage instability in vertical GaN trench MOSFETs characterized by charge pumping</t>
+        </is>
+      </c>
+      <c r="R665" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S665" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="T665" t="inlineStr"/>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr"/>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Simulation Research on PID Control of Single-Phase Full-Bridge Inverter Based on MATLAB/Simulink</t>
+        </is>
+      </c>
+      <c r="C666" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>EWA Publishing</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Applied and Computational Engineering</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>Su, Zerui</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr"/>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>10.54254/2755-2721/2026.34397</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54254/2755-2721/2026.34397</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K666" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L666" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M666" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N666" t="inlineStr"/>
+      <c r="O666" t="inlineStr"/>
+      <c r="P666" t="inlineStr"/>
+      <c r="Q666" t="inlineStr">
+        <is>
+          <t>Simulation Research on PID Control of Single-Phase Full-Bridge Inverter Based on MATLAB/Simulink</t>
+        </is>
+      </c>
+      <c r="R666" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S666" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="T666" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-17T00:20Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T666"/>
+  <dimension ref="A1:T670"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50812,6 +50812,310 @@
       </c>
       <c r="T666" t="inlineStr"/>
     </row>
+    <row r="667">
+      <c r="A667" t="inlineStr"/>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Performance Analysis of GAA Nanowire MOSFET through Dielectric Pocket and Tri Metal Gate Engineering</t>
+        </is>
+      </c>
+      <c r="C667" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>Swetha, A.; Balaji, B.; Cheerla, Sreevardhan; Sreenivasa Rao, Devireddy</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr"/>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae7e46</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae7e46</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K667" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L667" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M667" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N667" t="inlineStr"/>
+      <c r="O667" t="inlineStr"/>
+      <c r="P667" t="inlineStr"/>
+      <c r="Q667" t="inlineStr">
+        <is>
+          <t>Performance Analysis of GAA Nanowire MOSFET through Dielectric Pocket and Tri Metal Gate Engineering</t>
+        </is>
+      </c>
+      <c r="R667" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S667" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="T667" t="inlineStr"/>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr"/>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Performance Analysis of GAA Nanowire MOSFET through Dielectric Pocket and Tri Metal Gate Engineering</t>
+        </is>
+      </c>
+      <c r="C668" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>Swetha, A.; Balaji, B.; Cheerla, Sreevardhan; Sreenivasa Rao, Devireddy</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr"/>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae7e46</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae7e46</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K668" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L668" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M668" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N668" t="inlineStr"/>
+      <c r="O668" t="inlineStr"/>
+      <c r="P668" t="inlineStr"/>
+      <c r="Q668" t="inlineStr">
+        <is>
+          <t>Performance Analysis of GAA Nanowire MOSFET through Dielectric Pocket and Tri Metal Gate Engineering</t>
+        </is>
+      </c>
+      <c r="R668" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S668" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="T668" t="inlineStr"/>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr"/>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Performance Analysis of GAA Nanowire MOSFET through Dielectric Pocket and Tri Metal Gate Engineering</t>
+        </is>
+      </c>
+      <c r="C669" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>Swetha, A.; Balaji, B.; Cheerla, Sreevardhan; Sreenivasa Rao, Devireddy</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr"/>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae7e46</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae7e46</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K669" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L669" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M669" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N669" t="inlineStr"/>
+      <c r="O669" t="inlineStr"/>
+      <c r="P669" t="inlineStr"/>
+      <c r="Q669" t="inlineStr">
+        <is>
+          <t>Performance Analysis of GAA Nanowire MOSFET through Dielectric Pocket and Tri Metal Gate Engineering</t>
+        </is>
+      </c>
+      <c r="R669" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S669" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="T669" t="inlineStr"/>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr"/>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Performance Analysis of GAA Nanowire MOSFET through Dielectric Pocket and Tri Metal Gate Engineering</t>
+        </is>
+      </c>
+      <c r="C670" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>Swetha, A.; Balaji, B.; Cheerla, Sreevardhan; Sreenivasa Rao, Devireddy</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr"/>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae7e46</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae7e46</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K670" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L670" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M670" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N670" t="inlineStr"/>
+      <c r="O670" t="inlineStr"/>
+      <c r="P670" t="inlineStr"/>
+      <c r="Q670" t="inlineStr">
+        <is>
+          <t>Performance Analysis of GAA Nanowire MOSFET through Dielectric Pocket and Tri Metal Gate Engineering</t>
+        </is>
+      </c>
+      <c r="R670" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S670" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="T670" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-18T00:18Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T670"/>
+  <dimension ref="A1:T683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51116,6 +51116,994 @@
       </c>
       <c r="T670" t="inlineStr"/>
     </row>
+    <row r="671">
+      <c r="A671" t="inlineStr"/>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C671" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr"/>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K671" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L671" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M671" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N671" t="inlineStr"/>
+      <c r="O671" t="inlineStr"/>
+      <c r="P671" t="inlineStr"/>
+      <c r="Q671" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R671" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S671" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T671" t="inlineStr"/>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr"/>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Cross-Platform Neuromorphic Photodetectors: From Organic and Oxide to Perovskite, Wide-Bandgap, and Si-CMOS</t>
+        </is>
+      </c>
+      <c r="C672" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>Photonics</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>Weis, Martin</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr"/>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>10.3390/photonics13060589</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/photonics13060589</t>
+        </is>
+      </c>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K672" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L672" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M672" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N672" t="inlineStr"/>
+      <c r="O672" t="inlineStr"/>
+      <c r="P672" t="inlineStr"/>
+      <c r="Q672" t="inlineStr">
+        <is>
+          <t>Cross-Platform Neuromorphic Photodetectors: From Organic and Oxide to Perovskite, Wide-Bandgap, and Si-CMOS</t>
+        </is>
+      </c>
+      <c r="R672" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S672" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T672" t="inlineStr"/>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr"/>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Cross-Platform Neuromorphic Photodetectors: From Organic and Oxide to Perovskite, Wide-Bandgap, and Si-CMOS</t>
+        </is>
+      </c>
+      <c r="C673" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>Photonics</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>Weis, Martin</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr"/>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>10.3390/photonics13060589</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/photonics13060589</t>
+        </is>
+      </c>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K673" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L673" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M673" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N673" t="inlineStr"/>
+      <c r="O673" t="inlineStr"/>
+      <c r="P673" t="inlineStr"/>
+      <c r="Q673" t="inlineStr">
+        <is>
+          <t>Cross-Platform Neuromorphic Photodetectors: From Organic and Oxide to Perovskite, Wide-Bandgap, and Si-CMOS</t>
+        </is>
+      </c>
+      <c r="R673" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S673" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T673" t="inlineStr"/>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr"/>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C674" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr"/>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K674" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L674" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M674" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N674" t="inlineStr"/>
+      <c r="O674" t="inlineStr"/>
+      <c r="P674" t="inlineStr"/>
+      <c r="Q674" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R674" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S674" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T674" t="inlineStr"/>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr"/>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C675" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr"/>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K675" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L675" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M675" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N675" t="inlineStr"/>
+      <c r="O675" t="inlineStr"/>
+      <c r="P675" t="inlineStr"/>
+      <c r="Q675" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R675" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S675" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T675" t="inlineStr"/>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr"/>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C676" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr"/>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K676" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L676" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M676" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N676" t="inlineStr"/>
+      <c r="O676" t="inlineStr"/>
+      <c r="P676" t="inlineStr"/>
+      <c r="Q676" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R676" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S676" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T676" t="inlineStr"/>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr"/>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C677" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr"/>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K677" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L677" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M677" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N677" t="inlineStr"/>
+      <c r="O677" t="inlineStr"/>
+      <c r="P677" t="inlineStr"/>
+      <c r="Q677" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R677" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S677" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T677" t="inlineStr"/>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr"/>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C678" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr"/>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K678" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L678" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M678" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N678" t="inlineStr"/>
+      <c r="O678" t="inlineStr"/>
+      <c r="P678" t="inlineStr"/>
+      <c r="Q678" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R678" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S678" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T678" t="inlineStr"/>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr"/>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C679" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr"/>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K679" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L679" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M679" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N679" t="inlineStr"/>
+      <c r="O679" t="inlineStr"/>
+      <c r="P679" t="inlineStr"/>
+      <c r="Q679" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R679" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S679" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T679" t="inlineStr"/>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr"/>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C680" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr"/>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K680" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L680" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M680" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N680" t="inlineStr"/>
+      <c r="O680" t="inlineStr"/>
+      <c r="P680" t="inlineStr"/>
+      <c r="Q680" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R680" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S680" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T680" t="inlineStr"/>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr"/>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Cross-Platform Neuromorphic Photodetectors: From Organic and Oxide to Perovskite, Wide-Bandgap, and Si-CMOS</t>
+        </is>
+      </c>
+      <c r="C681" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Photonics</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Weis, Martin</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr"/>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>10.3390/photonics13060589</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/photonics13060589</t>
+        </is>
+      </c>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K681" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L681" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M681" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N681" t="inlineStr"/>
+      <c r="O681" t="inlineStr"/>
+      <c r="P681" t="inlineStr"/>
+      <c r="Q681" t="inlineStr">
+        <is>
+          <t>Cross-Platform Neuromorphic Photodetectors: From Organic and Oxide to Perovskite, Wide-Bandgap, and Si-CMOS</t>
+        </is>
+      </c>
+      <c r="R681" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S681" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T681" t="inlineStr"/>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr"/>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C682" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr"/>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J682" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K682" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L682" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M682" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N682" t="inlineStr"/>
+      <c r="O682" t="inlineStr"/>
+      <c r="P682" t="inlineStr"/>
+      <c r="Q682" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R682" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S682" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T682" t="inlineStr"/>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr"/>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="C683" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Gaillard, Pauline; Avertin, Sébastien; Drieu La Rochelle, Julien; Zeghouane, Mohammed; Chauveau, Hyon-Ju; Giorgino, Giovanni; Constant, Aurore; Iucolano, Ferdinando</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr"/>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122690</t>
+        </is>
+      </c>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K683" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L683" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M683" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N683" t="inlineStr"/>
+      <c r="O683" t="inlineStr"/>
+      <c r="P683" t="inlineStr"/>
+      <c r="Q683" t="inlineStr">
+        <is>
+          <t>p-GaN Layer Etch Engineering for Defect Reduction in 200 mm Enhanced-Mode AlGaN/GaN HEMT Processing</t>
+        </is>
+      </c>
+      <c r="R683" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S683" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="T683" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-19T01:45Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T683"/>
+  <dimension ref="A1:T687"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52104,6 +52104,310 @@
       </c>
       <c r="T683" t="inlineStr"/>
     </row>
+    <row r="684">
+      <c r="A684" t="inlineStr"/>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Bandgap engineering and high-throughput defect dynamics in two-terminal CsGeI3-Si monolithic tandem solar cells</t>
+        </is>
+      </c>
+      <c r="C684" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Singh, Sujata; Kaur, Gun Anit; Shandilya, Mamta; Sharma, Ajit; Singh, Pravin Kumar</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr"/>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-56282-2</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-56282-2</t>
+        </is>
+      </c>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K684" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L684" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M684" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N684" t="inlineStr"/>
+      <c r="O684" t="inlineStr"/>
+      <c r="P684" t="inlineStr"/>
+      <c r="Q684" t="inlineStr">
+        <is>
+          <t>Bandgap engineering and high-throughput defect dynamics in two-terminal CsGeI3-Si monolithic tandem solar cells</t>
+        </is>
+      </c>
+      <c r="R684" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S684" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="T684" t="inlineStr"/>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr"/>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Analysis of Multi-Finger GaN HEMTs Using Gate Resistance Thermometry, Raman Thermometry, and Infrared Thermal Microscopy</t>
+        </is>
+      </c>
+      <c r="C685" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>ASME International</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Journal of Electronic Packaging</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>Kim, Seokjun; Shoemaker, Daniel; Walwil, Husam; Wildeson, Isaac; Srivastava, Puneet; Zivasatienraj, Bill; Choi, Sukwon</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr"/>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>10.1115/1.4072184</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1115/1.4072184</t>
+        </is>
+      </c>
+      <c r="J685" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K685" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L685" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M685" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N685" t="inlineStr"/>
+      <c r="O685" t="inlineStr"/>
+      <c r="P685" t="inlineStr"/>
+      <c r="Q685" t="inlineStr">
+        <is>
+          <t>Analysis of Multi-Finger GaN HEMTs Using Gate Resistance Thermometry, Raman Thermometry, and Infrared Thermal Microscopy</t>
+        </is>
+      </c>
+      <c r="R685" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S685" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="T685" t="inlineStr"/>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr"/>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Analysis of Multi-Finger GaN HEMTs Using Gate Resistance Thermometry, Raman Thermometry, and Infrared Thermal Microscopy</t>
+        </is>
+      </c>
+      <c r="C686" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>ASME International</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Journal of Electronic Packaging</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>Kim, Seokjun; Shoemaker, Daniel; Walwil, Husam; Wildeson, Isaac; Srivastava, Puneet; Zivasatienraj, Bill; Choi, Sukwon</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr"/>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>10.1115/1.4072184</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1115/1.4072184</t>
+        </is>
+      </c>
+      <c r="J686" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K686" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L686" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M686" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N686" t="inlineStr"/>
+      <c r="O686" t="inlineStr"/>
+      <c r="P686" t="inlineStr"/>
+      <c r="Q686" t="inlineStr">
+        <is>
+          <t>Analysis of Multi-Finger GaN HEMTs Using Gate Resistance Thermometry, Raman Thermometry, and Infrared Thermal Microscopy</t>
+        </is>
+      </c>
+      <c r="R686" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S686" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="T686" t="inlineStr"/>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr"/>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Analysis of Multi-Finger GaN HEMTs Using Gate Resistance Thermometry, Raman Thermometry, and Infrared Thermal Microscopy</t>
+        </is>
+      </c>
+      <c r="C687" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>ASME International</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Journal of Electronic Packaging</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>Kim, Seokjun; Shoemaker, Daniel; Walwil, Husam; Wildeson, Isaac; Srivastava, Puneet; Zivasatienraj, Bill; Choi, Sukwon</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr"/>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>10.1115/1.4072184</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1115/1.4072184</t>
+        </is>
+      </c>
+      <c r="J687" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K687" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L687" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M687" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N687" t="inlineStr"/>
+      <c r="O687" t="inlineStr"/>
+      <c r="P687" t="inlineStr"/>
+      <c r="Q687" t="inlineStr">
+        <is>
+          <t>Analysis of Multi-Finger GaN HEMTs Using Gate Resistance Thermometry, Raman Thermometry, and Infrared Thermal Microscopy</t>
+        </is>
+      </c>
+      <c r="R687" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S687" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="T687" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-20T00:12Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T687"/>
+  <dimension ref="A1:T691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52408,6 +52408,310 @@
       </c>
       <c r="T687" t="inlineStr"/>
     </row>
+    <row r="688">
+      <c r="A688" t="inlineStr"/>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Online Parameter Identification for Sensorless PMSM Drives with Inverter Nonlinearity Compensation</t>
+        </is>
+      </c>
+      <c r="C688" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>Xiang, Fuyuan; Zhou, Zitong; Wang, Zuo</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr"/>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122722</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122722</t>
+        </is>
+      </c>
+      <c r="J688" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K688" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L688" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M688" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N688" t="inlineStr"/>
+      <c r="O688" t="inlineStr"/>
+      <c r="P688" t="inlineStr"/>
+      <c r="Q688" t="inlineStr">
+        <is>
+          <t>Online Parameter Identification for Sensorless PMSM Drives with Inverter Nonlinearity Compensation</t>
+        </is>
+      </c>
+      <c r="R688" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S688" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="T688" t="inlineStr"/>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr"/>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Online Parameter Identification for Sensorless PMSM Drives with Inverter Nonlinearity Compensation</t>
+        </is>
+      </c>
+      <c r="C689" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>Xiang, Fuyuan; Zhou, Zitong; Wang, Zuo</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr"/>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122722</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122722</t>
+        </is>
+      </c>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K689" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L689" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M689" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N689" t="inlineStr"/>
+      <c r="O689" t="inlineStr"/>
+      <c r="P689" t="inlineStr"/>
+      <c r="Q689" t="inlineStr">
+        <is>
+          <t>Online Parameter Identification for Sensorless PMSM Drives with Inverter Nonlinearity Compensation</t>
+        </is>
+      </c>
+      <c r="R689" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S689" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="T689" t="inlineStr"/>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr"/>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Online Parameter Identification for Sensorless PMSM Drives with Inverter Nonlinearity Compensation</t>
+        </is>
+      </c>
+      <c r="C690" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>Xiang, Fuyuan; Zhou, Zitong; Wang, Zuo</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr"/>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122722</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122722</t>
+        </is>
+      </c>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K690" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L690" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M690" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N690" t="inlineStr"/>
+      <c r="O690" t="inlineStr"/>
+      <c r="P690" t="inlineStr"/>
+      <c r="Q690" t="inlineStr">
+        <is>
+          <t>Online Parameter Identification for Sensorless PMSM Drives with Inverter Nonlinearity Compensation</t>
+        </is>
+      </c>
+      <c r="R690" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S690" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="T690" t="inlineStr"/>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr"/>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Online Parameter Identification for Sensorless PMSM Drives with Inverter Nonlinearity Compensation</t>
+        </is>
+      </c>
+      <c r="C691" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>Xiang, Fuyuan; Zhou, Zitong; Wang, Zuo</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr"/>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15122722</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15122722</t>
+        </is>
+      </c>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K691" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L691" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M691" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N691" t="inlineStr"/>
+      <c r="O691" t="inlineStr"/>
+      <c r="P691" t="inlineStr"/>
+      <c r="Q691" t="inlineStr">
+        <is>
+          <t>Online Parameter Identification for Sensorless PMSM Drives with Inverter Nonlinearity Compensation</t>
+        </is>
+      </c>
+      <c r="R691" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S691" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="T691" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-21T00:11Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T691"/>
+  <dimension ref="A1:T692"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52712,6 +52712,82 @@
       </c>
       <c r="T691" t="inlineStr"/>
     </row>
+    <row r="692">
+      <c r="A692" t="inlineStr"/>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Do sleep bruxism patients experience higher complication or failure rates with monolithic lithium disilicate or zirconia molar crowns?</t>
+        </is>
+      </c>
+      <c r="C692" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Evidence-Based Dentistry</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>Khalid, Afrida; Al-Jewair, Thikriat</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr"/>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>10.1038/s41432-026-01230-2</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41432-026-01230-2</t>
+        </is>
+      </c>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K692" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L692" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M692" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N692" t="inlineStr"/>
+      <c r="O692" t="inlineStr"/>
+      <c r="P692" t="inlineStr"/>
+      <c r="Q692" t="inlineStr">
+        <is>
+          <t>Do sleep bruxism patients experience higher complication or failure rates with monolithic lithium disilicate or zirconia molar crowns?</t>
+        </is>
+      </c>
+      <c r="R692" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S692" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="T692" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-23T00:10Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T692"/>
+  <dimension ref="A1:T696"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52788,6 +52788,310 @@
       </c>
       <c r="T692" t="inlineStr"/>
     </row>
+    <row r="693">
+      <c r="A693" t="inlineStr"/>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Experimental demonstration of acoustic complementary media for superscattering</t>
+        </is>
+      </c>
+      <c r="C693" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>American Physical Society (APS)</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Physical Review B</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>Gan, Tian; Yu, Zhaolun; Luo, Xudong; Wang, Xiaole; Huang, Zhenyu</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr"/>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>10.1103/j5tz-kwgq</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1103/j5tz-kwgq</t>
+        </is>
+      </c>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K693" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L693" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M693" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N693" t="inlineStr"/>
+      <c r="O693" t="inlineStr"/>
+      <c r="P693" t="inlineStr"/>
+      <c r="Q693" t="inlineStr">
+        <is>
+          <t>Experimental demonstration of acoustic complementary media for superscattering</t>
+        </is>
+      </c>
+      <c r="R693" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S693" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="T693" t="inlineStr"/>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr"/>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Experimental demonstration of acoustic complementary media for superscattering</t>
+        </is>
+      </c>
+      <c r="C694" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>American Physical Society (APS)</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Physical Review B</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>Gan, Tian; Yu, Zhaolun; Luo, Xudong; Wang, Xiaole; Huang, Zhenyu</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr"/>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>10.1103/j5tz-kwgq</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1103/j5tz-kwgq</t>
+        </is>
+      </c>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K694" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L694" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M694" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N694" t="inlineStr"/>
+      <c r="O694" t="inlineStr"/>
+      <c r="P694" t="inlineStr"/>
+      <c r="Q694" t="inlineStr">
+        <is>
+          <t>Experimental demonstration of acoustic complementary media for superscattering</t>
+        </is>
+      </c>
+      <c r="R694" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S694" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="T694" t="inlineStr"/>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr"/>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Effect of Channel Length Variation on the Electrical Conductivity of Passivated Back-Gated Graphene Field-Effect Transistor (GFET) Using Silvaco TCAD Tools</t>
+        </is>
+      </c>
+      <c r="C695" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>Guzali, Hazim; Ayob, Nur Idayu; Md Ralib, Aliza Aini; Md Zawawi, Mohamad Adzhar; Che Hak, Cik Rohaida; Ahmad, Zuraida</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr"/>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>10.4028/p-b57hzw</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-b57hzw</t>
+        </is>
+      </c>
+      <c r="J695" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K695" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L695" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M695" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N695" t="inlineStr"/>
+      <c r="O695" t="inlineStr"/>
+      <c r="P695" t="inlineStr"/>
+      <c r="Q695" t="inlineStr">
+        <is>
+          <t>Effect of Channel Length Variation on the Electrical Conductivity of Passivated Back-Gated Graphene Field-Effect Transistor (GFET) Using Silvaco TCAD Tools</t>
+        </is>
+      </c>
+      <c r="R695" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S695" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="T695" t="inlineStr"/>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr"/>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Effect of Channel Length Variation on the Electrical Conductivity of Passivated Back-Gated Graphene Field-Effect Transistor (GFET) Using Silvaco TCAD Tools</t>
+        </is>
+      </c>
+      <c r="C696" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Trans Tech Publications, Ltd.</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Key Engineering Materials</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>Guzali, Hazim; Ayob, Nur Idayu; Md Ralib, Aliza Aini; Md Zawawi, Mohamad Adzhar; Che Hak, Cik Rohaida; Ahmad, Zuraida</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr"/>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>10.4028/p-b57hzw</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4028/p-b57hzw</t>
+        </is>
+      </c>
+      <c r="J696" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K696" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L696" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M696" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N696" t="inlineStr"/>
+      <c r="O696" t="inlineStr"/>
+      <c r="P696" t="inlineStr"/>
+      <c r="Q696" t="inlineStr">
+        <is>
+          <t>Effect of Channel Length Variation on the Electrical Conductivity of Passivated Back-Gated Graphene Field-Effect Transistor (GFET) Using Silvaco TCAD Tools</t>
+        </is>
+      </c>
+      <c r="R696" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S696" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="T696" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-24T00:01Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T696"/>
+  <dimension ref="A1:T698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53092,6 +53092,158 @@
       </c>
       <c r="T696" t="inlineStr"/>
     </row>
+    <row r="697">
+      <c r="A697" t="inlineStr"/>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>A mixed-signal CMOS VLSI implementation of a spiking echo-state neural network for energy-efficient temporal signal processing</t>
+        </is>
+      </c>
+      <c r="C697" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Interactions</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>Nirmala, R.; Murugesan, Malathi; Duraisamy, Sasikala; Senthilkumar, V. M.</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr"/>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>10.1007/s10751-026-02615-6</t>
+        </is>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10751-026-02615-6</t>
+        </is>
+      </c>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K697" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L697" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M697" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N697" t="inlineStr"/>
+      <c r="O697" t="inlineStr"/>
+      <c r="P697" t="inlineStr"/>
+      <c r="Q697" t="inlineStr">
+        <is>
+          <t>A mixed-signal CMOS VLSI implementation of a spiking echo-state neural network for energy-efficient temporal signal processing</t>
+        </is>
+      </c>
+      <c r="R697" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S697" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T697" t="inlineStr"/>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr"/>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Graphical Proposal for a Quantum Simulation of the
+Two-Dimensional Dirac Oscillator: Optical Trapped-Ion and
+Microwave Implementations</t>
+        </is>
+      </c>
+      <c r="C698" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr"/>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>Boumali, Abdelmalek</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr"/>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10096167/v1</t>
+        </is>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10096167/v1</t>
+        </is>
+      </c>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K698" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L698" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M698" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N698" t="inlineStr"/>
+      <c r="O698" t="inlineStr"/>
+      <c r="P698" t="inlineStr"/>
+      <c r="Q698" t="inlineStr">
+        <is>
+          <t>Graphical Proposal for a Quantum Simulation of the
+Two-Dimensional Dirac Oscillator: Optical Trapped-Ion and
+Microwave Implementations</t>
+        </is>
+      </c>
+      <c r="R698" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S698" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T698" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-25T00:16Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T698"/>
+  <dimension ref="A1:T705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53244,6 +53244,566 @@
       </c>
       <c r="T698" t="inlineStr"/>
     </row>
+    <row r="699">
+      <c r="A699" t="inlineStr"/>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>A Thin Film Transistor Backplane for Scalable Chronic Neural Interfaces</t>
+        </is>
+      </c>
+      <c r="C699" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>openRxiv</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr"/>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>Bourhis, Andrew M; Vatsyayan, Ritwik; Tonsfeldt, Karen J; Galton, Ian; Dayeh, Shadi A</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr"/>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>10.64898/2026.06.23.733868</t>
+        </is>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.06.23.733868</t>
+        </is>
+      </c>
+      <c r="J699" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K699" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L699" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M699" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N699" t="inlineStr"/>
+      <c r="O699" t="inlineStr"/>
+      <c r="P699" t="inlineStr"/>
+      <c r="Q699" t="inlineStr">
+        <is>
+          <t>A Thin Film Transistor Backplane for Scalable Chronic Neural Interfaces</t>
+        </is>
+      </c>
+      <c r="R699" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S699" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="T699" t="inlineStr"/>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr"/>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Influence of ALD-Al
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    gate dielectric thickness on polarization and barrier strain under gate bias in AlGaN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="C700" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>Li, Weikang; Jiang, Guangyuan; Yang, Ming; Lv, Yuanjie; Cui, Peng; Wang, Minyan; Liu, Yang; Fu, Chen; Hou, Zhenfei; Cheng, Qianding; Zhang, Qingying; Zhang, Guangyuan</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr"/>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae8201</t>
+        </is>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae8201</t>
+        </is>
+      </c>
+      <c r="J700" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K700" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L700" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M700" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N700" t="inlineStr"/>
+      <c r="O700" t="inlineStr"/>
+      <c r="P700" t="inlineStr"/>
+      <c r="Q700" t="inlineStr">
+        <is>
+          <t>Influence of ALD-Al
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    gate dielectric thickness on polarization and barrier strain under gate bias in AlGaN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="R700" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S700" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="T700" t="inlineStr"/>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr"/>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>High‐Performance Neuromorphic Visual System With Image Pre‐Processing via Normally‐Off GaN MOS‐HEMT</t>
+        </is>
+      </c>
+      <c r="C701" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Advanced Materials Technologies</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>Yang, Ge; Du, Haitao; Qu, Haolan; Liu, Changshu; Li, Yudong; Zhou, Xuanling; Wang, Hongzhi; Li, Kerui; Zou, Xinbo</t>
+        </is>
+      </c>
+      <c r="G701" t="inlineStr"/>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>10.1002/admt.71128</t>
+        </is>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/admt.71128</t>
+        </is>
+      </c>
+      <c r="J701" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K701" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L701" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M701" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N701" t="inlineStr"/>
+      <c r="O701" t="inlineStr"/>
+      <c r="P701" t="inlineStr"/>
+      <c r="Q701" t="inlineStr">
+        <is>
+          <t>High‐Performance Neuromorphic Visual System With Image Pre‐Processing via Normally‐Off GaN MOS‐HEMT</t>
+        </is>
+      </c>
+      <c r="R701" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S701" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="T701" t="inlineStr"/>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr"/>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Influence of ALD-Al
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    gate dielectric thickness on polarization and barrier strain under gate bias in AlGaN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="C702" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>Li, Weikang; Jiang, Guangyuan; Yang, Ming; Lv, Yuanjie; Cui, Peng; Wang, Minyan; Liu, Yang; Fu, Chen; Hou, Zhenfei; Cheng, Qianding; Zhang, Qingying; Zhang, Guangyuan</t>
+        </is>
+      </c>
+      <c r="G702" t="inlineStr"/>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae8201</t>
+        </is>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae8201</t>
+        </is>
+      </c>
+      <c r="J702" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K702" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L702" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M702" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N702" t="inlineStr"/>
+      <c r="O702" t="inlineStr"/>
+      <c r="P702" t="inlineStr"/>
+      <c r="Q702" t="inlineStr">
+        <is>
+          <t>Influence of ALD-Al
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    gate dielectric thickness on polarization and barrier strain under gate bias in AlGaN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="R702" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S702" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="T702" t="inlineStr"/>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr"/>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>A Design for Single Event Transient Pulse Width Measurement in CMOS Technology</t>
+        </is>
+      </c>
+      <c r="C703" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>Journal of Electronic Testing</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>Liu, Baojun; Li, Chuang</t>
+        </is>
+      </c>
+      <c r="G703" t="inlineStr"/>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>10.1007/s10836-026-06242-5</t>
+        </is>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10836-026-06242-5</t>
+        </is>
+      </c>
+      <c r="J703" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K703" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L703" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M703" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N703" t="inlineStr"/>
+      <c r="O703" t="inlineStr"/>
+      <c r="P703" t="inlineStr"/>
+      <c r="Q703" t="inlineStr">
+        <is>
+          <t>A Design for Single Event Transient Pulse Width Measurement in CMOS Technology</t>
+        </is>
+      </c>
+      <c r="R703" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S703" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="T703" t="inlineStr"/>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr"/>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Influence of ALD-Al
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    gate dielectric thickness on polarization and barrier strain under gate bias in AlGaN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="C704" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>Li, Weikang; Jiang, Guangyuan; Yang, Ming; Lv, Yuanjie; Cui, Peng; Wang, Minyan; Liu, Yang; Fu, Chen; Hou, Zhenfei; Cheng, Qianding; Zhang, Qingying; Zhang, Guangyuan</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr"/>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae8201</t>
+        </is>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae8201</t>
+        </is>
+      </c>
+      <c r="J704" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K704" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L704" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M704" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N704" t="inlineStr"/>
+      <c r="O704" t="inlineStr"/>
+      <c r="P704" t="inlineStr"/>
+      <c r="Q704" t="inlineStr">
+        <is>
+          <t>Influence of ALD-Al
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    gate dielectric thickness on polarization and barrier strain under gate bias in AlGaN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="R704" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S704" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="T704" t="inlineStr"/>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr"/>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Influence of ALD-Al
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    gate dielectric thickness on polarization and barrier strain under gate bias in AlGaN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="C705" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>Li, Weikang; Jiang, Guangyuan; Yang, Ming; Lv, Yuanjie; Cui, Peng; Wang, Minyan; Liu, Yang; Fu, Chen; Hou, Zhenfei; Cheng, Qianding; Zhang, Qingying; Zhang, Guangyuan</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr"/>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae8201</t>
+        </is>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae8201</t>
+        </is>
+      </c>
+      <c r="J705" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K705" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L705" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M705" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N705" t="inlineStr"/>
+      <c r="O705" t="inlineStr"/>
+      <c r="P705" t="inlineStr"/>
+      <c r="Q705" t="inlineStr">
+        <is>
+          <t>Influence of ALD-Al
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    gate dielectric thickness on polarization and barrier strain under gate bias in AlGaN/GaN MIS-HEMTs</t>
+        </is>
+      </c>
+      <c r="R705" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S705" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="T705" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-26T00:14Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T705"/>
+  <dimension ref="A1:T707"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53804,6 +53804,158 @@
       </c>
       <c r="T705" t="inlineStr"/>
     </row>
+    <row r="706">
+      <c r="A706" t="inlineStr"/>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Monolithic triple auto-enhanced DNA nanoamplifier under orthogonal dual-response of direct-lock NIR photocage and endogenous APE1 gate for high-precision biosensing in live biosystems</t>
+        </is>
+      </c>
+      <c r="C706" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>Analytica Chimica Acta</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>Yao, Lejing; Sun, Xiaoming; Li, Cheng-Yu</t>
+        </is>
+      </c>
+      <c r="G706" t="inlineStr"/>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>10.1016/j.aca.2026.345880</t>
+        </is>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.aca.2026.345880</t>
+        </is>
+      </c>
+      <c r="J706" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K706" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L706" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M706" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N706" t="inlineStr"/>
+      <c r="O706" t="inlineStr"/>
+      <c r="P706" t="inlineStr"/>
+      <c r="Q706" t="inlineStr">
+        <is>
+          <t>Monolithic triple auto-enhanced DNA nanoamplifier under orthogonal dual-response of direct-lock NIR photocage and endogenous APE1 gate for high-precision biosensing in live biosystems</t>
+        </is>
+      </c>
+      <c r="R706" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S706" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="T706" t="inlineStr"/>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr"/>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Suppressing punch-through and boosting breakdown voltage in p-GaN gate HEMTs by employing a β-Ga2O3 back-barrier</t>
+        </is>
+      </c>
+      <c r="C707" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>Wu, Xinyu; Ren, Xinglin; Liao, Fuda; Wang, Xiao; Zhao, Wei; He, Chenguang; Miao, Zhenlin; Li, Shuti</t>
+        </is>
+      </c>
+      <c r="G707" t="inlineStr"/>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae82a0</t>
+        </is>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae82a0</t>
+        </is>
+      </c>
+      <c r="J707" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K707" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L707" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M707" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N707" t="inlineStr"/>
+      <c r="O707" t="inlineStr"/>
+      <c r="P707" t="inlineStr"/>
+      <c r="Q707" t="inlineStr">
+        <is>
+          <t>Suppressing punch-through and boosting breakdown voltage in p-GaN gate HEMTs by employing a β-Ga2O3 back-barrier</t>
+        </is>
+      </c>
+      <c r="R707" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S707" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="T707" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-27T00:12Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T707"/>
+  <dimension ref="A1:T709"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53956,6 +53956,158 @@
       </c>
       <c r="T707" t="inlineStr"/>
     </row>
+    <row r="708">
+      <c r="A708" t="inlineStr"/>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>A diagram illustrating layers of computing systems from application software to physics.In the diagram, the layers are Application Software with an icon showing 'greater than double quote hello world exclamation double quote', Operating Systems with a laptop icon, Architecture with a grid icon, Micro architecture with arrows between blocks, Logic with a logic gate icon, Digital Circuits with a digital gate icon, Analog Circuits with an amplifier icon, Devices with a transistor icon and Physics with an atomic structure icon.Design Verification</t>
+        </is>
+      </c>
+      <c r="C708" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>RISC-V System-on-Chip Design</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>Harris, David; Stine, James; Thompson, Rose; Harris, Sarah</t>
+        </is>
+      </c>
+      <c r="G708" t="inlineStr"/>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>10.1016/b978-0-323-99498-9.00005-0</t>
+        </is>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/b978-0-323-99498-9.00005-0</t>
+        </is>
+      </c>
+      <c r="J708" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K708" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L708" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M708" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N708" t="inlineStr"/>
+      <c r="O708" t="inlineStr"/>
+      <c r="P708" t="inlineStr"/>
+      <c r="Q708" t="inlineStr">
+        <is>
+          <t>A diagram illustrating layers of computing systems from application software to physics.In the diagram, the layers are Application Software with an icon showing 'greater than double quote hello world exclamation double quote', Operating Systems with a laptop icon, Architecture with a grid icon, Micro architecture with arrows between blocks, Logic with a logic gate icon, Digital Circuits with a digital gate icon, Analog Circuits with an amplifier icon, Devices with a transistor icon and Physics with an atomic structure icon.Design Verification</t>
+        </is>
+      </c>
+      <c r="R708" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S708" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="T708" t="inlineStr"/>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr"/>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>A diagram illustrating layers of computing systems from application software to physics.In the diagram, the layers are Application Software with an icon showing 'greater than double quote hello world exclamation double quote', Operating Systems with a laptop icon, Architecture with a grid icon, Micro architecture with arrows between blocks, Logic with a logic gate icon, Digital Circuits with a digital gate icon, Analog Circuits with an amplifier icon, Devices with a transistor icon and Physics with an atomic structure icon.A Brief History of Computer Design</t>
+        </is>
+      </c>
+      <c r="C709" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>RISC-V System-on-Chip Design</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>Harris, David; Stine, James; Thompson, Rose; Harris, Sarah</t>
+        </is>
+      </c>
+      <c r="G709" t="inlineStr"/>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>10.1016/b978-0-323-99498-9.00001-3</t>
+        </is>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/b978-0-323-99498-9.00001-3</t>
+        </is>
+      </c>
+      <c r="J709" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K709" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L709" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M709" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N709" t="inlineStr"/>
+      <c r="O709" t="inlineStr"/>
+      <c r="P709" t="inlineStr"/>
+      <c r="Q709" t="inlineStr">
+        <is>
+          <t>A diagram illustrating layers of computing systems from application software to physics.In the diagram, the layers are Application Software with an icon showing 'greater than double quote hello world exclamation double quote', Operating Systems with a laptop icon, Architecture with a grid icon, Micro architecture with arrows between blocks, Logic with a logic gate icon, Digital Circuits with a digital gate icon, Analog Circuits with an amplifier icon, Devices with a transistor icon and Physics with an atomic structure icon.A Brief History of Computer Design</t>
+        </is>
+      </c>
+      <c r="R709" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S709" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="T709" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-06-30T00:08Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T709"/>
+  <dimension ref="A1:T714"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54108,6 +54108,386 @@
       </c>
       <c r="T709" t="inlineStr"/>
     </row>
+    <row r="710">
+      <c r="A710" t="inlineStr"/>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Performance Analysis of Junctionless Gate-All-Around WSe₂ Nanowire MOSFET at Lg = 10 nm for IoT Applications</t>
+        </is>
+      </c>
+      <c r="C710" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>Majumdar, SANDIP</t>
+        </is>
+      </c>
+      <c r="G710" t="inlineStr"/>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae8403</t>
+        </is>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae8403</t>
+        </is>
+      </c>
+      <c r="J710" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K710" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L710" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M710" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N710" t="inlineStr"/>
+      <c r="O710" t="inlineStr"/>
+      <c r="P710" t="inlineStr"/>
+      <c r="Q710" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Performance Analysis of Junctionless Gate-All-Around WSe₂ Nanowire MOSFET at Lg = 10 nm for IoT Applications</t>
+        </is>
+      </c>
+      <c r="R710" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S710" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="T710" t="inlineStr"/>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr"/>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Performance Analysis of Junctionless Gate-All-Around WSe₂ Nanowire MOSFET at Lg = 10 nm for IoT Applications</t>
+        </is>
+      </c>
+      <c r="C711" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>Majumdar, SANDIP</t>
+        </is>
+      </c>
+      <c r="G711" t="inlineStr"/>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae8403</t>
+        </is>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae8403</t>
+        </is>
+      </c>
+      <c r="J711" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K711" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L711" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M711" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N711" t="inlineStr"/>
+      <c r="O711" t="inlineStr"/>
+      <c r="P711" t="inlineStr"/>
+      <c r="Q711" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Performance Analysis of Junctionless Gate-All-Around WSe₂ Nanowire MOSFET at Lg = 10 nm for IoT Applications</t>
+        </is>
+      </c>
+      <c r="R711" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S711" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="T711" t="inlineStr"/>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr"/>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Performance Analysis of Junctionless Gate-All-Around WSe₂ Nanowire MOSFET at Lg = 10 nm for IoT Applications</t>
+        </is>
+      </c>
+      <c r="C712" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>Majumdar, SANDIP</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr"/>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae8403</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae8403</t>
+        </is>
+      </c>
+      <c r="J712" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K712" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L712" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M712" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N712" t="inlineStr"/>
+      <c r="O712" t="inlineStr"/>
+      <c r="P712" t="inlineStr"/>
+      <c r="Q712" t="inlineStr">
+        <is>
+          <t>Temperature-Dependent Performance Analysis of Junctionless Gate-All-Around WSe₂ Nanowire MOSFET at Lg = 10 nm for IoT Applications</t>
+        </is>
+      </c>
+      <c r="R712" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S712" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="T712" t="inlineStr"/>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr"/>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Grid-connected inverter stability issues in modern electric power system</t>
+        </is>
+      </c>
+      <c r="C713" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Universe Scientific Publishing Pte. Ltd.</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Clean Energy Science and Technology</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>Sladic, Sasa; Zivic, Even; De Santis, Michele</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr"/>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>10.18686/cest855</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.18686/cest855</t>
+        </is>
+      </c>
+      <c r="J713" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K713" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L713" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M713" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N713" t="inlineStr"/>
+      <c r="O713" t="inlineStr"/>
+      <c r="P713" t="inlineStr"/>
+      <c r="Q713" t="inlineStr">
+        <is>
+          <t>Grid-connected inverter stability issues in modern electric power system</t>
+        </is>
+      </c>
+      <c r="R713" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S713" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="T713" t="inlineStr"/>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr"/>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>OR Logic Gate-Based NodeMCU (ESP8266) Supported IoT Simulation</t>
+        </is>
+      </c>
+      <c r="C714" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Cumhuriyet University</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Cumhuriyet Science Journal</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>Çoşkun, Özlem; Günay Demirel, Emine Canan</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr"/>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>10.17776/csj.1882678</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.17776/csj.1882678</t>
+        </is>
+      </c>
+      <c r="J714" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K714" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L714" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M714" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N714" t="inlineStr"/>
+      <c r="O714" t="inlineStr"/>
+      <c r="P714" t="inlineStr"/>
+      <c r="Q714" t="inlineStr">
+        <is>
+          <t>OR Logic Gate-Based NodeMCU (ESP8266) Supported IoT Simulation</t>
+        </is>
+      </c>
+      <c r="R714" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S714" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="T714" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-01T00:10Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T714"/>
+  <dimension ref="A1:T721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54488,6 +54488,534 @@
       </c>
       <c r="T714" t="inlineStr"/>
     </row>
+    <row r="715">
+      <c r="A715" t="inlineStr"/>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Monolithic kinetic algorithm for heterogeneous porous media systems using a continuous one-domain approach</t>
+        </is>
+      </c>
+      <c r="C715" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr"/>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>Gusev, Nikita; Karlin, Ilya</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr"/>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10169483/v1</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10169483/v1</t>
+        </is>
+      </c>
+      <c r="J715" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K715" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L715" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M715" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N715" t="inlineStr"/>
+      <c r="O715" t="inlineStr"/>
+      <c r="P715" t="inlineStr"/>
+      <c r="Q715" t="inlineStr">
+        <is>
+          <t>Monolithic kinetic algorithm for heterogeneous porous media systems using a continuous one-domain approach</t>
+        </is>
+      </c>
+      <c r="R715" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S715" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="T715" t="inlineStr"/>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr"/>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="C716" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>Zhang, Kuo; Liu, Kai; Wang, Chong; Luo, Yuhan; Ren, Jiahui; Zhang, Wentao; He, Yunlong; Zheng, Xuefeng; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G716" t="inlineStr"/>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="J716" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K716" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L716" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M716" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N716" t="inlineStr"/>
+      <c r="O716" t="inlineStr"/>
+      <c r="P716" t="inlineStr"/>
+      <c r="Q716" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="R716" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S716" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="T716" t="inlineStr"/>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr"/>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="C717" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>Zhang, Kuo; Liu, Kai; Wang, Chong; Luo, Yuhan; Ren, Jiahui; Zhang, Wentao; He, Yunlong; Zheng, Xuefeng; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G717" t="inlineStr"/>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="J717" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K717" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L717" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M717" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N717" t="inlineStr"/>
+      <c r="O717" t="inlineStr"/>
+      <c r="P717" t="inlineStr"/>
+      <c r="Q717" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="R717" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S717" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="T717" t="inlineStr"/>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr"/>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="C718" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>Zhang, Kuo; Liu, Kai; Wang, Chong; Luo, Yuhan; Ren, Jiahui; Zhang, Wentao; He, Yunlong; Zheng, Xuefeng; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr"/>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="J718" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K718" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L718" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M718" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N718" t="inlineStr"/>
+      <c r="O718" t="inlineStr"/>
+      <c r="P718" t="inlineStr"/>
+      <c r="Q718" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="R718" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S718" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="T718" t="inlineStr"/>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr"/>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="C719" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>Zhang, Kuo; Liu, Kai; Wang, Chong; Luo, Yuhan; Ren, Jiahui; Zhang, Wentao; He, Yunlong; Zheng, Xuefeng; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr"/>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="J719" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K719" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L719" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M719" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N719" t="inlineStr"/>
+      <c r="O719" t="inlineStr"/>
+      <c r="P719" t="inlineStr"/>
+      <c r="Q719" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="R719" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S719" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="T719" t="inlineStr"/>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr"/>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="C720" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>Zhang, Kuo; Liu, Kai; Wang, Chong; Luo, Yuhan; Ren, Jiahui; Zhang, Wentao; He, Yunlong; Zheng, Xuefeng; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr"/>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="J720" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K720" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L720" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M720" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N720" t="inlineStr"/>
+      <c r="O720" t="inlineStr"/>
+      <c r="P720" t="inlineStr"/>
+      <c r="Q720" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="R720" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S720" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="T720" t="inlineStr"/>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr"/>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="C721" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>Zhang, Kuo; Liu, Kai; Wang, Chong; Luo, Yuhan; Ren, Jiahui; Zhang, Wentao; He, Yunlong; Zheng, Xuefeng; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G721" t="inlineStr"/>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3696037</t>
+        </is>
+      </c>
+      <c r="J721" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K721" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L721" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M721" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N721" t="inlineStr"/>
+      <c r="O721" t="inlineStr"/>
+      <c r="P721" t="inlineStr"/>
+      <c r="Q721" t="inlineStr">
+        <is>
+          <t>Hybrid p-n Junction/Ohmic Gate p-GaN HEMT With Enhanced Threshold Voltage Stability and Large Gate Swing</t>
+        </is>
+      </c>
+      <c r="R721" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S721" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="T721" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-02T00:12Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T721"/>
+  <dimension ref="A1:T731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55016,6 +55016,766 @@
       </c>
       <c r="T721" t="inlineStr"/>
     </row>
+    <row r="722">
+      <c r="A722" t="inlineStr"/>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="C722" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>Zhang, Yanfang; Hao, Jinggang; Huang, Conggui; Dong, Yue; Chen, Quanhua; Fang, Ke; Qian, Dongjie; Xiao, Guoling</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr"/>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="J722" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K722" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L722" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M722" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N722" t="inlineStr"/>
+      <c r="O722" t="inlineStr"/>
+      <c r="P722" t="inlineStr"/>
+      <c r="Q722" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="R722" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S722" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T722" t="inlineStr"/>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr"/>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="C723" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>Zhang, Yanfang; Hao, Jinggang; Huang, Conggui; Dong, Yue; Chen, Quanhua; Fang, Ke; Qian, Dongjie; Xiao, Guoling</t>
+        </is>
+      </c>
+      <c r="G723" t="inlineStr"/>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="J723" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K723" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L723" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M723" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N723" t="inlineStr"/>
+      <c r="O723" t="inlineStr"/>
+      <c r="P723" t="inlineStr"/>
+      <c r="Q723" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="R723" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S723" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T723" t="inlineStr"/>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr"/>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="C724" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>Zhang, Yanfang; Hao, Jinggang; Huang, Conggui; Dong, Yue; Chen, Quanhua; Fang, Ke; Qian, Dongjie; Xiao, Guoling</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr"/>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="J724" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K724" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L724" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M724" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N724" t="inlineStr"/>
+      <c r="O724" t="inlineStr"/>
+      <c r="P724" t="inlineStr"/>
+      <c r="Q724" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="R724" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S724" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T724" t="inlineStr"/>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr"/>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="C725" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>Zhang, Yanfang; Hao, Jinggang; Huang, Conggui; Dong, Yue; Chen, Quanhua; Fang, Ke; Qian, Dongjie; Xiao, Guoling</t>
+        </is>
+      </c>
+      <c r="G725" t="inlineStr"/>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="J725" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K725" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L725" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M725" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N725" t="inlineStr"/>
+      <c r="O725" t="inlineStr"/>
+      <c r="P725" t="inlineStr"/>
+      <c r="Q725" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="R725" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S725" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T725" t="inlineStr"/>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr"/>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="C726" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>Zhang, Yanfang; Hao, Jinggang; Huang, Conggui; Dong, Yue; Chen, Quanhua; Fang, Ke; Qian, Dongjie; Xiao, Guoling</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr"/>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="J726" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K726" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L726" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M726" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N726" t="inlineStr"/>
+      <c r="O726" t="inlineStr"/>
+      <c r="P726" t="inlineStr"/>
+      <c r="Q726" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="R726" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S726" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T726" t="inlineStr"/>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr"/>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="C727" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>Zhang, Yanfang; Hao, Jinggang; Huang, Conggui; Dong, Yue; Chen, Quanhua; Fang, Ke; Qian, Dongjie; Xiao, Guoling</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr"/>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="J727" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K727" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L727" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M727" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N727" t="inlineStr"/>
+      <c r="O727" t="inlineStr"/>
+      <c r="P727" t="inlineStr"/>
+      <c r="Q727" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="R727" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S727" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T727" t="inlineStr"/>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr"/>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>GaN HEMT-Based Frequency Quadrupler Up-Converting from S Band to X Band with Conversion Gain in Narrowband</t>
+        </is>
+      </c>
+      <c r="C728" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>Morales-Fernandez, Ainhoa; Marante-Boado, Maria; Fernandez-Barciela, Monica; Martin-Rodriguez, Fernando</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr"/>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15132893</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15132893</t>
+        </is>
+      </c>
+      <c r="J728" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K728" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L728" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M728" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N728" t="inlineStr"/>
+      <c r="O728" t="inlineStr"/>
+      <c r="P728" t="inlineStr"/>
+      <c r="Q728" t="inlineStr">
+        <is>
+          <t>GaN HEMT-Based Frequency Quadrupler Up-Converting from S Band to X Band with Conversion Gain in Narrowband</t>
+        </is>
+      </c>
+      <c r="R728" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S728" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T728" t="inlineStr"/>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr"/>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="C729" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>Zhang, Yanfang; Hao, Jinggang; Huang, Conggui; Dong, Yue; Chen, Quanhua; Fang, Ke; Qian, Dongjie; Xiao, Guoling</t>
+        </is>
+      </c>
+      <c r="G729" t="inlineStr"/>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="J729" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K729" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L729" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M729" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N729" t="inlineStr"/>
+      <c r="O729" t="inlineStr"/>
+      <c r="P729" t="inlineStr"/>
+      <c r="Q729" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="R729" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S729" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T729" t="inlineStr"/>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr"/>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="C730" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>Zhang, Yanfang; Hao, Jinggang; Huang, Conggui; Dong, Yue; Chen, Quanhua; Fang, Ke; Qian, Dongjie; Xiao, Guoling</t>
+        </is>
+      </c>
+      <c r="G730" t="inlineStr"/>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="J730" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K730" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L730" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M730" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N730" t="inlineStr"/>
+      <c r="O730" t="inlineStr"/>
+      <c r="P730" t="inlineStr"/>
+      <c r="Q730" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="R730" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S730" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T730" t="inlineStr"/>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr"/>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="C731" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>Zhang, Yanfang; Hao, Jinggang; Huang, Conggui; Dong, Yue; Chen, Quanhua; Fang, Ke; Qian, Dongjie; Xiao, Guoling</t>
+        </is>
+      </c>
+      <c r="G731" t="inlineStr"/>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/micro6030048</t>
+        </is>
+      </c>
+      <c r="J731" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K731" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L731" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M731" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N731" t="inlineStr"/>
+      <c r="O731" t="inlineStr"/>
+      <c r="P731" t="inlineStr"/>
+      <c r="Q731" t="inlineStr">
+        <is>
+          <t>Performance of κ-Ga2O3/GaN HEMTs and Normally off Operation by p-GaN Gate</t>
+        </is>
+      </c>
+      <c r="R731" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S731" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T731" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-03T00:10Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T731"/>
+  <dimension ref="A1:T749"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55776,6 +55776,1374 @@
       </c>
       <c r="T731" t="inlineStr"/>
     </row>
+    <row r="732">
+      <c r="A732" t="inlineStr"/>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C732" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G732" t="inlineStr"/>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J732" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K732" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L732" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M732" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N732" t="inlineStr"/>
+      <c r="O732" t="inlineStr"/>
+      <c r="P732" t="inlineStr"/>
+      <c r="Q732" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R732" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S732" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T732" t="inlineStr"/>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr"/>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Continuous Sense-FET Current Measurement in a GaN-Based T-Type Bridge-Leg With Monolithic Bidirectional Switch</t>
+        </is>
+      </c>
+      <c r="C733" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Power Electronics</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>Basler, Michael; Reiner, Richard; Fugmann, Daniel; Benkhelifa, Fouad; Mönch, Stefan</t>
+        </is>
+      </c>
+      <c r="G733" t="inlineStr"/>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>10.1109/tpel.2026.3682261</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tpel.2026.3682261</t>
+        </is>
+      </c>
+      <c r="J733" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K733" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L733" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M733" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N733" t="inlineStr"/>
+      <c r="O733" t="inlineStr"/>
+      <c r="P733" t="inlineStr"/>
+      <c r="Q733" t="inlineStr">
+        <is>
+          <t>Continuous Sense-FET Current Measurement in a GaN-Based T-Type Bridge-Leg With Monolithic Bidirectional Switch</t>
+        </is>
+      </c>
+      <c r="R733" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S733" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T733" t="inlineStr"/>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr"/>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Method for Automated Decomposition of Monolithic Software Systems Based on Graph Neural Networks</t>
+        </is>
+      </c>
+      <c r="C734" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>Axioms</t>
+        </is>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>Kornaga, Yaroslav; Hubariev, Oleksandr; Yevseiev, Serhii; Yablonskyi, Petro; Pyrohovska, Tetiana</t>
+        </is>
+      </c>
+      <c r="G734" t="inlineStr"/>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>10.3390/axioms15070498</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/axioms15070498</t>
+        </is>
+      </c>
+      <c r="J734" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K734" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L734" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M734" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N734" t="inlineStr"/>
+      <c r="O734" t="inlineStr"/>
+      <c r="P734" t="inlineStr"/>
+      <c r="Q734" t="inlineStr">
+        <is>
+          <t>Method for Automated Decomposition of Monolithic Software Systems Based on Graph Neural Networks</t>
+        </is>
+      </c>
+      <c r="R734" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S734" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T734" t="inlineStr"/>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr"/>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C735" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G735" t="inlineStr"/>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J735" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K735" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L735" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M735" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N735" t="inlineStr"/>
+      <c r="O735" t="inlineStr"/>
+      <c r="P735" t="inlineStr"/>
+      <c r="Q735" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R735" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S735" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T735" t="inlineStr"/>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr"/>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Prediction of Thermal Stresses During the Construction of Massive Monolithic Foundation Slabs Using Temperature Monitoring Data</t>
+        </is>
+      </c>
+      <c r="C736" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>Bentham Science Publishers Ltd.</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>The Open Construction &amp;amp; Building Technology Journal</t>
+        </is>
+      </c>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>Kondratieva, Tatiana; Tyurina, Vasilina; Chepurnenko, Anton</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr"/>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>10.2174/0118748368503424260622093755</t>
+        </is>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2174/0118748368503424260622093755</t>
+        </is>
+      </c>
+      <c r="J736" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K736" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L736" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M736" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N736" t="inlineStr"/>
+      <c r="O736" t="inlineStr"/>
+      <c r="P736" t="inlineStr"/>
+      <c r="Q736" t="inlineStr">
+        <is>
+          <t>Prediction of Thermal Stresses During the Construction of Massive Monolithic Foundation Slabs Using Temperature Monitoring Data</t>
+        </is>
+      </c>
+      <c r="R736" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S736" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T736" t="inlineStr"/>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr"/>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C737" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G737" t="inlineStr"/>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J737" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K737" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L737" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M737" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N737" t="inlineStr"/>
+      <c r="O737" t="inlineStr"/>
+      <c r="P737" t="inlineStr"/>
+      <c r="Q737" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R737" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S737" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T737" t="inlineStr"/>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr"/>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C738" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr"/>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J738" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K738" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L738" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M738" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N738" t="inlineStr"/>
+      <c r="O738" t="inlineStr"/>
+      <c r="P738" t="inlineStr"/>
+      <c r="Q738" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R738" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S738" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T738" t="inlineStr"/>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr"/>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C739" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr"/>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J739" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K739" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L739" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M739" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N739" t="inlineStr"/>
+      <c r="O739" t="inlineStr"/>
+      <c r="P739" t="inlineStr"/>
+      <c r="Q739" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R739" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S739" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T739" t="inlineStr"/>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr"/>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Continuous Sense-FET Current Measurement in a GaN-Based T-Type Bridge-Leg With Monolithic Bidirectional Switch</t>
+        </is>
+      </c>
+      <c r="C740" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Power Electronics</t>
+        </is>
+      </c>
+      <c r="F740" t="inlineStr">
+        <is>
+          <t>Basler, Michael; Reiner, Richard; Fugmann, Daniel; Benkhelifa, Fouad; Mönch, Stefan</t>
+        </is>
+      </c>
+      <c r="G740" t="inlineStr"/>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>10.1109/tpel.2026.3682261</t>
+        </is>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tpel.2026.3682261</t>
+        </is>
+      </c>
+      <c r="J740" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K740" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L740" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M740" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N740" t="inlineStr"/>
+      <c r="O740" t="inlineStr"/>
+      <c r="P740" t="inlineStr"/>
+      <c r="Q740" t="inlineStr">
+        <is>
+          <t>Continuous Sense-FET Current Measurement in a GaN-Based T-Type Bridge-Leg With Monolithic Bidirectional Switch</t>
+        </is>
+      </c>
+      <c r="R740" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S740" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T740" t="inlineStr"/>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr"/>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C741" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F741" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G741" t="inlineStr"/>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J741" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K741" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L741" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M741" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N741" t="inlineStr"/>
+      <c r="O741" t="inlineStr"/>
+      <c r="P741" t="inlineStr"/>
+      <c r="Q741" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R741" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S741" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T741" t="inlineStr"/>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr"/>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C742" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G742" t="inlineStr"/>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J742" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K742" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L742" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M742" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N742" t="inlineStr"/>
+      <c r="O742" t="inlineStr"/>
+      <c r="P742" t="inlineStr"/>
+      <c r="Q742" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R742" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S742" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T742" t="inlineStr"/>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr"/>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C743" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G743" t="inlineStr"/>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J743" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K743" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L743" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M743" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N743" t="inlineStr"/>
+      <c r="O743" t="inlineStr"/>
+      <c r="P743" t="inlineStr"/>
+      <c r="Q743" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R743" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S743" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T743" t="inlineStr"/>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr"/>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C744" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G744" t="inlineStr"/>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J744" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K744" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L744" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M744" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N744" t="inlineStr"/>
+      <c r="O744" t="inlineStr"/>
+      <c r="P744" t="inlineStr"/>
+      <c r="Q744" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R744" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S744" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T744" t="inlineStr"/>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr"/>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="C745" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>Cao, Can; Thirupakuzi Vangipuram, Vijay Gopal; Mukit, Abdul; Helli, Motahareh; Hwang, Jinwoo; Zhao, Hongping; Lu, Wu</t>
+        </is>
+      </c>
+      <c r="G745" t="inlineStr"/>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0315706</t>
+        </is>
+      </c>
+      <c r="J745" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K745" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L745" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M745" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N745" t="inlineStr"/>
+      <c r="O745" t="inlineStr"/>
+      <c r="P745" t="inlineStr"/>
+      <c r="Q745" t="inlineStr">
+        <is>
+          <t>Microwave performance of all MOCVD-grown AlScN/GaN MIS-HEMTs on semi-insulating GaN substrates</t>
+        </is>
+      </c>
+      <c r="R745" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S745" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T745" t="inlineStr"/>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr"/>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Advanced gain-boosted CMOS LDO regulator for enhanced load regulation in RFSoC and mobile systems</t>
+        </is>
+      </c>
+      <c r="C746" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>Inderscience Publishers</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>International Journal of Automation and Control</t>
+        </is>
+      </c>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>Ameziane, Hatim; Yessef, Mourad</t>
+        </is>
+      </c>
+      <c r="G746" t="inlineStr"/>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>10.1504/ijaac.2027.10075192</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1504/ijaac.2027.10075192</t>
+        </is>
+      </c>
+      <c r="J746" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K746" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L746" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M746" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N746" t="inlineStr"/>
+      <c r="O746" t="inlineStr"/>
+      <c r="P746" t="inlineStr"/>
+      <c r="Q746" t="inlineStr">
+        <is>
+          <t>Advanced gain-boosted CMOS LDO regulator for enhanced load regulation in RFSoC and mobile systems</t>
+        </is>
+      </c>
+      <c r="R746" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S746" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T746" t="inlineStr"/>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr"/>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Continuous Sense-FET Current Measurement in a GaN-Based T-Type Bridge-Leg With Monolithic Bidirectional Switch</t>
+        </is>
+      </c>
+      <c r="C747" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Power Electronics</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>Basler, Michael; Reiner, Richard; Fugmann, Daniel; Benkhelifa, Fouad; Mönch, Stefan</t>
+        </is>
+      </c>
+      <c r="G747" t="inlineStr"/>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>10.1109/tpel.2026.3682261</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tpel.2026.3682261</t>
+        </is>
+      </c>
+      <c r="J747" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K747" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L747" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M747" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N747" t="inlineStr"/>
+      <c r="O747" t="inlineStr"/>
+      <c r="P747" t="inlineStr"/>
+      <c r="Q747" t="inlineStr">
+        <is>
+          <t>Continuous Sense-FET Current Measurement in a GaN-Based T-Type Bridge-Leg With Monolithic Bidirectional Switch</t>
+        </is>
+      </c>
+      <c r="R747" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S747" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T747" t="inlineStr"/>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr"/>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Influence of gate dielectric relative permittivity on polarization Coulomb field scattering in AlGaN/GaN metal–insulator–semiconductor high electron mobility transistors</t>
+        </is>
+      </c>
+      <c r="C748" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>Zhang, Qingying; Li, Weikang; Liu, Yang; Cui, Peng; Wang, Mingyan; Jiang, Guangyuan; Fu, Chen; Hou, Zhenfei; Zhang, Guangyuan</t>
+        </is>
+      </c>
+      <c r="G748" t="inlineStr"/>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>10.1063/5.0338452</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0338452</t>
+        </is>
+      </c>
+      <c r="J748" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K748" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L748" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M748" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N748" t="inlineStr"/>
+      <c r="O748" t="inlineStr"/>
+      <c r="P748" t="inlineStr"/>
+      <c r="Q748" t="inlineStr">
+        <is>
+          <t>Influence of gate dielectric relative permittivity on polarization Coulomb field scattering in AlGaN/GaN metal–insulator–semiconductor high electron mobility transistors</t>
+        </is>
+      </c>
+      <c r="R748" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S748" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T748" t="inlineStr"/>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr"/>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Influence of gate dielectric relative permittivity on polarization Coulomb field scattering in AlGaN/GaN metal–insulator–semiconductor high electron mobility transistors</t>
+        </is>
+      </c>
+      <c r="C749" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>Zhang, Qingying; Li, Weikang; Liu, Yang; Cui, Peng; Wang, Mingyan; Jiang, Guangyuan; Fu, Chen; Hou, Zhenfei; Zhang, Guangyuan</t>
+        </is>
+      </c>
+      <c r="G749" t="inlineStr"/>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>10.1063/5.0338452</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0338452</t>
+        </is>
+      </c>
+      <c r="J749" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K749" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L749" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M749" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N749" t="inlineStr"/>
+      <c r="O749" t="inlineStr"/>
+      <c r="P749" t="inlineStr"/>
+      <c r="Q749" t="inlineStr">
+        <is>
+          <t>Influence of gate dielectric relative permittivity on polarization Coulomb field scattering in AlGaN/GaN metal–insulator–semiconductor high electron mobility transistors</t>
+        </is>
+      </c>
+      <c r="R749" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S749" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="T749" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-04T00:09Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T749"/>
+  <dimension ref="A1:T768"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57144,6 +57144,1378 @@
       </c>
       <c r="T749" t="inlineStr"/>
     </row>
+    <row r="750">
+      <c r="A750" t="inlineStr"/>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C750" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr"/>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr"/>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J750" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K750" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L750" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M750" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N750" t="inlineStr"/>
+      <c r="O750" t="inlineStr"/>
+      <c r="P750" t="inlineStr"/>
+      <c r="Q750" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R750" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S750" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T750" t="inlineStr"/>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr"/>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Transistors to transmons: large-scale cryogenic CMOS control of superconducting qubits</t>
+        </is>
+      </c>
+      <c r="C751" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr"/>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>Underwood, Devin</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr"/>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10095152/v1</t>
+        </is>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10095152/v1</t>
+        </is>
+      </c>
+      <c r="J751" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K751" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L751" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M751" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N751" t="inlineStr"/>
+      <c r="O751" t="inlineStr"/>
+      <c r="P751" t="inlineStr"/>
+      <c r="Q751" t="inlineStr">
+        <is>
+          <t>Transistors to transmons: large-scale cryogenic CMOS control of superconducting qubits</t>
+        </is>
+      </c>
+      <c r="R751" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S751" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T751" t="inlineStr"/>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr"/>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C752" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr"/>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr"/>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J752" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K752" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L752" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M752" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N752" t="inlineStr"/>
+      <c r="O752" t="inlineStr"/>
+      <c r="P752" t="inlineStr"/>
+      <c r="Q752" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R752" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S752" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T752" t="inlineStr"/>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr"/>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C753" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr"/>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr"/>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J753" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K753" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L753" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M753" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N753" t="inlineStr"/>
+      <c r="O753" t="inlineStr"/>
+      <c r="P753" t="inlineStr"/>
+      <c r="Q753" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R753" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S753" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T753" t="inlineStr"/>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr"/>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Transistors to transmons: large-scale cryogenic CMOS control of superconducting qubits</t>
+        </is>
+      </c>
+      <c r="C754" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr"/>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>Underwood, Devin</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr"/>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10095152/v1</t>
+        </is>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10095152/v1</t>
+        </is>
+      </c>
+      <c r="J754" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K754" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L754" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M754" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N754" t="inlineStr"/>
+      <c r="O754" t="inlineStr"/>
+      <c r="P754" t="inlineStr"/>
+      <c r="Q754" t="inlineStr">
+        <is>
+          <t>Transistors to transmons: large-scale cryogenic CMOS control of superconducting qubits</t>
+        </is>
+      </c>
+      <c r="R754" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S754" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T754" t="inlineStr"/>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr"/>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C755" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr"/>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr"/>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J755" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K755" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L755" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M755" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N755" t="inlineStr"/>
+      <c r="O755" t="inlineStr"/>
+      <c r="P755" t="inlineStr"/>
+      <c r="Q755" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R755" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S755" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T755" t="inlineStr"/>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr"/>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C756" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr"/>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G756" t="inlineStr"/>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I756" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J756" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K756" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L756" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M756" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N756" t="inlineStr"/>
+      <c r="O756" t="inlineStr"/>
+      <c r="P756" t="inlineStr"/>
+      <c r="Q756" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R756" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S756" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T756" t="inlineStr"/>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr"/>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C757" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr"/>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G757" t="inlineStr"/>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J757" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K757" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L757" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M757" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N757" t="inlineStr"/>
+      <c r="O757" t="inlineStr"/>
+      <c r="P757" t="inlineStr"/>
+      <c r="Q757" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R757" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S757" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T757" t="inlineStr"/>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr"/>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C758" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr"/>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G758" t="inlineStr"/>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I758" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J758" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K758" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L758" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M758" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N758" t="inlineStr"/>
+      <c r="O758" t="inlineStr"/>
+      <c r="P758" t="inlineStr"/>
+      <c r="Q758" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R758" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S758" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T758" t="inlineStr"/>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr"/>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C759" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr"/>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G759" t="inlineStr"/>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I759" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J759" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K759" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L759" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M759" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N759" t="inlineStr"/>
+      <c r="O759" t="inlineStr"/>
+      <c r="P759" t="inlineStr"/>
+      <c r="Q759" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R759" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S759" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T759" t="inlineStr"/>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr"/>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C760" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr"/>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G760" t="inlineStr"/>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J760" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K760" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L760" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M760" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N760" t="inlineStr"/>
+      <c r="O760" t="inlineStr"/>
+      <c r="P760" t="inlineStr"/>
+      <c r="Q760" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R760" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S760" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T760" t="inlineStr"/>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr"/>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C761" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr"/>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G761" t="inlineStr"/>
+      <c r="H761" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I761" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J761" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K761" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L761" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M761" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N761" t="inlineStr"/>
+      <c r="O761" t="inlineStr"/>
+      <c r="P761" t="inlineStr"/>
+      <c r="Q761" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R761" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S761" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T761" t="inlineStr"/>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr"/>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Methodology for Harmonic Distortion Characterization and Modelling of GaN HEMT Varactors</t>
+        </is>
+      </c>
+      <c r="C762" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>Instruments</t>
+        </is>
+      </c>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>Chevas, Loukas; Bucher, Matthias; Makris, Nikolaos; Fosteris, Ioannis Spiridon; Fasarakis, Nikolaos; Stavrinidis, Antonios; Kayambaki, Maria; Kostopoulos, Athanasios; Konstantinidis, George</t>
+        </is>
+      </c>
+      <c r="G762" t="inlineStr"/>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>10.3390/instruments10030037</t>
+        </is>
+      </c>
+      <c r="I762" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/instruments10030037</t>
+        </is>
+      </c>
+      <c r="J762" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K762" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L762" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M762" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N762" t="inlineStr"/>
+      <c r="O762" t="inlineStr"/>
+      <c r="P762" t="inlineStr"/>
+      <c r="Q762" t="inlineStr">
+        <is>
+          <t>Methodology for Harmonic Distortion Characterization and Modelling of GaN HEMT Varactors</t>
+        </is>
+      </c>
+      <c r="R762" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S762" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T762" t="inlineStr"/>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr"/>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C763" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr"/>
+      <c r="F763" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G763" t="inlineStr"/>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I763" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J763" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K763" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L763" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M763" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N763" t="inlineStr"/>
+      <c r="O763" t="inlineStr"/>
+      <c r="P763" t="inlineStr"/>
+      <c r="Q763" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R763" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S763" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T763" t="inlineStr"/>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr"/>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C764" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr"/>
+      <c r="F764" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G764" t="inlineStr"/>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I764" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J764" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K764" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L764" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M764" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N764" t="inlineStr"/>
+      <c r="O764" t="inlineStr"/>
+      <c r="P764" t="inlineStr"/>
+      <c r="Q764" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R764" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S764" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T764" t="inlineStr"/>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr"/>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Transistors to transmons: large-scale cryogenic CMOS control of superconducting qubits</t>
+        </is>
+      </c>
+      <c r="C765" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr"/>
+      <c r="F765" t="inlineStr">
+        <is>
+          <t>Underwood, Devin</t>
+        </is>
+      </c>
+      <c r="G765" t="inlineStr"/>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10095152/v1</t>
+        </is>
+      </c>
+      <c r="I765" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10095152/v1</t>
+        </is>
+      </c>
+      <c r="J765" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K765" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L765" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M765" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N765" t="inlineStr"/>
+      <c r="O765" t="inlineStr"/>
+      <c r="P765" t="inlineStr"/>
+      <c r="Q765" t="inlineStr">
+        <is>
+          <t>Transistors to transmons: large-scale cryogenic CMOS control of superconducting qubits</t>
+        </is>
+      </c>
+      <c r="R765" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S765" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T765" t="inlineStr"/>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr"/>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C766" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr"/>
+      <c r="F766" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G766" t="inlineStr"/>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I766" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J766" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K766" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L766" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M766" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N766" t="inlineStr"/>
+      <c r="O766" t="inlineStr"/>
+      <c r="P766" t="inlineStr"/>
+      <c r="Q766" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R766" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S766" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T766" t="inlineStr"/>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr"/>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="C767" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr"/>
+      <c r="F767" t="inlineStr">
+        <is>
+          <t>Matys, Maciej; Yamada, Atsushi; Ohki, Toshihiro</t>
+        </is>
+      </c>
+      <c r="G767" t="inlineStr"/>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="I767" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15001376/v2</t>
+        </is>
+      </c>
+      <c r="J767" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K767" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L767" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M767" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N767" t="inlineStr"/>
+      <c r="O767" t="inlineStr"/>
+      <c r="P767" t="inlineStr"/>
+      <c r="Q767" t="inlineStr">
+        <is>
+          <t>Observation of ”negative” persistent photoconductivity effect at T &amp;gt; 200 oC in N-polar GaN/AlGaN/GaN heterostructures</t>
+        </is>
+      </c>
+      <c r="R767" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S767" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T767" t="inlineStr"/>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr"/>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Transistors to transmons: large-scale cryogenic CMOS control of superconducting qubits</t>
+        </is>
+      </c>
+      <c r="C768" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr"/>
+      <c r="F768" t="inlineStr">
+        <is>
+          <t>Underwood, Devin</t>
+        </is>
+      </c>
+      <c r="G768" t="inlineStr"/>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10095152/v1</t>
+        </is>
+      </c>
+      <c r="I768" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10095152/v1</t>
+        </is>
+      </c>
+      <c r="J768" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K768" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L768" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M768" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N768" t="inlineStr"/>
+      <c r="O768" t="inlineStr"/>
+      <c r="P768" t="inlineStr"/>
+      <c r="Q768" t="inlineStr">
+        <is>
+          <t>Transistors to transmons: large-scale cryogenic CMOS control of superconducting qubits</t>
+        </is>
+      </c>
+      <c r="R768" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S768" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T768" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-05T00:04Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T768"/>
+  <dimension ref="A1:T770"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58516,6 +58516,158 @@
       </c>
       <c r="T768" t="inlineStr"/>
     </row>
+    <row r="769">
+      <c r="A769" t="inlineStr"/>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Migration strategies from monolithic systems to Kubernetes-native microservices in enterprise environments</t>
+        </is>
+      </c>
+      <c r="C769" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>GSC Online Press</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>World Journal of Advanced Engineering Technology and Sciences</t>
+        </is>
+      </c>
+      <c r="F769" t="inlineStr">
+        <is>
+          <t>Srivastava, Shubham</t>
+        </is>
+      </c>
+      <c r="G769" t="inlineStr"/>
+      <c r="H769" t="inlineStr">
+        <is>
+          <t>10.30574/wjaets.2026.20.1.0329</t>
+        </is>
+      </c>
+      <c r="I769" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.30574/wjaets.2026.20.1.0329</t>
+        </is>
+      </c>
+      <c r="J769" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K769" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L769" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M769" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N769" t="inlineStr"/>
+      <c r="O769" t="inlineStr"/>
+      <c r="P769" t="inlineStr"/>
+      <c r="Q769" t="inlineStr">
+        <is>
+          <t>Migration strategies from monolithic systems to Kubernetes-native microservices in enterprise environments</t>
+        </is>
+      </c>
+      <c r="R769" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S769" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T769" t="inlineStr"/>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr"/>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>0.71% Lattice‐Mismatched Intergrowth Achieves 2000‐Cycle Stability in O3‐Type Na‐Layered Oxide Cathodes</t>
+        </is>
+      </c>
+      <c r="C770" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>Advanced Energy Materials</t>
+        </is>
+      </c>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>Yuan, Wei‐Wei; Yuan, Xin‐Guang; Yao, Hu‐Rong; Wen, Min; He, Wei‐Huan; Gan, Lu; Lin, Min; Shan, Pei‐Zhao; Yang, Yong; Guo, Yu‐Jie; Zheng, Lituo; Huang, Zhigao</t>
+        </is>
+      </c>
+      <c r="G770" t="inlineStr"/>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>10.1002/aenm.71237</t>
+        </is>
+      </c>
+      <c r="I770" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/aenm.71237</t>
+        </is>
+      </c>
+      <c r="J770" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K770" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L770" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M770" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N770" t="inlineStr"/>
+      <c r="O770" t="inlineStr"/>
+      <c r="P770" t="inlineStr"/>
+      <c r="Q770" t="inlineStr">
+        <is>
+          <t>0.71% Lattice‐Mismatched Intergrowth Achieves 2000‐Cycle Stability in O3‐Type Na‐Layered Oxide Cathodes</t>
+        </is>
+      </c>
+      <c r="R770" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S770" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T770" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-07T00:13Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T770"/>
+  <dimension ref="A1:T771"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58668,6 +58668,82 @@
       </c>
       <c r="T770" t="inlineStr"/>
     </row>
+    <row r="771">
+      <c r="A771" t="inlineStr"/>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Phase-controlled thermal amplification in a quantum thermal transistor</t>
+        </is>
+      </c>
+      <c r="C771" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>New Journal of Physics</t>
+        </is>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>Wang, Xiaoyun; Xu, Dazhi</t>
+        </is>
+      </c>
+      <c r="G771" t="inlineStr"/>
+      <c r="H771" t="inlineStr">
+        <is>
+          <t>10.1088/1367-2630/ae8690</t>
+        </is>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1367-2630/ae8690</t>
+        </is>
+      </c>
+      <c r="J771" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K771" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L771" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M771" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N771" t="inlineStr"/>
+      <c r="O771" t="inlineStr"/>
+      <c r="P771" t="inlineStr"/>
+      <c r="Q771" t="inlineStr">
+        <is>
+          <t>Phase-controlled thermal amplification in a quantum thermal transistor</t>
+        </is>
+      </c>
+      <c r="R771" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S771" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="T771" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-08T00:01Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T771"/>
+  <dimension ref="A1:T780"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58744,6 +58744,690 @@
       </c>
       <c r="T771" t="inlineStr"/>
     </row>
+    <row r="772">
+      <c r="A772" t="inlineStr"/>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Synergistic Enhancement of Threshold Voltage in AlGaN/GaN HEMTs Using Ferroelectric HfO₂/ZrO₂ Gate Dielectric and Partial Barrier Recess</t>
+        </is>
+      </c>
+      <c r="C772" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>Li, Xinghuan; Xie, Zijing; Liu, Xiaoyi; Ma, Xiao; Wang, Hong</t>
+        </is>
+      </c>
+      <c r="G772" t="inlineStr"/>
+      <c r="H772" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae8719</t>
+        </is>
+      </c>
+      <c r="I772" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae8719</t>
+        </is>
+      </c>
+      <c r="J772" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K772" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L772" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M772" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N772" t="inlineStr"/>
+      <c r="O772" t="inlineStr"/>
+      <c r="P772" t="inlineStr"/>
+      <c r="Q772" t="inlineStr">
+        <is>
+          <t>Synergistic Enhancement of Threshold Voltage in AlGaN/GaN HEMTs Using Ferroelectric HfO₂/ZrO₂ Gate Dielectric and Partial Barrier Recess</t>
+        </is>
+      </c>
+      <c r="R772" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S772" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="T772" t="inlineStr"/>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr"/>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Predictive modeling of Z-shaped gate source pocket TFET using machine learning and TCAD simulation data</t>
+        </is>
+      </c>
+      <c r="C773" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>Kondaveeti, Girija Sravani; Kumar, Rapolu Anil; Panigrahy, Asisa Kumar; Dwivedi, Amit Krishna; Ajayan, J.; Swain, Raghunandan; Karumuri, Srinivasa Rao</t>
+        </is>
+      </c>
+      <c r="G773" t="inlineStr"/>
+      <c r="H773" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-60414-z</t>
+        </is>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-60414-z</t>
+        </is>
+      </c>
+      <c r="J773" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K773" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L773" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M773" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N773" t="inlineStr"/>
+      <c r="O773" t="inlineStr"/>
+      <c r="P773" t="inlineStr"/>
+      <c r="Q773" t="inlineStr">
+        <is>
+          <t>Predictive modeling of Z-shaped gate source pocket TFET using machine learning and TCAD simulation data</t>
+        </is>
+      </c>
+      <c r="R773" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S773" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="T773" t="inlineStr"/>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr"/>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>MOSFET-Oriented Current Sharing Control Strategy for Scalable Parallel DC/DC Converters</t>
+        </is>
+      </c>
+      <c r="C774" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>Qu, Mingzhe; Zhou, Yuan; Zhang, Zhigang; Hu, Liangxing; Zhang, Yu</t>
+        </is>
+      </c>
+      <c r="G774" t="inlineStr"/>
+      <c r="H774" t="inlineStr">
+        <is>
+          <t>10.3390/mi17070818</t>
+        </is>
+      </c>
+      <c r="I774" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17070818</t>
+        </is>
+      </c>
+      <c r="J774" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K774" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L774" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M774" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N774" t="inlineStr"/>
+      <c r="O774" t="inlineStr"/>
+      <c r="P774" t="inlineStr"/>
+      <c r="Q774" t="inlineStr">
+        <is>
+          <t>MOSFET-Oriented Current Sharing Control Strategy for Scalable Parallel DC/DC Converters</t>
+        </is>
+      </c>
+      <c r="R774" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S774" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="T774" t="inlineStr"/>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr"/>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Synergistic Enhancement of Threshold Voltage in AlGaN/GaN HEMTs Using Ferroelectric HfO₂/ZrO₂ Gate Dielectric and Partial Barrier Recess</t>
+        </is>
+      </c>
+      <c r="C775" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>Li, Xinghuan; Xie, Zijing; Liu, Xiaoyi; Ma, Xiao; Wang, Hong</t>
+        </is>
+      </c>
+      <c r="G775" t="inlineStr"/>
+      <c r="H775" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae8719</t>
+        </is>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae8719</t>
+        </is>
+      </c>
+      <c r="J775" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K775" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L775" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M775" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N775" t="inlineStr"/>
+      <c r="O775" t="inlineStr"/>
+      <c r="P775" t="inlineStr"/>
+      <c r="Q775" t="inlineStr">
+        <is>
+          <t>Synergistic Enhancement of Threshold Voltage in AlGaN/GaN HEMTs Using Ferroelectric HfO₂/ZrO₂ Gate Dielectric and Partial Barrier Recess</t>
+        </is>
+      </c>
+      <c r="R775" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S775" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="T775" t="inlineStr"/>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr"/>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Predictive modeling of Z-shaped gate source pocket TFET using machine learning and TCAD simulation data</t>
+        </is>
+      </c>
+      <c r="C776" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F776" t="inlineStr">
+        <is>
+          <t>Kondaveeti, Girija Sravani; Kumar, Rapolu Anil; Panigrahy, Asisa Kumar; Dwivedi, Amit Krishna; Ajayan, J.; Swain, Raghunandan; Karumuri, Srinivasa Rao</t>
+        </is>
+      </c>
+      <c r="G776" t="inlineStr"/>
+      <c r="H776" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-60414-z</t>
+        </is>
+      </c>
+      <c r="I776" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-60414-z</t>
+        </is>
+      </c>
+      <c r="J776" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K776" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L776" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M776" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N776" t="inlineStr"/>
+      <c r="O776" t="inlineStr"/>
+      <c r="P776" t="inlineStr"/>
+      <c r="Q776" t="inlineStr">
+        <is>
+          <t>Predictive modeling of Z-shaped gate source pocket TFET using machine learning and TCAD simulation data</t>
+        </is>
+      </c>
+      <c r="R776" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S776" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="T776" t="inlineStr"/>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr"/>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>MOSFET-Oriented Current Sharing Control Strategy for Scalable Parallel DC/DC Converters</t>
+        </is>
+      </c>
+      <c r="C777" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F777" t="inlineStr">
+        <is>
+          <t>Qu, Mingzhe; Zhou, Yuan; Zhang, Zhigang; Hu, Liangxing; Zhang, Yu</t>
+        </is>
+      </c>
+      <c r="G777" t="inlineStr"/>
+      <c r="H777" t="inlineStr">
+        <is>
+          <t>10.3390/mi17070818</t>
+        </is>
+      </c>
+      <c r="I777" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17070818</t>
+        </is>
+      </c>
+      <c r="J777" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K777" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L777" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M777" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N777" t="inlineStr"/>
+      <c r="O777" t="inlineStr"/>
+      <c r="P777" t="inlineStr"/>
+      <c r="Q777" t="inlineStr">
+        <is>
+          <t>MOSFET-Oriented Current Sharing Control Strategy for Scalable Parallel DC/DC Converters</t>
+        </is>
+      </c>
+      <c r="R777" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S777" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="T777" t="inlineStr"/>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr"/>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Predictive modeling of Z-shaped gate source pocket TFET using machine learning and TCAD simulation data</t>
+        </is>
+      </c>
+      <c r="C778" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F778" t="inlineStr">
+        <is>
+          <t>Kondaveeti, Girija Sravani; Kumar, Rapolu Anil; Panigrahy, Asisa Kumar; Dwivedi, Amit Krishna; Ajayan, J.; Swain, Raghunandan; Karumuri, Srinivasa Rao</t>
+        </is>
+      </c>
+      <c r="G778" t="inlineStr"/>
+      <c r="H778" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-60414-z</t>
+        </is>
+      </c>
+      <c r="I778" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-60414-z</t>
+        </is>
+      </c>
+      <c r="J778" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K778" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L778" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M778" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N778" t="inlineStr"/>
+      <c r="O778" t="inlineStr"/>
+      <c r="P778" t="inlineStr"/>
+      <c r="Q778" t="inlineStr">
+        <is>
+          <t>Predictive modeling of Z-shaped gate source pocket TFET using machine learning and TCAD simulation data</t>
+        </is>
+      </c>
+      <c r="R778" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S778" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="T778" t="inlineStr"/>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr"/>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Synergistic Enhancement of Threshold Voltage in AlGaN/GaN HEMTs Using Ferroelectric HfO₂/ZrO₂ Gate Dielectric and Partial Barrier Recess</t>
+        </is>
+      </c>
+      <c r="C779" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F779" t="inlineStr">
+        <is>
+          <t>Li, Xinghuan; Xie, Zijing; Liu, Xiaoyi; Ma, Xiao; Wang, Hong</t>
+        </is>
+      </c>
+      <c r="G779" t="inlineStr"/>
+      <c r="H779" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae8719</t>
+        </is>
+      </c>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae8719</t>
+        </is>
+      </c>
+      <c r="J779" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K779" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L779" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M779" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N779" t="inlineStr"/>
+      <c r="O779" t="inlineStr"/>
+      <c r="P779" t="inlineStr"/>
+      <c r="Q779" t="inlineStr">
+        <is>
+          <t>Synergistic Enhancement of Threshold Voltage in AlGaN/GaN HEMTs Using Ferroelectric HfO₂/ZrO₂ Gate Dielectric and Partial Barrier Recess</t>
+        </is>
+      </c>
+      <c r="R779" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S779" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="T779" t="inlineStr"/>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr"/>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Synergistic Enhancement of Threshold Voltage in AlGaN/GaN HEMTs Using Ferroelectric HfO₂/ZrO₂ Gate Dielectric and Partial Barrier Recess</t>
+        </is>
+      </c>
+      <c r="C780" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F780" t="inlineStr">
+        <is>
+          <t>Li, Xinghuan; Xie, Zijing; Liu, Xiaoyi; Ma, Xiao; Wang, Hong</t>
+        </is>
+      </c>
+      <c r="G780" t="inlineStr"/>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae8719</t>
+        </is>
+      </c>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae8719</t>
+        </is>
+      </c>
+      <c r="J780" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K780" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L780" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M780" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N780" t="inlineStr"/>
+      <c r="O780" t="inlineStr"/>
+      <c r="P780" t="inlineStr"/>
+      <c r="Q780" t="inlineStr">
+        <is>
+          <t>Synergistic Enhancement of Threshold Voltage in AlGaN/GaN HEMTs Using Ferroelectric HfO₂/ZrO₂ Gate Dielectric and Partial Barrier Recess</t>
+        </is>
+      </c>
+      <c r="R780" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S780" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="T780" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-09T00:14Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T780"/>
+  <dimension ref="A1:T787"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59428,6 +59428,534 @@
       </c>
       <c r="T780" t="inlineStr"/>
     </row>
+    <row r="781">
+      <c r="A781" t="inlineStr"/>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="C781" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Cerebration Science Publishing Co., Limited</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>International Journal of Computer Information Systems and Industrial Management Applications</t>
+        </is>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>Hongyi Wei</t>
+        </is>
+      </c>
+      <c r="G781" t="inlineStr"/>
+      <c r="H781" t="inlineStr">
+        <is>
+          <t>10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="J781" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K781" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L781" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M781" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N781" t="inlineStr"/>
+      <c r="O781" t="inlineStr"/>
+      <c r="P781" t="inlineStr"/>
+      <c r="Q781" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="R781" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S781" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="T781" t="inlineStr"/>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr"/>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="C782" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Cerebration Science Publishing Co., Limited</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>International Journal of Computer Information Systems and Industrial Management Applications</t>
+        </is>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>Hongyi Wei</t>
+        </is>
+      </c>
+      <c r="G782" t="inlineStr"/>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="I782" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="J782" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K782" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L782" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M782" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N782" t="inlineStr"/>
+      <c r="O782" t="inlineStr"/>
+      <c r="P782" t="inlineStr"/>
+      <c r="Q782" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="R782" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S782" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="T782" t="inlineStr"/>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr"/>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Hollow-strut lattice architectures for distributed actuation and sensing in monolithic soft robots</t>
+        </is>
+      </c>
+      <c r="C783" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr"/>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>Coutinho, Altair; Exley, Trevor; Trunin, Petr; Nardin, Anderson Brazil; Beccai, Lucia</t>
+        </is>
+      </c>
+      <c r="G783" t="inlineStr"/>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10207223/v1</t>
+        </is>
+      </c>
+      <c r="I783" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10207223/v1</t>
+        </is>
+      </c>
+      <c r="J783" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K783" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L783" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M783" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N783" t="inlineStr"/>
+      <c r="O783" t="inlineStr"/>
+      <c r="P783" t="inlineStr"/>
+      <c r="Q783" t="inlineStr">
+        <is>
+          <t>Hollow-strut lattice architectures for distributed actuation and sensing in monolithic soft robots</t>
+        </is>
+      </c>
+      <c r="R783" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S783" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="T783" t="inlineStr"/>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr"/>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Degradation Mechanism of static and capacitance characteristic of 700 V p-GaN gate HEMT Under Repetitive Unclamped Inductive Switching Stress</t>
+        </is>
+      </c>
+      <c r="C784" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>Liu, Teng; Zhao, Linna; Li, Chenghao; Zhao, Ruijie; Gu, Xiaofeng; Zhu, Chenkai; Yang, Zhuo; Yang, Qian; Li, Zongqing</t>
+        </is>
+      </c>
+      <c r="G784" t="inlineStr"/>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae87c2</t>
+        </is>
+      </c>
+      <c r="I784" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae87c2</t>
+        </is>
+      </c>
+      <c r="J784" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K784" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L784" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M784" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N784" t="inlineStr"/>
+      <c r="O784" t="inlineStr"/>
+      <c r="P784" t="inlineStr"/>
+      <c r="Q784" t="inlineStr">
+        <is>
+          <t>Degradation Mechanism of static and capacitance characteristic of 700 V p-GaN gate HEMT Under Repetitive Unclamped Inductive Switching Stress</t>
+        </is>
+      </c>
+      <c r="R784" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S784" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="T784" t="inlineStr"/>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr"/>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="C785" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Cerebration Science Publishing Co., Limited</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>International Journal of Computer Information Systems and Industrial Management Applications</t>
+        </is>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>Hongyi Wei</t>
+        </is>
+      </c>
+      <c r="G785" t="inlineStr"/>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="I785" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="J785" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K785" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L785" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M785" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N785" t="inlineStr"/>
+      <c r="O785" t="inlineStr"/>
+      <c r="P785" t="inlineStr"/>
+      <c r="Q785" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="R785" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S785" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="T785" t="inlineStr"/>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr"/>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="C786" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>Cerebration Science Publishing Co., Limited</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>International Journal of Computer Information Systems and Industrial Management Applications</t>
+        </is>
+      </c>
+      <c r="F786" t="inlineStr">
+        <is>
+          <t>Hongyi Wei</t>
+        </is>
+      </c>
+      <c r="G786" t="inlineStr"/>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="I786" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="J786" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K786" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L786" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M786" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N786" t="inlineStr"/>
+      <c r="O786" t="inlineStr"/>
+      <c r="P786" t="inlineStr"/>
+      <c r="Q786" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="R786" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S786" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="T786" t="inlineStr"/>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr"/>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="C787" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Cerebration Science Publishing Co., Limited</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>International Journal of Computer Information Systems and Industrial Management Applications</t>
+        </is>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>Hongyi Wei</t>
+        </is>
+      </c>
+      <c r="G787" t="inlineStr"/>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.70917/ijcisim-2026-2818</t>
+        </is>
+      </c>
+      <c r="J787" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K787" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L787" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M787" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N787" t="inlineStr"/>
+      <c r="O787" t="inlineStr"/>
+      <c r="P787" t="inlineStr"/>
+      <c r="Q787" t="inlineStr">
+        <is>
+          <t>Silicon-Based GaN Power Devices and CMOS Monolithic Heterogeneous Integration with Driver Circuit Co-Optimization</t>
+        </is>
+      </c>
+      <c r="R787" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S787" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="T787" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-10T00:08Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T787"/>
+  <dimension ref="A1:T794"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59956,6 +59956,538 @@
       </c>
       <c r="T787" t="inlineStr"/>
     </row>
+    <row r="788">
+      <c r="A788" t="inlineStr"/>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Robust Inverter Synchronisation for Weak Grid Based on Impedance Estimation</t>
+        </is>
+      </c>
+      <c r="C788" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>Nguyen, Phuoc Sang; Nourbakhsh, Ghavameddin; Ledwich, Gerard</t>
+        </is>
+      </c>
+      <c r="G788" t="inlineStr"/>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>10.3390/en19143236</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19143236</t>
+        </is>
+      </c>
+      <c r="J788" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K788" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L788" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M788" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N788" t="inlineStr"/>
+      <c r="O788" t="inlineStr"/>
+      <c r="P788" t="inlineStr"/>
+      <c r="Q788" t="inlineStr">
+        <is>
+          <t>Robust Inverter Synchronisation for Weak Grid Based on Impedance Estimation</t>
+        </is>
+      </c>
+      <c r="R788" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S788" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="T788" t="inlineStr"/>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr"/>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Reliability-Oriented Performance Evaluation of a Photovoltaic Inverter Considering an Integrated Si–SiC IGBT</t>
+        </is>
+      </c>
+      <c r="C789" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>G, JAYALAXMI; Kottala, Padma; R.V.S, Lakshmi Kumari</t>
+        </is>
+      </c>
+      <c r="G789" t="inlineStr"/>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae88d8</t>
+        </is>
+      </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae88d8</t>
+        </is>
+      </c>
+      <c r="J789" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K789" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L789" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M789" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N789" t="inlineStr"/>
+      <c r="O789" t="inlineStr"/>
+      <c r="P789" t="inlineStr"/>
+      <c r="Q789" t="inlineStr">
+        <is>
+          <t>Reliability-Oriented Performance Evaluation of a Photovoltaic Inverter Considering an Integrated Si–SiC IGBT</t>
+        </is>
+      </c>
+      <c r="R789" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S789" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="T789" t="inlineStr"/>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr"/>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Robust Inverter Synchronisation for Weak Grid Based on Impedance Estimation</t>
+        </is>
+      </c>
+      <c r="C790" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>Nguyen, Phuoc Sang; Nourbakhsh, Ghavameddin; Ledwich, Gerard</t>
+        </is>
+      </c>
+      <c r="G790" t="inlineStr"/>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>10.3390/en19143236</t>
+        </is>
+      </c>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19143236</t>
+        </is>
+      </c>
+      <c r="J790" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K790" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L790" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M790" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N790" t="inlineStr"/>
+      <c r="O790" t="inlineStr"/>
+      <c r="P790" t="inlineStr"/>
+      <c r="Q790" t="inlineStr">
+        <is>
+          <t>Robust Inverter Synchronisation for Weak Grid Based on Impedance Estimation</t>
+        </is>
+      </c>
+      <c r="R790" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S790" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="T790" t="inlineStr"/>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr"/>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>The New Media Operating System (NMOS): A Synthesis Model of Deconglomeration, Decentralization, and Demassification in the New Media Communication Domain</t>
+        </is>
+      </c>
+      <c r="C791" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Yayasan Dharma Indonesia Tercinta (Dinasti)</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>Greenation International Journal of Law and Social Sciences</t>
+        </is>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>Revta Revolusi, Prabu; Kusubandio, Wishnutama; Febriandy, Radians Krisna</t>
+        </is>
+      </c>
+      <c r="G791" t="inlineStr"/>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>10.38035/gijlss.v4i3.1022</t>
+        </is>
+      </c>
+      <c r="I791" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.38035/gijlss.v4i3.1022</t>
+        </is>
+      </c>
+      <c r="J791" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K791" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L791" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M791" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N791" t="inlineStr"/>
+      <c r="O791" t="inlineStr"/>
+      <c r="P791" t="inlineStr"/>
+      <c r="Q791" t="inlineStr">
+        <is>
+          <t>The New Media Operating System (NMOS): A Synthesis Model of Deconglomeration, Decentralization, and Demassification in the New Media Communication Domain</t>
+        </is>
+      </c>
+      <c r="R791" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S791" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="T791" t="inlineStr"/>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr"/>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Robust Inverter Synchronisation for Weak Grid Based on Impedance Estimation</t>
+        </is>
+      </c>
+      <c r="C792" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>Nguyen, Phuoc Sang; Nourbakhsh, Ghavameddin; Ledwich, Gerard</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr"/>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>10.3390/en19143236</t>
+        </is>
+      </c>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19143236</t>
+        </is>
+      </c>
+      <c r="J792" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K792" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L792" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M792" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N792" t="inlineStr"/>
+      <c r="O792" t="inlineStr"/>
+      <c r="P792" t="inlineStr"/>
+      <c r="Q792" t="inlineStr">
+        <is>
+          <t>Robust Inverter Synchronisation for Weak Grid Based on Impedance Estimation</t>
+        </is>
+      </c>
+      <c r="R792" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S792" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="T792" t="inlineStr"/>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr"/>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Reliability-Oriented Performance Evaluation of a Photovoltaic Inverter Considering an Integrated Si–SiC IGBT</t>
+        </is>
+      </c>
+      <c r="C793" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>G, JAYALAXMI; Kottala, Padma; R.V.S, Lakshmi Kumari</t>
+        </is>
+      </c>
+      <c r="G793" t="inlineStr"/>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae88d8</t>
+        </is>
+      </c>
+      <c r="I793" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae88d8</t>
+        </is>
+      </c>
+      <c r="J793" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K793" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L793" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M793" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N793" t="inlineStr"/>
+      <c r="O793" t="inlineStr"/>
+      <c r="P793" t="inlineStr"/>
+      <c r="Q793" t="inlineStr">
+        <is>
+          <t>Reliability-Oriented Performance Evaluation of a Photovoltaic Inverter Considering an Integrated Si–SiC IGBT</t>
+        </is>
+      </c>
+      <c r="R793" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S793" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="T793" t="inlineStr"/>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr"/>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Robust Inverter Synchronisation for Weak Grid Based on Impedance Estimation</t>
+        </is>
+      </c>
+      <c r="C794" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>Nguyen, Phuoc Sang; Nourbakhsh, Ghavameddin; Ledwich, Gerard</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr"/>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>10.3390/en19143236</t>
+        </is>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19143236</t>
+        </is>
+      </c>
+      <c r="J794" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K794" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L794" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M794" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N794" t="inlineStr"/>
+      <c r="O794" t="inlineStr"/>
+      <c r="P794" t="inlineStr"/>
+      <c r="Q794" t="inlineStr">
+        <is>
+          <t>Robust Inverter Synchronisation for Weak Grid Based on Impedance Estimation</t>
+        </is>
+      </c>
+      <c r="R794" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S794" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="T794" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-11T00:01Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T794"/>
+  <dimension ref="A1:T799"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60488,6 +60488,386 @@
       </c>
       <c r="T794" t="inlineStr"/>
     </row>
+    <row r="795">
+      <c r="A795" t="inlineStr"/>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Operation Whole Health: An Operation Warp Speed Directed at Noncommunicable Diseases</t>
+        </is>
+      </c>
+      <c r="C795" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>Burdick, Ryan R.; Maiers, Michele J.; Albertson, Andrea K.; Sawyer, Charles E.</t>
+        </is>
+      </c>
+      <c r="G795" t="inlineStr"/>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261461166</t>
+        </is>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261461166</t>
+        </is>
+      </c>
+      <c r="J795" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K795" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L795" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M795" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N795" t="inlineStr"/>
+      <c r="O795" t="inlineStr"/>
+      <c r="P795" t="inlineStr"/>
+      <c r="Q795" t="inlineStr">
+        <is>
+          <t>Operation Whole Health: An Operation Warp Speed Directed at Noncommunicable Diseases</t>
+        </is>
+      </c>
+      <c r="R795" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S795" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="T795" t="inlineStr"/>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr"/>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Monolithic microcavity-metalens interfaces: bridging performance and complexity in quantum light sources</t>
+        </is>
+      </c>
+      <c r="C796" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>eLight</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>Betzold, Simon; Höfling, Sven</t>
+        </is>
+      </c>
+      <c r="G796" t="inlineStr"/>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>10.1186/s43593-026-00134-z</t>
+        </is>
+      </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s43593-026-00134-z</t>
+        </is>
+      </c>
+      <c r="J796" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K796" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L796" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M796" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N796" t="inlineStr"/>
+      <c r="O796" t="inlineStr"/>
+      <c r="P796" t="inlineStr"/>
+      <c r="Q796" t="inlineStr">
+        <is>
+          <t>Monolithic microcavity-metalens interfaces: bridging performance and complexity in quantum light sources</t>
+        </is>
+      </c>
+      <c r="R796" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S796" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="T796" t="inlineStr"/>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr"/>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>An Adaptive Gate-Side Feedback Active Gate Driver for GaN Devices with Optimized Switching Performance</t>
+        </is>
+      </c>
+      <c r="C797" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>Zhang, Yuxin; Huang, Baoqiang; Wu, Tiantian; Wang, Zhe; Zhang, Qiao; Zhang, Desheng; Lei, Jianming; Min, Run; Tong, Qiaoling</t>
+        </is>
+      </c>
+      <c r="G797" t="inlineStr"/>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>10.3390/mi17070826</t>
+        </is>
+      </c>
+      <c r="I797" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17070826</t>
+        </is>
+      </c>
+      <c r="J797" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K797" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L797" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M797" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N797" t="inlineStr"/>
+      <c r="O797" t="inlineStr"/>
+      <c r="P797" t="inlineStr"/>
+      <c r="Q797" t="inlineStr">
+        <is>
+          <t>An Adaptive Gate-Side Feedback Active Gate Driver for GaN Devices with Optimized Switching Performance</t>
+        </is>
+      </c>
+      <c r="R797" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S797" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="T797" t="inlineStr"/>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr"/>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>An Adaptive Gate-Side Feedback Active Gate Driver for GaN Devices with Optimized Switching Performance</t>
+        </is>
+      </c>
+      <c r="C798" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>Zhang, Yuxin; Huang, Baoqiang; Wu, Tiantian; Wang, Zhe; Zhang, Qiao; Zhang, Desheng; Lei, Jianming; Min, Run; Tong, Qiaoling</t>
+        </is>
+      </c>
+      <c r="G798" t="inlineStr"/>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>10.3390/mi17070826</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17070826</t>
+        </is>
+      </c>
+      <c r="J798" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K798" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L798" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M798" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N798" t="inlineStr"/>
+      <c r="O798" t="inlineStr"/>
+      <c r="P798" t="inlineStr"/>
+      <c r="Q798" t="inlineStr">
+        <is>
+          <t>An Adaptive Gate-Side Feedback Active Gate Driver for GaN Devices with Optimized Switching Performance</t>
+        </is>
+      </c>
+      <c r="R798" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S798" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="T798" t="inlineStr"/>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr"/>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>An Adaptive Gate-Side Feedback Active Gate Driver for GaN Devices with Optimized Switching Performance</t>
+        </is>
+      </c>
+      <c r="C799" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>Zhang, Yuxin; Huang, Baoqiang; Wu, Tiantian; Wang, Zhe; Zhang, Qiao; Zhang, Desheng; Lei, Jianming; Min, Run; Tong, Qiaoling</t>
+        </is>
+      </c>
+      <c r="G799" t="inlineStr"/>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>10.3390/mi17070826</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17070826</t>
+        </is>
+      </c>
+      <c r="J799" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K799" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L799" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M799" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N799" t="inlineStr"/>
+      <c r="O799" t="inlineStr"/>
+      <c r="P799" t="inlineStr"/>
+      <c r="Q799" t="inlineStr">
+        <is>
+          <t>An Adaptive Gate-Side Feedback Active Gate Driver for GaN Devices with Optimized Switching Performance</t>
+        </is>
+      </c>
+      <c r="R799" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S799" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="T799" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-11T23:58Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T799"/>
+  <dimension ref="A1:T801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60868,6 +60868,158 @@
       </c>
       <c r="T799" t="inlineStr"/>
     </row>
+    <row r="800">
+      <c r="A800" t="inlineStr"/>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Integrating device simulation with machine learning for improved characteristic of halo doped gate stack triple metal gate all around (HD-GS-TM-GAA) MOSFET</t>
+        </is>
+      </c>
+      <c r="C800" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>Memories - Materials, Devices, Circuits and Systems</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>Gupta, Rashmi; Gupta, Neeraj; Kumar, Prashant</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr"/>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>10.1016/j.memori.2026.100145</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.memori.2026.100145</t>
+        </is>
+      </c>
+      <c r="J800" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K800" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L800" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M800" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N800" t="inlineStr"/>
+      <c r="O800" t="inlineStr"/>
+      <c r="P800" t="inlineStr"/>
+      <c r="Q800" t="inlineStr">
+        <is>
+          <t>Integrating device simulation with machine learning for improved characteristic of halo doped gate stack triple metal gate all around (HD-GS-TM-GAA) MOSFET</t>
+        </is>
+      </c>
+      <c r="R800" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S800" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="T800" t="inlineStr"/>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr"/>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Advanced CMOS Scaling Challenges And Emerging Solutions For Future VLSI Systems</t>
+        </is>
+      </c>
+      <c r="C801" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Edtech Publishers (OPC) Private Limited</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>International Journal of Science, Strategic Management and Technology</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>Puttapaka Lokesh, Puttapaka Lokesh; Akula Sathvika, Akula Sathvika; P Kavitha, P Kavitha</t>
+        </is>
+      </c>
+      <c r="G801" t="inlineStr"/>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>10.55041/ijsmt.v2i7.013</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.55041/ijsmt.v2i7.013</t>
+        </is>
+      </c>
+      <c r="J801" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K801" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L801" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M801" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N801" t="inlineStr"/>
+      <c r="O801" t="inlineStr"/>
+      <c r="P801" t="inlineStr"/>
+      <c r="Q801" t="inlineStr">
+        <is>
+          <t>Advanced CMOS Scaling Challenges And Emerging Solutions For Future VLSI Systems</t>
+        </is>
+      </c>
+      <c r="R801" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S801" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="T801" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-13T23:56Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T801"/>
+  <dimension ref="A1:T806"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61020,6 +61020,386 @@
       </c>
       <c r="T801" t="inlineStr"/>
     </row>
+    <row r="802">
+      <c r="A802" t="inlineStr"/>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>EMI-Induced Eye Diagram Degradation in CMOS Inverter: Experimental Analysis and Predictive Modeling</t>
+        </is>
+      </c>
+      <c r="C802" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>Microelectronics</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>Abedi, Mohammad; Abedi, Zahra; Hemmady, Sameer; Schamiloglu, Edl; Zarkesh-Ha, Payman</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr"/>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>10.3390/microelectronics2030012</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/microelectronics2030012</t>
+        </is>
+      </c>
+      <c r="J802" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K802" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L802" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M802" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N802" t="inlineStr"/>
+      <c r="O802" t="inlineStr"/>
+      <c r="P802" t="inlineStr"/>
+      <c r="Q802" t="inlineStr">
+        <is>
+          <t>EMI-Induced Eye Diagram Degradation in CMOS Inverter: Experimental Analysis and Predictive Modeling</t>
+        </is>
+      </c>
+      <c r="R802" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S802" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="T802" t="inlineStr"/>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr"/>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>A voyage-level threshold analysis of planned turnaround vulnerability in cruise ports from an AIS big data perspective</t>
+        </is>
+      </c>
+      <c r="C803" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Frontiers Media SA</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Frontiers in Marine Science</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>Gan, Shengjun; Hu, Shikai; Zhang, Han; Luo, Kai; Yang, Rui; Biancardo, Salvatore Antonio</t>
+        </is>
+      </c>
+      <c r="G803" t="inlineStr"/>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>10.3389/fmars.2026.1886400</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/fmars.2026.1886400</t>
+        </is>
+      </c>
+      <c r="J803" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K803" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L803" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M803" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N803" t="inlineStr"/>
+      <c r="O803" t="inlineStr"/>
+      <c r="P803" t="inlineStr"/>
+      <c r="Q803" t="inlineStr">
+        <is>
+          <t>A voyage-level threshold analysis of planned turnaround vulnerability in cruise ports from an AIS big data perspective</t>
+        </is>
+      </c>
+      <c r="R803" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S803" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="T803" t="inlineStr"/>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr"/>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD-based geometry study on self-aligned coplanar top gate a-IGZO TFTs</t>
+        </is>
+      </c>
+      <c r="C804" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>Choudhary, Nikita; Daus, Alwin; Lahgere, Avinash; Gupta, Gangadhar; Duhan, Pardeep</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr"/>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>10.1063/5.0305029</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0305029</t>
+        </is>
+      </c>
+      <c r="J804" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K804" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L804" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M804" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N804" t="inlineStr"/>
+      <c r="O804" t="inlineStr"/>
+      <c r="P804" t="inlineStr"/>
+      <c r="Q804" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD-based geometry study on self-aligned coplanar top gate a-IGZO TFTs</t>
+        </is>
+      </c>
+      <c r="R804" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S804" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="T804" t="inlineStr"/>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr"/>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD-based geometry study on self-aligned coplanar top gate a-IGZO TFTs</t>
+        </is>
+      </c>
+      <c r="C805" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>Choudhary, Nikita; Daus, Alwin; Lahgere, Avinash; Gupta, Gangadhar; Duhan, Pardeep</t>
+        </is>
+      </c>
+      <c r="G805" t="inlineStr"/>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>10.1063/5.0305029</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0305029</t>
+        </is>
+      </c>
+      <c r="J805" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K805" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L805" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M805" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N805" t="inlineStr"/>
+      <c r="O805" t="inlineStr"/>
+      <c r="P805" t="inlineStr"/>
+      <c r="Q805" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD-based geometry study on self-aligned coplanar top gate a-IGZO TFTs</t>
+        </is>
+      </c>
+      <c r="R805" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S805" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="T805" t="inlineStr"/>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr"/>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD-based geometry study on self-aligned coplanar top gate a-IGZO TFTs</t>
+        </is>
+      </c>
+      <c r="C806" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>APL Electronic Devices</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>Choudhary, Nikita; Daus, Alwin; Lahgere, Avinash; Gupta, Gangadhar; Duhan, Pardeep</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr"/>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>10.1063/5.0305029</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0305029</t>
+        </is>
+      </c>
+      <c r="J806" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K806" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L806" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M806" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N806" t="inlineStr"/>
+      <c r="O806" t="inlineStr"/>
+      <c r="P806" t="inlineStr"/>
+      <c r="Q806" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD-based geometry study on self-aligned coplanar top gate a-IGZO TFTs</t>
+        </is>
+      </c>
+      <c r="R806" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S806" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="T806" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-14T23:55Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T806"/>
+  <dimension ref="A1:T816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61400,6 +61400,762 @@
       </c>
       <c r="T806" t="inlineStr"/>
     </row>
+    <row r="807">
+      <c r="A807" t="inlineStr"/>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Enhanced power performance and threshold voltage stability in quaternary InAlGaN/GaN MIS-HEMTs on Si with gate field plate</t>
+        </is>
+      </c>
+      <c r="C807" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>Discover Electronics</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>Rathaur, Shivendra Kr.; Ma, Cheng-Jun; Yang, Tsung-Ying; Dixit, Abhisek; Chang, Edward Yi</t>
+        </is>
+      </c>
+      <c r="G807" t="inlineStr"/>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>10.1007/s44291-026-00251-6</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s44291-026-00251-6</t>
+        </is>
+      </c>
+      <c r="J807" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K807" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L807" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M807" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N807" t="inlineStr"/>
+      <c r="O807" t="inlineStr"/>
+      <c r="P807" t="inlineStr"/>
+      <c r="Q807" t="inlineStr">
+        <is>
+          <t>Enhanced power performance and threshold voltage stability in quaternary InAlGaN/GaN MIS-HEMTs on Si with gate field plate</t>
+        </is>
+      </c>
+      <c r="R807" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S807" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T807" t="inlineStr"/>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr"/>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>High threshold voltage normally-off AlGaN/GaN MIS-HEMT using dielectric charge trap layer</t>
+        </is>
+      </c>
+      <c r="C808" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>Kanta, Shantveer; S, Niranjan; Venugopalrao, Anirudh; Gowrisankar, Aniruddhan; Chandrasekar, Hareesh; Raghavan, Srinivasan; Bhat, Navakanta</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr"/>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae8a28</t>
+        </is>
+      </c>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae8a28</t>
+        </is>
+      </c>
+      <c r="J808" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K808" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L808" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M808" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N808" t="inlineStr"/>
+      <c r="O808" t="inlineStr"/>
+      <c r="P808" t="inlineStr"/>
+      <c r="Q808" t="inlineStr">
+        <is>
+          <t>High threshold voltage normally-off AlGaN/GaN MIS-HEMT using dielectric charge trap layer</t>
+        </is>
+      </c>
+      <c r="R808" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S808" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T808" t="inlineStr"/>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr"/>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Comparative TCAD investigation of gate-all-around nanowire MOSFETs with emerging channel materials</t>
+        </is>
+      </c>
+      <c r="C809" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>Next Materials</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>Balaji, S.; Balaji, T.S.; Rathinakumar, P.; Karthik, S.</t>
+        </is>
+      </c>
+      <c r="G809" t="inlineStr"/>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>10.1016/j.nxmate.2026.102743</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.nxmate.2026.102743</t>
+        </is>
+      </c>
+      <c r="J809" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K809" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L809" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M809" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N809" t="inlineStr"/>
+      <c r="O809" t="inlineStr"/>
+      <c r="P809" t="inlineStr"/>
+      <c r="Q809" t="inlineStr">
+        <is>
+          <t>Comparative TCAD investigation of gate-all-around nanowire MOSFETs with emerging channel materials</t>
+        </is>
+      </c>
+      <c r="R809" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S809" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T809" t="inlineStr"/>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr"/>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Comparative TCAD investigation of gate-all-around nanowire MOSFETs with emerging channel materials</t>
+        </is>
+      </c>
+      <c r="C810" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>Next Materials</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>Balaji, S.; Balaji, T.S.; Rathinakumar, P.; Karthik, S.</t>
+        </is>
+      </c>
+      <c r="G810" t="inlineStr"/>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>10.1016/j.nxmate.2026.102743</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.nxmate.2026.102743</t>
+        </is>
+      </c>
+      <c r="J810" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K810" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L810" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M810" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N810" t="inlineStr"/>
+      <c r="O810" t="inlineStr"/>
+      <c r="P810" t="inlineStr"/>
+      <c r="Q810" t="inlineStr">
+        <is>
+          <t>Comparative TCAD investigation of gate-all-around nanowire MOSFETs with emerging channel materials</t>
+        </is>
+      </c>
+      <c r="R810" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S810" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T810" t="inlineStr"/>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr"/>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>High threshold voltage normally-off AlGaN/GaN MIS-HEMT using dielectric charge trap layer</t>
+        </is>
+      </c>
+      <c r="C811" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>Kanta, Shantveer; S, Niranjan; Venugopalrao, Anirudh; Gowrisankar, Aniruddhan; Chandrasekar, Hareesh; Raghavan, Srinivasan; Bhat, Navakanta</t>
+        </is>
+      </c>
+      <c r="G811" t="inlineStr"/>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae8a28</t>
+        </is>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae8a28</t>
+        </is>
+      </c>
+      <c r="J811" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K811" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L811" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M811" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N811" t="inlineStr"/>
+      <c r="O811" t="inlineStr"/>
+      <c r="P811" t="inlineStr"/>
+      <c r="Q811" t="inlineStr">
+        <is>
+          <t>High threshold voltage normally-off AlGaN/GaN MIS-HEMT using dielectric charge trap layer</t>
+        </is>
+      </c>
+      <c r="R811" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S811" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T811" t="inlineStr"/>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr"/>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Fabrication and DC Characterization of BST-Gated AlGaN/GaN MOS-HEMT Structures in Two- and Three-Terminal Configurations</t>
+        </is>
+      </c>
+      <c r="C812" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr"/>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>Abdullah</t>
+        </is>
+      </c>
+      <c r="G812" t="inlineStr"/>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10319963/v1</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10319963/v1</t>
+        </is>
+      </c>
+      <c r="J812" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K812" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L812" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M812" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N812" t="inlineStr"/>
+      <c r="O812" t="inlineStr"/>
+      <c r="P812" t="inlineStr"/>
+      <c r="Q812" t="inlineStr">
+        <is>
+          <t>Fabrication and DC Characterization of BST-Gated AlGaN/GaN MOS-HEMT Structures in Two- and Three-Terminal Configurations</t>
+        </is>
+      </c>
+      <c r="R812" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S812" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T812" t="inlineStr"/>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr"/>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Enhanced power performance and threshold voltage stability in quaternary InAlGaN/GaN MIS-HEMTs on Si with gate field plate</t>
+        </is>
+      </c>
+      <c r="C813" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>Discover Electronics</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>Rathaur, Shivendra Kr.; Ma, Cheng-Jun; Yang, Tsung-Ying; Dixit, Abhisek; Chang, Edward Yi</t>
+        </is>
+      </c>
+      <c r="G813" t="inlineStr"/>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>10.1007/s44291-026-00251-6</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s44291-026-00251-6</t>
+        </is>
+      </c>
+      <c r="J813" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K813" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L813" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M813" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N813" t="inlineStr"/>
+      <c r="O813" t="inlineStr"/>
+      <c r="P813" t="inlineStr"/>
+      <c r="Q813" t="inlineStr">
+        <is>
+          <t>Enhanced power performance and threshold voltage stability in quaternary InAlGaN/GaN MIS-HEMTs on Si with gate field plate</t>
+        </is>
+      </c>
+      <c r="R813" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S813" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T813" t="inlineStr"/>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr"/>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Comparative TCAD investigation of gate-all-around nanowire MOSFETs with emerging channel materials</t>
+        </is>
+      </c>
+      <c r="C814" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>Next Materials</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>Balaji, S.; Balaji, T.S.; Rathinakumar, P.; Karthik, S.</t>
+        </is>
+      </c>
+      <c r="G814" t="inlineStr"/>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>10.1016/j.nxmate.2026.102743</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.nxmate.2026.102743</t>
+        </is>
+      </c>
+      <c r="J814" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K814" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L814" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M814" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N814" t="inlineStr"/>
+      <c r="O814" t="inlineStr"/>
+      <c r="P814" t="inlineStr"/>
+      <c r="Q814" t="inlineStr">
+        <is>
+          <t>Comparative TCAD investigation of gate-all-around nanowire MOSFETs with emerging channel materials</t>
+        </is>
+      </c>
+      <c r="R814" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S814" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T814" t="inlineStr"/>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr"/>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Enhanced power performance and threshold voltage stability in quaternary InAlGaN/GaN MIS-HEMTs on Si with gate field plate</t>
+        </is>
+      </c>
+      <c r="C815" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>Discover Electronics</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>Rathaur, Shivendra Kr.; Ma, Cheng-Jun; Yang, Tsung-Ying; Dixit, Abhisek; Chang, Edward Yi</t>
+        </is>
+      </c>
+      <c r="G815" t="inlineStr"/>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>10.1007/s44291-026-00251-6</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s44291-026-00251-6</t>
+        </is>
+      </c>
+      <c r="J815" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K815" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L815" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M815" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N815" t="inlineStr"/>
+      <c r="O815" t="inlineStr"/>
+      <c r="P815" t="inlineStr"/>
+      <c r="Q815" t="inlineStr">
+        <is>
+          <t>Enhanced power performance and threshold voltage stability in quaternary InAlGaN/GaN MIS-HEMTs on Si with gate field plate</t>
+        </is>
+      </c>
+      <c r="R815" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S815" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T815" t="inlineStr"/>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr"/>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Comparative TCAD investigation of gate-all-around nanowire MOSFETs with emerging channel materials</t>
+        </is>
+      </c>
+      <c r="C816" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>Next Materials</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>Balaji, S.; Balaji, T.S.; Rathinakumar, P.; Karthik, S.</t>
+        </is>
+      </c>
+      <c r="G816" t="inlineStr"/>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>10.1016/j.nxmate.2026.102743</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.nxmate.2026.102743</t>
+        </is>
+      </c>
+      <c r="J816" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K816" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L816" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M816" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N816" t="inlineStr"/>
+      <c r="O816" t="inlineStr"/>
+      <c r="P816" t="inlineStr"/>
+      <c r="Q816" t="inlineStr">
+        <is>
+          <t>Comparative TCAD investigation of gate-all-around nanowire MOSFETs with emerging channel materials</t>
+        </is>
+      </c>
+      <c r="R816" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S816" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="T816" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-16T00:01Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T816"/>
+  <dimension ref="A1:T826"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62156,6 +62156,762 @@
       </c>
       <c r="T816" t="inlineStr"/>
     </row>
+    <row r="817">
+      <c r="A817" t="inlineStr"/>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Bridging Policy and Practice: Strengthening Complementary and Integrative Medicine Through the Lens of the Delhi Declaration</t>
+        </is>
+      </c>
+      <c r="C817" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>Thakur, Rinky; Mishra, Avishek; Vyas, Mahesh K.</t>
+        </is>
+      </c>
+      <c r="G817" t="inlineStr"/>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261469679</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261469679</t>
+        </is>
+      </c>
+      <c r="J817" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K817" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L817" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M817" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N817" t="inlineStr"/>
+      <c r="O817" t="inlineStr"/>
+      <c r="P817" t="inlineStr"/>
+      <c r="Q817" t="inlineStr">
+        <is>
+          <t>Bridging Policy and Practice: Strengthening Complementary and Integrative Medicine Through the Lens of the Delhi Declaration</t>
+        </is>
+      </c>
+      <c r="R817" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S817" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T817" t="inlineStr"/>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr"/>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Monolithic Integration of Piezo-Optomechanical Photonics and CMOS Electronics</t>
+        </is>
+      </c>
+      <c r="C818" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr"/>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>Zimmermann, Matthew; Zhai, Aileen; Leenheer, Andrew; Boyle, Julia; Mishra, Mayank; Dominguez, Daniel; Koppa, Matthew; Jehle, Wolfe; Panuski, Christopher; Dong, Mark; Gilbert, Gerald; Englund, Dirk</t>
+        </is>
+      </c>
+      <c r="G818" t="inlineStr"/>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10221147/v1</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10221147/v1</t>
+        </is>
+      </c>
+      <c r="J818" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K818" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L818" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M818" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N818" t="inlineStr"/>
+      <c r="O818" t="inlineStr"/>
+      <c r="P818" t="inlineStr"/>
+      <c r="Q818" t="inlineStr">
+        <is>
+          <t>Monolithic Integration of Piezo-Optomechanical Photonics and CMOS Electronics</t>
+        </is>
+      </c>
+      <c r="R818" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S818" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T818" t="inlineStr"/>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr"/>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Tail latency, throughput, and memory overhead of monolithic and microservices architectures in resource-constrained docker deployments</t>
+        </is>
+      </c>
+      <c r="C819" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Lembaga Penelitian dan Pengabdian kepada Masyarakat ITS</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>JUTI: Jurnal Ilmiah Teknologi Informasi</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>Tofan, Yoga Ari</t>
+        </is>
+      </c>
+      <c r="G819" t="inlineStr"/>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>10.12962/j24068535.v24i2.a1516</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.12962/j24068535.v24i2.a1516</t>
+        </is>
+      </c>
+      <c r="J819" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K819" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L819" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M819" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N819" t="inlineStr"/>
+      <c r="O819" t="inlineStr"/>
+      <c r="P819" t="inlineStr"/>
+      <c r="Q819" t="inlineStr">
+        <is>
+          <t>Tail latency, throughput, and memory overhead of monolithic and microservices architectures in resource-constrained docker deployments</t>
+        </is>
+      </c>
+      <c r="R819" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S819" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T819" t="inlineStr"/>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr"/>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Effect of different surface treatment protocols on surface topography, biaxial flexural strength and compositional alteration of monolithic translucent multi-layered zirconia</t>
+        </is>
+      </c>
+      <c r="C820" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>Discover Materials</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>Abdulgader, Areej; Shono, Nourah; AlNahedh, Hend</t>
+        </is>
+      </c>
+      <c r="G820" t="inlineStr"/>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>10.1007/s43939-026-00802-4</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s43939-026-00802-4</t>
+        </is>
+      </c>
+      <c r="J820" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K820" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L820" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M820" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N820" t="inlineStr"/>
+      <c r="O820" t="inlineStr"/>
+      <c r="P820" t="inlineStr"/>
+      <c r="Q820" t="inlineStr">
+        <is>
+          <t>Effect of different surface treatment protocols on surface topography, biaxial flexural strength and compositional alteration of monolithic translucent multi-layered zirconia</t>
+        </is>
+      </c>
+      <c r="R820" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S820" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T820" t="inlineStr"/>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr"/>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Bridging Policy and Practice: Strengthening Complementary and Integrative Medicine Through the Lens of the Delhi Declaration</t>
+        </is>
+      </c>
+      <c r="C821" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>Thakur, Rinky; Mishra, Avishek; Vyas, Mahesh K.</t>
+        </is>
+      </c>
+      <c r="G821" t="inlineStr"/>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261469679</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261469679</t>
+        </is>
+      </c>
+      <c r="J821" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K821" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L821" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M821" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N821" t="inlineStr"/>
+      <c r="O821" t="inlineStr"/>
+      <c r="P821" t="inlineStr"/>
+      <c r="Q821" t="inlineStr">
+        <is>
+          <t>Bridging Policy and Practice: Strengthening Complementary and Integrative Medicine Through the Lens of the Delhi Declaration</t>
+        </is>
+      </c>
+      <c r="R821" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S821" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T821" t="inlineStr"/>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr"/>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Manipulation of the symmetry of localized terahertz field in an AlGaN/GaN high-electron-mobility transistor integrated in a waveguide</t>
+        </is>
+      </c>
+      <c r="C822" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>Optics Express</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>You, Zhu; Xu, Boyang; Li, Xinxing; Sun, Jiandong; Qin, Chenyang; Xiang, Lanyong; Chen, Hanze; Jin, Chenyang; Shangguan, Yang; Qin, Hua</t>
+        </is>
+      </c>
+      <c r="G822" t="inlineStr"/>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>10.1364/oe.600020</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/oe.600020</t>
+        </is>
+      </c>
+      <c r="J822" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K822" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L822" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M822" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N822" t="inlineStr"/>
+      <c r="O822" t="inlineStr"/>
+      <c r="P822" t="inlineStr"/>
+      <c r="Q822" t="inlineStr">
+        <is>
+          <t>Manipulation of the symmetry of localized terahertz field in an AlGaN/GaN high-electron-mobility transistor integrated in a waveguide</t>
+        </is>
+      </c>
+      <c r="R822" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S822" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T822" t="inlineStr"/>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr"/>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Investigation on Geometrical Effects of FinFET Electronic Device Properties Using TCAD Simulations and Taguchi Optimization</t>
+        </is>
+      </c>
+      <c r="C823" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Penerbit Universiti Malaysia Perlis</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>International Journal of Nanoelectronics and Materials (IJNeaM)</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>Ahmad Syaiful Othman; Sabrina Reezal; Hanim Hussin; Rafidah Rosman; Maizan Muhamad; Nurul Ezaila Alias; Yasmin Abdul Wahab; Zaira Zaman Chowdhury; Md Fokhrul Islam</t>
+        </is>
+      </c>
+      <c r="G823" t="inlineStr"/>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>10.58915/ijneam.v19ijune.3294</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.58915/ijneam.v19ijune.3294</t>
+        </is>
+      </c>
+      <c r="J823" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K823" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L823" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M823" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N823" t="inlineStr"/>
+      <c r="O823" t="inlineStr"/>
+      <c r="P823" t="inlineStr"/>
+      <c r="Q823" t="inlineStr">
+        <is>
+          <t>Investigation on Geometrical Effects of FinFET Electronic Device Properties Using TCAD Simulations and Taguchi Optimization</t>
+        </is>
+      </c>
+      <c r="R823" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S823" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T823" t="inlineStr"/>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr"/>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Investigation on Geometrical Effects of FinFET Electronic Device Properties Using TCAD Simulations and Taguchi Optimization</t>
+        </is>
+      </c>
+      <c r="C824" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Penerbit Universiti Malaysia Perlis</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>International Journal of Nanoelectronics and Materials (IJNeaM)</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>Ahmad Syaiful Othman; Sabrina Reezal; Hanim Hussin; Rafidah Rosman; Maizan Muhamad; Nurul Ezaila Alias; Yasmin Abdul Wahab; Zaira Zaman Chowdhury; Md Fokhrul Islam</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr"/>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>10.58915/ijneam.v19ijune.3294</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.58915/ijneam.v19ijune.3294</t>
+        </is>
+      </c>
+      <c r="J824" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K824" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L824" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M824" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N824" t="inlineStr"/>
+      <c r="O824" t="inlineStr"/>
+      <c r="P824" t="inlineStr"/>
+      <c r="Q824" t="inlineStr">
+        <is>
+          <t>Investigation on Geometrical Effects of FinFET Electronic Device Properties Using TCAD Simulations and Taguchi Optimization</t>
+        </is>
+      </c>
+      <c r="R824" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S824" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T824" t="inlineStr"/>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr"/>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Analytical power system transient stability assessment considering nonlinear couplings among grid following inverter-based renewable resources</t>
+        </is>
+      </c>
+      <c r="C825" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>Applied Energy</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>Tang, Yingyi; Zhao, Junbo; Zhang, Baosen</t>
+        </is>
+      </c>
+      <c r="G825" t="inlineStr"/>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>10.1016/j.apenergy.2026.128396</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.apenergy.2026.128396</t>
+        </is>
+      </c>
+      <c r="J825" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K825" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L825" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M825" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N825" t="inlineStr"/>
+      <c r="O825" t="inlineStr"/>
+      <c r="P825" t="inlineStr"/>
+      <c r="Q825" t="inlineStr">
+        <is>
+          <t>Analytical power system transient stability assessment considering nonlinear couplings among grid following inverter-based renewable resources</t>
+        </is>
+      </c>
+      <c r="R825" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S825" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T825" t="inlineStr"/>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr"/>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Manipulation of the symmetry of localized terahertz field in an AlGaN/GaN high-electron-mobility transistor integrated in a waveguide</t>
+        </is>
+      </c>
+      <c r="C826" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>Optics Express</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>You, Zhu; Xu, Boyang; Li, Xinxing; Sun, Jiandong; Qin, Chenyang; Xiang, Lanyong; Chen, Hanze; Jin, Chenyang; Shangguan, Yang; Qin, Hua</t>
+        </is>
+      </c>
+      <c r="G826" t="inlineStr"/>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>10.1364/oe.600020</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/oe.600020</t>
+        </is>
+      </c>
+      <c r="J826" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K826" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L826" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M826" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N826" t="inlineStr"/>
+      <c r="O826" t="inlineStr"/>
+      <c r="P826" t="inlineStr"/>
+      <c r="Q826" t="inlineStr">
+        <is>
+          <t>Manipulation of the symmetry of localized terahertz field in an AlGaN/GaN high-electron-mobility transistor integrated in a waveguide</t>
+        </is>
+      </c>
+      <c r="R826" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S826" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="T826" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-17T00:01Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T826"/>
+  <dimension ref="A1:T828"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62912,6 +62912,158 @@
       </c>
       <c r="T826" t="inlineStr"/>
     </row>
+    <row r="827">
+      <c r="A827" t="inlineStr"/>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Beyond monolithic rankings: a cluster-based framework for MSME ecosystem performance in India with policy corroboration evidence</t>
+        </is>
+      </c>
+      <c r="C827" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>Journal of Economic and Administrative Sciences</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>Mukherjee, Kasturi; Majumdar, Malini; Chattopadhyay, Ayan</t>
+        </is>
+      </c>
+      <c r="G827" t="inlineStr"/>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>10.1108/jeas-10-2025-0750</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/jeas-10-2025-0750</t>
+        </is>
+      </c>
+      <c r="J827" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K827" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L827" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M827" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N827" t="inlineStr"/>
+      <c r="O827" t="inlineStr"/>
+      <c r="P827" t="inlineStr"/>
+      <c r="Q827" t="inlineStr">
+        <is>
+          <t>Beyond monolithic rankings: a cluster-based framework for MSME ecosystem performance in India with policy corroboration evidence</t>
+        </is>
+      </c>
+      <c r="R827" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S827" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="T827" t="inlineStr"/>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr"/>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Si-implanted ohmic contacts with modulated pulse activation annealing for down-scaled RF GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C828" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>Bassal, Amer; Koyucuoglu, Ali; Thies, Andreas; Ostermay, Ina; Paul, Pallabi; Chevtchenko, Serguei; Hilt, Oliver</t>
+        </is>
+      </c>
+      <c r="G828" t="inlineStr"/>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>10.1063/5.0331948</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0331948</t>
+        </is>
+      </c>
+      <c r="J828" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K828" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L828" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M828" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N828" t="inlineStr"/>
+      <c r="O828" t="inlineStr"/>
+      <c r="P828" t="inlineStr"/>
+      <c r="Q828" t="inlineStr">
+        <is>
+          <t>Si-implanted ohmic contacts with modulated pulse activation annealing for down-scaled RF GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R828" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S828" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="T828" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-17T23:55Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T828"/>
+  <dimension ref="A1:T830"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63064,6 +63064,154 @@
       </c>
       <c r="T828" t="inlineStr"/>
     </row>
+    <row r="829">
+      <c r="A829" t="inlineStr"/>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Circuit logic of oxytocin and vasopressin complementary actions</t>
+        </is>
+      </c>
+      <c r="C829" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Frontiers Media SA</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>Frontiers in Neuroscience</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>Jeanneteau, Freddy; Chakraborty, Prabahan; Petitjean, Hugues; Charlet, Alexandre</t>
+        </is>
+      </c>
+      <c r="G829" t="inlineStr"/>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>10.3389/fnins.2026.1875731</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/fnins.2026.1875731</t>
+        </is>
+      </c>
+      <c r="J829" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K829" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L829" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M829" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N829" t="inlineStr"/>
+      <c r="O829" t="inlineStr"/>
+      <c r="P829" t="inlineStr"/>
+      <c r="Q829" t="inlineStr">
+        <is>
+          <t>Circuit logic of oxytocin and vasopressin complementary actions</t>
+        </is>
+      </c>
+      <c r="R829" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S829" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="T829" t="inlineStr"/>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr"/>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Many-body quantum percolation sustains ohmic proton flux through the nanoconfined Fo motor</t>
+        </is>
+      </c>
+      <c r="C830" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>openRxiv</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr"/>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>Adeniran, Ismail; Lightfoot, Adam P</t>
+        </is>
+      </c>
+      <c r="G830" t="inlineStr"/>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>10.64898/2026.07.15.738743</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.07.15.738743</t>
+        </is>
+      </c>
+      <c r="J830" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K830" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L830" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M830" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N830" t="inlineStr"/>
+      <c r="O830" t="inlineStr"/>
+      <c r="P830" t="inlineStr"/>
+      <c r="Q830" t="inlineStr">
+        <is>
+          <t>Many-body quantum percolation sustains ohmic proton flux through the nanoconfined Fo motor</t>
+        </is>
+      </c>
+      <c r="R830" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S830" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="T830" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-20T00:01Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T830"/>
+  <dimension ref="A1:T832"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63212,6 +63212,158 @@
       </c>
       <c r="T830" t="inlineStr"/>
     </row>
+    <row r="831">
+      <c r="A831" t="inlineStr"/>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Robostness of precast monolithic concrete frames under special impacts</t>
+        </is>
+      </c>
+      <c r="C831" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Orel State University</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Building and Reconstruction</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>Kaydas, P. A.</t>
+        </is>
+      </c>
+      <c r="G831" t="inlineStr"/>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>10.33979/2073-7416-2026-125-3-60-70</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.33979/2073-7416-2026-125-3-60-70</t>
+        </is>
+      </c>
+      <c r="J831" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K831" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L831" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M831" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N831" t="inlineStr"/>
+      <c r="O831" t="inlineStr"/>
+      <c r="P831" t="inlineStr"/>
+      <c r="Q831" t="inlineStr">
+        <is>
+          <t>Robostness of precast monolithic concrete frames under special impacts</t>
+        </is>
+      </c>
+      <c r="R831" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S831" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T831" t="inlineStr"/>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr"/>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Design and Optimization of AlGaN/GaN Graded Barrier MOS-HEMT Biosensor for Breast Cancer Biomolecule detection</t>
+        </is>
+      </c>
+      <c r="C832" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>Scientific Reports</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>Karumuri, Srinivasa Rao; Prasanna, Rudra Lakshmi; Sreenivasulu, Vakkalakula Bharath; Kondavitee, Girija Sravani</t>
+        </is>
+      </c>
+      <c r="G832" t="inlineStr"/>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-026-61687-0</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-026-61687-0</t>
+        </is>
+      </c>
+      <c r="J832" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K832" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L832" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M832" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N832" t="inlineStr"/>
+      <c r="O832" t="inlineStr"/>
+      <c r="P832" t="inlineStr"/>
+      <c r="Q832" t="inlineStr">
+        <is>
+          <t>Design and Optimization of AlGaN/GaN Graded Barrier MOS-HEMT Biosensor for Breast Cancer Biomolecule detection</t>
+        </is>
+      </c>
+      <c r="R832" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S832" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T832" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-20T23:58Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T832"/>
+  <dimension ref="A1:T843"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63364,6 +63364,842 @@
       </c>
       <c r="T832" t="inlineStr"/>
     </row>
+    <row r="833">
+      <c r="A833" t="inlineStr"/>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Seed-assisted polarity control of flexible WSe2 transistors and demonstration of CMOS inverter</t>
+        </is>
+      </c>
+      <c r="C833" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>npj Flexible Electronics</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>Phùng, Quỳnh Thị; Nguyen, Kha Minh; Park, Ji-Yong; Daus, Alwin</t>
+        </is>
+      </c>
+      <c r="G833" t="inlineStr"/>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>10.1038/s41528-026-00621-w</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41528-026-00621-w</t>
+        </is>
+      </c>
+      <c r="J833" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K833" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L833" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M833" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N833" t="inlineStr"/>
+      <c r="O833" t="inlineStr"/>
+      <c r="P833" t="inlineStr"/>
+      <c r="Q833" t="inlineStr">
+        <is>
+          <t>Seed-assisted polarity control of flexible WSe2 transistors and demonstration of CMOS inverter</t>
+        </is>
+      </c>
+      <c r="R833" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S833" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T833" t="inlineStr"/>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr"/>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Naturopathic Knowledge and Approaches to Managing Hidradenitis Suppurativa: A Cross-Sectional Survey of Australian Naturopaths</t>
+        </is>
+      </c>
+      <c r="C834" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>Hentschel, Norelle; Schloss, Janet</t>
+        </is>
+      </c>
+      <c r="G834" t="inlineStr"/>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261469650</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261469650</t>
+        </is>
+      </c>
+      <c r="J834" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K834" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L834" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M834" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N834" t="inlineStr"/>
+      <c r="O834" t="inlineStr"/>
+      <c r="P834" t="inlineStr"/>
+      <c r="Q834" t="inlineStr">
+        <is>
+          <t>Naturopathic Knowledge and Approaches to Managing Hidradenitis Suppurativa: A Cross-Sectional Survey of Australian Naturopaths</t>
+        </is>
+      </c>
+      <c r="R834" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S834" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T834" t="inlineStr"/>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr"/>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Terahertz spatial dispersive engineering via a monolithic core-antiresonant cavity</t>
+        </is>
+      </c>
+      <c r="C835" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Communications Physics</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>Zhao, Jiayu; Yuan, Linlin; Tian, Yifu; Mei, Yangjun; Yang, Jiajun; Lao, Li; Peng, Yan; Zhu, Yiming; Zhuang, Songlin</t>
+        </is>
+      </c>
+      <c r="G835" t="inlineStr"/>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>10.1038/s42005-026-02776-4</t>
+        </is>
+      </c>
+      <c r="I835" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s42005-026-02776-4</t>
+        </is>
+      </c>
+      <c r="J835" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K835" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L835" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M835" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N835" t="inlineStr"/>
+      <c r="O835" t="inlineStr"/>
+      <c r="P835" t="inlineStr"/>
+      <c r="Q835" t="inlineStr">
+        <is>
+          <t>Terahertz spatial dispersive engineering via a monolithic core-antiresonant cavity</t>
+        </is>
+      </c>
+      <c r="R835" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S835" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T835" t="inlineStr"/>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr"/>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Naturopathic Knowledge and Approaches to Managing Hidradenitis Suppurativa: A Cross-Sectional Survey of Australian Naturopaths</t>
+        </is>
+      </c>
+      <c r="C836" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>Hentschel, Norelle; Schloss, Janet</t>
+        </is>
+      </c>
+      <c r="G836" t="inlineStr"/>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261469650</t>
+        </is>
+      </c>
+      <c r="I836" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261469650</t>
+        </is>
+      </c>
+      <c r="J836" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K836" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L836" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M836" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N836" t="inlineStr"/>
+      <c r="O836" t="inlineStr"/>
+      <c r="P836" t="inlineStr"/>
+      <c r="Q836" t="inlineStr">
+        <is>
+          <t>Naturopathic Knowledge and Approaches to Managing Hidradenitis Suppurativa: A Cross-Sectional Survey of Australian Naturopaths</t>
+        </is>
+      </c>
+      <c r="R836" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S836" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T836" t="inlineStr"/>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr"/>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="C837" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>Cui, Jiawei; Xu, Yuanyang; Fu, Xingyu; Chen, Zhenghao; Liu, Sihang; Qi, Hengyuan; Yang, Han; Yang, Junjie; Wang, Maojun; Yang, Xuelin; Shen, Bo; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G837" t="inlineStr"/>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="J837" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K837" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L837" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M837" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N837" t="inlineStr"/>
+      <c r="O837" t="inlineStr"/>
+      <c r="P837" t="inlineStr"/>
+      <c r="Q837" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="R837" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S837" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T837" t="inlineStr"/>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr"/>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="C838" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>Cui, Jiawei; Xu, Yuanyang; Fu, Xingyu; Chen, Zhenghao; Liu, Sihang; Qi, Hengyuan; Yang, Han; Yang, Junjie; Wang, Maojun; Yang, Xuelin; Shen, Bo; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G838" t="inlineStr"/>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="I838" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="J838" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K838" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L838" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M838" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N838" t="inlineStr"/>
+      <c r="O838" t="inlineStr"/>
+      <c r="P838" t="inlineStr"/>
+      <c r="Q838" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="R838" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S838" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T838" t="inlineStr"/>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr"/>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="C839" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>Cui, Jiawei; Xu, Yuanyang; Fu, Xingyu; Chen, Zhenghao; Liu, Sihang; Qi, Hengyuan; Yang, Han; Yang, Junjie; Wang, Maojun; Yang, Xuelin; Shen, Bo; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G839" t="inlineStr"/>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="I839" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="J839" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K839" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L839" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M839" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N839" t="inlineStr"/>
+      <c r="O839" t="inlineStr"/>
+      <c r="P839" t="inlineStr"/>
+      <c r="Q839" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="R839" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S839" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T839" t="inlineStr"/>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr"/>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="C840" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>Cui, Jiawei; Xu, Yuanyang; Fu, Xingyu; Chen, Zhenghao; Liu, Sihang; Qi, Hengyuan; Yang, Han; Yang, Junjie; Wang, Maojun; Yang, Xuelin; Shen, Bo; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G840" t="inlineStr"/>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="I840" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="J840" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K840" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L840" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M840" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N840" t="inlineStr"/>
+      <c r="O840" t="inlineStr"/>
+      <c r="P840" t="inlineStr"/>
+      <c r="Q840" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="R840" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S840" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T840" t="inlineStr"/>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr"/>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Enhancing Phishing Website Detection Using Artificial Neural Network with Logic Gate-Based Feature Interaction Modeling</t>
+        </is>
+      </c>
+      <c r="C841" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>Fakultas Sains dan Teknologi, Unira Malang</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>G-Tech: Jurnal Teknologi Terapan</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>Rahman, M. Halvi; Abidin, Zainal; Hariyadi, M. Amin</t>
+        </is>
+      </c>
+      <c r="G841" t="inlineStr"/>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>10.70609/g-tech.v10i3.10280</t>
+        </is>
+      </c>
+      <c r="I841" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.70609/g-tech.v10i3.10280</t>
+        </is>
+      </c>
+      <c r="J841" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K841" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L841" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M841" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N841" t="inlineStr"/>
+      <c r="O841" t="inlineStr"/>
+      <c r="P841" t="inlineStr"/>
+      <c r="Q841" t="inlineStr">
+        <is>
+          <t>Enhancing Phishing Website Detection Using Artificial Neural Network with Logic Gate-Based Feature Interaction Modeling</t>
+        </is>
+      </c>
+      <c r="R841" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S841" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T841" t="inlineStr"/>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr"/>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="C842" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>Cui, Jiawei; Xu, Yuanyang; Fu, Xingyu; Chen, Zhenghao; Liu, Sihang; Qi, Hengyuan; Yang, Han; Yang, Junjie; Wang, Maojun; Yang, Xuelin; Shen, Bo; Wei, Jin</t>
+        </is>
+      </c>
+      <c r="G842" t="inlineStr"/>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="I842" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0333796</t>
+        </is>
+      </c>
+      <c r="J842" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K842" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L842" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M842" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N842" t="inlineStr"/>
+      <c r="O842" t="inlineStr"/>
+      <c r="P842" t="inlineStr"/>
+      <c r="Q842" t="inlineStr">
+        <is>
+          <t>Achieving low ON-resistance in E-mode regrown U-shaped p-GaN gate multi-channel HEMT</t>
+        </is>
+      </c>
+      <c r="R842" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S842" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T842" t="inlineStr"/>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr"/>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Investigation of hot electrons in polarization-graded AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C843" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>Raychaudhuri, Jagori; Pomeroy, James W.; Anjali, Anjali; Smith, Matthew D.; Jeng, Yu-En; Fay, Patrick; Kuball, Martin</t>
+        </is>
+      </c>
+      <c r="G843" t="inlineStr"/>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>10.1063/5.0326723</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0326723</t>
+        </is>
+      </c>
+      <c r="J843" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K843" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L843" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M843" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="N843" t="inlineStr"/>
+      <c r="O843" t="inlineStr"/>
+      <c r="P843" t="inlineStr"/>
+      <c r="Q843" t="inlineStr">
+        <is>
+          <t>Investigation of hot electrons in polarization-graded AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R843" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S843" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="T843" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-21T23:58Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T843"/>
+  <dimension ref="A1:T845"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64200,6 +64200,170 @@
       </c>
       <c r="T843" t="inlineStr"/>
     </row>
+    <row r="844">
+      <c r="A844" t="inlineStr"/>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Smart Weave Revolution: Monolithic Fiber-Integrated Circuits for Next-Generation Intelligence</t>
+        </is>
+      </c>
+      <c r="C844" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>International Journal of Extreme Manufacturing</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>Xiong, Yao; Cho, Jeong Ho; Sun, Qijun</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr"/>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>10.1088/2631-7990/ae8e0c</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-7990/ae8e0c</t>
+        </is>
+      </c>
+      <c r="J844" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K844" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L844" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M844" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N844" t="inlineStr"/>
+      <c r="O844" t="inlineStr"/>
+      <c r="P844" t="inlineStr"/>
+      <c r="Q844" t="inlineStr">
+        <is>
+          <t>Smart Weave Revolution: Monolithic Fiber-Integrated Circuits for Next-Generation Intelligence</t>
+        </is>
+      </c>
+      <c r="R844" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S844" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="T844" t="inlineStr"/>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr"/>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Low-Temperature Monolithic Integration of a Polycrystalline Silicon Ferroelectric-Gate Field-Effect Transistor with Microwave-Annealed HfZrO
+                    &lt;sub&gt;
+                      &lt;sub&gt;
+                        &lt;i&gt;x&lt;/i&gt;
+                      &lt;/sub&gt;
+                    &lt;/sub&gt;
+                    for Energy-Efficient Neuromorphic Computing</t>
+        </is>
+      </c>
+      <c r="C845" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>ACS Materials Letters</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>Kim, Sang Woo; Kwak, Been; Kim, Hyun-Min; Kwak, Sangeun; Kwon, Daewoong</t>
+        </is>
+      </c>
+      <c r="G845" t="inlineStr"/>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>10.1021/acsmaterialslett.5c01261</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsmaterialslett.5c01261</t>
+        </is>
+      </c>
+      <c r="J845" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K845" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L845" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M845" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N845" t="inlineStr"/>
+      <c r="O845" t="inlineStr"/>
+      <c r="P845" t="inlineStr"/>
+      <c r="Q845" t="inlineStr">
+        <is>
+          <t>Low-Temperature Monolithic Integration of a Polycrystalline Silicon Ferroelectric-Gate Field-Effect Transistor with Microwave-Annealed HfZrO
+                    &lt;sub&gt;
+                      &lt;sub&gt;
+                        &lt;i&gt;x&lt;/i&gt;
+                      &lt;/sub&gt;
+                    &lt;/sub&gt;
+                    for Energy-Efficient Neuromorphic Computing</t>
+        </is>
+      </c>
+      <c r="R845" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S845" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="T845" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-23T00:02Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T845"/>
+  <dimension ref="A1:T846"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64364,6 +64364,82 @@
       </c>
       <c r="T845" t="inlineStr"/>
     </row>
+    <row r="846">
+      <c r="A846" t="inlineStr"/>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Awareness and attitudes toward traditional and complementary medicine among community-dwelling individuals in Türkiye: a cross-sectional online survey</t>
+        </is>
+      </c>
+      <c r="C846" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>BMC Complementary Medicine and Therapies</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>Süzer, Akın; Yenil-Kocabay, Sinem; Ünal-Süzer, Nevriye; Büker, Nihal</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr"/>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>10.1186/s12906-026-05480-6</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s12906-026-05480-6</t>
+        </is>
+      </c>
+      <c r="J846" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K846" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L846" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M846" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N846" t="inlineStr"/>
+      <c r="O846" t="inlineStr"/>
+      <c r="P846" t="inlineStr"/>
+      <c r="Q846" t="inlineStr">
+        <is>
+          <t>Awareness and attitudes toward traditional and complementary medicine among community-dwelling individuals in Türkiye: a cross-sectional online survey</t>
+        </is>
+      </c>
+      <c r="R846" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S846" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="T846" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-24T00:04Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T846"/>
+  <dimension ref="A1:T848"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64440,6 +64440,158 @@
       </c>
       <c r="T846" t="inlineStr"/>
     </row>
+    <row r="847">
+      <c r="A847" t="inlineStr"/>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Temperature and Bias Dependence of the DC and RF Characteristics of a 150 nm AlGaN/GaN-on-SiC HEMT for Microwave Applications</t>
+        </is>
+      </c>
+      <c r="C847" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>Alim, Mohammad Abdul; Gaquiere, Christophe</t>
+        </is>
+      </c>
+      <c r="G847" t="inlineStr"/>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>10.3390/mi17080874</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17080874</t>
+        </is>
+      </c>
+      <c r="J847" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K847" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L847" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M847" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N847" t="inlineStr"/>
+      <c r="O847" t="inlineStr"/>
+      <c r="P847" t="inlineStr"/>
+      <c r="Q847" t="inlineStr">
+        <is>
+          <t>Temperature and Bias Dependence of the DC and RF Characteristics of a 150 nm AlGaN/GaN-on-SiC HEMT for Microwave Applications</t>
+        </is>
+      </c>
+      <c r="R847" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S847" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="T847" t="inlineStr"/>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr"/>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>CMOS-Compatible AlScN Memristor on Silicon Exhibiting Short-Term Memory for Reservoir Computing</t>
+        </is>
+      </c>
+      <c r="C848" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Biomimetics</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>Park, Woohyun; Chae, Hyojeong; Rasheed, Maria; Kim, Sungjun</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr"/>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>10.3390/biomimetics11080519</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/biomimetics11080519</t>
+        </is>
+      </c>
+      <c r="J848" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K848" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L848" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M848" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N848" t="inlineStr"/>
+      <c r="O848" t="inlineStr"/>
+      <c r="P848" t="inlineStr"/>
+      <c r="Q848" t="inlineStr">
+        <is>
+          <t>CMOS-Compatible AlScN Memristor on Silicon Exhibiting Short-Term Memory for Reservoir Computing</t>
+        </is>
+      </c>
+      <c r="R848" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S848" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="T848" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-25T00:06Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T848"/>
+  <dimension ref="A1:T855"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64592,6 +64592,522 @@
       </c>
       <c r="T848" t="inlineStr"/>
     </row>
+    <row r="849">
+      <c r="A849" t="inlineStr"/>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD Investigation of RF Performance, Noise Characteristics, and Intrinsic Capacitances of InAlAs/InGaAs/InP HEMTs: Impact of Gate-to-Channel Distance and Gate Bias.</t>
+        </is>
+      </c>
+      <c r="C849" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr"/>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>Derrouiche, Soufiane</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr"/>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10451190/v1</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10451190/v1</t>
+        </is>
+      </c>
+      <c r="J849" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K849" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L849" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M849" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N849" t="inlineStr"/>
+      <c r="O849" t="inlineStr"/>
+      <c r="P849" t="inlineStr"/>
+      <c r="Q849" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD Investigation of RF Performance, Noise Characteristics, and Intrinsic Capacitances of InAlAs/InGaAs/InP HEMTs: Impact of Gate-to-Channel Distance and Gate Bias.</t>
+        </is>
+      </c>
+      <c r="R849" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S849" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="T849" t="inlineStr"/>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr"/>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD Investigation of RF Performance, Noise Characteristics, and Intrinsic Capacitances of InAlAs/InGaAs/InP HEMTs: Impact of Gate-to-Channel Distance and Gate Bias.</t>
+        </is>
+      </c>
+      <c r="C850" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr"/>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>Derrouiche, Soufiane</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr"/>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10451190/v1</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10451190/v1</t>
+        </is>
+      </c>
+      <c r="J850" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K850" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L850" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M850" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N850" t="inlineStr"/>
+      <c r="O850" t="inlineStr"/>
+      <c r="P850" t="inlineStr"/>
+      <c r="Q850" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD Investigation of RF Performance, Noise Characteristics, and Intrinsic Capacitances of InAlAs/InGaAs/InP HEMTs: Impact of Gate-to-Channel Distance and Gate Bias.</t>
+        </is>
+      </c>
+      <c r="R850" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S850" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="T850" t="inlineStr"/>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr"/>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD Investigation of RF Performance, Noise Characteristics, and Intrinsic Capacitances of InAlAs/InGaAs/InP HEMTs: Impact of Gate-to-Channel Distance and Gate Bias.</t>
+        </is>
+      </c>
+      <c r="C851" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr"/>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>Derrouiche, Soufiane</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr"/>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10451190/v1</t>
+        </is>
+      </c>
+      <c r="I851" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10451190/v1</t>
+        </is>
+      </c>
+      <c r="J851" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K851" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L851" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M851" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N851" t="inlineStr"/>
+      <c r="O851" t="inlineStr"/>
+      <c r="P851" t="inlineStr"/>
+      <c r="Q851" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD Investigation of RF Performance, Noise Characteristics, and Intrinsic Capacitances of InAlAs/InGaAs/InP HEMTs: Impact of Gate-to-Channel Distance and Gate Bias.</t>
+        </is>
+      </c>
+      <c r="R851" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S851" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="T851" t="inlineStr"/>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr"/>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Image encryption based on Tetris puzzle game and a ring oscillator coupled with a Van der Pol oscillator</t>
+        </is>
+      </c>
+      <c r="C852" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>Walter de Gruyter GmbH</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Zeitschrift für Naturforschung A</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>Takotue, Jean Ernest; Atchoffo, William Nodem; Kengne, Romanic; Tchiotsop, Daniel; Talla Mbé, Jimmi Hervé</t>
+        </is>
+      </c>
+      <c r="G852" t="inlineStr"/>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>10.1515/zna-2026-0107</t>
+        </is>
+      </c>
+      <c r="I852" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1515/zna-2026-0107</t>
+        </is>
+      </c>
+      <c r="J852" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K852" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L852" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M852" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N852" t="inlineStr"/>
+      <c r="O852" t="inlineStr"/>
+      <c r="P852" t="inlineStr"/>
+      <c r="Q852" t="inlineStr">
+        <is>
+          <t>Image encryption based on Tetris puzzle game and a ring oscillator coupled with a Van der Pol oscillator</t>
+        </is>
+      </c>
+      <c r="R852" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S852" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="T852" t="inlineStr"/>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr"/>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Co‐Localization‐Gated Multivalent DNA Logic Gate for Programmable Cell Recognition</t>
+        </is>
+      </c>
+      <c r="C853" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Angewandte Chemie</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>Mao, Miao; Yang, Yingxin; Chen, Yitong; Chen, Xi; Dou, Quanhao; Shui, Lingling; Zhang, Yuanqing</t>
+        </is>
+      </c>
+      <c r="G853" t="inlineStr"/>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>10.1002/ange.5650963</t>
+        </is>
+      </c>
+      <c r="I853" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/ange.5650963</t>
+        </is>
+      </c>
+      <c r="J853" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K853" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L853" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M853" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N853" t="inlineStr"/>
+      <c r="O853" t="inlineStr"/>
+      <c r="P853" t="inlineStr"/>
+      <c r="Q853" t="inlineStr">
+        <is>
+          <t>Co‐Localization‐Gated Multivalent DNA Logic Gate for Programmable Cell Recognition</t>
+        </is>
+      </c>
+      <c r="R853" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S853" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="T853" t="inlineStr"/>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr"/>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Co‐Localization‐Gated Multivalent DNA Logic Gate for Programmable Cell Recognition</t>
+        </is>
+      </c>
+      <c r="C854" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Angewandte Chemie International Edition</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>Mao, Miao; Yang, Yingxin; Chen, Yitong; Chen, Xi; Dou, Quanhao; Shui, Lingling; Zhang, Yuanqing</t>
+        </is>
+      </c>
+      <c r="G854" t="inlineStr"/>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>10.1002/anie.5650963</t>
+        </is>
+      </c>
+      <c r="I854" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/anie.5650963</t>
+        </is>
+      </c>
+      <c r="J854" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K854" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L854" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M854" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N854" t="inlineStr"/>
+      <c r="O854" t="inlineStr"/>
+      <c r="P854" t="inlineStr"/>
+      <c r="Q854" t="inlineStr">
+        <is>
+          <t>Co‐Localization‐Gated Multivalent DNA Logic Gate for Programmable Cell Recognition</t>
+        </is>
+      </c>
+      <c r="R854" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S854" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="T854" t="inlineStr"/>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr"/>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD Investigation of RF Performance, Noise Characteristics, and Intrinsic Capacitances of InAlAs/InGaAs/InP HEMTs: Impact of Gate-to-Channel Distance and Gate Bias.</t>
+        </is>
+      </c>
+      <c r="C855" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr"/>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>Derrouiche, Soufiane</t>
+        </is>
+      </c>
+      <c r="G855" t="inlineStr"/>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10451190/v1</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10451190/v1</t>
+        </is>
+      </c>
+      <c r="J855" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K855" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L855" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M855" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N855" t="inlineStr"/>
+      <c r="O855" t="inlineStr"/>
+      <c r="P855" t="inlineStr"/>
+      <c r="Q855" t="inlineStr">
+        <is>
+          <t>Comprehensive TCAD Investigation of RF Performance, Noise Characteristics, and Intrinsic Capacitances of InAlAs/InGaAs/InP HEMTs: Impact of Gate-to-Channel Distance and Gate Bias.</t>
+        </is>
+      </c>
+      <c r="R855" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S855" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="T855" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-28T00:05Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T855"/>
+  <dimension ref="A1:T860"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65108,6 +65108,378 @@
       </c>
       <c r="T855" t="inlineStr"/>
     </row>
+    <row r="856">
+      <c r="A856" t="inlineStr"/>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Monolithic Multifocal Diamond Metalens for High-Power Laser Systems</t>
+        </is>
+      </c>
+      <c r="C856" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr"/>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>Qiu, Min; Li, Xiaoxuan; Sun, Xiaoyu; Li, Ce; Xie, Zhiqiang; Liu, Fengjiang; Chen, Boqu; Zhao, Ding; Du, Kaikai</t>
+        </is>
+      </c>
+      <c r="G856" t="inlineStr"/>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10316543/v1</t>
+        </is>
+      </c>
+      <c r="I856" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10316543/v1</t>
+        </is>
+      </c>
+      <c r="J856" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K856" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L856" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M856" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N856" t="inlineStr"/>
+      <c r="O856" t="inlineStr"/>
+      <c r="P856" t="inlineStr"/>
+      <c r="Q856" t="inlineStr">
+        <is>
+          <t>Monolithic Multifocal Diamond Metalens for High-Power Laser Systems</t>
+        </is>
+      </c>
+      <c r="R856" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S856" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="T856" t="inlineStr"/>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr"/>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Effect of Different Surface Treatment Protocols on Surface Roughness, Topography, Composition, Shear Bond Strength, and Failure Mode of Monolithic Translucent Multi-Layered Zirconia</t>
+        </is>
+      </c>
+      <c r="C857" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr"/>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>Abdulgader, Areej; Shono, Nourah; AlNahedh, Hend</t>
+        </is>
+      </c>
+      <c r="G857" t="inlineStr"/>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10348986/v1</t>
+        </is>
+      </c>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10348986/v1</t>
+        </is>
+      </c>
+      <c r="J857" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K857" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L857" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M857" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N857" t="inlineStr"/>
+      <c r="O857" t="inlineStr"/>
+      <c r="P857" t="inlineStr"/>
+      <c r="Q857" t="inlineStr">
+        <is>
+          <t>Effect of Different Surface Treatment Protocols on Surface Roughness, Topography, Composition, Shear Bond Strength, and Failure Mode of Monolithic Translucent Multi-Layered Zirconia</t>
+        </is>
+      </c>
+      <c r="R857" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S857" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="T857" t="inlineStr"/>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr"/>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Flexible AlGaN/GaN HEMT devices exfoliated from Si substrate by electrochemical etching</t>
+        </is>
+      </c>
+      <c r="C858" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>Xu, Chenxi; Ye, Lei; Wang, Haodong; Feng, Meixin; Zhang, Shuming; Sun, Qian; Yang, Hui</t>
+        </is>
+      </c>
+      <c r="G858" t="inlineStr"/>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae90bb</t>
+        </is>
+      </c>
+      <c r="I858" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae90bb</t>
+        </is>
+      </c>
+      <c r="J858" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K858" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L858" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M858" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N858" t="inlineStr"/>
+      <c r="O858" t="inlineStr"/>
+      <c r="P858" t="inlineStr"/>
+      <c r="Q858" t="inlineStr">
+        <is>
+          <t>Flexible AlGaN/GaN HEMT devices exfoliated from Si substrate by electrochemical etching</t>
+        </is>
+      </c>
+      <c r="R858" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S858" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="T858" t="inlineStr"/>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr"/>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Design Parameter Optimization of FPGA-based Ring Oscillator TRNG and Its Application to P-bit Inverse Computation System</t>
+        </is>
+      </c>
+      <c r="C859" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>The Institute of Electronics Engineers of Korea</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>Journal of the Institute of Electronics and Information Engineers</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>Jang, Jaeyong; Ji, Changhun; Lee, Chanwook; Ishdorj, Bayartulga; Na, Taehui</t>
+        </is>
+      </c>
+      <c r="G859" t="inlineStr"/>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>10.5573/ieie.2026.63.7.36</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5573/ieie.2026.63.7.36</t>
+        </is>
+      </c>
+      <c r="J859" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K859" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L859" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M859" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N859" t="inlineStr"/>
+      <c r="O859" t="inlineStr"/>
+      <c r="P859" t="inlineStr"/>
+      <c r="Q859" t="inlineStr">
+        <is>
+          <t>Design Parameter Optimization of FPGA-based Ring Oscillator TRNG and Its Application to P-bit Inverse Computation System</t>
+        </is>
+      </c>
+      <c r="R859" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S859" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="T859" t="inlineStr"/>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr"/>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Double-Layer Sandwich Metasurface for Mid-Infrared Multi-Channel Polarization Detection</t>
+        </is>
+      </c>
+      <c r="C860" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Photonics</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>Ma, Lifeng; Huang, Yi; Zheng, Ting; Chang, Jun; Jiang, Huilin</t>
+        </is>
+      </c>
+      <c r="G860" t="inlineStr"/>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>10.3390/photonics13080708</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/photonics13080708</t>
+        </is>
+      </c>
+      <c r="J860" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K860" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L860" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M860" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N860" t="inlineStr"/>
+      <c r="O860" t="inlineStr"/>
+      <c r="P860" t="inlineStr"/>
+      <c r="Q860" t="inlineStr">
+        <is>
+          <t>Double-Layer Sandwich Metasurface for Mid-Infrared Multi-Channel Polarization Detection</t>
+        </is>
+      </c>
+      <c r="R860" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S860" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="T860" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-29T00:00Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T860"/>
+  <dimension ref="A1:T862"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65480,6 +65480,166 @@
       </c>
       <c r="T860" t="inlineStr"/>
     </row>
+    <row r="861">
+      <c r="A861" t="inlineStr"/>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>An Overload-Capability Enhancement Technique Leveraging Hybrid Frequency Modulation and Triple-Phase Shift Control for Single-Stage AC–DC Monolithic Bidirectional GaN DAB Converters</t>
+        </is>
+      </c>
+      <c r="C861" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Power Electronics</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>Gong, Linxiao; Zhou, Kehui; Lv, Wei; Wang, Minqian; Nie, Mingzhi; Li, Yuxuan; Xu, Junzhong; Wang, Yong</t>
+        </is>
+      </c>
+      <c r="G861" t="inlineStr"/>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>10.1109/tpel.2026.3692530</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tpel.2026.3692530</t>
+        </is>
+      </c>
+      <c r="J861" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K861" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L861" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M861" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N861" t="inlineStr"/>
+      <c r="O861" t="inlineStr"/>
+      <c r="P861" t="inlineStr"/>
+      <c r="Q861" t="inlineStr">
+        <is>
+          <t>An Overload-Capability Enhancement Technique Leveraging Hybrid Frequency Modulation and Triple-Phase Shift Control for Single-Stage AC–DC Monolithic Bidirectional GaN DAB Converters</t>
+        </is>
+      </c>
+      <c r="R861" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S861" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="T861" t="inlineStr"/>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr"/>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Power Gain-Stable AlN/GaN MIS-HEMTs With Pulsed N
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    Plasma-Treated In-Situ SiN
+                    &lt;sub&gt;x&lt;/sub&gt;
+                    Gate Dielectric</t>
+        </is>
+      </c>
+      <c r="C862" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>Zhang, Qingyi; Wei, Ke; Wang, Jianchao; Zhang, Sheng; Wang, Kaiyu; Guo, Jiaqi; He, Xiaoqiang; Ma, Zhuanli; Feng, Junjie; Fan, Shibo; Gao, Xinguo; Li, Yankui</t>
+        </is>
+      </c>
+      <c r="G862" t="inlineStr"/>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3703504</t>
+        </is>
+      </c>
+      <c r="I862" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3703504</t>
+        </is>
+      </c>
+      <c r="J862" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K862" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L862" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M862" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N862" t="inlineStr"/>
+      <c r="O862" t="inlineStr"/>
+      <c r="P862" t="inlineStr"/>
+      <c r="Q862" t="inlineStr">
+        <is>
+          <t>Power Gain-Stable AlN/GaN MIS-HEMTs With Pulsed N
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    Plasma-Treated In-Situ SiN
+                    &lt;sub&gt;x&lt;/sub&gt;
+                    Gate Dielectric</t>
+        </is>
+      </c>
+      <c r="R862" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S862" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="T862" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-07-30T00:02Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T862"/>
+  <dimension ref="A1:T868"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65640,6 +65640,458 @@
       </c>
       <c r="T862" t="inlineStr"/>
     </row>
+    <row r="863">
+      <c r="A863" t="inlineStr"/>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Complementary Indicators of Knowledge Purporting and Their Validity</t>
+        </is>
+      </c>
+      <c r="C863" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>Center for Open Science</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr"/>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>Goecke, Benjamin; Schittenhelm, Catherine; Wilhelm, Oliver</t>
+        </is>
+      </c>
+      <c r="G863" t="inlineStr"/>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>10.31234/osf.io/zgqu7_v5</t>
+        </is>
+      </c>
+      <c r="I863" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.31234/osf.io/zgqu7_v5</t>
+        </is>
+      </c>
+      <c r="J863" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K863" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L863" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M863" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N863" t="inlineStr"/>
+      <c r="O863" t="inlineStr"/>
+      <c r="P863" t="inlineStr"/>
+      <c r="Q863" t="inlineStr">
+        <is>
+          <t>Complementary Indicators of Knowledge Purporting and Their Validity</t>
+        </is>
+      </c>
+      <c r="R863" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S863" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="T863" t="inlineStr"/>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr"/>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>3D simulation study of decoupled dual-gate p-GaN power HEMT with high forward threshold voltage and low reverse conduction loss</t>
+        </is>
+      </c>
+      <c r="C864" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Hu, Jinwei; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G864" t="inlineStr"/>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9211</t>
+        </is>
+      </c>
+      <c r="I864" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9211</t>
+        </is>
+      </c>
+      <c r="J864" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K864" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L864" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M864" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N864" t="inlineStr"/>
+      <c r="O864" t="inlineStr"/>
+      <c r="P864" t="inlineStr"/>
+      <c r="Q864" t="inlineStr">
+        <is>
+          <t>3D simulation study of decoupled dual-gate p-GaN power HEMT with high forward threshold voltage and low reverse conduction loss</t>
+        </is>
+      </c>
+      <c r="R864" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S864" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="T864" t="inlineStr"/>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr"/>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Experimental demonstration of reverse blocking with dual-gate H-diamond MOSFET at low voltage</t>
+        </is>
+      </c>
+      <c r="C865" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>Yue, Xinyu; Ren, Zeyang; Fu, Yu; Xu, Qihui; Zhang, Jinfeng; Chen, Junfei; Zhang, Jing; Su, Kai; Hao, Yue; Zhang, Jincheng</t>
+        </is>
+      </c>
+      <c r="G865" t="inlineStr"/>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae91f4</t>
+        </is>
+      </c>
+      <c r="I865" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae91f4</t>
+        </is>
+      </c>
+      <c r="J865" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K865" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L865" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M865" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N865" t="inlineStr"/>
+      <c r="O865" t="inlineStr"/>
+      <c r="P865" t="inlineStr"/>
+      <c r="Q865" t="inlineStr">
+        <is>
+          <t>Experimental demonstration of reverse blocking with dual-gate H-diamond MOSFET at low voltage</t>
+        </is>
+      </c>
+      <c r="R865" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S865" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="T865" t="inlineStr"/>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr"/>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>3D simulation study of decoupled dual-gate p-GaN power HEMT with high forward threshold voltage and low reverse conduction loss</t>
+        </is>
+      </c>
+      <c r="C866" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Hu, Jinwei; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G866" t="inlineStr"/>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9211</t>
+        </is>
+      </c>
+      <c r="I866" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9211</t>
+        </is>
+      </c>
+      <c r="J866" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K866" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L866" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M866" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N866" t="inlineStr"/>
+      <c r="O866" t="inlineStr"/>
+      <c r="P866" t="inlineStr"/>
+      <c r="Q866" t="inlineStr">
+        <is>
+          <t>3D simulation study of decoupled dual-gate p-GaN power HEMT with high forward threshold voltage and low reverse conduction loss</t>
+        </is>
+      </c>
+      <c r="R866" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S866" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="T866" t="inlineStr"/>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr"/>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Single-frequency 1116 nm laser based on a monolithic nonplanar ring oscillator and reflective volume Bragg grating</t>
+        </is>
+      </c>
+      <c r="C867" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Optica Publishing Group</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Optics Express</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>Zhang, Zhiheng; Xu, Zhen; Yang, Suhui; Li, Jing; Ye, Qing; Hou, Yanzuo; Li, Chaofeng; Feng, Yiming; Luo, Yijia; Wu, Nuocen; Gong, Yifan</t>
+        </is>
+      </c>
+      <c r="G867" t="inlineStr"/>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>10.1364/oe.607750</t>
+        </is>
+      </c>
+      <c r="I867" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1364/oe.607750</t>
+        </is>
+      </c>
+      <c r="J867" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K867" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L867" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M867" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N867" t="inlineStr"/>
+      <c r="O867" t="inlineStr"/>
+      <c r="P867" t="inlineStr"/>
+      <c r="Q867" t="inlineStr">
+        <is>
+          <t>Single-frequency 1116 nm laser based on a monolithic nonplanar ring oscillator and reflective volume Bragg grating</t>
+        </is>
+      </c>
+      <c r="R867" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S867" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="T867" t="inlineStr"/>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr"/>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>3D simulation study of decoupled dual-gate p-GaN power HEMT with high forward threshold voltage and low reverse conduction loss</t>
+        </is>
+      </c>
+      <c r="C868" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Hu, Jinwei; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G868" t="inlineStr"/>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9211</t>
+        </is>
+      </c>
+      <c r="I868" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9211</t>
+        </is>
+      </c>
+      <c r="J868" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K868" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L868" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M868" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N868" t="inlineStr"/>
+      <c r="O868" t="inlineStr"/>
+      <c r="P868" t="inlineStr"/>
+      <c r="Q868" t="inlineStr">
+        <is>
+          <t>3D simulation study of decoupled dual-gate p-GaN power HEMT with high forward threshold voltage and low reverse conduction loss</t>
+        </is>
+      </c>
+      <c r="R868" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S868" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="T868" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-01T00:04Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T868"/>
+  <dimension ref="A1:T872"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66092,6 +66092,306 @@
       </c>
       <c r="T868" t="inlineStr"/>
     </row>
+    <row r="869">
+      <c r="A869" t="inlineStr"/>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Scalable Biomimetic Solar Evaporators Via Monolithic 3D Printing of Magnetic-Fluid Photocurable Composites</t>
+        </is>
+      </c>
+      <c r="C869" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr"/>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>Rao, Longshi; Liu, Jiaying; Huo, Xiang; Liu, Yang; Tang, Junsong; Xie, Shu; Liu, Qingxian; Zhong, Guisheng; Yu, shudong</t>
+        </is>
+      </c>
+      <c r="G869" t="inlineStr"/>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>10.22541/authorea.15006827/v1</t>
+        </is>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22541/authorea.15006827/v1</t>
+        </is>
+      </c>
+      <c r="J869" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K869" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L869" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M869" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N869" t="inlineStr"/>
+      <c r="O869" t="inlineStr"/>
+      <c r="P869" t="inlineStr"/>
+      <c r="Q869" t="inlineStr">
+        <is>
+          <t>Scalable Biomimetic Solar Evaporators Via Monolithic 3D Printing of Magnetic-Fluid Photocurable Composites</t>
+        </is>
+      </c>
+      <c r="R869" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S869" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="T869" t="inlineStr"/>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr"/>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Simulations of p‐Channel GaN‐Based Metal‐Oxide‐Semiconductor Heterostructure Field‐Effect Transistors for Normally Off Operation</t>
+        </is>
+      </c>
+      <c r="C870" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>Ubochi, Brendan; Ahmeda, Khaled; Benbakhti, Brahim; Kalna, Karol</t>
+        </is>
+      </c>
+      <c r="G870" t="inlineStr"/>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.70448</t>
+        </is>
+      </c>
+      <c r="I870" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.70448</t>
+        </is>
+      </c>
+      <c r="J870" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K870" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L870" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M870" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N870" t="inlineStr"/>
+      <c r="O870" t="inlineStr"/>
+      <c r="P870" t="inlineStr"/>
+      <c r="Q870" t="inlineStr">
+        <is>
+          <t>Simulations of p‐Channel GaN‐Based Metal‐Oxide‐Semiconductor Heterostructure Field‐Effect Transistors for Normally Off Operation</t>
+        </is>
+      </c>
+      <c r="R870" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S870" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="T870" t="inlineStr"/>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr"/>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Simulations of p‐Channel GaN‐Based Metal‐Oxide‐Semiconductor Heterostructure Field‐Effect Transistors for Normally Off Operation</t>
+        </is>
+      </c>
+      <c r="C871" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>Ubochi, Brendan; Ahmeda, Khaled; Benbakhti, Brahim; Kalna, Karol</t>
+        </is>
+      </c>
+      <c r="G871" t="inlineStr"/>
+      <c r="H871" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.70448</t>
+        </is>
+      </c>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.70448</t>
+        </is>
+      </c>
+      <c r="J871" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K871" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L871" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M871" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N871" t="inlineStr"/>
+      <c r="O871" t="inlineStr"/>
+      <c r="P871" t="inlineStr"/>
+      <c r="Q871" t="inlineStr">
+        <is>
+          <t>Simulations of p‐Channel GaN‐Based Metal‐Oxide‐Semiconductor Heterostructure Field‐Effect Transistors for Normally Off Operation</t>
+        </is>
+      </c>
+      <c r="R871" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S871" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="T871" t="inlineStr"/>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr"/>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Simulations of p‐Channel GaN‐Based Metal‐Oxide‐Semiconductor Heterostructure Field‐Effect Transistors for Normally Off Operation</t>
+        </is>
+      </c>
+      <c r="C872" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>Ubochi, Brendan; Ahmeda, Khaled; Benbakhti, Brahim; Kalna, Karol</t>
+        </is>
+      </c>
+      <c r="G872" t="inlineStr"/>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.70448</t>
+        </is>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.70448</t>
+        </is>
+      </c>
+      <c r="J872" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K872" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L872" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M872" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N872" t="inlineStr"/>
+      <c r="O872" t="inlineStr"/>
+      <c r="P872" t="inlineStr"/>
+      <c r="Q872" t="inlineStr">
+        <is>
+          <t>Simulations of p‐Channel GaN‐Based Metal‐Oxide‐Semiconductor Heterostructure Field‐Effect Transistors for Normally Off Operation</t>
+        </is>
+      </c>
+      <c r="R872" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S872" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="T872" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-04T00:12Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T872"/>
+  <dimension ref="A1:T889"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66392,6 +66392,1298 @@
       </c>
       <c r="T872" t="inlineStr"/>
     </row>
+    <row r="873">
+      <c r="A873" t="inlineStr"/>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C873" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G873" t="inlineStr"/>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I873" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J873" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K873" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L873" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M873" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N873" t="inlineStr"/>
+      <c r="O873" t="inlineStr"/>
+      <c r="P873" t="inlineStr"/>
+      <c r="Q873" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R873" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S873" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T873" t="inlineStr"/>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr"/>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Dual‐Peak Friction Upon Traversing a Monolithic Subsurface Step in Layered Materials</t>
+        </is>
+      </c>
+      <c r="C874" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>Advanced Materials</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>He, Wenjie; Zhang, Honglin; Sun, Junhui; Huang, Xuanyu; Qian, Linmao; Wang, Wen</t>
+        </is>
+      </c>
+      <c r="G874" t="inlineStr"/>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>10.1002/adma.74468</t>
+        </is>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/adma.74468</t>
+        </is>
+      </c>
+      <c r="J874" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K874" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L874" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M874" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N874" t="inlineStr"/>
+      <c r="O874" t="inlineStr"/>
+      <c r="P874" t="inlineStr"/>
+      <c r="Q874" t="inlineStr">
+        <is>
+          <t>Dual‐Peak Friction Upon Traversing a Monolithic Subsurface Step in Layered Materials</t>
+        </is>
+      </c>
+      <c r="R874" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S874" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T874" t="inlineStr"/>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr"/>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C875" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G875" t="inlineStr"/>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J875" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K875" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L875" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M875" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N875" t="inlineStr"/>
+      <c r="O875" t="inlineStr"/>
+      <c r="P875" t="inlineStr"/>
+      <c r="Q875" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R875" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S875" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T875" t="inlineStr"/>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr"/>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Ultrathin fully strained GaN channel high electron mobility transistors on AlN-on-sapphire templates engineered by ferroelectric ScAlN epilayers</t>
+        </is>
+      </c>
+      <c r="C876" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>Yao, JiaJia; Xue, JunShuai; Wu, GuanLin; Zhao, Cheng; Li, ZeHui; Yuan, JinYuan; Zhang, YuYing; Zhang, ChenKai; Hu, HaoRan; Wang, XinPeng; Tong, Yi; Zhang, JinCheng</t>
+        </is>
+      </c>
+      <c r="G876" t="inlineStr"/>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325273</t>
+        </is>
+      </c>
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325273</t>
+        </is>
+      </c>
+      <c r="J876" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K876" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L876" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M876" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N876" t="inlineStr"/>
+      <c r="O876" t="inlineStr"/>
+      <c r="P876" t="inlineStr"/>
+      <c r="Q876" t="inlineStr">
+        <is>
+          <t>Ultrathin fully strained GaN channel high electron mobility transistors on AlN-on-sapphire templates engineered by ferroelectric ScAlN epilayers</t>
+        </is>
+      </c>
+      <c r="R876" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S876" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T876" t="inlineStr"/>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr"/>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C877" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G877" t="inlineStr"/>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J877" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K877" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L877" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M877" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N877" t="inlineStr"/>
+      <c r="O877" t="inlineStr"/>
+      <c r="P877" t="inlineStr"/>
+      <c r="Q877" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R877" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S877" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T877" t="inlineStr"/>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr"/>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Ultrathin fully strained GaN channel high electron mobility transistors on AlN-on-sapphire templates engineered by ferroelectric ScAlN epilayers</t>
+        </is>
+      </c>
+      <c r="C878" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>Yao, JiaJia; Xue, JunShuai; Wu, GuanLin; Zhao, Cheng; Li, ZeHui; Yuan, JinYuan; Zhang, YuYing; Zhang, ChenKai; Hu, HaoRan; Wang, XinPeng; Tong, Yi; Zhang, JinCheng</t>
+        </is>
+      </c>
+      <c r="G878" t="inlineStr"/>
+      <c r="H878" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325273</t>
+        </is>
+      </c>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325273</t>
+        </is>
+      </c>
+      <c r="J878" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K878" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L878" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M878" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N878" t="inlineStr"/>
+      <c r="O878" t="inlineStr"/>
+      <c r="P878" t="inlineStr"/>
+      <c r="Q878" t="inlineStr">
+        <is>
+          <t>Ultrathin fully strained GaN channel high electron mobility transistors on AlN-on-sapphire templates engineered by ferroelectric ScAlN epilayers</t>
+        </is>
+      </c>
+      <c r="R878" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S878" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T878" t="inlineStr"/>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr"/>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C879" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G879" t="inlineStr"/>
+      <c r="H879" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I879" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J879" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K879" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L879" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M879" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N879" t="inlineStr"/>
+      <c r="O879" t="inlineStr"/>
+      <c r="P879" t="inlineStr"/>
+      <c r="Q879" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R879" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S879" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T879" t="inlineStr"/>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr"/>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>1.7kV Fully-Vertical GaN Trench MOSFET with Nitrogen Ion-Implanted Guard Rings</t>
+        </is>
+      </c>
+      <c r="C880" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>Nanotechnology</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr">
+        <is>
+          <t>Xie, Yuanyuan; Yang, Cui; Mao, Wei; Peng, Guoliang; Fan, Dongguo; Wang, Maojun; Ma, Yuchuan; sun, changfa; Liu, Chao; Zheng, Li; Zhang, Yachao; Zhang, Chunfu</t>
+        </is>
+      </c>
+      <c r="G880" t="inlineStr"/>
+      <c r="H880" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6528/ae93c2</t>
+        </is>
+      </c>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6528/ae93c2</t>
+        </is>
+      </c>
+      <c r="J880" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K880" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L880" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M880" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N880" t="inlineStr"/>
+      <c r="O880" t="inlineStr"/>
+      <c r="P880" t="inlineStr"/>
+      <c r="Q880" t="inlineStr">
+        <is>
+          <t>1.7kV Fully-Vertical GaN Trench MOSFET with Nitrogen Ion-Implanted Guard Rings</t>
+        </is>
+      </c>
+      <c r="R880" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S880" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T880" t="inlineStr"/>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr"/>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C881" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G881" t="inlineStr"/>
+      <c r="H881" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I881" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J881" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K881" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L881" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M881" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N881" t="inlineStr"/>
+      <c r="O881" t="inlineStr"/>
+      <c r="P881" t="inlineStr"/>
+      <c r="Q881" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R881" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S881" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T881" t="inlineStr"/>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr"/>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C882" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G882" t="inlineStr"/>
+      <c r="H882" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I882" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J882" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K882" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L882" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M882" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N882" t="inlineStr"/>
+      <c r="O882" t="inlineStr"/>
+      <c r="P882" t="inlineStr"/>
+      <c r="Q882" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R882" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S882" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T882" t="inlineStr"/>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr"/>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>1.7kV Fully-Vertical GaN Trench MOSFET with Nitrogen Ion-Implanted Guard Rings</t>
+        </is>
+      </c>
+      <c r="C883" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>Nanotechnology</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>Xie, Yuanyuan; Yang, Cui; Mao, Wei; Peng, Guoliang; Fan, Dongguo; Wang, Maojun; Ma, Yuchuan; sun, changfa; Liu, Chao; Zheng, Li; Zhang, Yachao; Zhang, Chunfu</t>
+        </is>
+      </c>
+      <c r="G883" t="inlineStr"/>
+      <c r="H883" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6528/ae93c2</t>
+        </is>
+      </c>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6528/ae93c2</t>
+        </is>
+      </c>
+      <c r="J883" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K883" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L883" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M883" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N883" t="inlineStr"/>
+      <c r="O883" t="inlineStr"/>
+      <c r="P883" t="inlineStr"/>
+      <c r="Q883" t="inlineStr">
+        <is>
+          <t>1.7kV Fully-Vertical GaN Trench MOSFET with Nitrogen Ion-Implanted Guard Rings</t>
+        </is>
+      </c>
+      <c r="R883" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S883" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T883" t="inlineStr"/>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr"/>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>1.7kV Fully-Vertical GaN Trench MOSFET with Nitrogen Ion-Implanted Guard Rings</t>
+        </is>
+      </c>
+      <c r="C884" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>Nanotechnology</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>Xie, Yuanyuan; Yang, Cui; Mao, Wei; Peng, Guoliang; Fan, Dongguo; Wang, Maojun; Ma, Yuchuan; sun, changfa; Liu, Chao; Zheng, Li; Zhang, Yachao; Zhang, Chunfu</t>
+        </is>
+      </c>
+      <c r="G884" t="inlineStr"/>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6528/ae93c2</t>
+        </is>
+      </c>
+      <c r="I884" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6528/ae93c2</t>
+        </is>
+      </c>
+      <c r="J884" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K884" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L884" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M884" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N884" t="inlineStr"/>
+      <c r="O884" t="inlineStr"/>
+      <c r="P884" t="inlineStr"/>
+      <c r="Q884" t="inlineStr">
+        <is>
+          <t>1.7kV Fully-Vertical GaN Trench MOSFET with Nitrogen Ion-Implanted Guard Rings</t>
+        </is>
+      </c>
+      <c r="R884" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S884" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T884" t="inlineStr"/>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr"/>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C885" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G885" t="inlineStr"/>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I885" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J885" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K885" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L885" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M885" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N885" t="inlineStr"/>
+      <c r="O885" t="inlineStr"/>
+      <c r="P885" t="inlineStr"/>
+      <c r="Q885" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R885" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S885" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T885" t="inlineStr"/>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr"/>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C886" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G886" t="inlineStr"/>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J886" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K886" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L886" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M886" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N886" t="inlineStr"/>
+      <c r="O886" t="inlineStr"/>
+      <c r="P886" t="inlineStr"/>
+      <c r="Q886" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R886" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S886" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T886" t="inlineStr"/>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr"/>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C887" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G887" t="inlineStr"/>
+      <c r="H887" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I887" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J887" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K887" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L887" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M887" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N887" t="inlineStr"/>
+      <c r="O887" t="inlineStr"/>
+      <c r="P887" t="inlineStr"/>
+      <c r="Q887" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R887" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S887" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T887" t="inlineStr"/>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr"/>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C888" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G888" t="inlineStr"/>
+      <c r="H888" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I888" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J888" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K888" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L888" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M888" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N888" t="inlineStr"/>
+      <c r="O888" t="inlineStr"/>
+      <c r="P888" t="inlineStr"/>
+      <c r="Q888" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R888" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S888" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T888" t="inlineStr"/>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr"/>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="C889" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>Fan, Xuancong; Zhu, Renqiang; Luo, Haowen; Li, Jialun; Guo, Hui; He, Yuanzhi; Lau, Kei May; Jiang, Huaxing</t>
+        </is>
+      </c>
+      <c r="G889" t="inlineStr"/>
+      <c r="H889" t="inlineStr">
+        <is>
+          <t>10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="I889" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0325399</t>
+        </is>
+      </c>
+      <c r="J889" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K889" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L889" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M889" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N889" t="inlineStr"/>
+      <c r="O889" t="inlineStr"/>
+      <c r="P889" t="inlineStr"/>
+      <c r="Q889" t="inlineStr">
+        <is>
+          <t>Homoepitaxial GaN-on-GaN trench MOSFETs with 438 MW/cm2 figure of merit and improved gate reliability</t>
+        </is>
+      </c>
+      <c r="R889" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S889" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="T889" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-05T00:06Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T889"/>
+  <dimension ref="A1:T896"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67684,6 +67684,538 @@
       </c>
       <c r="T889" t="inlineStr"/>
     </row>
+    <row r="890">
+      <c r="A890" t="inlineStr"/>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>The Role of CMOS Technology in Modern Microprocessor Design: A Review</t>
+        </is>
+      </c>
+      <c r="C890" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>EWA Publishing</t>
+        </is>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>Applied and Computational Engineering</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>Yao, Zeyu</t>
+        </is>
+      </c>
+      <c r="G890" t="inlineStr"/>
+      <c r="H890" t="inlineStr">
+        <is>
+          <t>10.54254/2755-2721/2026.ba35893</t>
+        </is>
+      </c>
+      <c r="I890" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54254/2755-2721/2026.ba35893</t>
+        </is>
+      </c>
+      <c r="J890" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K890" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L890" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M890" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N890" t="inlineStr"/>
+      <c r="O890" t="inlineStr"/>
+      <c r="P890" t="inlineStr"/>
+      <c r="Q890" t="inlineStr">
+        <is>
+          <t>The Role of CMOS Technology in Modern Microprocessor Design: A Review</t>
+        </is>
+      </c>
+      <c r="R890" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S890" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="T890" t="inlineStr"/>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr"/>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>The Role of CMOS Technology in Modern Microprocessor Design: A Review</t>
+        </is>
+      </c>
+      <c r="C891" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>EWA Publishing</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>Applied and Computational Engineering</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>Yao, Zeyu</t>
+        </is>
+      </c>
+      <c r="G891" t="inlineStr"/>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>10.54254/2755-2721/2026.ba35893</t>
+        </is>
+      </c>
+      <c r="I891" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54254/2755-2721/2026.ba35893</t>
+        </is>
+      </c>
+      <c r="J891" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K891" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L891" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M891" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N891" t="inlineStr"/>
+      <c r="O891" t="inlineStr"/>
+      <c r="P891" t="inlineStr"/>
+      <c r="Q891" t="inlineStr">
+        <is>
+          <t>The Role of CMOS Technology in Modern Microprocessor Design: A Review</t>
+        </is>
+      </c>
+      <c r="R891" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S891" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="T891" t="inlineStr"/>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr"/>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Gate-metal-dependent transition of leakage mechanisms in AlGaN/GaN HEMTs under temperature-dependent conditions</t>
+        </is>
+      </c>
+      <c r="C892" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>Microelectronics Reliability</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>Caño de Andrade, Maria Glória; Cândido, Josué; Simoen, Eddy</t>
+        </is>
+      </c>
+      <c r="G892" t="inlineStr"/>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>10.1016/j.microrel.2026.116260</t>
+        </is>
+      </c>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.microrel.2026.116260</t>
+        </is>
+      </c>
+      <c r="J892" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K892" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L892" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M892" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N892" t="inlineStr"/>
+      <c r="O892" t="inlineStr"/>
+      <c r="P892" t="inlineStr"/>
+      <c r="Q892" t="inlineStr">
+        <is>
+          <t>Gate-metal-dependent transition of leakage mechanisms in AlGaN/GaN HEMTs under temperature-dependent conditions</t>
+        </is>
+      </c>
+      <c r="R892" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S892" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="T892" t="inlineStr"/>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr"/>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>The Role of CMOS Technology in Modern Microprocessor Design: A Review</t>
+        </is>
+      </c>
+      <c r="C893" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>EWA Publishing</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>Applied and Computational Engineering</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>Yao, Zeyu</t>
+        </is>
+      </c>
+      <c r="G893" t="inlineStr"/>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>10.54254/2755-2721/2026.ba35893</t>
+        </is>
+      </c>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54254/2755-2721/2026.ba35893</t>
+        </is>
+      </c>
+      <c r="J893" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K893" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L893" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M893" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N893" t="inlineStr"/>
+      <c r="O893" t="inlineStr"/>
+      <c r="P893" t="inlineStr"/>
+      <c r="Q893" t="inlineStr">
+        <is>
+          <t>The Role of CMOS Technology in Modern Microprocessor Design: A Review</t>
+        </is>
+      </c>
+      <c r="R893" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S893" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="T893" t="inlineStr"/>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr"/>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>A Practical Methodology for Designing and Optimizing a Three-Stage Ring Oscillator in 180-nm CMOS Technology using Particle Swarm Optimization (PSO)</t>
+        </is>
+      </c>
+      <c r="C894" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>World Scientific and Engineering Academy and Society (WSEAS)</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>WSEAS TRANSACTIONS ON CIRCUITS AND SYSTEMS</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>Sanae, Elhafidi; Asmae, Elbeqal; Ismail, Maaroufi; Bachir, Benhala</t>
+        </is>
+      </c>
+      <c r="G894" t="inlineStr"/>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>10.37394/23201.2026.25.25</t>
+        </is>
+      </c>
+      <c r="I894" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.37394/23201.2026.25.25</t>
+        </is>
+      </c>
+      <c r="J894" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K894" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L894" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M894" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N894" t="inlineStr"/>
+      <c r="O894" t="inlineStr"/>
+      <c r="P894" t="inlineStr"/>
+      <c r="Q894" t="inlineStr">
+        <is>
+          <t>A Practical Methodology for Designing and Optimizing a Three-Stage Ring Oscillator in 180-nm CMOS Technology using Particle Swarm Optimization (PSO)</t>
+        </is>
+      </c>
+      <c r="R894" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S894" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="T894" t="inlineStr"/>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr"/>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Gate-metal-dependent transition of leakage mechanisms in AlGaN/GaN HEMTs under temperature-dependent conditions</t>
+        </is>
+      </c>
+      <c r="C895" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>Microelectronics Reliability</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>Caño de Andrade, Maria Glória; Cândido, Josué; Simoen, Eddy</t>
+        </is>
+      </c>
+      <c r="G895" t="inlineStr"/>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>10.1016/j.microrel.2026.116260</t>
+        </is>
+      </c>
+      <c r="I895" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.microrel.2026.116260</t>
+        </is>
+      </c>
+      <c r="J895" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K895" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L895" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M895" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N895" t="inlineStr"/>
+      <c r="O895" t="inlineStr"/>
+      <c r="P895" t="inlineStr"/>
+      <c r="Q895" t="inlineStr">
+        <is>
+          <t>Gate-metal-dependent transition of leakage mechanisms in AlGaN/GaN HEMTs under temperature-dependent conditions</t>
+        </is>
+      </c>
+      <c r="R895" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S895" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="T895" t="inlineStr"/>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr"/>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Gate-metal-dependent transition of leakage mechanisms in AlGaN/GaN HEMTs under temperature-dependent conditions</t>
+        </is>
+      </c>
+      <c r="C896" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>Microelectronics Reliability</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>Caño de Andrade, Maria Glória; Cândido, Josué; Simoen, Eddy</t>
+        </is>
+      </c>
+      <c r="G896" t="inlineStr"/>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>10.1016/j.microrel.2026.116260</t>
+        </is>
+      </c>
+      <c r="I896" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.microrel.2026.116260</t>
+        </is>
+      </c>
+      <c r="J896" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K896" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L896" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M896" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N896" t="inlineStr"/>
+      <c r="O896" t="inlineStr"/>
+      <c r="P896" t="inlineStr"/>
+      <c r="Q896" t="inlineStr">
+        <is>
+          <t>Gate-metal-dependent transition of leakage mechanisms in AlGaN/GaN HEMTs under temperature-dependent conditions</t>
+        </is>
+      </c>
+      <c r="R896" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S896" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="T896" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-06T00:02Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T896"/>
+  <dimension ref="A1:T902"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68216,6 +68216,464 @@
       </c>
       <c r="T896" t="inlineStr"/>
     </row>
+    <row r="897">
+      <c r="A897" t="inlineStr"/>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Hybrid MPPT optimization for solar powered cascaded DC–DC converters interfaced with grid-connected multilevel inverter</t>
+        </is>
+      </c>
+      <c r="C897" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>World Journal of Engineering</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>J., Veerabhadra; Sulake, Nagaraja Rao</t>
+        </is>
+      </c>
+      <c r="G897" t="inlineStr"/>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>10.1108/wje-02-2026-0068</t>
+        </is>
+      </c>
+      <c r="I897" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/wje-02-2026-0068</t>
+        </is>
+      </c>
+      <c r="J897" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K897" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L897" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M897" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N897" t="inlineStr"/>
+      <c r="O897" t="inlineStr"/>
+      <c r="P897" t="inlineStr"/>
+      <c r="Q897" t="inlineStr">
+        <is>
+          <t>Hybrid MPPT optimization for solar powered cascaded DC–DC converters interfaced with grid-connected multilevel inverter</t>
+        </is>
+      </c>
+      <c r="R897" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S897" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="T897" t="inlineStr"/>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr"/>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Monolithic Porous Polymer Architectures for Visible‐to‐UV Upconversion‐Driven Photochemical Reactions</t>
+        </is>
+      </c>
+      <c r="C898" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>Angewandte Chemie</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>Nakagawa, Sakura; Matsumoto, Naoto; Uji, Masanori; Bertrams, Maria‐Sophie; Kerzig, Christoph; Yanai, Nobuhiro</t>
+        </is>
+      </c>
+      <c r="G898" t="inlineStr"/>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>10.1002/ange.3019584</t>
+        </is>
+      </c>
+      <c r="I898" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/ange.3019584</t>
+        </is>
+      </c>
+      <c r="J898" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K898" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L898" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M898" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N898" t="inlineStr"/>
+      <c r="O898" t="inlineStr"/>
+      <c r="P898" t="inlineStr"/>
+      <c r="Q898" t="inlineStr">
+        <is>
+          <t>Monolithic Porous Polymer Architectures for Visible‐to‐UV Upconversion‐Driven Photochemical Reactions</t>
+        </is>
+      </c>
+      <c r="R898" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S898" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="T898" t="inlineStr"/>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr"/>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Effects of Powder Purity and SPS Conditions on Microstructure and Mechanical Properties of Monolithic TiB2 Ceramics</t>
+        </is>
+      </c>
+      <c r="C899" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>Ceramics</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>Çelik, Azmi Mert; Haber, Richard A.; Mann, Adrian B.</t>
+        </is>
+      </c>
+      <c r="G899" t="inlineStr"/>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>10.3390/ceramics9080083</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ceramics9080083</t>
+        </is>
+      </c>
+      <c r="J899" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K899" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L899" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M899" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N899" t="inlineStr"/>
+      <c r="O899" t="inlineStr"/>
+      <c r="P899" t="inlineStr"/>
+      <c r="Q899" t="inlineStr">
+        <is>
+          <t>Effects of Powder Purity and SPS Conditions on Microstructure and Mechanical Properties of Monolithic TiB2 Ceramics</t>
+        </is>
+      </c>
+      <c r="R899" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S899" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="T899" t="inlineStr"/>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr"/>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Monolithic III–V Membrane Photodetectors on
+SOI with 240 Gb/s Data Reception</t>
+        </is>
+      </c>
+      <c r="C900" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>ACS Photonics</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>Zhao, Yingzhi; Liang, Zhiwei; Fu, Donghui; Ren, Zhaojie; Chen, Antai; Zeng, Cong; Han, Yu; Jin, Yunjiang; Yu, Siyuan</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr"/>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>10.1021/acsphotonics.6c01040</t>
+        </is>
+      </c>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsphotonics.6c01040</t>
+        </is>
+      </c>
+      <c r="J900" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K900" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L900" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M900" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N900" t="inlineStr"/>
+      <c r="O900" t="inlineStr"/>
+      <c r="P900" t="inlineStr"/>
+      <c r="Q900" t="inlineStr">
+        <is>
+          <t>Monolithic III–V Membrane Photodetectors on
+SOI with 240 Gb/s Data Reception</t>
+        </is>
+      </c>
+      <c r="R900" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S900" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="T900" t="inlineStr"/>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr"/>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Hybrid MPPT optimization for solar powered cascaded DC–DC converters interfaced with grid-connected multilevel inverter</t>
+        </is>
+      </c>
+      <c r="C901" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>World Journal of Engineering</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>J., Veerabhadra; Sulake, Nagaraja Rao</t>
+        </is>
+      </c>
+      <c r="G901" t="inlineStr"/>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>10.1108/wje-02-2026-0068</t>
+        </is>
+      </c>
+      <c r="I901" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/wje-02-2026-0068</t>
+        </is>
+      </c>
+      <c r="J901" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K901" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L901" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M901" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N901" t="inlineStr"/>
+      <c r="O901" t="inlineStr"/>
+      <c r="P901" t="inlineStr"/>
+      <c r="Q901" t="inlineStr">
+        <is>
+          <t>Hybrid MPPT optimization for solar powered cascaded DC–DC converters interfaced with grid-connected multilevel inverter</t>
+        </is>
+      </c>
+      <c r="R901" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S901" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="T901" t="inlineStr"/>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr"/>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Optical determination of cyanide in water using an anthraquinone-based chemosensing system with DFT-assisted mechanistic insights and Logic gate functionality</t>
+        </is>
+      </c>
+      <c r="C902" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>Microchemical Journal</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>Shastri, Priyanka; Kaur, Navneet</t>
+        </is>
+      </c>
+      <c r="G902" t="inlineStr"/>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>10.1016/j.microc.2026.119253</t>
+        </is>
+      </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.microc.2026.119253</t>
+        </is>
+      </c>
+      <c r="J902" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K902" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L902" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M902" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N902" t="inlineStr"/>
+      <c r="O902" t="inlineStr"/>
+      <c r="P902" t="inlineStr"/>
+      <c r="Q902" t="inlineStr">
+        <is>
+          <t>Optical determination of cyanide in water using an anthraquinone-based chemosensing system with DFT-assisted mechanistic insights and Logic gate functionality</t>
+        </is>
+      </c>
+      <c r="R902" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S902" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="T902" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-07T01:42Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T902"/>
+  <dimension ref="A1:T914"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68674,6 +68674,918 @@
       </c>
       <c r="T902" t="inlineStr"/>
     </row>
+    <row r="903">
+      <c r="A903" t="inlineStr"/>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="C903" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>Liu, Haoran; Wang, Manjing; Yuan, Jiancheng; Li, Xuan; Chen, Jiamao; Zhang, Lin; Gao, Sheng</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr"/>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="I903" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="J903" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K903" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L903" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M903" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N903" t="inlineStr"/>
+      <c r="O903" t="inlineStr"/>
+      <c r="P903" t="inlineStr"/>
+      <c r="Q903" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="R903" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S903" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T903" t="inlineStr"/>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr"/>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="C904" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>Liu, Haoran; Wang, Manjing; Yuan, Jiancheng; Li, Xuan; Chen, Jiamao; Zhang, Lin; Gao, Sheng</t>
+        </is>
+      </c>
+      <c r="G904" t="inlineStr"/>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="J904" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K904" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L904" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M904" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N904" t="inlineStr"/>
+      <c r="O904" t="inlineStr"/>
+      <c r="P904" t="inlineStr"/>
+      <c r="Q904" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="R904" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S904" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T904" t="inlineStr"/>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr"/>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="C905" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>Liu, Haoran; Wang, Manjing; Yuan, Jiancheng; Li, Xuan; Chen, Jiamao; Zhang, Lin; Gao, Sheng</t>
+        </is>
+      </c>
+      <c r="G905" t="inlineStr"/>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="I905" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="J905" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K905" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L905" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M905" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N905" t="inlineStr"/>
+      <c r="O905" t="inlineStr"/>
+      <c r="P905" t="inlineStr"/>
+      <c r="Q905" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="R905" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S905" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T905" t="inlineStr"/>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr"/>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="C906" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>Liu, Haoran; Wang, Manjing; Yuan, Jiancheng; Li, Xuan; Chen, Jiamao; Zhang, Lin; Gao, Sheng</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr"/>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="I906" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="J906" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K906" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L906" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M906" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N906" t="inlineStr"/>
+      <c r="O906" t="inlineStr"/>
+      <c r="P906" t="inlineStr"/>
+      <c r="Q906" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="R906" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S906" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T906" t="inlineStr"/>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr"/>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Simulation study of a split-gate superjunction SiC MOSFET with a p-type shielding layer</t>
+        </is>
+      </c>
+      <c r="C907" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>Huang, Jun-Sheng; Luo, Xin-Yi; Chen, Chun-Pei; Hsin, Yue-Ming</t>
+        </is>
+      </c>
+      <c r="G907" t="inlineStr"/>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae9661</t>
+        </is>
+      </c>
+      <c r="I907" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae9661</t>
+        </is>
+      </c>
+      <c r="J907" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K907" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L907" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M907" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N907" t="inlineStr"/>
+      <c r="O907" t="inlineStr"/>
+      <c r="P907" t="inlineStr"/>
+      <c r="Q907" t="inlineStr">
+        <is>
+          <t>Simulation study of a split-gate superjunction SiC MOSFET with a p-type shielding layer</t>
+        </is>
+      </c>
+      <c r="R907" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S907" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T907" t="inlineStr"/>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr"/>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="C908" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>Liu, Haoran; Wang, Manjing; Yuan, Jiancheng; Li, Xuan; Chen, Jiamao; Zhang, Lin; Gao, Sheng</t>
+        </is>
+      </c>
+      <c r="G908" t="inlineStr"/>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="I908" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="J908" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K908" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L908" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M908" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N908" t="inlineStr"/>
+      <c r="O908" t="inlineStr"/>
+      <c r="P908" t="inlineStr"/>
+      <c r="Q908" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="R908" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S908" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T908" t="inlineStr"/>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr"/>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Simulation study of a split-gate superjunction SiC MOSFET with a p-type shielding layer</t>
+        </is>
+      </c>
+      <c r="C909" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>Huang, Jun-Sheng; Luo, Xin-Yi; Chen, Chun-Pei; Hsin, Yue-Ming</t>
+        </is>
+      </c>
+      <c r="G909" t="inlineStr"/>
+      <c r="H909" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae9661</t>
+        </is>
+      </c>
+      <c r="I909" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae9661</t>
+        </is>
+      </c>
+      <c r="J909" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K909" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L909" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M909" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N909" t="inlineStr"/>
+      <c r="O909" t="inlineStr"/>
+      <c r="P909" t="inlineStr"/>
+      <c r="Q909" t="inlineStr">
+        <is>
+          <t>Simulation study of a split-gate superjunction SiC MOSFET with a p-type shielding layer</t>
+        </is>
+      </c>
+      <c r="R909" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S909" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T909" t="inlineStr"/>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr"/>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Simulation study of a split-gate superjunction SiC MOSFET with a p-type shielding layer</t>
+        </is>
+      </c>
+      <c r="C910" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>Japanese Journal of Applied Physics</t>
+        </is>
+      </c>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>Huang, Jun-Sheng; Luo, Xin-Yi; Chen, Chun-Pei; Hsin, Yue-Ming</t>
+        </is>
+      </c>
+      <c r="G910" t="inlineStr"/>
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>10.35848/1347-4065/ae9661</t>
+        </is>
+      </c>
+      <c r="I910" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.35848/1347-4065/ae9661</t>
+        </is>
+      </c>
+      <c r="J910" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K910" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L910" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M910" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N910" t="inlineStr"/>
+      <c r="O910" t="inlineStr"/>
+      <c r="P910" t="inlineStr"/>
+      <c r="Q910" t="inlineStr">
+        <is>
+          <t>Simulation study of a split-gate superjunction SiC MOSFET with a p-type shielding layer</t>
+        </is>
+      </c>
+      <c r="R910" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S910" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T910" t="inlineStr"/>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr"/>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="C911" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>Liu, Haoran; Wang, Manjing; Yuan, Jiancheng; Li, Xuan; Chen, Jiamao; Zhang, Lin; Gao, Sheng</t>
+        </is>
+      </c>
+      <c r="G911" t="inlineStr"/>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="I911" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="J911" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K911" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L911" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M911" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N911" t="inlineStr"/>
+      <c r="O911" t="inlineStr"/>
+      <c r="P911" t="inlineStr"/>
+      <c r="Q911" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="R911" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S911" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T911" t="inlineStr"/>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr"/>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="C912" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>Liu, Haoran; Wang, Manjing; Yuan, Jiancheng; Li, Xuan; Chen, Jiamao; Zhang, Lin; Gao, Sheng</t>
+        </is>
+      </c>
+      <c r="G912" t="inlineStr"/>
+      <c r="H912" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="I912" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="J912" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K912" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L912" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M912" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N912" t="inlineStr"/>
+      <c r="O912" t="inlineStr"/>
+      <c r="P912" t="inlineStr"/>
+      <c r="Q912" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="R912" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S912" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T912" t="inlineStr"/>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr"/>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Enhancing frequency stability of IBR-dominated low-inertia power grids using virtual synchronous generator (VSG)-based GFM inverter control</t>
+        </is>
+      </c>
+      <c r="C913" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>Sharif, Suriya; Rahman, Asadur</t>
+        </is>
+      </c>
+      <c r="G913" t="inlineStr"/>
+      <c r="H913" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae95f0</t>
+        </is>
+      </c>
+      <c r="I913" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae95f0</t>
+        </is>
+      </c>
+      <c r="J913" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K913" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L913" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M913" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N913" t="inlineStr"/>
+      <c r="O913" t="inlineStr"/>
+      <c r="P913" t="inlineStr"/>
+      <c r="Q913" t="inlineStr">
+        <is>
+          <t>Enhancing frequency stability of IBR-dominated low-inertia power grids using virtual synchronous generator (VSG)-based GFM inverter control</t>
+        </is>
+      </c>
+      <c r="R913" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S913" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T913" t="inlineStr"/>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr"/>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="C914" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>Semiconductor Science and Technology</t>
+        </is>
+      </c>
+      <c r="F914" t="inlineStr">
+        <is>
+          <t>Liu, Haoran; Wang, Manjing; Yuan, Jiancheng; Li, Xuan; Chen, Jiamao; Zhang, Lin; Gao, Sheng</t>
+        </is>
+      </c>
+      <c r="G914" t="inlineStr"/>
+      <c r="H914" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="I914" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6641/ae9638</t>
+        </is>
+      </c>
+      <c r="J914" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K914" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L914" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M914" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N914" t="inlineStr"/>
+      <c r="O914" t="inlineStr"/>
+      <c r="P914" t="inlineStr"/>
+      <c r="Q914" t="inlineStr">
+        <is>
+          <t>Simulation of Enhanced Short-Circuit Ruggedness in GaN HEMTs with a Step-Graded-Doped p-GaN Buried Layer</t>
+        </is>
+      </c>
+      <c r="R914" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S914" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="T914" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-10T23:38Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T914"/>
+  <dimension ref="A1:T922"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69586,6 +69586,610 @@
       </c>
       <c r="T914" t="inlineStr"/>
     </row>
+    <row r="915">
+      <c r="A915" t="inlineStr"/>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>π-Armor Strategy: Shape-Complementary Encapsulation of Aromatics</t>
+        </is>
+      </c>
+      <c r="C915" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E915" t="inlineStr"/>
+      <c r="F915" t="inlineStr">
+        <is>
+          <t>Kano, Haruka; Harimoto, Takashi; Segawa, Yasutomo</t>
+        </is>
+      </c>
+      <c r="G915" t="inlineStr"/>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>10.26434/chemrxiv.15007230/v1</t>
+        </is>
+      </c>
+      <c r="I915" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.26434/chemrxiv.15007230/v1</t>
+        </is>
+      </c>
+      <c r="J915" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K915" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L915" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M915" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N915" t="inlineStr"/>
+      <c r="O915" t="inlineStr"/>
+      <c r="P915" t="inlineStr"/>
+      <c r="Q915" t="inlineStr">
+        <is>
+          <t>π-Armor Strategy: Shape-Complementary Encapsulation of Aromatics</t>
+        </is>
+      </c>
+      <c r="R915" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S915" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="T915" t="inlineStr"/>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr"/>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>3D-printed monolithic zeolite structures for terrestrial decarbonization and space life support systems</t>
+        </is>
+      </c>
+      <c r="C916" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>Chemical Engineering Journal</t>
+        </is>
+      </c>
+      <c r="F916" t="inlineStr">
+        <is>
+          <t>Agata, Noah; Cesarano, Joseph; Richardson, Tra-My Justine; Bigham, Sajjad</t>
+        </is>
+      </c>
+      <c r="G916" t="inlineStr"/>
+      <c r="H916" t="inlineStr">
+        <is>
+          <t>10.1016/j.cej.2026.179476</t>
+        </is>
+      </c>
+      <c r="I916" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.cej.2026.179476</t>
+        </is>
+      </c>
+      <c r="J916" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K916" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L916" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M916" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N916" t="inlineStr"/>
+      <c r="O916" t="inlineStr"/>
+      <c r="P916" t="inlineStr"/>
+      <c r="Q916" t="inlineStr">
+        <is>
+          <t>3D-printed monolithic zeolite structures for terrestrial decarbonization and space life support systems</t>
+        </is>
+      </c>
+      <c r="R916" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S916" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="T916" t="inlineStr"/>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr"/>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Sequential Channel Activation in Multi-Channel AlGaN/AlN/GaN HEMTs: From 4-Channel to Double-Sided 5-Channel Configurations</t>
+        </is>
+      </c>
+      <c r="C917" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>ACS Applied Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>Kocherla, Maria Kiran; Huang, Kun-Pin; Chiu, Shih-Hsuan; Kao, Yu-Cheng; Rather, Safeer Hussain; Lin, Der-Yuh; Yang, Hongta; Lin, Chia-Feng</t>
+        </is>
+      </c>
+      <c r="G917" t="inlineStr"/>
+      <c r="H917" t="inlineStr">
+        <is>
+          <t>10.1021/acsaelm.6c00929</t>
+        </is>
+      </c>
+      <c r="I917" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsaelm.6c00929</t>
+        </is>
+      </c>
+      <c r="J917" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K917" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L917" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M917" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N917" t="inlineStr"/>
+      <c r="O917" t="inlineStr"/>
+      <c r="P917" t="inlineStr"/>
+      <c r="Q917" t="inlineStr">
+        <is>
+          <t>Sequential Channel Activation in Multi-Channel AlGaN/AlN/GaN HEMTs: From 4-Channel to Double-Sided 5-Channel Configurations</t>
+        </is>
+      </c>
+      <c r="R917" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S917" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="T917" t="inlineStr"/>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr"/>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Linearity metrics of pre-matched AlGaN/GaN RF transistor: multi-tone simulation and measurement analysis</t>
+        </is>
+      </c>
+      <c r="C918" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>Cambridge University Press (CUP)</t>
+        </is>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>International Journal of Microwave and Wireless Technologies</t>
+        </is>
+      </c>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>Silva Dos Santos, José Anderson; Alleman, Julien; Leventoux, Margot; Medrel, Pierre; Chang, Christophe; Sommet, Raphael; Courrèges, Fabien; Nallatamby, Jean-Christophe</t>
+        </is>
+      </c>
+      <c r="G918" t="inlineStr"/>
+      <c r="H918" t="inlineStr">
+        <is>
+          <t>10.1017/s1759078726103699</t>
+        </is>
+      </c>
+      <c r="I918" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1017/s1759078726103699</t>
+        </is>
+      </c>
+      <c r="J918" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K918" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L918" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M918" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N918" t="inlineStr"/>
+      <c r="O918" t="inlineStr"/>
+      <c r="P918" t="inlineStr"/>
+      <c r="Q918" t="inlineStr">
+        <is>
+          <t>Linearity metrics of pre-matched AlGaN/GaN RF transistor: multi-tone simulation and measurement analysis</t>
+        </is>
+      </c>
+      <c r="R918" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S918" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="T918" t="inlineStr"/>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr"/>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Sequential Channel Activation in Multi-Channel AlGaN/AlN/GaN HEMTs: From 4-Channel to Double-Sided 5-Channel Configurations</t>
+        </is>
+      </c>
+      <c r="C919" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>ACS Applied Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>Kocherla, Maria Kiran; Huang, Kun-Pin; Chiu, Shih-Hsuan; Kao, Yu-Cheng; Rather, Safeer Hussain; Lin, Der-Yuh; Yang, Hongta; Lin, Chia-Feng</t>
+        </is>
+      </c>
+      <c r="G919" t="inlineStr"/>
+      <c r="H919" t="inlineStr">
+        <is>
+          <t>10.1021/acsaelm.6c00929</t>
+        </is>
+      </c>
+      <c r="I919" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsaelm.6c00929</t>
+        </is>
+      </c>
+      <c r="J919" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K919" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L919" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M919" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N919" t="inlineStr"/>
+      <c r="O919" t="inlineStr"/>
+      <c r="P919" t="inlineStr"/>
+      <c r="Q919" t="inlineStr">
+        <is>
+          <t>Sequential Channel Activation in Multi-Channel AlGaN/AlN/GaN HEMTs: From 4-Channel to Double-Sided 5-Channel Configurations</t>
+        </is>
+      </c>
+      <c r="R919" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S919" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="T919" t="inlineStr"/>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr"/>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Linearity metrics of pre-matched AlGaN/GaN RF transistor: multi-tone simulation and measurement analysis</t>
+        </is>
+      </c>
+      <c r="C920" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>Cambridge University Press (CUP)</t>
+        </is>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>International Journal of Microwave and Wireless Technologies</t>
+        </is>
+      </c>
+      <c r="F920" t="inlineStr">
+        <is>
+          <t>Silva Dos Santos, José Anderson; Alleman, Julien; Leventoux, Margot; Medrel, Pierre; Chang, Christophe; Sommet, Raphael; Courrèges, Fabien; Nallatamby, Jean-Christophe</t>
+        </is>
+      </c>
+      <c r="G920" t="inlineStr"/>
+      <c r="H920" t="inlineStr">
+        <is>
+          <t>10.1017/s1759078726103699</t>
+        </is>
+      </c>
+      <c r="I920" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1017/s1759078726103699</t>
+        </is>
+      </c>
+      <c r="J920" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K920" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L920" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M920" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N920" t="inlineStr"/>
+      <c r="O920" t="inlineStr"/>
+      <c r="P920" t="inlineStr"/>
+      <c r="Q920" t="inlineStr">
+        <is>
+          <t>Linearity metrics of pre-matched AlGaN/GaN RF transistor: multi-tone simulation and measurement analysis</t>
+        </is>
+      </c>
+      <c r="R920" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S920" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="T920" t="inlineStr"/>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr"/>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Sequential Channel Activation in Multi-Channel AlGaN/AlN/GaN HEMTs: From 4-Channel to Double-Sided 5-Channel Configurations</t>
+        </is>
+      </c>
+      <c r="C921" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>ACS Applied Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F921" t="inlineStr">
+        <is>
+          <t>Kocherla, Maria Kiran; Huang, Kun-Pin; Chiu, Shih-Hsuan; Kao, Yu-Cheng; Rather, Safeer Hussain; Lin, Der-Yuh; Yang, Hongta; Lin, Chia-Feng</t>
+        </is>
+      </c>
+      <c r="G921" t="inlineStr"/>
+      <c r="H921" t="inlineStr">
+        <is>
+          <t>10.1021/acsaelm.6c00929</t>
+        </is>
+      </c>
+      <c r="I921" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsaelm.6c00929</t>
+        </is>
+      </c>
+      <c r="J921" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K921" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L921" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M921" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N921" t="inlineStr"/>
+      <c r="O921" t="inlineStr"/>
+      <c r="P921" t="inlineStr"/>
+      <c r="Q921" t="inlineStr">
+        <is>
+          <t>Sequential Channel Activation in Multi-Channel AlGaN/AlN/GaN HEMTs: From 4-Channel to Double-Sided 5-Channel Configurations</t>
+        </is>
+      </c>
+      <c r="R921" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S921" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="T921" t="inlineStr"/>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr"/>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Sequential Channel Activation in Multi-Channel AlGaN/AlN/GaN HEMTs: From 4-Channel to Double-Sided 5-Channel Configurations</t>
+        </is>
+      </c>
+      <c r="C922" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>ACS Applied Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F922" t="inlineStr">
+        <is>
+          <t>Kocherla, Maria Kiran; Huang, Kun-Pin; Chiu, Shih-Hsuan; Kao, Yu-Cheng; Rather, Safeer Hussain; Lin, Der-Yuh; Yang, Hongta; Lin, Chia-Feng</t>
+        </is>
+      </c>
+      <c r="G922" t="inlineStr"/>
+      <c r="H922" t="inlineStr">
+        <is>
+          <t>10.1021/acsaelm.6c00929</t>
+        </is>
+      </c>
+      <c r="I922" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsaelm.6c00929</t>
+        </is>
+      </c>
+      <c r="J922" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K922" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L922" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M922" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N922" t="inlineStr"/>
+      <c r="O922" t="inlineStr"/>
+      <c r="P922" t="inlineStr"/>
+      <c r="Q922" t="inlineStr">
+        <is>
+          <t>Sequential Channel Activation in Multi-Channel AlGaN/AlN/GaN HEMTs: From 4-Channel to Double-Sided 5-Channel Configurations</t>
+        </is>
+      </c>
+      <c r="R922" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S922" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="T922" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-12T23:44Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T922"/>
+  <dimension ref="A1:T940"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70190,6 +70190,1362 @@
       </c>
       <c r="T922" t="inlineStr"/>
     </row>
+    <row r="923">
+      <c r="A923" t="inlineStr"/>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C923" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E923" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F923" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G923" t="inlineStr"/>
+      <c r="H923" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I923" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J923" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K923" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L923" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M923" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N923" t="inlineStr"/>
+      <c r="O923" t="inlineStr"/>
+      <c r="P923" t="inlineStr"/>
+      <c r="Q923" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R923" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S923" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T923" t="inlineStr"/>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr"/>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Sistem Kontrol PLC dan Inverter pada Vacuum Mesin Industri</t>
+        </is>
+      </c>
+      <c r="C924" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>Institute of Advanced Knowledge and Science</t>
+        </is>
+      </c>
+      <c r="E924" t="inlineStr">
+        <is>
+          <t>Journal of Engineering and Science Application</t>
+        </is>
+      </c>
+      <c r="F924" t="inlineStr">
+        <is>
+          <t>Budiarjo, Wisnu; Sugiyanto, Didik</t>
+        </is>
+      </c>
+      <c r="G924" t="inlineStr"/>
+      <c r="H924" t="inlineStr">
+        <is>
+          <t>10.69693/jesa.v3i2.42</t>
+        </is>
+      </c>
+      <c r="I924" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.69693/jesa.v3i2.42</t>
+        </is>
+      </c>
+      <c r="J924" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K924" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L924" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M924" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N924" t="inlineStr"/>
+      <c r="O924" t="inlineStr"/>
+      <c r="P924" t="inlineStr"/>
+      <c r="Q924" t="inlineStr">
+        <is>
+          <t>Sistem Kontrol PLC dan Inverter pada Vacuum Mesin Industri</t>
+        </is>
+      </c>
+      <c r="R924" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S924" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T924" t="inlineStr"/>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr"/>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C925" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E925" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F925" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G925" t="inlineStr"/>
+      <c r="H925" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I925" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J925" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K925" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L925" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M925" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N925" t="inlineStr"/>
+      <c r="O925" t="inlineStr"/>
+      <c r="P925" t="inlineStr"/>
+      <c r="Q925" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R925" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S925" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T925" t="inlineStr"/>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr"/>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C926" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E926" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F926" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G926" t="inlineStr"/>
+      <c r="H926" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I926" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J926" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K926" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L926" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M926" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N926" t="inlineStr"/>
+      <c r="O926" t="inlineStr"/>
+      <c r="P926" t="inlineStr"/>
+      <c r="Q926" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R926" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S926" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T926" t="inlineStr"/>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr"/>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Ferroelectric Polarization Enabled Threshold Voltage Modulation in High Electron Mobility Transistor</t>
+        </is>
+      </c>
+      <c r="C927" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E927" t="inlineStr">
+        <is>
+          <t>Advanced Functional Materials</t>
+        </is>
+      </c>
+      <c r="F927" t="inlineStr">
+        <is>
+          <t>Gao, Wentian; Wachowiak, Andre; Mikolajick, Thomas; Schroeder, Uwe; Guido, Roberto</t>
+        </is>
+      </c>
+      <c r="G927" t="inlineStr"/>
+      <c r="H927" t="inlineStr">
+        <is>
+          <t>10.1002/adfm.77470</t>
+        </is>
+      </c>
+      <c r="I927" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/adfm.77470</t>
+        </is>
+      </c>
+      <c r="J927" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K927" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L927" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M927" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N927" t="inlineStr"/>
+      <c r="O927" t="inlineStr"/>
+      <c r="P927" t="inlineStr"/>
+      <c r="Q927" t="inlineStr">
+        <is>
+          <t>Ferroelectric Polarization Enabled Threshold Voltage Modulation in High Electron Mobility Transistor</t>
+        </is>
+      </c>
+      <c r="R927" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S927" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T927" t="inlineStr"/>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr"/>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Fabrication and characterization of a hydrogen-terminated diamond MOSFET with buried p+ type electrodes formed by ion implantation</t>
+        </is>
+      </c>
+      <c r="C928" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E928" t="inlineStr">
+        <is>
+          <t>Diamond and Related Materials</t>
+        </is>
+      </c>
+      <c r="F928" t="inlineStr">
+        <is>
+          <t>Uehara, Sakura; Seki, Yuhei; Hoshino, Yasushi; Umezawa, Hitoshi; Kaneko, Junichi H.</t>
+        </is>
+      </c>
+      <c r="G928" t="inlineStr"/>
+      <c r="H928" t="inlineStr">
+        <is>
+          <t>10.1016/j.diamond.2026.114054</t>
+        </is>
+      </c>
+      <c r="I928" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.diamond.2026.114054</t>
+        </is>
+      </c>
+      <c r="J928" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K928" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L928" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M928" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N928" t="inlineStr"/>
+      <c r="O928" t="inlineStr"/>
+      <c r="P928" t="inlineStr"/>
+      <c r="Q928" t="inlineStr">
+        <is>
+          <t>Fabrication and characterization of a hydrogen-terminated diamond MOSFET with buried p+ type electrodes formed by ion implantation</t>
+        </is>
+      </c>
+      <c r="R928" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S928" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T928" t="inlineStr"/>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr"/>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C929" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E929" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F929" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G929" t="inlineStr"/>
+      <c r="H929" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I929" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J929" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K929" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L929" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M929" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N929" t="inlineStr"/>
+      <c r="O929" t="inlineStr"/>
+      <c r="P929" t="inlineStr"/>
+      <c r="Q929" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R929" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S929" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T929" t="inlineStr"/>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr"/>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C930" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F930" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G930" t="inlineStr"/>
+      <c r="H930" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I930" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J930" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K930" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L930" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M930" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N930" t="inlineStr"/>
+      <c r="O930" t="inlineStr"/>
+      <c r="P930" t="inlineStr"/>
+      <c r="Q930" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R930" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S930" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T930" t="inlineStr"/>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr"/>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Fabrication and Electrical Characterization of AlGaN/GaN HEMTs with BST Gate Dielectric: A Comparative Study of Two- and Three-Terminal Devices</t>
+        </is>
+      </c>
+      <c r="C931" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E931" t="inlineStr"/>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>., Abdullah</t>
+        </is>
+      </c>
+      <c r="G931" t="inlineStr"/>
+      <c r="H931" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10638750/v1</t>
+        </is>
+      </c>
+      <c r="I931" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10638750/v1</t>
+        </is>
+      </c>
+      <c r="J931" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K931" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L931" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M931" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N931" t="inlineStr"/>
+      <c r="O931" t="inlineStr"/>
+      <c r="P931" t="inlineStr"/>
+      <c r="Q931" t="inlineStr">
+        <is>
+          <t>Fabrication and Electrical Characterization of AlGaN/GaN HEMTs with BST Gate Dielectric: A Comparative Study of Two- and Three-Terminal Devices</t>
+        </is>
+      </c>
+      <c r="R931" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S931" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T931" t="inlineStr"/>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr"/>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C932" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G932" t="inlineStr"/>
+      <c r="H932" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I932" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J932" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K932" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L932" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M932" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N932" t="inlineStr"/>
+      <c r="O932" t="inlineStr"/>
+      <c r="P932" t="inlineStr"/>
+      <c r="Q932" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R932" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S932" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T932" t="inlineStr"/>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr"/>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C933" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F933" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G933" t="inlineStr"/>
+      <c r="H933" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I933" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J933" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K933" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L933" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M933" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N933" t="inlineStr"/>
+      <c r="O933" t="inlineStr"/>
+      <c r="P933" t="inlineStr"/>
+      <c r="Q933" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R933" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S933" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T933" t="inlineStr"/>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr"/>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Sistem Kontrol PLC dan Inverter pada Vacuum Mesin Industri</t>
+        </is>
+      </c>
+      <c r="C934" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>Institute of Advanced Knowledge and Science</t>
+        </is>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>Journal of Engineering and Science Application</t>
+        </is>
+      </c>
+      <c r="F934" t="inlineStr">
+        <is>
+          <t>Budiarjo, Wisnu; Sugiyanto, Didik</t>
+        </is>
+      </c>
+      <c r="G934" t="inlineStr"/>
+      <c r="H934" t="inlineStr">
+        <is>
+          <t>10.69693/jesa.v3i2.42</t>
+        </is>
+      </c>
+      <c r="I934" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.69693/jesa.v3i2.42</t>
+        </is>
+      </c>
+      <c r="J934" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K934" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L934" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M934" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N934" t="inlineStr"/>
+      <c r="O934" t="inlineStr"/>
+      <c r="P934" t="inlineStr"/>
+      <c r="Q934" t="inlineStr">
+        <is>
+          <t>Sistem Kontrol PLC dan Inverter pada Vacuum Mesin Industri</t>
+        </is>
+      </c>
+      <c r="R934" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S934" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T934" t="inlineStr"/>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr"/>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C935" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F935" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G935" t="inlineStr"/>
+      <c r="H935" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I935" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J935" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K935" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L935" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M935" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N935" t="inlineStr"/>
+      <c r="O935" t="inlineStr"/>
+      <c r="P935" t="inlineStr"/>
+      <c r="Q935" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R935" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S935" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T935" t="inlineStr"/>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr"/>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>A Bandgap-Referenced Current-Mode VCSEL Driver in CMOS for Short-Range LiDAR Sensors</t>
+        </is>
+      </c>
+      <c r="C936" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F936" t="inlineStr">
+        <is>
+          <t>Li, Yiyao; Hu, Yu; Park, Sung-Min</t>
+        </is>
+      </c>
+      <c r="G936" t="inlineStr"/>
+      <c r="H936" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15163578</t>
+        </is>
+      </c>
+      <c r="I936" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15163578</t>
+        </is>
+      </c>
+      <c r="J936" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K936" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L936" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M936" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N936" t="inlineStr"/>
+      <c r="O936" t="inlineStr"/>
+      <c r="P936" t="inlineStr"/>
+      <c r="Q936" t="inlineStr">
+        <is>
+          <t>A Bandgap-Referenced Current-Mode VCSEL Driver in CMOS for Short-Range LiDAR Sensors</t>
+        </is>
+      </c>
+      <c r="R936" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S936" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T936" t="inlineStr"/>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr"/>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C937" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F937" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G937" t="inlineStr"/>
+      <c r="H937" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I937" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J937" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K937" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L937" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M937" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N937" t="inlineStr"/>
+      <c r="O937" t="inlineStr"/>
+      <c r="P937" t="inlineStr"/>
+      <c r="Q937" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R937" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S937" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T937" t="inlineStr"/>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr"/>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Fabrication and Electrical Characterization of AlGaN/GaN HEMTs with BST Gate Dielectric: A Comparative Study of Two- and Three-Terminal Devices</t>
+        </is>
+      </c>
+      <c r="C938" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E938" t="inlineStr"/>
+      <c r="F938" t="inlineStr">
+        <is>
+          <t>., Abdullah</t>
+        </is>
+      </c>
+      <c r="G938" t="inlineStr"/>
+      <c r="H938" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10638750/v1</t>
+        </is>
+      </c>
+      <c r="I938" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10638750/v1</t>
+        </is>
+      </c>
+      <c r="J938" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K938" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L938" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M938" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N938" t="inlineStr"/>
+      <c r="O938" t="inlineStr"/>
+      <c r="P938" t="inlineStr"/>
+      <c r="Q938" t="inlineStr">
+        <is>
+          <t>Fabrication and Electrical Characterization of AlGaN/GaN HEMTs with BST Gate Dielectric: A Comparative Study of Two- and Three-Terminal Devices</t>
+        </is>
+      </c>
+      <c r="R938" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S938" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T938" t="inlineStr"/>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr"/>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>Fabrication and Electrical Characterization of AlGaN/GaN HEMTs with BST Gate Dielectric: A Comparative Study of Two- and Three-Terminal Devices</t>
+        </is>
+      </c>
+      <c r="C939" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E939" t="inlineStr"/>
+      <c r="F939" t="inlineStr">
+        <is>
+          <t>., Abdullah</t>
+        </is>
+      </c>
+      <c r="G939" t="inlineStr"/>
+      <c r="H939" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10638750/v1</t>
+        </is>
+      </c>
+      <c r="I939" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10638750/v1</t>
+        </is>
+      </c>
+      <c r="J939" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K939" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L939" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M939" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N939" t="inlineStr"/>
+      <c r="O939" t="inlineStr"/>
+      <c r="P939" t="inlineStr"/>
+      <c r="Q939" t="inlineStr">
+        <is>
+          <t>Fabrication and Electrical Characterization of AlGaN/GaN HEMTs with BST Gate Dielectric: A Comparative Study of Two- and Three-Terminal Devices</t>
+        </is>
+      </c>
+      <c r="R939" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S939" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T939" t="inlineStr"/>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr"/>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="C940" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E940" t="inlineStr">
+        <is>
+          <t>Microelectronics Journal</t>
+        </is>
+      </c>
+      <c r="F940" t="inlineStr">
+        <is>
+          <t>Zhao, Yapeng; Liu, Chengyi; Li, You; Quan, Guoyu; Du, Jiangfeng</t>
+        </is>
+      </c>
+      <c r="G940" t="inlineStr"/>
+      <c r="H940" t="inlineStr">
+        <is>
+          <t>10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="I940" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mejo.2026.107436</t>
+        </is>
+      </c>
+      <c r="J940" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K940" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L940" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M940" t="inlineStr">
+        <is>
+          <t>Electrostatics</t>
+        </is>
+      </c>
+      <c r="N940" t="inlineStr"/>
+      <c r="O940" t="inlineStr"/>
+      <c r="P940" t="inlineStr"/>
+      <c r="Q940" t="inlineStr">
+        <is>
+          <t>Trap-induced gate transient current variation in E-mode p-GaN gate GaN power HEMTs: characterization and physical mechanism</t>
+        </is>
+      </c>
+      <c r="R940" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S940" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="T940" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-13T23:44Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T940"/>
+  <dimension ref="A1:T945"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71546,6 +71546,382 @@
       </c>
       <c r="T940" t="inlineStr"/>
     </row>
+    <row r="941">
+      <c r="A941" t="inlineStr"/>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>Metaheuristic-Based PV–BESS Planning for Radial Distribution Networks with Inverter-Based Voltage Support</t>
+        </is>
+      </c>
+      <c r="C941" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E941" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F941" t="inlineStr">
+        <is>
+          <t>Ceylan, Oğuzhan</t>
+        </is>
+      </c>
+      <c r="G941" t="inlineStr"/>
+      <c r="H941" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15163604</t>
+        </is>
+      </c>
+      <c r="I941" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15163604</t>
+        </is>
+      </c>
+      <c r="J941" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K941" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L941" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M941" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N941" t="inlineStr"/>
+      <c r="O941" t="inlineStr"/>
+      <c r="P941" t="inlineStr"/>
+      <c r="Q941" t="inlineStr">
+        <is>
+          <t>Metaheuristic-Based PV–BESS Planning for Radial Distribution Networks with Inverter-Based Voltage Support</t>
+        </is>
+      </c>
+      <c r="R941" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S941" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="T941" t="inlineStr"/>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr"/>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>Metaheuristic-Based PV–BESS Planning for Radial Distribution Networks with Inverter-Based Voltage Support</t>
+        </is>
+      </c>
+      <c r="C942" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E942" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F942" t="inlineStr">
+        <is>
+          <t>Ceylan, Oğuzhan</t>
+        </is>
+      </c>
+      <c r="G942" t="inlineStr"/>
+      <c r="H942" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15163604</t>
+        </is>
+      </c>
+      <c r="I942" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15163604</t>
+        </is>
+      </c>
+      <c r="J942" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K942" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L942" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M942" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N942" t="inlineStr"/>
+      <c r="O942" t="inlineStr"/>
+      <c r="P942" t="inlineStr"/>
+      <c r="Q942" t="inlineStr">
+        <is>
+          <t>Metaheuristic-Based PV–BESS Planning for Radial Distribution Networks with Inverter-Based Voltage Support</t>
+        </is>
+      </c>
+      <c r="R942" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S942" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="T942" t="inlineStr"/>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr"/>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Inverse Airfoil Design as Constrained Root-Finding: A Monolithic CST-Newton Formulation</t>
+        </is>
+      </c>
+      <c r="C943" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E943" t="inlineStr"/>
+      <c r="F943" t="inlineStr">
+        <is>
+          <t>Sathish, Sharath</t>
+        </is>
+      </c>
+      <c r="G943" t="inlineStr"/>
+      <c r="H943" t="inlineStr">
+        <is>
+          <t>10.20944/preprints202608.0845.v1</t>
+        </is>
+      </c>
+      <c r="I943" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20944/preprints202608.0845.v1</t>
+        </is>
+      </c>
+      <c r="J943" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K943" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L943" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M943" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N943" t="inlineStr"/>
+      <c r="O943" t="inlineStr"/>
+      <c r="P943" t="inlineStr"/>
+      <c r="Q943" t="inlineStr">
+        <is>
+          <t>Inverse Airfoil Design as Constrained Root-Finding: A Monolithic CST-Newton Formulation</t>
+        </is>
+      </c>
+      <c r="R943" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S943" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="T943" t="inlineStr"/>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr"/>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Metaheuristic-Based PV–BESS Planning for Radial Distribution Networks with Inverter-Based Voltage Support</t>
+        </is>
+      </c>
+      <c r="C944" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E944" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F944" t="inlineStr">
+        <is>
+          <t>Ceylan, Oğuzhan</t>
+        </is>
+      </c>
+      <c r="G944" t="inlineStr"/>
+      <c r="H944" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15163604</t>
+        </is>
+      </c>
+      <c r="I944" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15163604</t>
+        </is>
+      </c>
+      <c r="J944" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K944" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L944" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M944" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N944" t="inlineStr"/>
+      <c r="O944" t="inlineStr"/>
+      <c r="P944" t="inlineStr"/>
+      <c r="Q944" t="inlineStr">
+        <is>
+          <t>Metaheuristic-Based PV–BESS Planning for Radial Distribution Networks with Inverter-Based Voltage Support</t>
+        </is>
+      </c>
+      <c r="R944" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S944" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="T944" t="inlineStr"/>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr"/>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Metaheuristic-Based PV–BESS Planning for Radial Distribution Networks with Inverter-Based Voltage Support</t>
+        </is>
+      </c>
+      <c r="C945" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E945" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F945" t="inlineStr">
+        <is>
+          <t>Ceylan, Oğuzhan</t>
+        </is>
+      </c>
+      <c r="G945" t="inlineStr"/>
+      <c r="H945" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15163604</t>
+        </is>
+      </c>
+      <c r="I945" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15163604</t>
+        </is>
+      </c>
+      <c r="J945" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K945" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L945" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M945" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N945" t="inlineStr"/>
+      <c r="O945" t="inlineStr"/>
+      <c r="P945" t="inlineStr"/>
+      <c r="Q945" t="inlineStr">
+        <is>
+          <t>Metaheuristic-Based PV–BESS Planning for Radial Distribution Networks with Inverter-Based Voltage Support</t>
+        </is>
+      </c>
+      <c r="R945" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S945" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="T945" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-14T23:24Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T945"/>
+  <dimension ref="A1:T946"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71922,6 +71922,82 @@
       </c>
       <c r="T945" t="inlineStr"/>
     </row>
+    <row r="946">
+      <c r="A946" t="inlineStr"/>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>A hybrid random forest–ANFIS framework for accurate power estimation in CMOS VLSI circuits</t>
+        </is>
+      </c>
+      <c r="C946" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E946" t="inlineStr">
+        <is>
+          <t>Discover Computing</t>
+        </is>
+      </c>
+      <c r="F946" t="inlineStr">
+        <is>
+          <t>Govindaraj, V.; Sahaya Sheela, M.; Muthu Krishnammal, P.; Hari Kumar, S.; Jayanthi, T.; Shoban Babu, B.</t>
+        </is>
+      </c>
+      <c r="G946" t="inlineStr"/>
+      <c r="H946" t="inlineStr">
+        <is>
+          <t>10.1007/s10791-026-10430-4</t>
+        </is>
+      </c>
+      <c r="I946" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10791-026-10430-4</t>
+        </is>
+      </c>
+      <c r="J946" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K946" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L946" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M946" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N946" t="inlineStr"/>
+      <c r="O946" t="inlineStr"/>
+      <c r="P946" t="inlineStr"/>
+      <c r="Q946" t="inlineStr">
+        <is>
+          <t>A hybrid random forest–ANFIS framework for accurate power estimation in CMOS VLSI circuits</t>
+        </is>
+      </c>
+      <c r="R946" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S946" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="T946" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-17T23:25Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T946"/>
+  <dimension ref="A1:T952"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71998,6 +71998,466 @@
       </c>
       <c r="T946" t="inlineStr"/>
     </row>
+    <row r="947">
+      <c r="A947" t="inlineStr"/>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>RDA-ANN Based Real-Time Selective Harmonic Elimination in Multilevel Inverter Fed by PV Panels</t>
+        </is>
+      </c>
+      <c r="C947" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E947" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F947" t="inlineStr">
+        <is>
+          <t>Karaca, Hulusi; Şahman, Mehmet Akif; Bektaş, Yasin</t>
+        </is>
+      </c>
+      <c r="G947" t="inlineStr"/>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>10.3390/en19163849</t>
+        </is>
+      </c>
+      <c r="I947" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19163849</t>
+        </is>
+      </c>
+      <c r="J947" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K947" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L947" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M947" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N947" t="inlineStr"/>
+      <c r="O947" t="inlineStr"/>
+      <c r="P947" t="inlineStr"/>
+      <c r="Q947" t="inlineStr">
+        <is>
+          <t>RDA-ANN Based Real-Time Selective Harmonic Elimination in Multilevel Inverter Fed by PV Panels</t>
+        </is>
+      </c>
+      <c r="R947" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S947" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="T947" t="inlineStr"/>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr"/>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Monolithic 3D-Printed
+Interdigitated Cement-Based
+Supercapacitors for Structural Energy Storage</t>
+        </is>
+      </c>
+      <c r="C948" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>ACS Nano</t>
+        </is>
+      </c>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>Wu, Haiping; Zhong, Jing; Ren, Wencai</t>
+        </is>
+      </c>
+      <c r="G948" t="inlineStr"/>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>10.1021/acsnano.6c09927</t>
+        </is>
+      </c>
+      <c r="I948" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsnano.6c09927</t>
+        </is>
+      </c>
+      <c r="J948" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K948" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L948" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M948" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N948" t="inlineStr"/>
+      <c r="O948" t="inlineStr"/>
+      <c r="P948" t="inlineStr"/>
+      <c r="Q948" t="inlineStr">
+        <is>
+          <t>Monolithic 3D-Printed
+Interdigitated Cement-Based
+Supercapacitors for Structural Energy Storage</t>
+        </is>
+      </c>
+      <c r="R948" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S948" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="T948" t="inlineStr"/>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr"/>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>RDA-ANN Based Real-Time Selective Harmonic Elimination in Multilevel Inverter Fed by PV Panels</t>
+        </is>
+      </c>
+      <c r="C949" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>Karaca, Hulusi; Şahman, Mehmet Akif; Bektaş, Yasin</t>
+        </is>
+      </c>
+      <c r="G949" t="inlineStr"/>
+      <c r="H949" t="inlineStr">
+        <is>
+          <t>10.3390/en19163849</t>
+        </is>
+      </c>
+      <c r="I949" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19163849</t>
+        </is>
+      </c>
+      <c r="J949" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K949" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L949" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M949" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N949" t="inlineStr"/>
+      <c r="O949" t="inlineStr"/>
+      <c r="P949" t="inlineStr"/>
+      <c r="Q949" t="inlineStr">
+        <is>
+          <t>RDA-ANN Based Real-Time Selective Harmonic Elimination in Multilevel Inverter Fed by PV Panels</t>
+        </is>
+      </c>
+      <c r="R949" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S949" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="T949" t="inlineStr"/>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr"/>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>A CMOS VCII-Based Multi-Waveform Generator with Reduced Harmonic Distortion</t>
+        </is>
+      </c>
+      <c r="C950" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E950" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>Olivieri, Riccardo; Barile, Gianluca; Stornelli, Vincenzo; Ferri, Giuseppe; Minaei, Shahram</t>
+        </is>
+      </c>
+      <c r="G950" t="inlineStr"/>
+      <c r="H950" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15163675</t>
+        </is>
+      </c>
+      <c r="I950" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15163675</t>
+        </is>
+      </c>
+      <c r="J950" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K950" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L950" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M950" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N950" t="inlineStr"/>
+      <c r="O950" t="inlineStr"/>
+      <c r="P950" t="inlineStr"/>
+      <c r="Q950" t="inlineStr">
+        <is>
+          <t>A CMOS VCII-Based Multi-Waveform Generator with Reduced Harmonic Distortion</t>
+        </is>
+      </c>
+      <c r="R950" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S950" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="T950" t="inlineStr"/>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr"/>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Bandgap Engineering of Si-Ge-Sn Alloys for CMOS-Compatible Infrared Optoelectronic Devices</t>
+        </is>
+      </c>
+      <c r="C951" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>EWA Publishing</t>
+        </is>
+      </c>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>Theoretical and Natural Science</t>
+        </is>
+      </c>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>Yuan, Rongbin</t>
+        </is>
+      </c>
+      <c r="G951" t="inlineStr"/>
+      <c r="H951" t="inlineStr">
+        <is>
+          <t>10.54254/2753-8818/2026.gl36171</t>
+        </is>
+      </c>
+      <c r="I951" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54254/2753-8818/2026.gl36171</t>
+        </is>
+      </c>
+      <c r="J951" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K951" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L951" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M951" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N951" t="inlineStr"/>
+      <c r="O951" t="inlineStr"/>
+      <c r="P951" t="inlineStr"/>
+      <c r="Q951" t="inlineStr">
+        <is>
+          <t>Bandgap Engineering of Si-Ge-Sn Alloys for CMOS-Compatible Infrared Optoelectronic Devices</t>
+        </is>
+      </c>
+      <c r="R951" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S951" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="T951" t="inlineStr"/>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr"/>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>CMOS-compatible Si/Pd ohmic contact to n-InP for Si photonics</t>
+        </is>
+      </c>
+      <c r="C952" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>Cong, Riyu; Ouyang, Wenyuan; Li, Hao; Li, Yanping; Xu, Wanjin; Ran, Guangzhao</t>
+        </is>
+      </c>
+      <c r="G952" t="inlineStr"/>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae9317</t>
+        </is>
+      </c>
+      <c r="I952" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae9317</t>
+        </is>
+      </c>
+      <c r="J952" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K952" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L952" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M952" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N952" t="inlineStr"/>
+      <c r="O952" t="inlineStr"/>
+      <c r="P952" t="inlineStr"/>
+      <c r="Q952" t="inlineStr">
+        <is>
+          <t>CMOS-compatible Si/Pd ohmic contact to n-InP for Si photonics</t>
+        </is>
+      </c>
+      <c r="R952" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S952" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="T952" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-18T23:25Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T952"/>
+  <dimension ref="A1:T954"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72458,6 +72458,158 @@
       </c>
       <c r="T952" t="inlineStr"/>
     </row>
+    <row r="953">
+      <c r="A953" t="inlineStr"/>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Mitigation of Dead-Time Voltage Spikes in High-Frequency WPT Inverters: A Comparative Study of GaN HEMT and Si IGBT Technologies</t>
+        </is>
+      </c>
+      <c r="C953" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>Bogdanović, Miroslav; Despotović, Živadin; Marčetić, Darko; Herceg, Dejana; Popadić, Bane; Brkić, Miodrag; Batinić, Branislav; Rajs, Vladimir M.</t>
+        </is>
+      </c>
+      <c r="G953" t="inlineStr"/>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15163688</t>
+        </is>
+      </c>
+      <c r="I953" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15163688</t>
+        </is>
+      </c>
+      <c r="J953" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K953" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L953" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M953" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N953" t="inlineStr"/>
+      <c r="O953" t="inlineStr"/>
+      <c r="P953" t="inlineStr"/>
+      <c r="Q953" t="inlineStr">
+        <is>
+          <t>Mitigation of Dead-Time Voltage Spikes in High-Frequency WPT Inverters: A Comparative Study of GaN HEMT and Si IGBT Technologies</t>
+        </is>
+      </c>
+      <c r="R953" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S953" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="T953" t="inlineStr"/>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr"/>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Logic and SRAM design co-optimization for A7 monolithic CFETs using backside gate contact-enabled hybrid power delivery</t>
+        </is>
+      </c>
+      <c r="C954" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E954" t="inlineStr">
+        <is>
+          <t>Microelectronic Engineering</t>
+        </is>
+      </c>
+      <c r="F954" t="inlineStr">
+        <is>
+          <t>He, Hao; Xu, Lijun; Ma, Xiaoning; An, Kunlong; Jia, Yuntian; Zhang, Yajia; Li, Zhiqiang; Liu, Jianyun; Cao, He; Wu, Zhenhua; Xu, Qinzhi</t>
+        </is>
+      </c>
+      <c r="G954" t="inlineStr"/>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>10.1016/j.mee.2026.112501</t>
+        </is>
+      </c>
+      <c r="I954" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.mee.2026.112501</t>
+        </is>
+      </c>
+      <c r="J954" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K954" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L954" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M954" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N954" t="inlineStr"/>
+      <c r="O954" t="inlineStr"/>
+      <c r="P954" t="inlineStr"/>
+      <c r="Q954" t="inlineStr">
+        <is>
+          <t>Logic and SRAM design co-optimization for A7 monolithic CFETs using backside gate contact-enabled hybrid power delivery</t>
+        </is>
+      </c>
+      <c r="R954" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S954" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="T954" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-19T23:25Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T954"/>
+  <dimension ref="A1:T963"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72610,6 +72610,690 @@
       </c>
       <c r="T954" t="inlineStr"/>
     </row>
+    <row r="955">
+      <c r="A955" t="inlineStr"/>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Experimental evaluation of reduced component nine -level switched capacitor boost inverter with self-balancing capacitors</t>
+        </is>
+      </c>
+      <c r="C955" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>Arun, Vijayakumar; K, Saravanan; Kumar, Tharwin</t>
+        </is>
+      </c>
+      <c r="G955" t="inlineStr"/>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae9b68</t>
+        </is>
+      </c>
+      <c r="I955" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae9b68</t>
+        </is>
+      </c>
+      <c r="J955" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K955" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L955" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M955" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N955" t="inlineStr"/>
+      <c r="O955" t="inlineStr"/>
+      <c r="P955" t="inlineStr"/>
+      <c r="Q955" t="inlineStr">
+        <is>
+          <t>Experimental evaluation of reduced component nine -level switched capacitor boost inverter with self-balancing capacitors</t>
+        </is>
+      </c>
+      <c r="R955" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S955" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="T955" t="inlineStr"/>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr"/>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Dynamic Fault Detection and Protection Strategies for Medium-Voltage Networks Supplied by Grid-Forming Inverter Sources</t>
+        </is>
+      </c>
+      <c r="C956" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E956" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>Rauf, Muhammad Abdul; Batool, Munira; Madni, Imtiaz</t>
+        </is>
+      </c>
+      <c r="G956" t="inlineStr"/>
+      <c r="H956" t="inlineStr">
+        <is>
+          <t>10.3390/en19163897</t>
+        </is>
+      </c>
+      <c r="I956" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19163897</t>
+        </is>
+      </c>
+      <c r="J956" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K956" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L956" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M956" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N956" t="inlineStr"/>
+      <c r="O956" t="inlineStr"/>
+      <c r="P956" t="inlineStr"/>
+      <c r="Q956" t="inlineStr">
+        <is>
+          <t>Dynamic Fault Detection and Protection Strategies for Medium-Voltage Networks Supplied by Grid-Forming Inverter Sources</t>
+        </is>
+      </c>
+      <c r="R956" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S956" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="T956" t="inlineStr"/>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr"/>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Proof of concept for IR-SOIPIX, a monolithic midinfrared image sensor fabricated using a standard CMOS process</t>
+        </is>
+      </c>
+      <c r="C957" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>SPIE</t>
+        </is>
+      </c>
+      <c r="E957" t="inlineStr">
+        <is>
+          <t>X-Ray, Optical, and Infrared Detectors for Astronomy XII</t>
+        </is>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>Wada, Takehiko; Nakaoka, Toshihiro; Suzuki, Toyoaki; Tanaka, Youta</t>
+        </is>
+      </c>
+      <c r="G957" t="inlineStr"/>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>10.1117/12.3105612</t>
+        </is>
+      </c>
+      <c r="I957" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1117/12.3105612</t>
+        </is>
+      </c>
+      <c r="J957" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K957" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L957" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M957" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N957" t="inlineStr"/>
+      <c r="O957" t="inlineStr"/>
+      <c r="P957" t="inlineStr"/>
+      <c r="Q957" t="inlineStr">
+        <is>
+          <t>Proof of concept for IR-SOIPIX, a monolithic midinfrared image sensor fabricated using a standard CMOS process</t>
+        </is>
+      </c>
+      <c r="R957" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S957" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="T957" t="inlineStr"/>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr"/>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>A Comprehensive Review of MOSFET Switching Loss Modelling Techniques for Power Electronic Converters</t>
+        </is>
+      </c>
+      <c r="C958" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E958" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>Darwish, Ahmed; Rohouma, Wesam</t>
+        </is>
+      </c>
+      <c r="G958" t="inlineStr"/>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15163706</t>
+        </is>
+      </c>
+      <c r="I958" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15163706</t>
+        </is>
+      </c>
+      <c r="J958" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K958" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L958" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M958" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N958" t="inlineStr"/>
+      <c r="O958" t="inlineStr"/>
+      <c r="P958" t="inlineStr"/>
+      <c r="Q958" t="inlineStr">
+        <is>
+          <t>A Comprehensive Review of MOSFET Switching Loss Modelling Techniques for Power Electronic Converters</t>
+        </is>
+      </c>
+      <c r="R958" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S958" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="T958" t="inlineStr"/>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr"/>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>A Comprehensive Review of MOSFET Switching Loss Modelling Techniques for Power Electronic Converters</t>
+        </is>
+      </c>
+      <c r="C959" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>Darwish, Ahmed; Rohouma, Wesam</t>
+        </is>
+      </c>
+      <c r="G959" t="inlineStr"/>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15163706</t>
+        </is>
+      </c>
+      <c r="I959" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15163706</t>
+        </is>
+      </c>
+      <c r="J959" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K959" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L959" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M959" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N959" t="inlineStr"/>
+      <c r="O959" t="inlineStr"/>
+      <c r="P959" t="inlineStr"/>
+      <c r="Q959" t="inlineStr">
+        <is>
+          <t>A Comprehensive Review of MOSFET Switching Loss Modelling Techniques for Power Electronic Converters</t>
+        </is>
+      </c>
+      <c r="R959" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S959" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="T959" t="inlineStr"/>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr"/>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Experimental evaluation of reduced component nine -level switched capacitor boost inverter with self-balancing capacitors</t>
+        </is>
+      </c>
+      <c r="C960" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E960" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F960" t="inlineStr">
+        <is>
+          <t>Arun, Vijayakumar; K, Saravanan; Kumar, Tharwin</t>
+        </is>
+      </c>
+      <c r="G960" t="inlineStr"/>
+      <c r="H960" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/ae9b68</t>
+        </is>
+      </c>
+      <c r="I960" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/ae9b68</t>
+        </is>
+      </c>
+      <c r="J960" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K960" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L960" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M960" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N960" t="inlineStr"/>
+      <c r="O960" t="inlineStr"/>
+      <c r="P960" t="inlineStr"/>
+      <c r="Q960" t="inlineStr">
+        <is>
+          <t>Experimental evaluation of reduced component nine -level switched capacitor boost inverter with self-balancing capacitors</t>
+        </is>
+      </c>
+      <c r="R960" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S960" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="T960" t="inlineStr"/>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr"/>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Dynamic Fault Detection and Protection Strategies for Medium-Voltage Networks Supplied by Grid-Forming Inverter Sources</t>
+        </is>
+      </c>
+      <c r="C961" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E961" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F961" t="inlineStr">
+        <is>
+          <t>Rauf, Muhammad Abdul; Batool, Munira; Madni, Imtiaz</t>
+        </is>
+      </c>
+      <c r="G961" t="inlineStr"/>
+      <c r="H961" t="inlineStr">
+        <is>
+          <t>10.3390/en19163897</t>
+        </is>
+      </c>
+      <c r="I961" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19163897</t>
+        </is>
+      </c>
+      <c r="J961" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K961" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L961" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M961" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N961" t="inlineStr"/>
+      <c r="O961" t="inlineStr"/>
+      <c r="P961" t="inlineStr"/>
+      <c r="Q961" t="inlineStr">
+        <is>
+          <t>Dynamic Fault Detection and Protection Strategies for Medium-Voltage Networks Supplied by Grid-Forming Inverter Sources</t>
+        </is>
+      </c>
+      <c r="R961" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S961" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="T961" t="inlineStr"/>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr"/>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Post-Silicon Timing Characterization of Dynamic Logic Using a Single Ring-Oscillator-Based Test Structure</t>
+        </is>
+      </c>
+      <c r="C962" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>Naksh Solutions</t>
+        </is>
+      </c>
+      <c r="E962" t="inlineStr">
+        <is>
+          <t>International Journal of Advanced Research in Science Communication and Technology</t>
+        </is>
+      </c>
+      <c r="F962" t="inlineStr">
+        <is>
+          <t>A. Baloji, B. Radhika, Varda Manasa, Kammampati Saisri</t>
+        </is>
+      </c>
+      <c r="G962" t="inlineStr"/>
+      <c r="H962" t="inlineStr">
+        <is>
+          <t>10.48175/ijarsct-38082</t>
+        </is>
+      </c>
+      <c r="I962" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48175/ijarsct-38082</t>
+        </is>
+      </c>
+      <c r="J962" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K962" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L962" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M962" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N962" t="inlineStr"/>
+      <c r="O962" t="inlineStr"/>
+      <c r="P962" t="inlineStr"/>
+      <c r="Q962" t="inlineStr">
+        <is>
+          <t>Post-Silicon Timing Characterization of Dynamic Logic Using a Single Ring-Oscillator-Based Test Structure</t>
+        </is>
+      </c>
+      <c r="R962" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S962" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="T962" t="inlineStr"/>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr"/>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>Detection and translation of logic gate images into Boolean functions</t>
+        </is>
+      </c>
+      <c r="C963" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>Institute of Advanced Engineering and Science</t>
+        </is>
+      </c>
+      <c r="E963" t="inlineStr">
+        <is>
+          <t>Computer Science and Information Technologies</t>
+        </is>
+      </c>
+      <c r="F963" t="inlineStr">
+        <is>
+          <t>Taqiyyuddin, Muhammad Shidqii; Subali, Muhammad</t>
+        </is>
+      </c>
+      <c r="G963" t="inlineStr"/>
+      <c r="H963" t="inlineStr">
+        <is>
+          <t>10.11591/csit.v7i3.p346-352</t>
+        </is>
+      </c>
+      <c r="I963" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.11591/csit.v7i3.p346-352</t>
+        </is>
+      </c>
+      <c r="J963" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K963" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L963" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M963" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N963" t="inlineStr"/>
+      <c r="O963" t="inlineStr"/>
+      <c r="P963" t="inlineStr"/>
+      <c r="Q963" t="inlineStr">
+        <is>
+          <t>Detection and translation of logic gate images into Boolean functions</t>
+        </is>
+      </c>
+      <c r="R963" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S963" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="T963" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-20T23:28Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T963"/>
+  <dimension ref="A1:T967"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -73294,6 +73294,310 @@
       </c>
       <c r="T963" t="inlineStr"/>
     </row>
+    <row r="964">
+      <c r="A964" t="inlineStr"/>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>Optomechanical Response Analysis of a Tunable Monolithic Littrow WDM System Under Different Mechanical Boundary Conditions</t>
+        </is>
+      </c>
+      <c r="C964" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>Bon View Publishing Pte</t>
+        </is>
+      </c>
+      <c r="E964" t="inlineStr">
+        <is>
+          <t>Journal of Optics and Photonics Research</t>
+        </is>
+      </c>
+      <c r="F964" t="inlineStr">
+        <is>
+          <t>Kharazmi, Mehdi; Pottier, Pierre; Ozhikandathil, Jayan; Packirisamy, Muthukumaran</t>
+        </is>
+      </c>
+      <c r="G964" t="inlineStr"/>
+      <c r="H964" t="inlineStr">
+        <is>
+          <t>10.47852/bonviewjopr62029619</t>
+        </is>
+      </c>
+      <c r="I964" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.47852/bonviewjopr62029619</t>
+        </is>
+      </c>
+      <c r="J964" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K964" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L964" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M964" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N964" t="inlineStr"/>
+      <c r="O964" t="inlineStr"/>
+      <c r="P964" t="inlineStr"/>
+      <c r="Q964" t="inlineStr">
+        <is>
+          <t>Optomechanical Response Analysis of a Tunable Monolithic Littrow WDM System Under Different Mechanical Boundary Conditions</t>
+        </is>
+      </c>
+      <c r="R964" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S964" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="T964" t="inlineStr"/>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr"/>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Radiation-Induced Charge Trapping Effect in BST/AlGaN/GaN Transistor: Gamma-Ray Dosimeter</t>
+        </is>
+      </c>
+      <c r="C965" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E965" t="inlineStr">
+        <is>
+          <t>ACS Applied Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F965" t="inlineStr">
+        <is>
+          <t>Pandey, Vikas; Gupta, Vishal; Auti, Chaitanya B.; Jingar, Naresh; Kumar, Pradeep; Sahu, Satyajit; Gupta, Ankur; Tripathy, Sudhiranjan; Barala, Surendra Singh; Kumar, Mahesh</t>
+        </is>
+      </c>
+      <c r="G965" t="inlineStr"/>
+      <c r="H965" t="inlineStr">
+        <is>
+          <t>10.1021/acsaelm.6c01298</t>
+        </is>
+      </c>
+      <c r="I965" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsaelm.6c01298</t>
+        </is>
+      </c>
+      <c r="J965" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K965" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L965" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M965" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N965" t="inlineStr"/>
+      <c r="O965" t="inlineStr"/>
+      <c r="P965" t="inlineStr"/>
+      <c r="Q965" t="inlineStr">
+        <is>
+          <t>Radiation-Induced Charge Trapping Effect in BST/AlGaN/GaN Transistor: Gamma-Ray Dosimeter</t>
+        </is>
+      </c>
+      <c r="R965" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S965" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="T965" t="inlineStr"/>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr"/>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>PWM-induced lifetime enhancement in commercial 4H-SiC MOSFET gate oxides and the associated physical mechanisms of interface traps</t>
+        </is>
+      </c>
+      <c r="C966" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E966" t="inlineStr">
+        <is>
+          <t>Journal of Physics D: Applied Physics</t>
+        </is>
+      </c>
+      <c r="F966" t="inlineStr">
+        <is>
+          <t>Yan, Jiahui; Cheng, Faci; Luo, Xi; Liu, Yuebo; Yang, Wen</t>
+        </is>
+      </c>
+      <c r="G966" t="inlineStr"/>
+      <c r="H966" t="inlineStr">
+        <is>
+          <t>10.1088/1361-6463/ae9c4e</t>
+        </is>
+      </c>
+      <c r="I966" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1361-6463/ae9c4e</t>
+        </is>
+      </c>
+      <c r="J966" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K966" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L966" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M966" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N966" t="inlineStr"/>
+      <c r="O966" t="inlineStr"/>
+      <c r="P966" t="inlineStr"/>
+      <c r="Q966" t="inlineStr">
+        <is>
+          <t>PWM-induced lifetime enhancement in commercial 4H-SiC MOSFET gate oxides and the associated physical mechanisms of interface traps</t>
+        </is>
+      </c>
+      <c r="R966" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S966" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="T966" t="inlineStr"/>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr"/>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>Radiation-Induced Charge Trapping Effect in BST/AlGaN/GaN Transistor: Gamma-Ray Dosimeter</t>
+        </is>
+      </c>
+      <c r="C967" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E967" t="inlineStr">
+        <is>
+          <t>ACS Applied Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F967" t="inlineStr">
+        <is>
+          <t>Pandey, Vikas; Gupta, Vishal; Auti, Chaitanya B.; Jingar, Naresh; Kumar, Pradeep; Sahu, Satyajit; Gupta, Ankur; Tripathy, Sudhiranjan; Barala, Surendra Singh; Kumar, Mahesh</t>
+        </is>
+      </c>
+      <c r="G967" t="inlineStr"/>
+      <c r="H967" t="inlineStr">
+        <is>
+          <t>10.1021/acsaelm.6c01298</t>
+        </is>
+      </c>
+      <c r="I967" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acsaelm.6c01298</t>
+        </is>
+      </c>
+      <c r="J967" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K967" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L967" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M967" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N967" t="inlineStr"/>
+      <c r="O967" t="inlineStr"/>
+      <c r="P967" t="inlineStr"/>
+      <c r="Q967" t="inlineStr">
+        <is>
+          <t>Radiation-Induced Charge Trapping Effect in BST/AlGaN/GaN Transistor: Gamma-Ray Dosimeter</t>
+        </is>
+      </c>
+      <c r="R967" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S967" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="T967" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-23T23:24Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T967"/>
+  <dimension ref="A1:T976"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -73598,6 +73598,690 @@
       </c>
       <c r="T967" t="inlineStr"/>
     </row>
+    <row r="968">
+      <c r="A968" t="inlineStr"/>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>The Present Situation, Challenges and Development of CMOS 3D Stacking Technology</t>
+        </is>
+      </c>
+      <c r="C968" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>Darcy &amp; Roy Press Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="E968" t="inlineStr">
+        <is>
+          <t>Highlights in Science, Engineering and Technology</t>
+        </is>
+      </c>
+      <c r="F968" t="inlineStr">
+        <is>
+          <t>Hao, Yijun</t>
+        </is>
+      </c>
+      <c r="G968" t="inlineStr"/>
+      <c r="H968" t="inlineStr">
+        <is>
+          <t>10.54097/33gah778</t>
+        </is>
+      </c>
+      <c r="I968" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54097/33gah778</t>
+        </is>
+      </c>
+      <c r="J968" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K968" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L968" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M968" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N968" t="inlineStr"/>
+      <c r="O968" t="inlineStr"/>
+      <c r="P968" t="inlineStr"/>
+      <c r="Q968" t="inlineStr">
+        <is>
+          <t>The Present Situation, Challenges and Development of CMOS 3D Stacking Technology</t>
+        </is>
+      </c>
+      <c r="R968" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S968" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="T968" t="inlineStr"/>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr"/>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Performance of Monolithic CMOS Pixel Sensors Under X-Rays</t>
+        </is>
+      </c>
+      <c r="C969" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E969" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="F969" t="inlineStr">
+        <is>
+          <t>Ameen, Mohammad Mobassir; Dash, Ganapati; Vijay, Anushree; Chembakan, Theertha; Behera, Prafulla Kumar</t>
+        </is>
+      </c>
+      <c r="G969" t="inlineStr"/>
+      <c r="H969" t="inlineStr">
+        <is>
+          <t>10.3390/physics8030062</t>
+        </is>
+      </c>
+      <c r="I969" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/physics8030062</t>
+        </is>
+      </c>
+      <c r="J969" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K969" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L969" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M969" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N969" t="inlineStr"/>
+      <c r="O969" t="inlineStr"/>
+      <c r="P969" t="inlineStr"/>
+      <c r="Q969" t="inlineStr">
+        <is>
+          <t>Performance of Monolithic CMOS Pixel Sensors Under X-Rays</t>
+        </is>
+      </c>
+      <c r="R969" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S969" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="T969" t="inlineStr"/>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr"/>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Thermal Management of AlGaN/GaN Metal–Insulator–Semiconductor High‐Electron‐Mobility Transistor by AlN Buffer Engineering for Smart Power Chip Technologies</t>
+        </is>
+      </c>
+      <c r="C970" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E970" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F970" t="inlineStr">
+        <is>
+          <t>Jaiswal, Nilesh Kumar; Ebel, Thomas; Sharbati, Samaneh</t>
+        </is>
+      </c>
+      <c r="G970" t="inlineStr"/>
+      <c r="H970" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.70474</t>
+        </is>
+      </c>
+      <c r="I970" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.70474</t>
+        </is>
+      </c>
+      <c r="J970" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K970" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L970" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M970" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N970" t="inlineStr"/>
+      <c r="O970" t="inlineStr"/>
+      <c r="P970" t="inlineStr"/>
+      <c r="Q970" t="inlineStr">
+        <is>
+          <t>Thermal Management of AlGaN/GaN Metal–Insulator–Semiconductor High‐Electron‐Mobility Transistor by AlN Buffer Engineering for Smart Power Chip Technologies</t>
+        </is>
+      </c>
+      <c r="R970" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S970" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="T970" t="inlineStr"/>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr"/>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Response of a Commercial MOSFET to Clinical Photon and Electron Beams Used in Radiotherapy</t>
+        </is>
+      </c>
+      <c r="C971" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>Sociedade Brasileira de Proteção Radiológica - SBPR</t>
+        </is>
+      </c>
+      <c r="E971" t="inlineStr">
+        <is>
+          <t>Brazilian Journal of Radiation Sciences</t>
+        </is>
+      </c>
+      <c r="F971" t="inlineStr">
+        <is>
+          <t>Telles, Luiz Flavio Kalil; Maria, L. M.; Souza, Divanízia N.; Luiz Antonio Pereira dos; Benevides, Clayton Augusto</t>
+        </is>
+      </c>
+      <c r="G971" t="inlineStr"/>
+      <c r="H971" t="inlineStr">
+        <is>
+          <t>10.15392/2319-0612.2026.2995</t>
+        </is>
+      </c>
+      <c r="I971" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.15392/2319-0612.2026.2995</t>
+        </is>
+      </c>
+      <c r="J971" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K971" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L971" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M971" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N971" t="inlineStr"/>
+      <c r="O971" t="inlineStr"/>
+      <c r="P971" t="inlineStr"/>
+      <c r="Q971" t="inlineStr">
+        <is>
+          <t>Response of a Commercial MOSFET to Clinical Photon and Electron Beams Used in Radiotherapy</t>
+        </is>
+      </c>
+      <c r="R971" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S971" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="T971" t="inlineStr"/>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr"/>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>Response of a Commercial MOSFET to Clinical Photon and Electron Beams Used in Radiotherapy</t>
+        </is>
+      </c>
+      <c r="C972" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>Sociedade Brasileira de Proteção Radiológica - SBPR</t>
+        </is>
+      </c>
+      <c r="E972" t="inlineStr">
+        <is>
+          <t>Brazilian Journal of Radiation Sciences</t>
+        </is>
+      </c>
+      <c r="F972" t="inlineStr">
+        <is>
+          <t>Telles, Luiz Flavio Kalil; Maria, L. M.; Souza, Divanízia N.; Luiz Antonio Pereira dos; Benevides, Clayton Augusto</t>
+        </is>
+      </c>
+      <c r="G972" t="inlineStr"/>
+      <c r="H972" t="inlineStr">
+        <is>
+          <t>10.15392/2319-0612.2026.2995</t>
+        </is>
+      </c>
+      <c r="I972" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.15392/2319-0612.2026.2995</t>
+        </is>
+      </c>
+      <c r="J972" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K972" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L972" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M972" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N972" t="inlineStr"/>
+      <c r="O972" t="inlineStr"/>
+      <c r="P972" t="inlineStr"/>
+      <c r="Q972" t="inlineStr">
+        <is>
+          <t>Response of a Commercial MOSFET to Clinical Photon and Electron Beams Used in Radiotherapy</t>
+        </is>
+      </c>
+      <c r="R972" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S972" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="T972" t="inlineStr"/>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr"/>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>The Present Situation, Challenges and Development of CMOS 3D Stacking Technology</t>
+        </is>
+      </c>
+      <c r="C973" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>Darcy &amp; Roy Press Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="E973" t="inlineStr">
+        <is>
+          <t>Highlights in Science, Engineering and Technology</t>
+        </is>
+      </c>
+      <c r="F973" t="inlineStr">
+        <is>
+          <t>Hao, Yijun</t>
+        </is>
+      </c>
+      <c r="G973" t="inlineStr"/>
+      <c r="H973" t="inlineStr">
+        <is>
+          <t>10.54097/33gah778</t>
+        </is>
+      </c>
+      <c r="I973" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.54097/33gah778</t>
+        </is>
+      </c>
+      <c r="J973" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K973" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L973" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M973" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N973" t="inlineStr"/>
+      <c r="O973" t="inlineStr"/>
+      <c r="P973" t="inlineStr"/>
+      <c r="Q973" t="inlineStr">
+        <is>
+          <t>The Present Situation, Challenges and Development of CMOS 3D Stacking Technology</t>
+        </is>
+      </c>
+      <c r="R973" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S973" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="T973" t="inlineStr"/>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr"/>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Emerging Device-Based Hardware Security Primitives: From CMOS PUFs to Ferroelectric and Memristive Technologies</t>
+        </is>
+      </c>
+      <c r="C974" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>World Scientific Pub Co Pte Ltd</t>
+        </is>
+      </c>
+      <c r="E974" t="inlineStr">
+        <is>
+          <t>International Journal of Nanoscience</t>
+        </is>
+      </c>
+      <c r="F974" t="inlineStr">
+        <is>
+          <t>Jha, Rajesh Kumar</t>
+        </is>
+      </c>
+      <c r="G974" t="inlineStr"/>
+      <c r="H974" t="inlineStr">
+        <is>
+          <t>10.1142/s0219581x26400284</t>
+        </is>
+      </c>
+      <c r="I974" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1142/s0219581x26400284</t>
+        </is>
+      </c>
+      <c r="J974" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K974" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L974" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M974" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N974" t="inlineStr"/>
+      <c r="O974" t="inlineStr"/>
+      <c r="P974" t="inlineStr"/>
+      <c r="Q974" t="inlineStr">
+        <is>
+          <t>Emerging Device-Based Hardware Security Primitives: From CMOS PUFs to Ferroelectric and Memristive Technologies</t>
+        </is>
+      </c>
+      <c r="R974" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S974" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="T974" t="inlineStr"/>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr"/>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Thermal Management of AlGaN/GaN Metal–Insulator–Semiconductor High‐Electron‐Mobility Transistor by AlN Buffer Engineering for Smart Power Chip Technologies</t>
+        </is>
+      </c>
+      <c r="C975" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E975" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F975" t="inlineStr">
+        <is>
+          <t>Jaiswal, Nilesh Kumar; Ebel, Thomas; Sharbati, Samaneh</t>
+        </is>
+      </c>
+      <c r="G975" t="inlineStr"/>
+      <c r="H975" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.70474</t>
+        </is>
+      </c>
+      <c r="I975" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.70474</t>
+        </is>
+      </c>
+      <c r="J975" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K975" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L975" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M975" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N975" t="inlineStr"/>
+      <c r="O975" t="inlineStr"/>
+      <c r="P975" t="inlineStr"/>
+      <c r="Q975" t="inlineStr">
+        <is>
+          <t>Thermal Management of AlGaN/GaN Metal–Insulator–Semiconductor High‐Electron‐Mobility Transistor by AlN Buffer Engineering for Smart Power Chip Technologies</t>
+        </is>
+      </c>
+      <c r="R975" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S975" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="T975" t="inlineStr"/>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr"/>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Demonstration of Low-Voltage Lateral Trench Split-Gate Tri-Gate MOSFETs in 4H-SiC</t>
+        </is>
+      </c>
+      <c r="C976" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>The Electrochemical Society</t>
+        </is>
+      </c>
+      <c r="E976" t="inlineStr">
+        <is>
+          <t>ECS Journal of Solid State Science and Technology</t>
+        </is>
+      </c>
+      <c r="F976" t="inlineStr">
+        <is>
+          <t>Kang, Kuan-Min; HU, JIAWEI; Huang, Chih-Fang; Castellazzi, Alberto</t>
+        </is>
+      </c>
+      <c r="G976" t="inlineStr"/>
+      <c r="H976" t="inlineStr">
+        <is>
+          <t>10.1149/2162-8777/ae9ce0</t>
+        </is>
+      </c>
+      <c r="I976" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1149/2162-8777/ae9ce0</t>
+        </is>
+      </c>
+      <c r="J976" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K976" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L976" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M976" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N976" t="inlineStr"/>
+      <c r="O976" t="inlineStr"/>
+      <c r="P976" t="inlineStr"/>
+      <c r="Q976" t="inlineStr">
+        <is>
+          <t>Demonstration of Low-Voltage Lateral Trench Split-Gate Tri-Gate MOSFETs in 4H-SiC</t>
+        </is>
+      </c>
+      <c r="R976" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S976" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="T976" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-24T23:25Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T976"/>
+  <dimension ref="A1:T979"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74282,6 +74282,246 @@
       </c>
       <c r="T976" t="inlineStr"/>
     </row>
+    <row r="977">
+      <c r="A977" t="inlineStr"/>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>BV–Ron,sp Trade-Off Optimization in a Floating-P-Island-Assisted Silicon Shielded-Gate Trench MOSFET</t>
+        </is>
+      </c>
+      <c r="C977" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E977" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F977" t="inlineStr">
+        <is>
+          <t>Han, Zequ; Luo, Juan; Deng, Yunhao; Lin, Zhi; Duan, Yifei; Hu, Shengdong</t>
+        </is>
+      </c>
+      <c r="G977" t="inlineStr"/>
+      <c r="H977" t="inlineStr">
+        <is>
+          <t>10.3390/mi17090999</t>
+        </is>
+      </c>
+      <c r="I977" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17090999</t>
+        </is>
+      </c>
+      <c r="J977" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K977" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L977" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M977" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N977" t="inlineStr"/>
+      <c r="O977" t="inlineStr"/>
+      <c r="P977" t="inlineStr"/>
+      <c r="Q977" t="inlineStr">
+        <is>
+          <t>BV–Ron,sp Trade-Off Optimization in a Floating-P-Island-Assisted Silicon Shielded-Gate Trench MOSFET</t>
+        </is>
+      </c>
+      <c r="R977" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S977" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="T977" t="inlineStr"/>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr"/>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>BV–Ron,sp Trade-Off Optimization in a Floating-P-Island-Assisted Silicon Shielded-Gate Trench MOSFET</t>
+        </is>
+      </c>
+      <c r="C978" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E978" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F978" t="inlineStr">
+        <is>
+          <t>Han, Zequ; Luo, Juan; Deng, Yunhao; Lin, Zhi; Duan, Yifei; Hu, Shengdong</t>
+        </is>
+      </c>
+      <c r="G978" t="inlineStr"/>
+      <c r="H978" t="inlineStr">
+        <is>
+          <t>10.3390/mi17090999</t>
+        </is>
+      </c>
+      <c r="I978" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17090999</t>
+        </is>
+      </c>
+      <c r="J978" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K978" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L978" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M978" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N978" t="inlineStr"/>
+      <c r="O978" t="inlineStr"/>
+      <c r="P978" t="inlineStr"/>
+      <c r="Q978" t="inlineStr">
+        <is>
+          <t>BV–Ron,sp Trade-Off Optimization in a Floating-P-Island-Assisted Silicon Shielded-Gate Trench MOSFET</t>
+        </is>
+      </c>
+      <c r="R978" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S978" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="T978" t="inlineStr"/>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr"/>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Engineered AlGaN/GaN HEMT With
+                    &lt;i&gt;β&lt;/i&gt;
+                    ‐Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    Buffer, Graded AlGaN Back Barrier, and Gate Field Plate for Enhanced Breakdown of 544  V and RF Performance of 110  GHz</t>
+        </is>
+      </c>
+      <c r="C979" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E979" t="inlineStr">
+        <is>
+          <t>physica status solidi (a)</t>
+        </is>
+      </c>
+      <c r="F979" t="inlineStr">
+        <is>
+          <t>Prakash, Ellapu Bhanu; Bordoloi, Sushanta</t>
+        </is>
+      </c>
+      <c r="G979" t="inlineStr"/>
+      <c r="H979" t="inlineStr">
+        <is>
+          <t>10.1002/pssa.70496</t>
+        </is>
+      </c>
+      <c r="I979" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pssa.70496</t>
+        </is>
+      </c>
+      <c r="J979" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K979" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L979" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M979" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N979" t="inlineStr"/>
+      <c r="O979" t="inlineStr"/>
+      <c r="P979" t="inlineStr"/>
+      <c r="Q979" t="inlineStr">
+        <is>
+          <t>Engineered AlGaN/GaN HEMT With
+                    &lt;i&gt;β&lt;/i&gt;
+                    ‐Ga
+                    &lt;sub&gt;2&lt;/sub&gt;
+                    O
+                    &lt;sub&gt;3&lt;/sub&gt;
+                    Buffer, Graded AlGaN Back Barrier, and Gate Field Plate for Enhanced Breakdown of 544  V and RF Performance of 110  GHz</t>
+        </is>
+      </c>
+      <c r="R979" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S979" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="T979" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-25T23:27Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T979"/>
+  <dimension ref="A1:T996"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74522,6 +74522,1298 @@
       </c>
       <c r="T979" t="inlineStr"/>
     </row>
+    <row r="980">
+      <c r="A980" t="inlineStr"/>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C980" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E980" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F980" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G980" t="inlineStr"/>
+      <c r="H980" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I980" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J980" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K980" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L980" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M980" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N980" t="inlineStr"/>
+      <c r="O980" t="inlineStr"/>
+      <c r="P980" t="inlineStr"/>
+      <c r="Q980" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R980" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S980" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T980" t="inlineStr"/>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr"/>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C981" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E981" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F981" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G981" t="inlineStr"/>
+      <c r="H981" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I981" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J981" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K981" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L981" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M981" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N981" t="inlineStr"/>
+      <c r="O981" t="inlineStr"/>
+      <c r="P981" t="inlineStr"/>
+      <c r="Q981" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R981" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S981" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T981" t="inlineStr"/>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr"/>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C982" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E982" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F982" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G982" t="inlineStr"/>
+      <c r="H982" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I982" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J982" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K982" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L982" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M982" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N982" t="inlineStr"/>
+      <c r="O982" t="inlineStr"/>
+      <c r="P982" t="inlineStr"/>
+      <c r="Q982" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R982" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S982" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T982" t="inlineStr"/>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr"/>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Temperature dependence of on-resistance components in recessed p-Channel GaN MOSFETs</t>
+        </is>
+      </c>
+      <c r="C983" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E983" t="inlineStr">
+        <is>
+          <t>Solid-State Electronics</t>
+        </is>
+      </c>
+      <c r="F983" t="inlineStr">
+        <is>
+          <t>Kim, Seung-Su; Kim, Hyun-Seop; Cha, Ho-Young</t>
+        </is>
+      </c>
+      <c r="G983" t="inlineStr"/>
+      <c r="H983" t="inlineStr">
+        <is>
+          <t>10.1016/j.sse.2026.109407</t>
+        </is>
+      </c>
+      <c r="I983" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.sse.2026.109407</t>
+        </is>
+      </c>
+      <c r="J983" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K983" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L983" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M983" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N983" t="inlineStr"/>
+      <c r="O983" t="inlineStr"/>
+      <c r="P983" t="inlineStr"/>
+      <c r="Q983" t="inlineStr">
+        <is>
+          <t>Temperature dependence of on-resistance components in recessed p-Channel GaN MOSFETs</t>
+        </is>
+      </c>
+      <c r="R983" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S983" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T983" t="inlineStr"/>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr"/>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C984" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F984" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G984" t="inlineStr"/>
+      <c r="H984" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I984" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J984" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K984" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L984" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M984" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N984" t="inlineStr"/>
+      <c r="O984" t="inlineStr"/>
+      <c r="P984" t="inlineStr"/>
+      <c r="Q984" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R984" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S984" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T984" t="inlineStr"/>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr"/>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C985" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F985" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G985" t="inlineStr"/>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I985" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J985" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K985" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L985" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M985" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N985" t="inlineStr"/>
+      <c r="O985" t="inlineStr"/>
+      <c r="P985" t="inlineStr"/>
+      <c r="Q985" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R985" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S985" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T985" t="inlineStr"/>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr"/>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Temperature dependence of on-resistance components in recessed p-Channel GaN MOSFETs</t>
+        </is>
+      </c>
+      <c r="C986" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>Solid-State Electronics</t>
+        </is>
+      </c>
+      <c r="F986" t="inlineStr">
+        <is>
+          <t>Kim, Seung-Su; Kim, Hyun-Seop; Cha, Ho-Young</t>
+        </is>
+      </c>
+      <c r="G986" t="inlineStr"/>
+      <c r="H986" t="inlineStr">
+        <is>
+          <t>10.1016/j.sse.2026.109407</t>
+        </is>
+      </c>
+      <c r="I986" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.sse.2026.109407</t>
+        </is>
+      </c>
+      <c r="J986" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K986" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L986" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M986" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N986" t="inlineStr"/>
+      <c r="O986" t="inlineStr"/>
+      <c r="P986" t="inlineStr"/>
+      <c r="Q986" t="inlineStr">
+        <is>
+          <t>Temperature dependence of on-resistance components in recessed p-Channel GaN MOSFETs</t>
+        </is>
+      </c>
+      <c r="R986" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S986" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T986" t="inlineStr"/>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr"/>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C987" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E987" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F987" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G987" t="inlineStr"/>
+      <c r="H987" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I987" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J987" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K987" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L987" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M987" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N987" t="inlineStr"/>
+      <c r="O987" t="inlineStr"/>
+      <c r="P987" t="inlineStr"/>
+      <c r="Q987" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R987" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S987" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T987" t="inlineStr"/>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr"/>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C988" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G988" t="inlineStr"/>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J988" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K988" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L988" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M988" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N988" t="inlineStr"/>
+      <c r="O988" t="inlineStr"/>
+      <c r="P988" t="inlineStr"/>
+      <c r="Q988" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R988" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S988" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T988" t="inlineStr"/>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr"/>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C989" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G989" t="inlineStr"/>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I989" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J989" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K989" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L989" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M989" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N989" t="inlineStr"/>
+      <c r="O989" t="inlineStr"/>
+      <c r="P989" t="inlineStr"/>
+      <c r="Q989" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R989" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S989" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T989" t="inlineStr"/>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr"/>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C990" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G990" t="inlineStr"/>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I990" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J990" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K990" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L990" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M990" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N990" t="inlineStr"/>
+      <c r="O990" t="inlineStr"/>
+      <c r="P990" t="inlineStr"/>
+      <c r="Q990" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R990" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S990" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T990" t="inlineStr"/>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr"/>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>A Standalone GaN HEMT‐Based pH Sensing System for Agricultural, Industrial, and Biomedical Applications</t>
+        </is>
+      </c>
+      <c r="C991" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>Advanced Materials Technologies</t>
+        </is>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>Thakur, Rajiv; Saini, Anil Kumar; Suri, Nikhil; Kharbanda, Dheeraj Kumar; Chaturvedi, Nidhi</t>
+        </is>
+      </c>
+      <c r="G991" t="inlineStr"/>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>10.1002/admt.71259</t>
+        </is>
+      </c>
+      <c r="I991" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/admt.71259</t>
+        </is>
+      </c>
+      <c r="J991" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K991" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L991" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M991" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N991" t="inlineStr"/>
+      <c r="O991" t="inlineStr"/>
+      <c r="P991" t="inlineStr"/>
+      <c r="Q991" t="inlineStr">
+        <is>
+          <t>A Standalone GaN HEMT‐Based pH Sensing System for Agricultural, Industrial, and Biomedical Applications</t>
+        </is>
+      </c>
+      <c r="R991" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S991" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T991" t="inlineStr"/>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr"/>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C992" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G992" t="inlineStr"/>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I992" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J992" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K992" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L992" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M992" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N992" t="inlineStr"/>
+      <c r="O992" t="inlineStr"/>
+      <c r="P992" t="inlineStr"/>
+      <c r="Q992" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R992" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S992" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T992" t="inlineStr"/>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr"/>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C993" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G993" t="inlineStr"/>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J993" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K993" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L993" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M993" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N993" t="inlineStr"/>
+      <c r="O993" t="inlineStr"/>
+      <c r="P993" t="inlineStr"/>
+      <c r="Q993" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R993" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S993" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T993" t="inlineStr"/>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr"/>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="C994" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>Physica Scripta</t>
+        </is>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>P, Muthu Subramanian; Subhashini, T; Daniel, Jackson; Natarajan, Ramkumar</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr"/>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="I994" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1402-4896/ae9e94</t>
+        </is>
+      </c>
+      <c r="J994" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K994" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L994" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M994" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N994" t="inlineStr"/>
+      <c r="O994" t="inlineStr"/>
+      <c r="P994" t="inlineStr"/>
+      <c r="Q994" t="inlineStr">
+        <is>
+          <t>Impact of Doped AlGaN and GaN Buffer Layers on the Performance of AlGaN/GaN HEMTs for RF Applications</t>
+        </is>
+      </c>
+      <c r="R994" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S994" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T994" t="inlineStr"/>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr"/>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Temperature dependence of on-resistance components in recessed p-Channel GaN MOSFETs</t>
+        </is>
+      </c>
+      <c r="C995" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>Solid-State Electronics</t>
+        </is>
+      </c>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>Kim, Seung-Su; Kim, Hyun-Seop; Cha, Ho-Young</t>
+        </is>
+      </c>
+      <c r="G995" t="inlineStr"/>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>10.1016/j.sse.2026.109407</t>
+        </is>
+      </c>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.sse.2026.109407</t>
+        </is>
+      </c>
+      <c r="J995" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K995" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L995" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M995" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N995" t="inlineStr"/>
+      <c r="O995" t="inlineStr"/>
+      <c r="P995" t="inlineStr"/>
+      <c r="Q995" t="inlineStr">
+        <is>
+          <t>Temperature dependence of on-resistance components in recessed p-Channel GaN MOSFETs</t>
+        </is>
+      </c>
+      <c r="R995" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S995" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T995" t="inlineStr"/>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr"/>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>Temperature dependence of on-resistance components in recessed p-Channel GaN MOSFETs</t>
+        </is>
+      </c>
+      <c r="C996" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>Solid-State Electronics</t>
+        </is>
+      </c>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>Kim, Seung-Su; Kim, Hyun-Seop; Cha, Ho-Young</t>
+        </is>
+      </c>
+      <c r="G996" t="inlineStr"/>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>10.1016/j.sse.2026.109407</t>
+        </is>
+      </c>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.sse.2026.109407</t>
+        </is>
+      </c>
+      <c r="J996" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K996" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L996" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M996" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N996" t="inlineStr"/>
+      <c r="O996" t="inlineStr"/>
+      <c r="P996" t="inlineStr"/>
+      <c r="Q996" t="inlineStr">
+        <is>
+          <t>Temperature dependence of on-resistance components in recessed p-Channel GaN MOSFETs</t>
+        </is>
+      </c>
+      <c r="R996" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S996" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="T996" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-27T04:24Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T996"/>
+  <dimension ref="A1:T1002"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75814,6 +75814,450 @@
       </c>
       <c r="T996" t="inlineStr"/>
     </row>
+    <row r="997">
+      <c r="A997" t="inlineStr"/>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Physics-Informed Closed-Loop Python–OpenDSS Co-Simulation for Fault Detection and Localization in Inverter-Dominated Microgrids</t>
+        </is>
+      </c>
+      <c r="C997" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr"/>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>Nante, Zukisa Emerson; Wang, Zenghui</t>
+        </is>
+      </c>
+      <c r="G997" t="inlineStr"/>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>10.20944/preprints202608.1890.v1</t>
+        </is>
+      </c>
+      <c r="I997" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20944/preprints202608.1890.v1</t>
+        </is>
+      </c>
+      <c r="J997" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K997" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L997" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M997" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N997" t="inlineStr"/>
+      <c r="O997" t="inlineStr"/>
+      <c r="P997" t="inlineStr"/>
+      <c r="Q997" t="inlineStr">
+        <is>
+          <t>Physics-Informed Closed-Loop Python–OpenDSS Co-Simulation for Fault Detection and Localization in Inverter-Dominated Microgrids</t>
+        </is>
+      </c>
+      <c r="R997" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S997" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="T997" t="inlineStr"/>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr"/>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Constraint-Aware Framework for Inertia–Security Boundary Extraction in Grid-Forming Inverter-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="C998" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>Matsila, Hulisani T.; Bokoro, Pitshou Ntambu</t>
+        </is>
+      </c>
+      <c r="G998" t="inlineStr"/>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>10.3390/en19174002</t>
+        </is>
+      </c>
+      <c r="I998" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19174002</t>
+        </is>
+      </c>
+      <c r="J998" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K998" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L998" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M998" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N998" t="inlineStr"/>
+      <c r="O998" t="inlineStr"/>
+      <c r="P998" t="inlineStr"/>
+      <c r="Q998" t="inlineStr">
+        <is>
+          <t>Constraint-Aware Framework for Inertia–Security Boundary Extraction in Grid-Forming Inverter-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="R998" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S998" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="T998" t="inlineStr"/>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr"/>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Physics-Informed Closed-Loop Python–OpenDSS Co-Simulation for Fault Detection and Localization in Inverter-Dominated Microgrids</t>
+        </is>
+      </c>
+      <c r="C999" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr"/>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>Nante, Zukisa Emerson; Wang, Zenghui</t>
+        </is>
+      </c>
+      <c r="G999" t="inlineStr"/>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>10.20944/preprints202608.1890.v1</t>
+        </is>
+      </c>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20944/preprints202608.1890.v1</t>
+        </is>
+      </c>
+      <c r="J999" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K999" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L999" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M999" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N999" t="inlineStr"/>
+      <c r="O999" t="inlineStr"/>
+      <c r="P999" t="inlineStr"/>
+      <c r="Q999" t="inlineStr">
+        <is>
+          <t>Physics-Informed Closed-Loop Python–OpenDSS Co-Simulation for Fault Detection and Localization in Inverter-Dominated Microgrids</t>
+        </is>
+      </c>
+      <c r="R999" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S999" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="T999" t="inlineStr"/>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr"/>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Constraint-Aware Framework for Inertia–Security Boundary Extraction in Grid-Forming Inverter-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="C1000" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>Matsila, Hulisani T.; Bokoro, Pitshou Ntambu</t>
+        </is>
+      </c>
+      <c r="G1000" t="inlineStr"/>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>10.3390/en19174002</t>
+        </is>
+      </c>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en19174002</t>
+        </is>
+      </c>
+      <c r="J1000" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1000" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1000" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1000" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1000" t="inlineStr"/>
+      <c r="O1000" t="inlineStr"/>
+      <c r="P1000" t="inlineStr"/>
+      <c r="Q1000" t="inlineStr">
+        <is>
+          <t>Constraint-Aware Framework for Inertia–Security Boundary Extraction in Grid-Forming Inverter-Dominated Power Systems</t>
+        </is>
+      </c>
+      <c r="R1000" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1000" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="T1000" t="inlineStr"/>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr"/>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Physics-Informed Closed-Loop Python–OpenDSS Co-Simulation for Fault Detection and Localization in Inverter-Dominated Microgrids</t>
+        </is>
+      </c>
+      <c r="C1001" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr"/>
+      <c r="F1001" t="inlineStr">
+        <is>
+          <t>Nante, Zukisa Emerson; Wang, Zenghui</t>
+        </is>
+      </c>
+      <c r="G1001" t="inlineStr"/>
+      <c r="H1001" t="inlineStr">
+        <is>
+          <t>10.20944/preprints202608.1890.v1</t>
+        </is>
+      </c>
+      <c r="I1001" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20944/preprints202608.1890.v1</t>
+        </is>
+      </c>
+      <c r="J1001" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1001" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1001" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1001" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1001" t="inlineStr"/>
+      <c r="O1001" t="inlineStr"/>
+      <c r="P1001" t="inlineStr"/>
+      <c r="Q1001" t="inlineStr">
+        <is>
+          <t>Physics-Informed Closed-Loop Python–OpenDSS Co-Simulation for Fault Detection and Localization in Inverter-Dominated Microgrids</t>
+        </is>
+      </c>
+      <c r="R1001" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1001" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="T1001" t="inlineStr"/>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr"/>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Noise-shaped synchrony in neuronal oscillator networks</t>
+        </is>
+      </c>
+      <c r="C1002" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>American Physical Society (APS)</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>Physical Review E</t>
+        </is>
+      </c>
+      <c r="F1002" t="inlineStr">
+        <is>
+          <t>Contreras, Max; Hövel, Philipp</t>
+        </is>
+      </c>
+      <c r="G1002" t="inlineStr"/>
+      <c r="H1002" t="inlineStr">
+        <is>
+          <t>10.1103/sxl4-6mdm</t>
+        </is>
+      </c>
+      <c r="I1002" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1103/sxl4-6mdm</t>
+        </is>
+      </c>
+      <c r="J1002" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1002" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1002" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1002" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N1002" t="inlineStr"/>
+      <c r="O1002" t="inlineStr"/>
+      <c r="P1002" t="inlineStr"/>
+      <c r="Q1002" t="inlineStr">
+        <is>
+          <t>Noise-shaped synchrony in neuronal oscillator networks</t>
+        </is>
+      </c>
+      <c r="R1002" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1002" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="T1002" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-28T06:49Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1002"/>
+  <dimension ref="A1:T1013"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76258,6 +76258,830 @@
       </c>
       <c r="T1002" t="inlineStr"/>
     </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr"/>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>A 95.3% Efficiency APT/AET/SPT Multimode Multiband CMOS/GaN Envelope Tracking for 6G-Oriented Systems</t>
+        </is>
+      </c>
+      <c r="C1003" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>IEEE Journal of Solid-State Circuits</t>
+        </is>
+      </c>
+      <c r="F1003" t="inlineStr">
+        <is>
+          <t>Chen, Chun-Yuan; Huang, Yi-Chun; Chen, Ke-Horng; Lin, Ying-Hsi; Lin, Shian-Ru; Tsai, Tsung-Yen</t>
+        </is>
+      </c>
+      <c r="G1003" t="inlineStr"/>
+      <c r="H1003" t="inlineStr">
+        <is>
+          <t>10.1109/jssc.2026.3681319</t>
+        </is>
+      </c>
+      <c r="I1003" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/jssc.2026.3681319</t>
+        </is>
+      </c>
+      <c r="J1003" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1003" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1003" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1003" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1003" t="inlineStr"/>
+      <c r="O1003" t="inlineStr"/>
+      <c r="P1003" t="inlineStr"/>
+      <c r="Q1003" t="inlineStr">
+        <is>
+          <t>A 95.3% Efficiency APT/AET/SPT Multimode Multiband CMOS/GaN Envelope Tracking for 6G-Oriented Systems</t>
+        </is>
+      </c>
+      <c r="R1003" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1003" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1003" t="inlineStr"/>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr"/>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Stability-Constrained Decentralized Control and Energy Management for Grid-Forming Inverter-Based Microgrids</t>
+        </is>
+      </c>
+      <c r="C1004" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr"/>
+      <c r="F1004" t="inlineStr">
+        <is>
+          <t>Bagdadee, Amam Hossain; Mamoon, Ishtiak Al; Dewi, Deshinta Arrova; Islam, A. K.M. Muzahidul; Zhang, Li</t>
+        </is>
+      </c>
+      <c r="G1004" t="inlineStr"/>
+      <c r="H1004" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10601339/v1</t>
+        </is>
+      </c>
+      <c r="I1004" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10601339/v1</t>
+        </is>
+      </c>
+      <c r="J1004" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1004" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1004" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1004" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1004" t="inlineStr"/>
+      <c r="O1004" t="inlineStr"/>
+      <c r="P1004" t="inlineStr"/>
+      <c r="Q1004" t="inlineStr">
+        <is>
+          <t>Stability-Constrained Decentralized Control and Energy Management for Grid-Forming Inverter-Based Microgrids</t>
+        </is>
+      </c>
+      <c r="R1004" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1004" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1004" t="inlineStr"/>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr"/>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>A 95.3% Efficiency APT/AET/SPT Multimode Multiband CMOS/GaN Envelope Tracking for 6G-Oriented Systems</t>
+        </is>
+      </c>
+      <c r="C1005" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>IEEE Journal of Solid-State Circuits</t>
+        </is>
+      </c>
+      <c r="F1005" t="inlineStr">
+        <is>
+          <t>Chen, Chun-Yuan; Huang, Yi-Chun; Chen, Ke-Horng; Lin, Ying-Hsi; Lin, Shian-Ru; Tsai, Tsung-Yen</t>
+        </is>
+      </c>
+      <c r="G1005" t="inlineStr"/>
+      <c r="H1005" t="inlineStr">
+        <is>
+          <t>10.1109/jssc.2026.3681319</t>
+        </is>
+      </c>
+      <c r="I1005" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/jssc.2026.3681319</t>
+        </is>
+      </c>
+      <c r="J1005" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1005" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1005" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1005" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1005" t="inlineStr"/>
+      <c r="O1005" t="inlineStr"/>
+      <c r="P1005" t="inlineStr"/>
+      <c r="Q1005" t="inlineStr">
+        <is>
+          <t>A 95.3% Efficiency APT/AET/SPT Multimode Multiband CMOS/GaN Envelope Tracking for 6G-Oriented Systems</t>
+        </is>
+      </c>
+      <c r="R1005" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1005" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1005" t="inlineStr"/>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr"/>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Quasi-Vertical GaN-Based Trench Gate MOSFETs Treated with Fluorine-Plasma</t>
+        </is>
+      </c>
+      <c r="C1006" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F1006" t="inlineStr">
+        <is>
+          <t>Zhang, Peng; Li, Dong-Yang; Xu, Jia-Rui; Chang, Qing-Yuan; Hou, Bin; Xi, He; Ma, Xiao-Hua</t>
+        </is>
+      </c>
+      <c r="G1006" t="inlineStr"/>
+      <c r="H1006" t="inlineStr">
+        <is>
+          <t>10.3390/mi17091019</t>
+        </is>
+      </c>
+      <c r="I1006" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17091019</t>
+        </is>
+      </c>
+      <c r="J1006" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1006" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1006" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1006" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1006" t="inlineStr"/>
+      <c r="O1006" t="inlineStr"/>
+      <c r="P1006" t="inlineStr"/>
+      <c r="Q1006" t="inlineStr">
+        <is>
+          <t>Quasi-Vertical GaN-Based Trench Gate MOSFETs Treated with Fluorine-Plasma</t>
+        </is>
+      </c>
+      <c r="R1006" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1006" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1006" t="inlineStr"/>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr"/>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Stability-Constrained Decentralized Control and Energy Management for Grid-Forming Inverter-Based Microgrids</t>
+        </is>
+      </c>
+      <c r="C1007" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr"/>
+      <c r="F1007" t="inlineStr">
+        <is>
+          <t>Bagdadee, Amam Hossain; Mamoon, Ishtiak Al; Dewi, Deshinta Arrova; Islam, A. K.M. Muzahidul; Zhang, Li</t>
+        </is>
+      </c>
+      <c r="G1007" t="inlineStr"/>
+      <c r="H1007" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10601339/v1</t>
+        </is>
+      </c>
+      <c r="I1007" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10601339/v1</t>
+        </is>
+      </c>
+      <c r="J1007" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1007" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1007" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1007" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1007" t="inlineStr"/>
+      <c r="O1007" t="inlineStr"/>
+      <c r="P1007" t="inlineStr"/>
+      <c r="Q1007" t="inlineStr">
+        <is>
+          <t>Stability-Constrained Decentralized Control and Energy Management for Grid-Forming Inverter-Based Microgrids</t>
+        </is>
+      </c>
+      <c r="R1007" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1007" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1007" t="inlineStr"/>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr"/>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>System-level modeling and energy-performance assessment of frosting in inverter-driven air-source heat pumps under constant-heating-capacity operation</t>
+        </is>
+      </c>
+      <c r="C1008" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F1008" t="inlineStr">
+        <is>
+          <t>Sezen, Kutbay</t>
+        </is>
+      </c>
+      <c r="G1008" t="inlineStr"/>
+      <c r="H1008" t="inlineStr">
+        <is>
+          <t>10.1016/j.energy.2026.142252</t>
+        </is>
+      </c>
+      <c r="I1008" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.energy.2026.142252</t>
+        </is>
+      </c>
+      <c r="J1008" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1008" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1008" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1008" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1008" t="inlineStr"/>
+      <c r="O1008" t="inlineStr"/>
+      <c r="P1008" t="inlineStr"/>
+      <c r="Q1008" t="inlineStr">
+        <is>
+          <t>System-level modeling and energy-performance assessment of frosting in inverter-driven air-source heat pumps under constant-heating-capacity operation</t>
+        </is>
+      </c>
+      <c r="R1008" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1008" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1008" t="inlineStr"/>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr"/>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>A 95.3% Efficiency APT/AET/SPT Multimode Multiband CMOS/GaN Envelope Tracking for 6G-Oriented Systems</t>
+        </is>
+      </c>
+      <c r="C1009" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>IEEE Journal of Solid-State Circuits</t>
+        </is>
+      </c>
+      <c r="F1009" t="inlineStr">
+        <is>
+          <t>Chen, Chun-Yuan; Huang, Yi-Chun; Chen, Ke-Horng; Lin, Ying-Hsi; Lin, Shian-Ru; Tsai, Tsung-Yen</t>
+        </is>
+      </c>
+      <c r="G1009" t="inlineStr"/>
+      <c r="H1009" t="inlineStr">
+        <is>
+          <t>10.1109/jssc.2026.3681319</t>
+        </is>
+      </c>
+      <c r="I1009" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/jssc.2026.3681319</t>
+        </is>
+      </c>
+      <c r="J1009" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1009" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1009" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1009" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1009" t="inlineStr"/>
+      <c r="O1009" t="inlineStr"/>
+      <c r="P1009" t="inlineStr"/>
+      <c r="Q1009" t="inlineStr">
+        <is>
+          <t>A 95.3% Efficiency APT/AET/SPT Multimode Multiband CMOS/GaN Envelope Tracking for 6G-Oriented Systems</t>
+        </is>
+      </c>
+      <c r="R1009" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1009" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1009" t="inlineStr"/>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr"/>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Quasi-Vertical GaN-Based Trench Gate MOSFETs Treated with Fluorine-Plasma</t>
+        </is>
+      </c>
+      <c r="C1010" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F1010" t="inlineStr">
+        <is>
+          <t>Zhang, Peng; Li, Dong-Yang; Xu, Jia-Rui; Chang, Qing-Yuan; Hou, Bin; Xi, He; Ma, Xiao-Hua</t>
+        </is>
+      </c>
+      <c r="G1010" t="inlineStr"/>
+      <c r="H1010" t="inlineStr">
+        <is>
+          <t>10.3390/mi17091019</t>
+        </is>
+      </c>
+      <c r="I1010" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17091019</t>
+        </is>
+      </c>
+      <c r="J1010" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1010" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1010" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1010" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1010" t="inlineStr"/>
+      <c r="O1010" t="inlineStr"/>
+      <c r="P1010" t="inlineStr"/>
+      <c r="Q1010" t="inlineStr">
+        <is>
+          <t>Quasi-Vertical GaN-Based Trench Gate MOSFETs Treated with Fluorine-Plasma</t>
+        </is>
+      </c>
+      <c r="R1010" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1010" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1010" t="inlineStr"/>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr"/>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Universal Electrical Resistivity in Iron-Based High-Temperature Superconductors</t>
+        </is>
+      </c>
+      <c r="C1011" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr"/>
+      <c r="F1011" t="inlineStr">
+        <is>
+          <t>Talantsev, Evgeny F.</t>
+        </is>
+      </c>
+      <c r="G1011" t="inlineStr"/>
+      <c r="H1011" t="inlineStr">
+        <is>
+          <t>10.20944/preprints202608.1997.v1</t>
+        </is>
+      </c>
+      <c r="I1011" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.20944/preprints202608.1997.v1</t>
+        </is>
+      </c>
+      <c r="J1011" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1011" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1011" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1011" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1011" t="inlineStr"/>
+      <c r="O1011" t="inlineStr"/>
+      <c r="P1011" t="inlineStr"/>
+      <c r="Q1011" t="inlineStr">
+        <is>
+          <t>Universal Electrical Resistivity in Iron-Based High-Temperature Superconductors</t>
+        </is>
+      </c>
+      <c r="R1011" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1011" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1011" t="inlineStr"/>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr"/>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Study of n-Channel 4H-SiC MOSFETs with a High-k/SiO2 Stacked Gate Dielectric and a p+-Polysilicon Gate</t>
+        </is>
+      </c>
+      <c r="C1012" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>Micromachines</t>
+        </is>
+      </c>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>Lin, Zhi; Cheng, Nuo; Cai, Weicheng; Hu, Jianyu; Hu, Shengdong</t>
+        </is>
+      </c>
+      <c r="G1012" t="inlineStr"/>
+      <c r="H1012" t="inlineStr">
+        <is>
+          <t>10.3390/mi17091017</t>
+        </is>
+      </c>
+      <c r="I1012" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/mi17091017</t>
+        </is>
+      </c>
+      <c r="J1012" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1012" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1012" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1012" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1012" t="inlineStr"/>
+      <c r="O1012" t="inlineStr"/>
+      <c r="P1012" t="inlineStr"/>
+      <c r="Q1012" t="inlineStr">
+        <is>
+          <t>Study of n-Channel 4H-SiC MOSFETs with a High-k/SiO2 Stacked Gate Dielectric and a p+-Polysilicon Gate</t>
+        </is>
+      </c>
+      <c r="R1012" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1012" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1012" t="inlineStr"/>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr"/>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>A 95.3% Efficiency APT/AET/SPT Multimode Multiband CMOS/GaN Envelope Tracking for 6G-Oriented Systems</t>
+        </is>
+      </c>
+      <c r="C1013" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>IEEE Journal of Solid-State Circuits</t>
+        </is>
+      </c>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>Chen, Chun-Yuan; Huang, Yi-Chun; Chen, Ke-Horng; Lin, Ying-Hsi; Lin, Shian-Ru; Tsai, Tsung-Yen</t>
+        </is>
+      </c>
+      <c r="G1013" t="inlineStr"/>
+      <c r="H1013" t="inlineStr">
+        <is>
+          <t>10.1109/jssc.2026.3681319</t>
+        </is>
+      </c>
+      <c r="I1013" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/jssc.2026.3681319</t>
+        </is>
+      </c>
+      <c r="J1013" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1013" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1013" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1013" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1013" t="inlineStr"/>
+      <c r="O1013" t="inlineStr"/>
+      <c r="P1013" t="inlineStr"/>
+      <c r="Q1013" t="inlineStr">
+        <is>
+          <t>A 95.3% Efficiency APT/AET/SPT Multimode Multiband CMOS/GaN Envelope Tracking for 6G-Oriented Systems</t>
+        </is>
+      </c>
+      <c r="R1013" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1013" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="T1013" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-30T01:09Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1013"/>
+  <dimension ref="A1:T1019"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77082,6 +77082,458 @@
       </c>
       <c r="T1013" t="inlineStr"/>
     </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr"/>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>High-PSRR, fast-settling inverter-based LDO voltage regulator with integrated TOS circuit for advanced CMOS systems</t>
+        </is>
+      </c>
+      <c r="C1014" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="F1014" t="inlineStr">
+        <is>
+          <t>Borule, Nivedita; Bhukya, Sunitha; Vadthiya, Narendar; Naresh Kumar Reddy, B.; Varshney, Vikrant</t>
+        </is>
+      </c>
+      <c r="G1014" t="inlineStr"/>
+      <c r="H1014" t="inlineStr">
+        <is>
+          <t>10.1016/j.vlsi.2026.102859</t>
+        </is>
+      </c>
+      <c r="I1014" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.vlsi.2026.102859</t>
+        </is>
+      </c>
+      <c r="J1014" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1014" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1014" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1014" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1014" t="inlineStr"/>
+      <c r="O1014" t="inlineStr"/>
+      <c r="P1014" t="inlineStr"/>
+      <c r="Q1014" t="inlineStr">
+        <is>
+          <t>High-PSRR, fast-settling inverter-based LDO voltage regulator with integrated TOS circuit for advanced CMOS systems</t>
+        </is>
+      </c>
+      <c r="R1014" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1014" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="T1014" t="inlineStr"/>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr"/>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Facile fabrication of Cu-TiO2@Ti monolithic catalyst for effective catalytic reduction of p-nitrophenol</t>
+        </is>
+      </c>
+      <c r="C1015" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>Solid State Sciences</t>
+        </is>
+      </c>
+      <c r="F1015" t="inlineStr">
+        <is>
+          <t>Tuo, Qingwen; He, Jingwei; Li, Gang</t>
+        </is>
+      </c>
+      <c r="G1015" t="inlineStr"/>
+      <c r="H1015" t="inlineStr">
+        <is>
+          <t>10.1016/j.solidstatesciences.2026.108463</t>
+        </is>
+      </c>
+      <c r="I1015" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.solidstatesciences.2026.108463</t>
+        </is>
+      </c>
+      <c r="J1015" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1015" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1015" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1015" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="N1015" t="inlineStr"/>
+      <c r="O1015" t="inlineStr"/>
+      <c r="P1015" t="inlineStr"/>
+      <c r="Q1015" t="inlineStr">
+        <is>
+          <t>Facile fabrication of Cu-TiO2@Ti monolithic catalyst for effective catalytic reduction of p-nitrophenol</t>
+        </is>
+      </c>
+      <c r="R1015" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1015" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="T1015" t="inlineStr"/>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr"/>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>SWCNTs thin film transistor circuits fabricated on flexible substrates with inkjet-printed silver electrodes for photodetectors</t>
+        </is>
+      </c>
+      <c r="C1016" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr"/>
+      <c r="F1016" t="inlineStr">
+        <is>
+          <t>Singh, Subhash; Ranjan, Piyush; Sambandan, Sanjiv</t>
+        </is>
+      </c>
+      <c r="G1016" t="inlineStr"/>
+      <c r="H1016" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10650690/v1</t>
+        </is>
+      </c>
+      <c r="I1016" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10650690/v1</t>
+        </is>
+      </c>
+      <c r="J1016" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1016" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L1016" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1016" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1016" t="inlineStr"/>
+      <c r="O1016" t="inlineStr"/>
+      <c r="P1016" t="inlineStr"/>
+      <c r="Q1016" t="inlineStr">
+        <is>
+          <t>SWCNTs thin film transistor circuits fabricated on flexible substrates with inkjet-printed silver electrodes for photodetectors</t>
+        </is>
+      </c>
+      <c r="R1016" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1016" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="T1016" t="inlineStr"/>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr"/>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Semi-On State Hole Generation in GaN HEMTs: Experimental Evidence and TCAD Modeling</t>
+        </is>
+      </c>
+      <c r="C1017" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F1017" t="inlineStr">
+        <is>
+          <t>Kuo, Ying-Chun; Yu, Hao; Braga, Nelson de Almeida; Fang, Jingtian; Gupta, Amratansh; Yadav, Sachin; Sibaja-Hernandez, Arturo; Alian, Alireza; Peralagu, Uthayasankaran; Collaert, Nadine; Parvais, Bertrand</t>
+        </is>
+      </c>
+      <c r="G1017" t="inlineStr"/>
+      <c r="H1017" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3711655</t>
+        </is>
+      </c>
+      <c r="I1017" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3711655</t>
+        </is>
+      </c>
+      <c r="J1017" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1017" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1017" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1017" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N1017" t="inlineStr"/>
+      <c r="O1017" t="inlineStr"/>
+      <c r="P1017" t="inlineStr"/>
+      <c r="Q1017" t="inlineStr">
+        <is>
+          <t>Semi-On State Hole Generation in GaN HEMTs: Experimental Evidence and TCAD Modeling</t>
+        </is>
+      </c>
+      <c r="R1017" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1017" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="T1017" t="inlineStr"/>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr"/>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Semi-On State Hole Generation in GaN HEMTs: Experimental Evidence and TCAD Modeling</t>
+        </is>
+      </c>
+      <c r="C1018" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>Kuo, Ying-Chun; Yu, Hao; Braga, Nelson de Almeida; Fang, Jingtian; Gupta, Amratansh; Yadav, Sachin; Sibaja-Hernandez, Arturo; Alian, Alireza; Peralagu, Uthayasankaran; Collaert, Nadine; Parvais, Bertrand</t>
+        </is>
+      </c>
+      <c r="G1018" t="inlineStr"/>
+      <c r="H1018" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3711655</t>
+        </is>
+      </c>
+      <c r="I1018" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3711655</t>
+        </is>
+      </c>
+      <c r="J1018" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1018" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1018" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1018" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N1018" t="inlineStr"/>
+      <c r="O1018" t="inlineStr"/>
+      <c r="P1018" t="inlineStr"/>
+      <c r="Q1018" t="inlineStr">
+        <is>
+          <t>Semi-On State Hole Generation in GaN HEMTs: Experimental Evidence and TCAD Modeling</t>
+        </is>
+      </c>
+      <c r="R1018" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1018" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="T1018" t="inlineStr"/>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr"/>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Semi-On State Hole Generation in GaN HEMTs: Experimental Evidence and TCAD Modeling</t>
+        </is>
+      </c>
+      <c r="C1019" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>Institute of Electrical and Electronics Engineers (IEEE)</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>IEEE Electron Device Letters</t>
+        </is>
+      </c>
+      <c r="F1019" t="inlineStr">
+        <is>
+          <t>Kuo, Ying-Chun; Yu, Hao; Braga, Nelson de Almeida; Fang, Jingtian; Gupta, Amratansh; Yadav, Sachin; Sibaja-Hernandez, Arturo; Alian, Alireza; Peralagu, Uthayasankaran; Collaert, Nadine; Parvais, Bertrand</t>
+        </is>
+      </c>
+      <c r="G1019" t="inlineStr"/>
+      <c r="H1019" t="inlineStr">
+        <is>
+          <t>10.1109/led.2026.3711655</t>
+        </is>
+      </c>
+      <c r="I1019" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/led.2026.3711655</t>
+        </is>
+      </c>
+      <c r="J1019" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1019" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1019" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1019" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="N1019" t="inlineStr"/>
+      <c r="O1019" t="inlineStr"/>
+      <c r="P1019" t="inlineStr"/>
+      <c r="Q1019" t="inlineStr">
+        <is>
+          <t>Semi-On State Hole Generation in GaN HEMTs: Experimental Evidence and TCAD Modeling</t>
+        </is>
+      </c>
+      <c r="R1019" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1019" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="T1019" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-08-31T01:12Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1019"/>
+  <dimension ref="A1:T1021"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77534,6 +77534,158 @@
       </c>
       <c r="T1019" t="inlineStr"/>
     </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr"/>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Performance Enhancement of MOSFET Circuits Using Evolutionary and Nature-Inspired Optimization Algorithms</t>
+        </is>
+      </c>
+      <c r="C1020" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>Mustansiriyah University College of Engineering</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>Academic Journal of Electrical and Computer Engineering</t>
+        </is>
+      </c>
+      <c r="F1020" t="inlineStr">
+        <is>
+          <t>Hathal, Hussein; A. Alhilali, Riyadh; M. Hathal, Reeman</t>
+        </is>
+      </c>
+      <c r="G1020" t="inlineStr"/>
+      <c r="H1020" t="inlineStr">
+        <is>
+          <t>10.31272/ajece.47</t>
+        </is>
+      </c>
+      <c r="I1020" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.31272/ajece.47</t>
+        </is>
+      </c>
+      <c r="J1020" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1020" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1020" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M1020" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1020" t="inlineStr"/>
+      <c r="O1020" t="inlineStr"/>
+      <c r="P1020" t="inlineStr"/>
+      <c r="Q1020" t="inlineStr">
+        <is>
+          <t>Performance Enhancement of MOSFET Circuits Using Evolutionary and Nature-Inspired Optimization Algorithms</t>
+        </is>
+      </c>
+      <c r="R1020" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1020" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="T1020" t="inlineStr"/>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr"/>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Performance Enhancement of MOSFET Circuits Using Evolutionary and Nature-Inspired Optimization Algorithms</t>
+        </is>
+      </c>
+      <c r="C1021" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>Mustansiriyah University College of Engineering</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>Academic Journal of Electrical and Computer Engineering</t>
+        </is>
+      </c>
+      <c r="F1021" t="inlineStr">
+        <is>
+          <t>Hathal, Hussein; A. Alhilali, Riyadh; M. Hathal, Reeman</t>
+        </is>
+      </c>
+      <c r="G1021" t="inlineStr"/>
+      <c r="H1021" t="inlineStr">
+        <is>
+          <t>10.31272/ajece.47</t>
+        </is>
+      </c>
+      <c r="I1021" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.31272/ajece.47</t>
+        </is>
+      </c>
+      <c r="J1021" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1021" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1021" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M1021" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1021" t="inlineStr"/>
+      <c r="O1021" t="inlineStr"/>
+      <c r="P1021" t="inlineStr"/>
+      <c r="Q1021" t="inlineStr">
+        <is>
+          <t>Performance Enhancement of MOSFET Circuits Using Evolutionary and Nature-Inspired Optimization Algorithms</t>
+        </is>
+      </c>
+      <c r="R1021" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1021" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="T1021" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-09-01T01:44Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1021"/>
+  <dimension ref="A1:T1025"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77686,6 +77686,306 @@
       </c>
       <c r="T1021" t="inlineStr"/>
     </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr"/>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Low‐Power Column‐Parallel Single‐Slope Analog‐to‐Digital Converter With Floating Inverter Amplifier for CMOS Image Sensors</t>
+        </is>
+      </c>
+      <c r="C1022" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>International Journal of Circuit Theory and Applications</t>
+        </is>
+      </c>
+      <c r="F1022" t="inlineStr">
+        <is>
+          <t>Nie, Kaiming; Zou, Weipeng; Zhang, Zihang; Chen, Sirong; Xu, Jiangtao; Gao, Jing</t>
+        </is>
+      </c>
+      <c r="G1022" t="inlineStr"/>
+      <c r="H1022" t="inlineStr">
+        <is>
+          <t>10.1002/cta.70630</t>
+        </is>
+      </c>
+      <c r="I1022" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/cta.70630</t>
+        </is>
+      </c>
+      <c r="J1022" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1022" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1022" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1022" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1022" t="inlineStr"/>
+      <c r="O1022" t="inlineStr"/>
+      <c r="P1022" t="inlineStr"/>
+      <c r="Q1022" t="inlineStr">
+        <is>
+          <t>Low‐Power Column‐Parallel Single‐Slope Analog‐to‐Digital Converter With Floating Inverter Amplifier for CMOS Image Sensors</t>
+        </is>
+      </c>
+      <c r="R1022" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1022" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="T1022" t="inlineStr"/>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr"/>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>An Improved Switched-Inductor-Capacitor Z-Source Inverter with Enhanced Boost Capability and Reduced Voltage Stress</t>
+        </is>
+      </c>
+      <c r="C1023" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr"/>
+      <c r="F1023" t="inlineStr">
+        <is>
+          <t>Gholami, Masoumeh; Noroozian, Reza; Bajestan, Mehran Moslehi; Bizhani, Hamed</t>
+        </is>
+      </c>
+      <c r="G1023" t="inlineStr"/>
+      <c r="H1023" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10572008/v1</t>
+        </is>
+      </c>
+      <c r="I1023" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10572008/v1</t>
+        </is>
+      </c>
+      <c r="J1023" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1023" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1023" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1023" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1023" t="inlineStr"/>
+      <c r="O1023" t="inlineStr"/>
+      <c r="P1023" t="inlineStr"/>
+      <c r="Q1023" t="inlineStr">
+        <is>
+          <t>An Improved Switched-Inductor-Capacitor Z-Source Inverter with Enhanced Boost Capability and Reduced Voltage Stress</t>
+        </is>
+      </c>
+      <c r="R1023" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1023" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="T1023" t="inlineStr"/>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr"/>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Design of DC gate electric field redistribution under high drain voltage for high linearity, wide gain control range, and low
+                    &lt;i&gt;C&lt;/i&gt;
+                    off in GaN dual-mode integrated devices</t>
+        </is>
+      </c>
+      <c r="C1024" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>AIP Publishing</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>Applied Physics Letters</t>
+        </is>
+      </c>
+      <c r="F1024" t="inlineStr">
+        <is>
+          <t>Zou, Xu; Zhang, Meng; Yang, Ling; Jiang, Yutong; Yu, Qian; Ren, Weiyu; Wu, Mei; Hou, Bin; Lu, Hao; Jia, Mao; Ma, Xiaohua; Hao, Yue</t>
+        </is>
+      </c>
+      <c r="G1024" t="inlineStr"/>
+      <c r="H1024" t="inlineStr">
+        <is>
+          <t>10.1063/5.0344361</t>
+        </is>
+      </c>
+      <c r="I1024" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1063/5.0344361</t>
+        </is>
+      </c>
+      <c r="J1024" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1024" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1024" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1024" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1024" t="inlineStr"/>
+      <c r="O1024" t="inlineStr"/>
+      <c r="P1024" t="inlineStr"/>
+      <c r="Q1024" t="inlineStr">
+        <is>
+          <t>Design of DC gate electric field redistribution under high drain voltage for high linearity, wide gain control range, and low
+                    &lt;i&gt;C&lt;/i&gt;
+                    off in GaN dual-mode integrated devices</t>
+        </is>
+      </c>
+      <c r="R1024" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1024" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="T1024" t="inlineStr"/>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr"/>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>An Improved Switched-Inductor-Capacitor Z-Source Inverter with Enhanced Boost Capability and Reduced Voltage Stress</t>
+        </is>
+      </c>
+      <c r="C1025" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr"/>
+      <c r="F1025" t="inlineStr">
+        <is>
+          <t>Gholami, Masoumeh; Noroozian, Reza; Bajestan, Mehran Moslehi; Bizhani, Hamed</t>
+        </is>
+      </c>
+      <c r="G1025" t="inlineStr"/>
+      <c r="H1025" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10572008/v1</t>
+        </is>
+      </c>
+      <c r="I1025" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10572008/v1</t>
+        </is>
+      </c>
+      <c r="J1025" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1025" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1025" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1025" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1025" t="inlineStr"/>
+      <c r="O1025" t="inlineStr"/>
+      <c r="P1025" t="inlineStr"/>
+      <c r="Q1025" t="inlineStr">
+        <is>
+          <t>An Improved Switched-Inductor-Capacitor Z-Source Inverter with Enhanced Boost Capability and Reduced Voltage Stress</t>
+        </is>
+      </c>
+      <c r="R1025" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1025" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="T1025" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-09-02T00:54Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1025"/>
+  <dimension ref="A1:T1031"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77986,6 +77986,446 @@
       </c>
       <c r="T1025" t="inlineStr"/>
     </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr"/>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Life as Form: Biomimetic Transport Networks in Complementary Active Matter</t>
+        </is>
+      </c>
+      <c r="C1026" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1026" t="inlineStr"/>
+      <c r="F1026" t="inlineStr">
+        <is>
+          <t>Scirè, Alessandro</t>
+        </is>
+      </c>
+      <c r="G1026" t="inlineStr"/>
+      <c r="H1026" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10876418/v1</t>
+        </is>
+      </c>
+      <c r="I1026" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10876418/v1</t>
+        </is>
+      </c>
+      <c r="J1026" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1026" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1026" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1026" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1026" t="inlineStr"/>
+      <c r="O1026" t="inlineStr"/>
+      <c r="P1026" t="inlineStr"/>
+      <c r="Q1026" t="inlineStr">
+        <is>
+          <t>Life as Form: Biomimetic Transport Networks in Complementary Active Matter</t>
+        </is>
+      </c>
+      <c r="R1026" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1026" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T1026" t="inlineStr"/>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr"/>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Total ionizing dose effects on backside-illuminated CMOS image sensors through experiments and TCAD simulations</t>
+        </is>
+      </c>
+      <c r="C1027" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>Informa UK Limited</t>
+        </is>
+      </c>
+      <c r="E1027" t="inlineStr">
+        <is>
+          <t>Radiation Effects and Defects in Solids</t>
+        </is>
+      </c>
+      <c r="F1027" t="inlineStr">
+        <is>
+          <t>Liu, Mingyu; liu, Bingkai; Wen, Lin; Pan, Chen; Cui, Yihao; Zhao, Zitao; Guo, Qi; Li, Yudong</t>
+        </is>
+      </c>
+      <c r="G1027" t="inlineStr"/>
+      <c r="H1027" t="inlineStr">
+        <is>
+          <t>10.1080/10420150.2026.2721519</t>
+        </is>
+      </c>
+      <c r="I1027" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/10420150.2026.2721519</t>
+        </is>
+      </c>
+      <c r="J1027" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1027" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1027" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1027" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1027" t="inlineStr"/>
+      <c r="O1027" t="inlineStr"/>
+      <c r="P1027" t="inlineStr"/>
+      <c r="Q1027" t="inlineStr">
+        <is>
+          <t>Total ionizing dose effects on backside-illuminated CMOS image sensors through experiments and TCAD simulations</t>
+        </is>
+      </c>
+      <c r="R1027" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1027" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T1027" t="inlineStr"/>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr"/>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Bending-strain-resilient threshold and RF stability of a La2O3/Al0.43Ga0.57As cylindrical surrounding double-gate MOSFET on a cellulose nanofiber substrate</t>
+        </is>
+      </c>
+      <c r="C1028" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr"/>
+      <c r="F1028" t="inlineStr">
+        <is>
+          <t>Gowthaman, Naveenbalaji; SRIVASTAVA, VIRANJAY</t>
+        </is>
+      </c>
+      <c r="G1028" t="inlineStr"/>
+      <c r="H1028" t="inlineStr">
+        <is>
+          <t>10.22541/authorea.15008145/v1</t>
+        </is>
+      </c>
+      <c r="I1028" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22541/authorea.15008145/v1</t>
+        </is>
+      </c>
+      <c r="J1028" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1028" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1028" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M1028" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1028" t="inlineStr"/>
+      <c r="O1028" t="inlineStr"/>
+      <c r="P1028" t="inlineStr"/>
+      <c r="Q1028" t="inlineStr">
+        <is>
+          <t>Bending-strain-resilient threshold and RF stability of a La2O3/Al0.43Ga0.57As cylindrical surrounding double-gate MOSFET on a cellulose nanofiber substrate</t>
+        </is>
+      </c>
+      <c r="R1028" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1028" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T1028" t="inlineStr"/>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr"/>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Bending-strain-resilient threshold and RF stability of a La2O3/Al0.43Ga0.57As cylindrical surrounding double-gate MOSFET on a cellulose nanofiber substrate</t>
+        </is>
+      </c>
+      <c r="C1029" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E1029" t="inlineStr"/>
+      <c r="F1029" t="inlineStr">
+        <is>
+          <t>Gowthaman, Naveenbalaji; SRIVASTAVA, VIRANJAY</t>
+        </is>
+      </c>
+      <c r="G1029" t="inlineStr"/>
+      <c r="H1029" t="inlineStr">
+        <is>
+          <t>10.22541/authorea.15008145/v1</t>
+        </is>
+      </c>
+      <c r="I1029" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22541/authorea.15008145/v1</t>
+        </is>
+      </c>
+      <c r="J1029" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1029" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1029" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M1029" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1029" t="inlineStr"/>
+      <c r="O1029" t="inlineStr"/>
+      <c r="P1029" t="inlineStr"/>
+      <c r="Q1029" t="inlineStr">
+        <is>
+          <t>Bending-strain-resilient threshold and RF stability of a La2O3/Al0.43Ga0.57As cylindrical surrounding double-gate MOSFET on a cellulose nanofiber substrate</t>
+        </is>
+      </c>
+      <c r="R1029" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1029" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T1029" t="inlineStr"/>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr"/>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Bending-strain-resilient threshold and RF stability of a La2O3/Al0.43Ga0.57As cylindrical surrounding double-gate MOSFET on a cellulose nanofiber substrate</t>
+        </is>
+      </c>
+      <c r="C1030" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="E1030" t="inlineStr"/>
+      <c r="F1030" t="inlineStr">
+        <is>
+          <t>Gowthaman, Naveenbalaji; SRIVASTAVA, VIRANJAY</t>
+        </is>
+      </c>
+      <c r="G1030" t="inlineStr"/>
+      <c r="H1030" t="inlineStr">
+        <is>
+          <t>10.22541/authorea.15008145/v1</t>
+        </is>
+      </c>
+      <c r="I1030" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22541/authorea.15008145/v1</t>
+        </is>
+      </c>
+      <c r="J1030" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1030" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1030" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M1030" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1030" t="inlineStr"/>
+      <c r="O1030" t="inlineStr"/>
+      <c r="P1030" t="inlineStr"/>
+      <c r="Q1030" t="inlineStr">
+        <is>
+          <t>Bending-strain-resilient threshold and RF stability of a La2O3/Al0.43Ga0.57As cylindrical surrounding double-gate MOSFET on a cellulose nanofiber substrate</t>
+        </is>
+      </c>
+      <c r="R1030" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1030" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T1030" t="inlineStr"/>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr"/>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Total ionizing dose effects on backside-illuminated CMOS image sensors through experiments and TCAD simulations</t>
+        </is>
+      </c>
+      <c r="C1031" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>Informa UK Limited</t>
+        </is>
+      </c>
+      <c r="E1031" t="inlineStr">
+        <is>
+          <t>Radiation Effects and Defects in Solids</t>
+        </is>
+      </c>
+      <c r="F1031" t="inlineStr">
+        <is>
+          <t>Liu, Mingyu; liu, Bingkai; Wen, Lin; Pan, Chen; Cui, Yihao; Zhao, Zitao; Guo, Qi; Li, Yudong</t>
+        </is>
+      </c>
+      <c r="G1031" t="inlineStr"/>
+      <c r="H1031" t="inlineStr">
+        <is>
+          <t>10.1080/10420150.2026.2721519</t>
+        </is>
+      </c>
+      <c r="I1031" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/10420150.2026.2721519</t>
+        </is>
+      </c>
+      <c r="J1031" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1031" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1031" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1031" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1031" t="inlineStr"/>
+      <c r="O1031" t="inlineStr"/>
+      <c r="P1031" t="inlineStr"/>
+      <c r="Q1031" t="inlineStr">
+        <is>
+          <t>Total ionizing dose effects on backside-illuminated CMOS image sensors through experiments and TCAD simulations</t>
+        </is>
+      </c>
+      <c r="R1031" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1031" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="T1031" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-09-04T00:51Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1031"/>
+  <dimension ref="A1:T1044"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78426,6 +78426,994 @@
       </c>
       <c r="T1031" t="inlineStr"/>
     </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr"/>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Power System Operating and Managing Under Rapidly Changing Amounts of Grid-Inverter-Connected RES</t>
+        </is>
+      </c>
+      <c r="C1032" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>MDPI</t>
+        </is>
+      </c>
+      <c r="E1032" t="inlineStr">
+        <is>
+          <t>EEPES 2026</t>
+        </is>
+      </c>
+      <c r="F1032" t="inlineStr">
+        <is>
+          <t>Koeva, Dimitrina; Ivanov, Ivaylo; Slavov, Dimitar; Bankov, Georgi; Dimitrov, Metodi</t>
+        </is>
+      </c>
+      <c r="G1032" t="inlineStr"/>
+      <c r="H1032" t="inlineStr">
+        <is>
+          <t>10.3390/engproc2026154027</t>
+        </is>
+      </c>
+      <c r="I1032" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/engproc2026154027</t>
+        </is>
+      </c>
+      <c r="J1032" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1032" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1032" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1032" t="inlineStr">
+        <is>
+          <t>Reliability</t>
+        </is>
+      </c>
+      <c r="N1032" t="inlineStr"/>
+      <c r="O1032" t="inlineStr"/>
+      <c r="P1032" t="inlineStr"/>
+      <c r="Q1032" t="inlineStr">
+        <is>
+          <t>Power System Operating and Managing Under Rapidly Changing Amounts of Grid-Inverter-Connected RES</t>
+        </is>
+      </c>
+      <c r="R1032" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1032" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1032" t="inlineStr"/>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr"/>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Bounded Integration: The Regulation of Traditional and Complementary Medicine in Türkiye</t>
+        </is>
+      </c>
+      <c r="C1033" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E1033" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F1033" t="inlineStr">
+        <is>
+          <t>Polat, Ayşe</t>
+        </is>
+      </c>
+      <c r="G1033" t="inlineStr"/>
+      <c r="H1033" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261483924</t>
+        </is>
+      </c>
+      <c r="I1033" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261483924</t>
+        </is>
+      </c>
+      <c r="J1033" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1033" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1033" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1033" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1033" t="inlineStr"/>
+      <c r="O1033" t="inlineStr"/>
+      <c r="P1033" t="inlineStr"/>
+      <c r="Q1033" t="inlineStr">
+        <is>
+          <t>Bounded Integration: The Regulation of Traditional and Complementary Medicine in Türkiye</t>
+        </is>
+      </c>
+      <c r="R1033" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1033" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1033" t="inlineStr"/>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr"/>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Bounded Integration: The Regulation of Traditional and Complementary Medicine in Türkiye</t>
+        </is>
+      </c>
+      <c r="C1034" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>SAGE Publications</t>
+        </is>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>Journal of Integrative and Complementary Medicine</t>
+        </is>
+      </c>
+      <c r="F1034" t="inlineStr">
+        <is>
+          <t>Polat, Ayşe</t>
+        </is>
+      </c>
+      <c r="G1034" t="inlineStr"/>
+      <c r="H1034" t="inlineStr">
+        <is>
+          <t>10.1177/27683605261483924</t>
+        </is>
+      </c>
+      <c r="I1034" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/27683605261483924</t>
+        </is>
+      </c>
+      <c r="J1034" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1034" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1034" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1034" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1034" t="inlineStr"/>
+      <c r="O1034" t="inlineStr"/>
+      <c r="P1034" t="inlineStr"/>
+      <c r="Q1034" t="inlineStr">
+        <is>
+          <t>Bounded Integration: The Regulation of Traditional and Complementary Medicine in Türkiye</t>
+        </is>
+      </c>
+      <c r="R1034" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1034" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1034" t="inlineStr"/>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr"/>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C1035" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>Micro and Nanostructures</t>
+        </is>
+      </c>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>Alem, R.; Mattalah, M.; Benzekkour, N.; Soltani, A.</t>
+        </is>
+      </c>
+      <c r="G1035" t="inlineStr"/>
+      <c r="H1035" t="inlineStr">
+        <is>
+          <t>10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="I1035" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="J1035" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1035" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1035" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1035" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1035" t="inlineStr"/>
+      <c r="O1035" t="inlineStr"/>
+      <c r="P1035" t="inlineStr"/>
+      <c r="Q1035" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R1035" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1035" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1035" t="inlineStr"/>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr"/>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C1036" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>Micro and Nanostructures</t>
+        </is>
+      </c>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>Alem, R.; Mattalah, M.; Benzekkour, N.; Soltani, A.</t>
+        </is>
+      </c>
+      <c r="G1036" t="inlineStr"/>
+      <c r="H1036" t="inlineStr">
+        <is>
+          <t>10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="I1036" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="J1036" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1036" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1036" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1036" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1036" t="inlineStr"/>
+      <c r="O1036" t="inlineStr"/>
+      <c r="P1036" t="inlineStr"/>
+      <c r="Q1036" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R1036" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1036" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1036" t="inlineStr"/>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr"/>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C1037" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>Micro and Nanostructures</t>
+        </is>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>Alem, R.; Mattalah, M.; Benzekkour, N.; Soltani, A.</t>
+        </is>
+      </c>
+      <c r="G1037" t="inlineStr"/>
+      <c r="H1037" t="inlineStr">
+        <is>
+          <t>10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="I1037" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="J1037" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1037" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1037" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1037" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1037" t="inlineStr"/>
+      <c r="O1037" t="inlineStr"/>
+      <c r="P1037" t="inlineStr"/>
+      <c r="Q1037" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R1037" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1037" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1037" t="inlineStr"/>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr"/>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C1038" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>Micro and Nanostructures</t>
+        </is>
+      </c>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>Alem, R.; Mattalah, M.; Benzekkour, N.; Soltani, A.</t>
+        </is>
+      </c>
+      <c r="G1038" t="inlineStr"/>
+      <c r="H1038" t="inlineStr">
+        <is>
+          <t>10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="I1038" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="J1038" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1038" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1038" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1038" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1038" t="inlineStr"/>
+      <c r="O1038" t="inlineStr"/>
+      <c r="P1038" t="inlineStr"/>
+      <c r="Q1038" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R1038" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1038" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1038" t="inlineStr"/>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr"/>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Power System Operating and Managing Under Rapidly Changing Amounts of Grid-Inverter-Connected RES</t>
+        </is>
+      </c>
+      <c r="C1039" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>MDPI</t>
+        </is>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>EEPES 2026</t>
+        </is>
+      </c>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>Koeva, Dimitrina; Ivanov, Ivaylo; Slavov, Dimitar; Bankov, Georgi; Dimitrov, Metodi</t>
+        </is>
+      </c>
+      <c r="G1039" t="inlineStr"/>
+      <c r="H1039" t="inlineStr">
+        <is>
+          <t>10.3390/engproc2026154027</t>
+        </is>
+      </c>
+      <c r="I1039" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/engproc2026154027</t>
+        </is>
+      </c>
+      <c r="J1039" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1039" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1039" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1039" t="inlineStr">
+        <is>
+          <t>Reliability</t>
+        </is>
+      </c>
+      <c r="N1039" t="inlineStr"/>
+      <c r="O1039" t="inlineStr"/>
+      <c r="P1039" t="inlineStr"/>
+      <c r="Q1039" t="inlineStr">
+        <is>
+          <t>Power System Operating and Managing Under Rapidly Changing Amounts of Grid-Inverter-Connected RES</t>
+        </is>
+      </c>
+      <c r="R1039" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1039" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1039" t="inlineStr"/>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr"/>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Machine Learning-Assisted Optimization of CMOS VLSI Circuits for Low-Power and High-Speed Applications</t>
+        </is>
+      </c>
+      <c r="C1040" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>Naksh Solutions</t>
+        </is>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>International Journal of Advanced Research in Science Communication and Technology</t>
+        </is>
+      </c>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>Ankit Soni</t>
+        </is>
+      </c>
+      <c r="G1040" t="inlineStr"/>
+      <c r="H1040" t="inlineStr">
+        <is>
+          <t>10.48175/ijarsct-38215</t>
+        </is>
+      </c>
+      <c r="I1040" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48175/ijarsct-38215</t>
+        </is>
+      </c>
+      <c r="J1040" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1040" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1040" t="inlineStr">
+        <is>
+          <t>Compact</t>
+        </is>
+      </c>
+      <c r="M1040" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1040" t="inlineStr"/>
+      <c r="O1040" t="inlineStr"/>
+      <c r="P1040" t="inlineStr"/>
+      <c r="Q1040" t="inlineStr">
+        <is>
+          <t>Machine Learning-Assisted Optimization of CMOS VLSI Circuits for Low-Power and High-Speed Applications</t>
+        </is>
+      </c>
+      <c r="R1040" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1040" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1040" t="inlineStr"/>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr"/>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Beyond CMOS: performance-driven hybrid PMOS–memristor logic for scalable computing</t>
+        </is>
+      </c>
+      <c r="C1041" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>Microsystem Technologies</t>
+        </is>
+      </c>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>Pahsyntiew, Marbaremdor Wahlang; Saha, Prabir; Dandapat, Anup</t>
+        </is>
+      </c>
+      <c r="G1041" t="inlineStr"/>
+      <c r="H1041" t="inlineStr">
+        <is>
+          <t>10.1007/s00542-026-06144-8</t>
+        </is>
+      </c>
+      <c r="I1041" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s00542-026-06144-8</t>
+        </is>
+      </c>
+      <c r="J1041" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1041" t="inlineStr">
+        <is>
+          <t>p-FET</t>
+        </is>
+      </c>
+      <c r="L1041" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M1041" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1041" t="inlineStr"/>
+      <c r="O1041" t="inlineStr"/>
+      <c r="P1041" t="inlineStr"/>
+      <c r="Q1041" t="inlineStr">
+        <is>
+          <t>Beyond CMOS: performance-driven hybrid PMOS–memristor logic for scalable computing</t>
+        </is>
+      </c>
+      <c r="R1041" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1041" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1041" t="inlineStr"/>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr"/>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C1042" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>Micro and Nanostructures</t>
+        </is>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>Alem, R.; Mattalah, M.; Benzekkour, N.; Soltani, A.</t>
+        </is>
+      </c>
+      <c r="G1042" t="inlineStr"/>
+      <c r="H1042" t="inlineStr">
+        <is>
+          <t>10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="I1042" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="J1042" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1042" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1042" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1042" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1042" t="inlineStr"/>
+      <c r="O1042" t="inlineStr"/>
+      <c r="P1042" t="inlineStr"/>
+      <c r="Q1042" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R1042" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1042" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1042" t="inlineStr"/>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr"/>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>Structural interconversion of tin hybrids: solvent-driven fluorescence modulation for logic gate and anticounterfeiting applications</t>
+        </is>
+      </c>
+      <c r="C1043" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>Journal of Molecular Structure</t>
+        </is>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>Das, Deblina; Kwak, Seoyoung; Mal, Sourav; Mandal, Tarak Nath; Jana, Atanu; Cho, Sangeun</t>
+        </is>
+      </c>
+      <c r="G1043" t="inlineStr"/>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>10.1016/j.molstruc.2026.147328</t>
+        </is>
+      </c>
+      <c r="I1043" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.molstruc.2026.147328</t>
+        </is>
+      </c>
+      <c r="J1043" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1043" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1043" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M1043" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1043" t="inlineStr"/>
+      <c r="O1043" t="inlineStr"/>
+      <c r="P1043" t="inlineStr"/>
+      <c r="Q1043" t="inlineStr">
+        <is>
+          <t>Structural interconversion of tin hybrids: solvent-driven fluorescence modulation for logic gate and anticounterfeiting applications</t>
+        </is>
+      </c>
+      <c r="R1043" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1043" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1043" t="inlineStr"/>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr"/>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="C1044" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>Micro and Nanostructures</t>
+        </is>
+      </c>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>Alem, R.; Mattalah, M.; Benzekkour, N.; Soltani, A.</t>
+        </is>
+      </c>
+      <c r="G1044" t="inlineStr"/>
+      <c r="H1044" t="inlineStr">
+        <is>
+          <t>10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="I1044" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.micrna.2026.208887</t>
+        </is>
+      </c>
+      <c r="J1044" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1044" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1044" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1044" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1044" t="inlineStr"/>
+      <c r="O1044" t="inlineStr"/>
+      <c r="P1044" t="inlineStr"/>
+      <c r="Q1044" t="inlineStr">
+        <is>
+          <t>Decoupling interface and border trap effects in recessed-gate AlGaN/GaN MOSHEMTs via TCAD simulation</t>
+        </is>
+      </c>
+      <c r="R1044" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1044" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="T1044" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-09-05T00:43Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1044"/>
+  <dimension ref="A1:T1047"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79414,6 +79414,234 @@
       </c>
       <c r="T1044" t="inlineStr"/>
     </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr"/>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Compact and Reliable Design of Thin-Body MOSFET for Advanced Artificial Intelligence-Driven Sensing Systems</t>
+        </is>
+      </c>
+      <c r="C1045" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1045" t="inlineStr">
+        <is>
+          <t>Journal of Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F1045" t="inlineStr">
+        <is>
+          <t>Sentamilselvi, M.; Karthikeyan, K.; Srither, S. R.; Ramachandran, Balaji</t>
+        </is>
+      </c>
+      <c r="G1045" t="inlineStr"/>
+      <c r="H1045" t="inlineStr">
+        <is>
+          <t>10.1007/s11664-026-13116-1</t>
+        </is>
+      </c>
+      <c r="I1045" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s11664-026-13116-1</t>
+        </is>
+      </c>
+      <c r="J1045" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1045" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1045" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1045" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1045" t="inlineStr"/>
+      <c r="O1045" t="inlineStr"/>
+      <c r="P1045" t="inlineStr"/>
+      <c r="Q1045" t="inlineStr">
+        <is>
+          <t>Compact and Reliable Design of Thin-Body MOSFET for Advanced Artificial Intelligence-Driven Sensing Systems</t>
+        </is>
+      </c>
+      <c r="R1045" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1045" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="T1045" t="inlineStr"/>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr"/>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>Optimization of work function in triple-metal junctionless dual-gate-all-around MOSFET for nanoscale switching and electrostatic performance</t>
+        </is>
+      </c>
+      <c r="C1046" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>IOP Publishing</t>
+        </is>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>Engineering Research Express</t>
+        </is>
+      </c>
+      <c r="F1046" t="inlineStr">
+        <is>
+          <t>Khaja Shabuddin, Ad; Sreenivasa Rao, Devireddy; Balaji, B; Cheerla, Sreevardhan; Agarwal, Vipul; Koteswara Rao Devana, V N</t>
+        </is>
+      </c>
+      <c r="G1046" t="inlineStr"/>
+      <c r="H1046" t="inlineStr">
+        <is>
+          <t>10.1088/2631-8695/aea2f2</t>
+        </is>
+      </c>
+      <c r="I1046" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/2631-8695/aea2f2</t>
+        </is>
+      </c>
+      <c r="J1046" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1046" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1046" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1046" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1046" t="inlineStr"/>
+      <c r="O1046" t="inlineStr"/>
+      <c r="P1046" t="inlineStr"/>
+      <c r="Q1046" t="inlineStr">
+        <is>
+          <t>Optimization of work function in triple-metal junctionless dual-gate-all-around MOSFET for nanoscale switching and electrostatic performance</t>
+        </is>
+      </c>
+      <c r="R1046" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1046" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="T1046" t="inlineStr"/>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr"/>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>Compact and Reliable Design of Thin-Body MOSFET for Advanced Artificial Intelligence-Driven Sensing Systems</t>
+        </is>
+      </c>
+      <c r="C1047" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>Journal of Electronic Materials</t>
+        </is>
+      </c>
+      <c r="F1047" t="inlineStr">
+        <is>
+          <t>Sentamilselvi, M.; Karthikeyan, K.; Srither, S. R.; Ramachandran, Balaji</t>
+        </is>
+      </c>
+      <c r="G1047" t="inlineStr"/>
+      <c r="H1047" t="inlineStr">
+        <is>
+          <t>10.1007/s11664-026-13116-1</t>
+        </is>
+      </c>
+      <c r="I1047" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s11664-026-13116-1</t>
+        </is>
+      </c>
+      <c r="J1047" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1047" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1047" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1047" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1047" t="inlineStr"/>
+      <c r="O1047" t="inlineStr"/>
+      <c r="P1047" t="inlineStr"/>
+      <c r="Q1047" t="inlineStr">
+        <is>
+          <t>Compact and Reliable Design of Thin-Body MOSFET for Advanced Artificial Intelligence-Driven Sensing Systems</t>
+        </is>
+      </c>
+      <c r="R1047" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1047" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="T1047" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-09-06T00:43Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1047"/>
+  <dimension ref="A1:T1050"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79642,6 +79642,234 @@
       </c>
       <c r="T1047" t="inlineStr"/>
     </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr"/>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>TCAD-calibrated ML for trap-induced degradation in AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C1048" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>Microelectronics Reliability</t>
+        </is>
+      </c>
+      <c r="F1048" t="inlineStr">
+        <is>
+          <t>Sharma, Niketa; Sharma, Amit Kumar; Kachhawa, Pharyanshu</t>
+        </is>
+      </c>
+      <c r="G1048" t="inlineStr"/>
+      <c r="H1048" t="inlineStr">
+        <is>
+          <t>10.1016/j.microrel.2026.116293</t>
+        </is>
+      </c>
+      <c r="I1048" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.microrel.2026.116293</t>
+        </is>
+      </c>
+      <c r="J1048" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1048" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1048" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1048" t="inlineStr">
+        <is>
+          <t>Reliability</t>
+        </is>
+      </c>
+      <c r="N1048" t="inlineStr"/>
+      <c r="O1048" t="inlineStr"/>
+      <c r="P1048" t="inlineStr"/>
+      <c r="Q1048" t="inlineStr">
+        <is>
+          <t>TCAD-calibrated ML for trap-induced degradation in AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R1048" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1048" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="T1048" t="inlineStr"/>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr"/>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>TCAD-calibrated ML for trap-induced degradation in AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C1049" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>Microelectronics Reliability</t>
+        </is>
+      </c>
+      <c r="F1049" t="inlineStr">
+        <is>
+          <t>Sharma, Niketa; Sharma, Amit Kumar; Kachhawa, Pharyanshu</t>
+        </is>
+      </c>
+      <c r="G1049" t="inlineStr"/>
+      <c r="H1049" t="inlineStr">
+        <is>
+          <t>10.1016/j.microrel.2026.116293</t>
+        </is>
+      </c>
+      <c r="I1049" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.microrel.2026.116293</t>
+        </is>
+      </c>
+      <c r="J1049" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1049" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1049" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1049" t="inlineStr">
+        <is>
+          <t>Reliability</t>
+        </is>
+      </c>
+      <c r="N1049" t="inlineStr"/>
+      <c r="O1049" t="inlineStr"/>
+      <c r="P1049" t="inlineStr"/>
+      <c r="Q1049" t="inlineStr">
+        <is>
+          <t>TCAD-calibrated ML for trap-induced degradation in AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R1049" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1049" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="T1049" t="inlineStr"/>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr"/>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>TCAD-calibrated ML for trap-induced degradation in AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C1050" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>Elsevier BV</t>
+        </is>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>Microelectronics Reliability</t>
+        </is>
+      </c>
+      <c r="F1050" t="inlineStr">
+        <is>
+          <t>Sharma, Niketa; Sharma, Amit Kumar; Kachhawa, Pharyanshu</t>
+        </is>
+      </c>
+      <c r="G1050" t="inlineStr"/>
+      <c r="H1050" t="inlineStr">
+        <is>
+          <t>10.1016/j.microrel.2026.116293</t>
+        </is>
+      </c>
+      <c r="I1050" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.microrel.2026.116293</t>
+        </is>
+      </c>
+      <c r="J1050" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1050" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1050" t="inlineStr">
+        <is>
+          <t>TCAD</t>
+        </is>
+      </c>
+      <c r="M1050" t="inlineStr">
+        <is>
+          <t>Reliability</t>
+        </is>
+      </c>
+      <c r="N1050" t="inlineStr"/>
+      <c r="O1050" t="inlineStr"/>
+      <c r="P1050" t="inlineStr"/>
+      <c r="Q1050" t="inlineStr">
+        <is>
+          <t>TCAD-calibrated ML for trap-induced degradation in AlGaN/GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R1050" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1050" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="T1050" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-09-07T00:46Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1050"/>
+  <dimension ref="A1:T1051"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79870,6 +79870,86 @@
       </c>
       <c r="T1050" t="inlineStr"/>
     </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr"/>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>Multivariate-Activated
+DNA Logic Gate for Predicting
+Responses to Cisplatin-Based Chemotherapy</t>
+        </is>
+      </c>
+      <c r="C1051" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>American Chemical Society (ACS)</t>
+        </is>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>Analytical Chemistry</t>
+        </is>
+      </c>
+      <c r="F1051" t="inlineStr">
+        <is>
+          <t>Li, Bin; Yan, Jueyue; Wang, Danyang; Li, Xiao; Liu, Xueling; Ding, Yuxi; Zhao, Feng; Fan, Yingcong; Yin, Jiayi; Xia, Yaokun</t>
+        </is>
+      </c>
+      <c r="G1051" t="inlineStr"/>
+      <c r="H1051" t="inlineStr">
+        <is>
+          <t>10.1021/acs.analchem.6c04574</t>
+        </is>
+      </c>
+      <c r="I1051" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acs.analchem.6c04574</t>
+        </is>
+      </c>
+      <c r="J1051" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1051" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1051" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1051" t="inlineStr">
+        <is>
+          <t>Gate Stack</t>
+        </is>
+      </c>
+      <c r="N1051" t="inlineStr"/>
+      <c r="O1051" t="inlineStr"/>
+      <c r="P1051" t="inlineStr"/>
+      <c r="Q1051" t="inlineStr">
+        <is>
+          <t>Multivariate-Activated
+DNA Logic Gate for Predicting
+Responses to Cisplatin-Based Chemotherapy</t>
+        </is>
+      </c>
+      <c r="R1051" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1051" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="T1051" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-09-08T01:00Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1051"/>
+  <dimension ref="A1:T1052"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79950,6 +79950,82 @@
       </c>
       <c r="T1051" t="inlineStr"/>
     </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr"/>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>Climate-responsive robotic brickwork for monolithic building envelopes</t>
+        </is>
+      </c>
+      <c r="C1052" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>Construction Robotics</t>
+        </is>
+      </c>
+      <c r="F1052" t="inlineStr">
+        <is>
+          <t>Fleckenstein, Julia; Dörfler, Kathrin; Molter, Philipp L.; Santucci, Daniele</t>
+        </is>
+      </c>
+      <c r="G1052" t="inlineStr"/>
+      <c r="H1052" t="inlineStr">
+        <is>
+          <t>10.1007/s41693-026-00219-8</t>
+        </is>
+      </c>
+      <c r="I1052" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s41693-026-00219-8</t>
+        </is>
+      </c>
+      <c r="J1052" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1052" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1052" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1052" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1052" t="inlineStr"/>
+      <c r="O1052" t="inlineStr"/>
+      <c r="P1052" t="inlineStr"/>
+      <c r="Q1052" t="inlineStr">
+        <is>
+          <t>Climate-responsive robotic brickwork for monolithic building envelopes</t>
+        </is>
+      </c>
+      <c r="R1052" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1052" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="T1052" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IKD update: GaN CMOS 2026-09-09T01:06Z
</commit_message>
<xml_diff>
--- a/01_literature/IKD_Literature_Master.xlsx
+++ b/01_literature/IKD_Literature_Master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1052"/>
+  <dimension ref="A1:T1058"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80026,6 +80026,446 @@
       </c>
       <c r="T1052" t="inlineStr"/>
     </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr"/>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>High Gain Low Elements Counts Switched Capacitor based Multi-Level Inverter</t>
+        </is>
+      </c>
+      <c r="C1053" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1053" t="inlineStr"/>
+      <c r="F1053" t="inlineStr">
+        <is>
+          <t>Kojabadi, Hossein Madadi; Hallaji, Erfan; Esfahlan, Amir Ghorbani; Panahgholi, Ataollah</t>
+        </is>
+      </c>
+      <c r="G1053" t="inlineStr"/>
+      <c r="H1053" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10537879/v1</t>
+        </is>
+      </c>
+      <c r="I1053" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10537879/v1</t>
+        </is>
+      </c>
+      <c r="J1053" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1053" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1053" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1053" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1053" t="inlineStr"/>
+      <c r="O1053" t="inlineStr"/>
+      <c r="P1053" t="inlineStr"/>
+      <c r="Q1053" t="inlineStr">
+        <is>
+          <t>High Gain Low Elements Counts Switched Capacitor based Multi-Level Inverter</t>
+        </is>
+      </c>
+      <c r="R1053" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1053" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="T1053" t="inlineStr"/>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr"/>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>High Gain Low Elements Counts Switched Capacitor based Multi-Level Inverter</t>
+        </is>
+      </c>
+      <c r="C1054" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1054" t="inlineStr"/>
+      <c r="F1054" t="inlineStr">
+        <is>
+          <t>Kojabadi, Hossein Madadi; Hallaji, Erfan; Esfahlan, Amir Ghorbani; Panahgholi, Ataollah</t>
+        </is>
+      </c>
+      <c r="G1054" t="inlineStr"/>
+      <c r="H1054" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10537879/v1</t>
+        </is>
+      </c>
+      <c r="I1054" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10537879/v1</t>
+        </is>
+      </c>
+      <c r="J1054" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1054" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1054" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1054" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1054" t="inlineStr"/>
+      <c r="O1054" t="inlineStr"/>
+      <c r="P1054" t="inlineStr"/>
+      <c r="Q1054" t="inlineStr">
+        <is>
+          <t>High Gain Low Elements Counts Switched Capacitor based Multi-Level Inverter</t>
+        </is>
+      </c>
+      <c r="R1054" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1054" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="T1054" t="inlineStr"/>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr"/>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>Calibration Robustness and Cross-Device Transferability of Four Temperature-Sensitive Electrical Parameters in Enhancement-Mode GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="C1055" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>MDPI AG</t>
+        </is>
+      </c>
+      <c r="E1055" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="F1055" t="inlineStr">
+        <is>
+          <t>Lee, Kwangsun; Lee, Hojoon</t>
+        </is>
+      </c>
+      <c r="G1055" t="inlineStr"/>
+      <c r="H1055" t="inlineStr">
+        <is>
+          <t>10.3390/electronics15184068</t>
+        </is>
+      </c>
+      <c r="I1055" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/electronics15184068</t>
+        </is>
+      </c>
+      <c r="J1055" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1055" t="inlineStr">
+        <is>
+          <t>n-FET</t>
+        </is>
+      </c>
+      <c r="L1055" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1055" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1055" t="inlineStr"/>
+      <c r="O1055" t="inlineStr"/>
+      <c r="P1055" t="inlineStr"/>
+      <c r="Q1055" t="inlineStr">
+        <is>
+          <t>Calibration Robustness and Cross-Device Transferability of Four Temperature-Sensitive Electrical Parameters in Enhancement-Mode GaN HEMTs</t>
+        </is>
+      </c>
+      <c r="R1055" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1055" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="T1055" t="inlineStr"/>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr"/>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>High Gain Low Elements Counts Switched Capacitor based Multi-Level Inverter</t>
+        </is>
+      </c>
+      <c r="C1056" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1056" t="inlineStr"/>
+      <c r="F1056" t="inlineStr">
+        <is>
+          <t>Kojabadi, Hossein Madadi; Hallaji, Erfan; Esfahlan, Amir Ghorbani; Panahgholi, Ataollah</t>
+        </is>
+      </c>
+      <c r="G1056" t="inlineStr"/>
+      <c r="H1056" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10537879/v1</t>
+        </is>
+      </c>
+      <c r="I1056" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10537879/v1</t>
+        </is>
+      </c>
+      <c r="J1056" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1056" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1056" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1056" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1056" t="inlineStr"/>
+      <c r="O1056" t="inlineStr"/>
+      <c r="P1056" t="inlineStr"/>
+      <c r="Q1056" t="inlineStr">
+        <is>
+          <t>High Gain Low Elements Counts Switched Capacitor based Multi-Level Inverter</t>
+        </is>
+      </c>
+      <c r="R1056" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1056" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="T1056" t="inlineStr"/>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr"/>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>A Novel Design of Energy Efficient CNTFET-Based Full Adder for VLSI Applications</t>
+        </is>
+      </c>
+      <c r="C1057" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>Bentham Science Publishers Ltd.</t>
+        </is>
+      </c>
+      <c r="E1057" t="inlineStr">
+        <is>
+          <t>Micro and Nanosystems</t>
+        </is>
+      </c>
+      <c r="F1057" t="inlineStr">
+        <is>
+          <t>Niharika, Lakkireddy; Machupalli, Madhusudhan Reddy; Rao, Tirumalasetty Venkata</t>
+        </is>
+      </c>
+      <c r="G1057" t="inlineStr"/>
+      <c r="H1057" t="inlineStr">
+        <is>
+          <t>10.2174/0118764029413710251122014017</t>
+        </is>
+      </c>
+      <c r="I1057" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2174/0118764029413710251122014017</t>
+        </is>
+      </c>
+      <c r="J1057" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1057" t="inlineStr">
+        <is>
+          <t>Co-integration</t>
+        </is>
+      </c>
+      <c r="L1057" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1057" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1057" t="inlineStr"/>
+      <c r="O1057" t="inlineStr"/>
+      <c r="P1057" t="inlineStr"/>
+      <c r="Q1057" t="inlineStr">
+        <is>
+          <t>A Novel Design of Energy Efficient CNTFET-Based Full Adder for VLSI Applications</t>
+        </is>
+      </c>
+      <c r="R1057" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1057" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="T1057" t="inlineStr"/>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr"/>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>High Gain Low Elements Counts Switched Capacitor based Multi-Level Inverter</t>
+        </is>
+      </c>
+      <c r="C1058" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>Springer Science and Business Media LLC</t>
+        </is>
+      </c>
+      <c r="E1058" t="inlineStr"/>
+      <c r="F1058" t="inlineStr">
+        <is>
+          <t>Kojabadi, Hossein Madadi; Hallaji, Erfan; Esfahlan, Amir Ghorbani; Panahgholi, Ataollah</t>
+        </is>
+      </c>
+      <c r="G1058" t="inlineStr"/>
+      <c r="H1058" t="inlineStr">
+        <is>
+          <t>10.21203/rs.3.rs-10537879/v1</t>
+        </is>
+      </c>
+      <c r="I1058" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-10537879/v1</t>
+        </is>
+      </c>
+      <c r="J1058" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="K1058" t="inlineStr">
+        <is>
+          <t>Inverter</t>
+        </is>
+      </c>
+      <c r="L1058" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="M1058" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="N1058" t="inlineStr"/>
+      <c r="O1058" t="inlineStr"/>
+      <c r="P1058" t="inlineStr"/>
+      <c r="Q1058" t="inlineStr">
+        <is>
+          <t>High Gain Low Elements Counts Switched Capacitor based Multi-Level Inverter</t>
+        </is>
+      </c>
+      <c r="R1058" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S1058" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="T1058" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>